<commit_message>
Split long advance warning literal without changing calculation
</commit_message>
<xml_diff>
--- a/tools/candidates/s1-oplata-za-raboty/04-uchet-raschetov-i-otpravok.xlsx
+++ b/tools/candidates/s1-oplata-za-raboty/04-uchet-raschetov-i-otpravok.xlsx
@@ -611,7 +611,7 @@
         <v/>
       </c>
       <c r="I5" s="6">
-        <f>IF(AND(B5="",C5="",D5="",E5="",F5=""),"",IF(OR(B5="",C5="",E5=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E5)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H5&lt;&gt;0,F5=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G5&lt;&gt;0,F5=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F5&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F5)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C5)*($E$5:$E$504=E5)*(($D$5:$D$504=D5)*(D5&lt;&gt;"")+($B$5:$B$504=B5)*(B5&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C5="Оплата",K5&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E5)&gt;0,ROUND(E5-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B5="",C5="",D5="",E5="",F5=""),"",IF(OR(B5="",C5="",E5=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E5)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H5&lt;&gt;0,F5=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G5&lt;&gt;0,F5=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F5&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F5)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C5)*($E$5:$E$504=E5)*(($D$5:$D$504=D5)*(D5&lt;&gt;"")+($B$5:$B$504=B5)*(B5&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C5="Оплата",K5&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E5)&gt;0,ROUND(E5-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J5" s="5">
@@ -647,7 +647,7 @@
         <v/>
       </c>
       <c r="I6" s="6">
-        <f>IF(AND(B6="",C6="",D6="",E6="",F6=""),"",IF(OR(B6="",C6="",E6=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E6)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H6&lt;&gt;0,F6=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G6&lt;&gt;0,F6=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F6&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F6)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C6)*($E$5:$E$504=E6)*(($D$5:$D$504=D6)*(D6&lt;&gt;"")+($B$5:$B$504=B6)*(B6&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C6="Оплата",K6&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E6)&gt;0,ROUND(E6-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B6="",C6="",D6="",E6="",F6=""),"",IF(OR(B6="",C6="",E6=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E6)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H6&lt;&gt;0,F6=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G6&lt;&gt;0,F6=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F6&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F6)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C6)*($E$5:$E$504=E6)*(($D$5:$D$504=D6)*(D6&lt;&gt;"")+($B$5:$B$504=B6)*(B6&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C6="Оплата",K6&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E6)&gt;0,ROUND(E6-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J6" s="5">
@@ -683,7 +683,7 @@
         <v/>
       </c>
       <c r="I7" s="6">
-        <f>IF(AND(B7="",C7="",D7="",E7="",F7=""),"",IF(OR(B7="",C7="",E7=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E7)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H7&lt;&gt;0,F7=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G7&lt;&gt;0,F7=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F7&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F7)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C7)*($E$5:$E$504=E7)*(($D$5:$D$504=D7)*(D7&lt;&gt;"")+($B$5:$B$504=B7)*(B7&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C7="Оплата",K7&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E7)&gt;0,ROUND(E7-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B7="",C7="",D7="",E7="",F7=""),"",IF(OR(B7="",C7="",E7=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E7)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H7&lt;&gt;0,F7=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G7&lt;&gt;0,F7=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F7&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F7)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C7)*($E$5:$E$504=E7)*(($D$5:$D$504=D7)*(D7&lt;&gt;"")+($B$5:$B$504=B7)*(B7&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C7="Оплата",K7&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E7)&gt;0,ROUND(E7-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J7" s="5">
@@ -719,7 +719,7 @@
         <v/>
       </c>
       <c r="I8" s="6">
-        <f>IF(AND(B8="",C8="",D8="",E8="",F8=""),"",IF(OR(B8="",C8="",E8=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E8)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H8&lt;&gt;0,F8=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G8&lt;&gt;0,F8=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F8&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F8)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C8)*($E$5:$E$504=E8)*(($D$5:$D$504=D8)*(D8&lt;&gt;"")+($B$5:$B$504=B8)*(B8&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C8="Оплата",K8&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E8)&gt;0,ROUND(E8-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B8="",C8="",D8="",E8="",F8=""),"",IF(OR(B8="",C8="",E8=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E8)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H8&lt;&gt;0,F8=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G8&lt;&gt;0,F8=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F8&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F8)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C8)*($E$5:$E$504=E8)*(($D$5:$D$504=D8)*(D8&lt;&gt;"")+($B$5:$B$504=B8)*(B8&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C8="Оплата",K8&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E8)&gt;0,ROUND(E8-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J8" s="5">
@@ -755,7 +755,7 @@
         <v/>
       </c>
       <c r="I9" s="6">
-        <f>IF(AND(B9="",C9="",D9="",E9="",F9=""),"",IF(OR(B9="",C9="",E9=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E9)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H9&lt;&gt;0,F9=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G9&lt;&gt;0,F9=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F9&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F9)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C9)*($E$5:$E$504=E9)*(($D$5:$D$504=D9)*(D9&lt;&gt;"")+($B$5:$B$504=B9)*(B9&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C9="Оплата",K9&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E9)&gt;0,ROUND(E9-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B9="",C9="",D9="",E9="",F9=""),"",IF(OR(B9="",C9="",E9=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E9)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H9&lt;&gt;0,F9=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G9&lt;&gt;0,F9=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F9&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F9)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C9)*($E$5:$E$504=E9)*(($D$5:$D$504=D9)*(D9&lt;&gt;"")+($B$5:$B$504=B9)*(B9&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C9="Оплата",K9&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E9)&gt;0,ROUND(E9-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J9" s="5">
@@ -791,7 +791,7 @@
         <v/>
       </c>
       <c r="I10" s="6">
-        <f>IF(AND(B10="",C10="",D10="",E10="",F10=""),"",IF(OR(B10="",C10="",E10=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E10)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H10&lt;&gt;0,F10=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G10&lt;&gt;0,F10=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F10&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F10)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C10)*($E$5:$E$504=E10)*(($D$5:$D$504=D10)*(D10&lt;&gt;"")+($B$5:$B$504=B10)*(B10&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C10="Оплата",K10&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E10)&gt;0,ROUND(E10-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B10="",C10="",D10="",E10="",F10=""),"",IF(OR(B10="",C10="",E10=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E10)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H10&lt;&gt;0,F10=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G10&lt;&gt;0,F10=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F10&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F10)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C10)*($E$5:$E$504=E10)*(($D$5:$D$504=D10)*(D10&lt;&gt;"")+($B$5:$B$504=B10)*(B10&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C10="Оплата",K10&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E10)&gt;0,ROUND(E10-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J10" s="5">
@@ -827,7 +827,7 @@
         <v/>
       </c>
       <c r="I11" s="6">
-        <f>IF(AND(B11="",C11="",D11="",E11="",F11=""),"",IF(OR(B11="",C11="",E11=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E11)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H11&lt;&gt;0,F11=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G11&lt;&gt;0,F11=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F11&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F11)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C11)*($E$5:$E$504=E11)*(($D$5:$D$504=D11)*(D11&lt;&gt;"")+($B$5:$B$504=B11)*(B11&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C11="Оплата",K11&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E11)&gt;0,ROUND(E11-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B11="",C11="",D11="",E11="",F11=""),"",IF(OR(B11="",C11="",E11=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E11)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H11&lt;&gt;0,F11=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G11&lt;&gt;0,F11=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F11&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F11)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C11)*($E$5:$E$504=E11)*(($D$5:$D$504=D11)*(D11&lt;&gt;"")+($B$5:$B$504=B11)*(B11&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C11="Оплата",K11&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E11)&gt;0,ROUND(E11-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J11" s="5">
@@ -863,7 +863,7 @@
         <v/>
       </c>
       <c r="I12" s="6">
-        <f>IF(AND(B12="",C12="",D12="",E12="",F12=""),"",IF(OR(B12="",C12="",E12=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E12)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H12&lt;&gt;0,F12=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G12&lt;&gt;0,F12=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F12&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F12)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C12)*($E$5:$E$504=E12)*(($D$5:$D$504=D12)*(D12&lt;&gt;"")+($B$5:$B$504=B12)*(B12&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C12="Оплата",K12&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E12)&gt;0,ROUND(E12-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B12="",C12="",D12="",E12="",F12=""),"",IF(OR(B12="",C12="",E12=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E12)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H12&lt;&gt;0,F12=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G12&lt;&gt;0,F12=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F12&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F12)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C12)*($E$5:$E$504=E12)*(($D$5:$D$504=D12)*(D12&lt;&gt;"")+($B$5:$B$504=B12)*(B12&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C12="Оплата",K12&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E12)&gt;0,ROUND(E12-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J12" s="5">
@@ -899,7 +899,7 @@
         <v/>
       </c>
       <c r="I13" s="6">
-        <f>IF(AND(B13="",C13="",D13="",E13="",F13=""),"",IF(OR(B13="",C13="",E13=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E13)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H13&lt;&gt;0,F13=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G13&lt;&gt;0,F13=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F13&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F13)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C13)*($E$5:$E$504=E13)*(($D$5:$D$504=D13)*(D13&lt;&gt;"")+($B$5:$B$504=B13)*(B13&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C13="Оплата",K13&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E13)&gt;0,ROUND(E13-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B13="",C13="",D13="",E13="",F13=""),"",IF(OR(B13="",C13="",E13=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E13)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H13&lt;&gt;0,F13=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G13&lt;&gt;0,F13=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F13&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F13)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C13)*($E$5:$E$504=E13)*(($D$5:$D$504=D13)*(D13&lt;&gt;"")+($B$5:$B$504=B13)*(B13&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C13="Оплата",K13&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E13)&gt;0,ROUND(E13-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J13" s="5">
@@ -935,7 +935,7 @@
         <v/>
       </c>
       <c r="I14" s="6">
-        <f>IF(AND(B14="",C14="",D14="",E14="",F14=""),"",IF(OR(B14="",C14="",E14=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E14)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H14&lt;&gt;0,F14=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G14&lt;&gt;0,F14=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F14&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F14)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C14)*($E$5:$E$504=E14)*(($D$5:$D$504=D14)*(D14&lt;&gt;"")+($B$5:$B$504=B14)*(B14&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C14="Оплата",K14&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E14)&gt;0,ROUND(E14-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B14="",C14="",D14="",E14="",F14=""),"",IF(OR(B14="",C14="",E14=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E14)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H14&lt;&gt;0,F14=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G14&lt;&gt;0,F14=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F14&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F14)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C14)*($E$5:$E$504=E14)*(($D$5:$D$504=D14)*(D14&lt;&gt;"")+($B$5:$B$504=B14)*(B14&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C14="Оплата",K14&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E14)&gt;0,ROUND(E14-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J14" s="5">
@@ -971,7 +971,7 @@
         <v/>
       </c>
       <c r="I15" s="6">
-        <f>IF(AND(B15="",C15="",D15="",E15="",F15=""),"",IF(OR(B15="",C15="",E15=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E15)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H15&lt;&gt;0,F15=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G15&lt;&gt;0,F15=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F15&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F15)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C15)*($E$5:$E$504=E15)*(($D$5:$D$504=D15)*(D15&lt;&gt;"")+($B$5:$B$504=B15)*(B15&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C15="Оплата",K15&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E15)&gt;0,ROUND(E15-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B15="",C15="",D15="",E15="",F15=""),"",IF(OR(B15="",C15="",E15=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E15)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H15&lt;&gt;0,F15=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G15&lt;&gt;0,F15=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F15&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F15)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C15)*($E$5:$E$504=E15)*(($D$5:$D$504=D15)*(D15&lt;&gt;"")+($B$5:$B$504=B15)*(B15&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C15="Оплата",K15&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E15)&gt;0,ROUND(E15-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J15" s="5">
@@ -1007,7 +1007,7 @@
         <v/>
       </c>
       <c r="I16" s="6">
-        <f>IF(AND(B16="",C16="",D16="",E16="",F16=""),"",IF(OR(B16="",C16="",E16=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E16)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H16&lt;&gt;0,F16=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G16&lt;&gt;0,F16=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F16&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F16)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C16)*($E$5:$E$504=E16)*(($D$5:$D$504=D16)*(D16&lt;&gt;"")+($B$5:$B$504=B16)*(B16&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C16="Оплата",K16&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E16)&gt;0,ROUND(E16-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B16="",C16="",D16="",E16="",F16=""),"",IF(OR(B16="",C16="",E16=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E16)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H16&lt;&gt;0,F16=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G16&lt;&gt;0,F16=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F16&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F16)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C16)*($E$5:$E$504=E16)*(($D$5:$D$504=D16)*(D16&lt;&gt;"")+($B$5:$B$504=B16)*(B16&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C16="Оплата",K16&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E16)&gt;0,ROUND(E16-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J16" s="5">
@@ -1034,7 +1034,7 @@
         <v/>
       </c>
       <c r="I17" s="6">
-        <f>IF(AND(B17="",C17="",D17="",E17="",F17=""),"",IF(OR(B17="",C17="",E17=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E17)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H17&lt;&gt;0,F17=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G17&lt;&gt;0,F17=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F17&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F17)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C17)*($E$5:$E$504=E17)*(($D$5:$D$504=D17)*(D17&lt;&gt;"")+($B$5:$B$504=B17)*(B17&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C17="Оплата",K17&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E17)&gt;0,ROUND(E17-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B17="",C17="",D17="",E17="",F17=""),"",IF(OR(B17="",C17="",E17=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E17)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H17&lt;&gt;0,F17=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G17&lt;&gt;0,F17=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F17&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F17)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C17)*($E$5:$E$504=E17)*(($D$5:$D$504=D17)*(D17&lt;&gt;"")+($B$5:$B$504=B17)*(B17&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C17="Оплата",K17&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E17)&gt;0,ROUND(E17-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J17" s="5">
@@ -1061,7 +1061,7 @@
         <v/>
       </c>
       <c r="I18" s="6">
-        <f>IF(AND(B18="",C18="",D18="",E18="",F18=""),"",IF(OR(B18="",C18="",E18=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E18)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H18&lt;&gt;0,F18=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G18&lt;&gt;0,F18=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F18&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F18)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C18)*($E$5:$E$504=E18)*(($D$5:$D$504=D18)*(D18&lt;&gt;"")+($B$5:$B$504=B18)*(B18&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C18="Оплата",K18&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E18)&gt;0,ROUND(E18-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B18="",C18="",D18="",E18="",F18=""),"",IF(OR(B18="",C18="",E18=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E18)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H18&lt;&gt;0,F18=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G18&lt;&gt;0,F18=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F18&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F18)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C18)*($E$5:$E$504=E18)*(($D$5:$D$504=D18)*(D18&lt;&gt;"")+($B$5:$B$504=B18)*(B18&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C18="Оплата",K18&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E18)&gt;0,ROUND(E18-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J18" s="5">
@@ -1093,7 +1093,7 @@
         <v/>
       </c>
       <c r="I19" s="6">
-        <f>IF(AND(B19="",C19="",D19="",E19="",F19=""),"",IF(OR(B19="",C19="",E19=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E19)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H19&lt;&gt;0,F19=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G19&lt;&gt;0,F19=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F19&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F19)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C19)*($E$5:$E$504=E19)*(($D$5:$D$504=D19)*(D19&lt;&gt;"")+($B$5:$B$504=B19)*(B19&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C19="Оплата",K19&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E19)&gt;0,ROUND(E19-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B19="",C19="",D19="",E19="",F19=""),"",IF(OR(B19="",C19="",E19=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E19)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H19&lt;&gt;0,F19=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G19&lt;&gt;0,F19=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F19&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F19)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C19)*($E$5:$E$504=E19)*(($D$5:$D$504=D19)*(D19&lt;&gt;"")+($B$5:$B$504=B19)*(B19&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C19="Оплата",K19&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E19)&gt;0,ROUND(E19-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J19" s="5">
@@ -1120,7 +1120,7 @@
         <v/>
       </c>
       <c r="I20" s="6">
-        <f>IF(AND(B20="",C20="",D20="",E20="",F20=""),"",IF(OR(B20="",C20="",E20=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E20)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H20&lt;&gt;0,F20=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G20&lt;&gt;0,F20=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F20&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F20)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C20)*($E$5:$E$504=E20)*(($D$5:$D$504=D20)*(D20&lt;&gt;"")+($B$5:$B$504=B20)*(B20&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C20="Оплата",K20&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E20)&gt;0,ROUND(E20-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B20="",C20="",D20="",E20="",F20=""),"",IF(OR(B20="",C20="",E20=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E20)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H20&lt;&gt;0,F20=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G20&lt;&gt;0,F20=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F20&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F20)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C20)*($E$5:$E$504=E20)*(($D$5:$D$504=D20)*(D20&lt;&gt;"")+($B$5:$B$504=B20)*(B20&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C20="Оплата",K20&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E20)&gt;0,ROUND(E20-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J20" s="5">
@@ -1147,7 +1147,7 @@
         <v/>
       </c>
       <c r="I21" s="6">
-        <f>IF(AND(B21="",C21="",D21="",E21="",F21=""),"",IF(OR(B21="",C21="",E21=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E21)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H21&lt;&gt;0,F21=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G21&lt;&gt;0,F21=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F21&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F21)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C21)*($E$5:$E$504=E21)*(($D$5:$D$504=D21)*(D21&lt;&gt;"")+($B$5:$B$504=B21)*(B21&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C21="Оплата",K21&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E21)&gt;0,ROUND(E21-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B21="",C21="",D21="",E21="",F21=""),"",IF(OR(B21="",C21="",E21=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E21)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H21&lt;&gt;0,F21=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G21&lt;&gt;0,F21=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F21&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F21)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C21)*($E$5:$E$504=E21)*(($D$5:$D$504=D21)*(D21&lt;&gt;"")+($B$5:$B$504=B21)*(B21&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C21="Оплата",K21&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E21)&gt;0,ROUND(E21-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J21" s="5">
@@ -1174,7 +1174,7 @@
         <v/>
       </c>
       <c r="I22" s="6">
-        <f>IF(AND(B22="",C22="",D22="",E22="",F22=""),"",IF(OR(B22="",C22="",E22=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E22)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H22&lt;&gt;0,F22=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G22&lt;&gt;0,F22=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F22&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F22)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C22)*($E$5:$E$504=E22)*(($D$5:$D$504=D22)*(D22&lt;&gt;"")+($B$5:$B$504=B22)*(B22&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C22="Оплата",K22&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E22)&gt;0,ROUND(E22-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B22="",C22="",D22="",E22="",F22=""),"",IF(OR(B22="",C22="",E22=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E22)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H22&lt;&gt;0,F22=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G22&lt;&gt;0,F22=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F22&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F22)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C22)*($E$5:$E$504=E22)*(($D$5:$D$504=D22)*(D22&lt;&gt;"")+($B$5:$B$504=B22)*(B22&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C22="Оплата",K22&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E22)&gt;0,ROUND(E22-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J22" s="5">
@@ -1201,7 +1201,7 @@
         <v/>
       </c>
       <c r="I23" s="6">
-        <f>IF(AND(B23="",C23="",D23="",E23="",F23=""),"",IF(OR(B23="",C23="",E23=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E23)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H23&lt;&gt;0,F23=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G23&lt;&gt;0,F23=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F23&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F23)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C23)*($E$5:$E$504=E23)*(($D$5:$D$504=D23)*(D23&lt;&gt;"")+($B$5:$B$504=B23)*(B23&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C23="Оплата",K23&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E23)&gt;0,ROUND(E23-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B23="",C23="",D23="",E23="",F23=""),"",IF(OR(B23="",C23="",E23=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E23)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H23&lt;&gt;0,F23=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G23&lt;&gt;0,F23=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F23&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F23)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C23)*($E$5:$E$504=E23)*(($D$5:$D$504=D23)*(D23&lt;&gt;"")+($B$5:$B$504=B23)*(B23&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C23="Оплата",K23&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E23)&gt;0,ROUND(E23-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J23" s="5">
@@ -1228,7 +1228,7 @@
         <v/>
       </c>
       <c r="I24" s="6">
-        <f>IF(AND(B24="",C24="",D24="",E24="",F24=""),"",IF(OR(B24="",C24="",E24=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E24)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H24&lt;&gt;0,F24=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G24&lt;&gt;0,F24=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F24&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F24)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C24)*($E$5:$E$504=E24)*(($D$5:$D$504=D24)*(D24&lt;&gt;"")+($B$5:$B$504=B24)*(B24&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C24="Оплата",K24&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E24)&gt;0,ROUND(E24-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B24="",C24="",D24="",E24="",F24=""),"",IF(OR(B24="",C24="",E24=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E24)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H24&lt;&gt;0,F24=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G24&lt;&gt;0,F24=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F24&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F24)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C24)*($E$5:$E$504=E24)*(($D$5:$D$504=D24)*(D24&lt;&gt;"")+($B$5:$B$504=B24)*(B24&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C24="Оплата",K24&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E24)&gt;0,ROUND(E24-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J24" s="5">
@@ -1255,7 +1255,7 @@
         <v/>
       </c>
       <c r="I25" s="6">
-        <f>IF(AND(B25="",C25="",D25="",E25="",F25=""),"",IF(OR(B25="",C25="",E25=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E25)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H25&lt;&gt;0,F25=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G25&lt;&gt;0,F25=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F25&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F25)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C25)*($E$5:$E$504=E25)*(($D$5:$D$504=D25)*(D25&lt;&gt;"")+($B$5:$B$504=B25)*(B25&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C25="Оплата",K25&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E25)&gt;0,ROUND(E25-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B25="",C25="",D25="",E25="",F25=""),"",IF(OR(B25="",C25="",E25=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E25)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H25&lt;&gt;0,F25=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G25&lt;&gt;0,F25=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F25&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F25)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C25)*($E$5:$E$504=E25)*(($D$5:$D$504=D25)*(D25&lt;&gt;"")+($B$5:$B$504=B25)*(B25&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C25="Оплата",K25&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E25)&gt;0,ROUND(E25-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J25" s="5">
@@ -1282,7 +1282,7 @@
         <v/>
       </c>
       <c r="I26" s="6">
-        <f>IF(AND(B26="",C26="",D26="",E26="",F26=""),"",IF(OR(B26="",C26="",E26=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E26)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H26&lt;&gt;0,F26=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G26&lt;&gt;0,F26=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F26&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F26)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C26)*($E$5:$E$504=E26)*(($D$5:$D$504=D26)*(D26&lt;&gt;"")+($B$5:$B$504=B26)*(B26&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C26="Оплата",K26&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E26)&gt;0,ROUND(E26-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B26="",C26="",D26="",E26="",F26=""),"",IF(OR(B26="",C26="",E26=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E26)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H26&lt;&gt;0,F26=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G26&lt;&gt;0,F26=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F26&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F26)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C26)*($E$5:$E$504=E26)*(($D$5:$D$504=D26)*(D26&lt;&gt;"")+($B$5:$B$504=B26)*(B26&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C26="Оплата",K26&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E26)&gt;0,ROUND(E26-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J26" s="5">
@@ -1309,7 +1309,7 @@
         <v/>
       </c>
       <c r="I27" s="6">
-        <f>IF(AND(B27="",C27="",D27="",E27="",F27=""),"",IF(OR(B27="",C27="",E27=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E27)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H27&lt;&gt;0,F27=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G27&lt;&gt;0,F27=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F27&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F27)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C27)*($E$5:$E$504=E27)*(($D$5:$D$504=D27)*(D27&lt;&gt;"")+($B$5:$B$504=B27)*(B27&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C27="Оплата",K27&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E27)&gt;0,ROUND(E27-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B27="",C27="",D27="",E27="",F27=""),"",IF(OR(B27="",C27="",E27=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E27)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H27&lt;&gt;0,F27=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G27&lt;&gt;0,F27=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F27&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F27)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C27)*($E$5:$E$504=E27)*(($D$5:$D$504=D27)*(D27&lt;&gt;"")+($B$5:$B$504=B27)*(B27&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C27="Оплата",K27&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E27)&gt;0,ROUND(E27-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J27" s="5">
@@ -1336,7 +1336,7 @@
         <v/>
       </c>
       <c r="I28" s="6">
-        <f>IF(AND(B28="",C28="",D28="",E28="",F28=""),"",IF(OR(B28="",C28="",E28=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E28)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H28&lt;&gt;0,F28=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G28&lt;&gt;0,F28=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F28&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F28)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C28)*($E$5:$E$504=E28)*(($D$5:$D$504=D28)*(D28&lt;&gt;"")+($B$5:$B$504=B28)*(B28&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C28="Оплата",K28&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E28)&gt;0,ROUND(E28-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B28="",C28="",D28="",E28="",F28=""),"",IF(OR(B28="",C28="",E28=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E28)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H28&lt;&gt;0,F28=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G28&lt;&gt;0,F28=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F28&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F28)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C28)*($E$5:$E$504=E28)*(($D$5:$D$504=D28)*(D28&lt;&gt;"")+($B$5:$B$504=B28)*(B28&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C28="Оплата",K28&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E28)&gt;0,ROUND(E28-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J28" s="5">
@@ -1363,7 +1363,7 @@
         <v/>
       </c>
       <c r="I29" s="6">
-        <f>IF(AND(B29="",C29="",D29="",E29="",F29=""),"",IF(OR(B29="",C29="",E29=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E29)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H29&lt;&gt;0,F29=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G29&lt;&gt;0,F29=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F29&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F29)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C29)*($E$5:$E$504=E29)*(($D$5:$D$504=D29)*(D29&lt;&gt;"")+($B$5:$B$504=B29)*(B29&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C29="Оплата",K29&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E29)&gt;0,ROUND(E29-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B29="",C29="",D29="",E29="",F29=""),"",IF(OR(B29="",C29="",E29=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E29)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H29&lt;&gt;0,F29=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G29&lt;&gt;0,F29=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F29&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F29)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C29)*($E$5:$E$504=E29)*(($D$5:$D$504=D29)*(D29&lt;&gt;"")+($B$5:$B$504=B29)*(B29&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C29="Оплата",K29&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E29)&gt;0,ROUND(E29-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J29" s="5">
@@ -1390,7 +1390,7 @@
         <v/>
       </c>
       <c r="I30" s="6">
-        <f>IF(AND(B30="",C30="",D30="",E30="",F30=""),"",IF(OR(B30="",C30="",E30=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E30)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H30&lt;&gt;0,F30=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G30&lt;&gt;0,F30=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F30&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F30)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C30)*($E$5:$E$504=E30)*(($D$5:$D$504=D30)*(D30&lt;&gt;"")+($B$5:$B$504=B30)*(B30&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C30="Оплата",K30&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E30)&gt;0,ROUND(E30-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B30="",C30="",D30="",E30="",F30=""),"",IF(OR(B30="",C30="",E30=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E30)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H30&lt;&gt;0,F30=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G30&lt;&gt;0,F30=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F30&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F30)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C30)*($E$5:$E$504=E30)*(($D$5:$D$504=D30)*(D30&lt;&gt;"")+($B$5:$B$504=B30)*(B30&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C30="Оплата",K30&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E30)&gt;0,ROUND(E30-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J30" s="5">
@@ -1417,7 +1417,7 @@
         <v/>
       </c>
       <c r="I31" s="6">
-        <f>IF(AND(B31="",C31="",D31="",E31="",F31=""),"",IF(OR(B31="",C31="",E31=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E31)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H31&lt;&gt;0,F31=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G31&lt;&gt;0,F31=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F31&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F31)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C31)*($E$5:$E$504=E31)*(($D$5:$D$504=D31)*(D31&lt;&gt;"")+($B$5:$B$504=B31)*(B31&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C31="Оплата",K31&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E31)&gt;0,ROUND(E31-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B31="",C31="",D31="",E31="",F31=""),"",IF(OR(B31="",C31="",E31=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E31)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H31&lt;&gt;0,F31=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G31&lt;&gt;0,F31=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F31&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F31)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C31)*($E$5:$E$504=E31)*(($D$5:$D$504=D31)*(D31&lt;&gt;"")+($B$5:$B$504=B31)*(B31&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C31="Оплата",K31&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E31)&gt;0,ROUND(E31-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J31" s="5">
@@ -1444,7 +1444,7 @@
         <v/>
       </c>
       <c r="I32" s="6">
-        <f>IF(AND(B32="",C32="",D32="",E32="",F32=""),"",IF(OR(B32="",C32="",E32=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E32)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H32&lt;&gt;0,F32=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G32&lt;&gt;0,F32=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F32&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F32)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C32)*($E$5:$E$504=E32)*(($D$5:$D$504=D32)*(D32&lt;&gt;"")+($B$5:$B$504=B32)*(B32&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C32="Оплата",K32&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E32)&gt;0,ROUND(E32-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B32="",C32="",D32="",E32="",F32=""),"",IF(OR(B32="",C32="",E32=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E32)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H32&lt;&gt;0,F32=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G32&lt;&gt;0,F32=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F32&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F32)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C32)*($E$5:$E$504=E32)*(($D$5:$D$504=D32)*(D32&lt;&gt;"")+($B$5:$B$504=B32)*(B32&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C32="Оплата",K32&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E32)&gt;0,ROUND(E32-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J32" s="5">
@@ -1471,7 +1471,7 @@
         <v/>
       </c>
       <c r="I33" s="6">
-        <f>IF(AND(B33="",C33="",D33="",E33="",F33=""),"",IF(OR(B33="",C33="",E33=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E33)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H33&lt;&gt;0,F33=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G33&lt;&gt;0,F33=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F33&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F33)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C33)*($E$5:$E$504=E33)*(($D$5:$D$504=D33)*(D33&lt;&gt;"")+($B$5:$B$504=B33)*(B33&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C33="Оплата",K33&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E33)&gt;0,ROUND(E33-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B33="",C33="",D33="",E33="",F33=""),"",IF(OR(B33="",C33="",E33=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E33)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H33&lt;&gt;0,F33=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G33&lt;&gt;0,F33=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F33&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F33)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C33)*($E$5:$E$504=E33)*(($D$5:$D$504=D33)*(D33&lt;&gt;"")+($B$5:$B$504=B33)*(B33&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C33="Оплата",K33&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E33)&gt;0,ROUND(E33-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J33" s="5">
@@ -1498,7 +1498,7 @@
         <v/>
       </c>
       <c r="I34" s="6">
-        <f>IF(AND(B34="",C34="",D34="",E34="",F34=""),"",IF(OR(B34="",C34="",E34=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E34)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H34&lt;&gt;0,F34=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G34&lt;&gt;0,F34=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F34&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F34)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C34)*($E$5:$E$504=E34)*(($D$5:$D$504=D34)*(D34&lt;&gt;"")+($B$5:$B$504=B34)*(B34&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C34="Оплата",K34&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E34)&gt;0,ROUND(E34-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B34="",C34="",D34="",E34="",F34=""),"",IF(OR(B34="",C34="",E34=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E34)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H34&lt;&gt;0,F34=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G34&lt;&gt;0,F34=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F34&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F34)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C34)*($E$5:$E$504=E34)*(($D$5:$D$504=D34)*(D34&lt;&gt;"")+($B$5:$B$504=B34)*(B34&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C34="Оплата",K34&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E34)&gt;0,ROUND(E34-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J34" s="5">
@@ -1525,7 +1525,7 @@
         <v/>
       </c>
       <c r="I35" s="6">
-        <f>IF(AND(B35="",C35="",D35="",E35="",F35=""),"",IF(OR(B35="",C35="",E35=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E35)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H35&lt;&gt;0,F35=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G35&lt;&gt;0,F35=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F35&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F35)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C35)*($E$5:$E$504=E35)*(($D$5:$D$504=D35)*(D35&lt;&gt;"")+($B$5:$B$504=B35)*(B35&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C35="Оплата",K35&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E35)&gt;0,ROUND(E35-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B35="",C35="",D35="",E35="",F35=""),"",IF(OR(B35="",C35="",E35=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E35)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H35&lt;&gt;0,F35=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G35&lt;&gt;0,F35=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F35&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F35)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C35)*($E$5:$E$504=E35)*(($D$5:$D$504=D35)*(D35&lt;&gt;"")+($B$5:$B$504=B35)*(B35&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C35="Оплата",K35&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E35)&gt;0,ROUND(E35-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J35" s="5">
@@ -1552,7 +1552,7 @@
         <v/>
       </c>
       <c r="I36" s="6">
-        <f>IF(AND(B36="",C36="",D36="",E36="",F36=""),"",IF(OR(B36="",C36="",E36=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E36)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H36&lt;&gt;0,F36=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G36&lt;&gt;0,F36=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F36&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F36)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C36)*($E$5:$E$504=E36)*(($D$5:$D$504=D36)*(D36&lt;&gt;"")+($B$5:$B$504=B36)*(B36&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C36="Оплата",K36&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E36)&gt;0,ROUND(E36-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B36="",C36="",D36="",E36="",F36=""),"",IF(OR(B36="",C36="",E36=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E36)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H36&lt;&gt;0,F36=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G36&lt;&gt;0,F36=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F36&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F36)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C36)*($E$5:$E$504=E36)*(($D$5:$D$504=D36)*(D36&lt;&gt;"")+($B$5:$B$504=B36)*(B36&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C36="Оплата",K36&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E36)&gt;0,ROUND(E36-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J36" s="5">
@@ -1579,7 +1579,7 @@
         <v/>
       </c>
       <c r="I37" s="6">
-        <f>IF(AND(B37="",C37="",D37="",E37="",F37=""),"",IF(OR(B37="",C37="",E37=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E37)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H37&lt;&gt;0,F37=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G37&lt;&gt;0,F37=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F37&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F37)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C37)*($E$5:$E$504=E37)*(($D$5:$D$504=D37)*(D37&lt;&gt;"")+($B$5:$B$504=B37)*(B37&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C37="Оплата",K37&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E37)&gt;0,ROUND(E37-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B37="",C37="",D37="",E37="",F37=""),"",IF(OR(B37="",C37="",E37=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E37)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H37&lt;&gt;0,F37=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G37&lt;&gt;0,F37=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F37&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F37)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C37)*($E$5:$E$504=E37)*(($D$5:$D$504=D37)*(D37&lt;&gt;"")+($B$5:$B$504=B37)*(B37&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C37="Оплата",K37&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E37)&gt;0,ROUND(E37-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J37" s="5">
@@ -1606,7 +1606,7 @@
         <v/>
       </c>
       <c r="I38" s="6">
-        <f>IF(AND(B38="",C38="",D38="",E38="",F38=""),"",IF(OR(B38="",C38="",E38=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E38)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H38&lt;&gt;0,F38=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G38&lt;&gt;0,F38=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F38&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F38)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C38)*($E$5:$E$504=E38)*(($D$5:$D$504=D38)*(D38&lt;&gt;"")+($B$5:$B$504=B38)*(B38&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C38="Оплата",K38&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E38)&gt;0,ROUND(E38-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B38="",C38="",D38="",E38="",F38=""),"",IF(OR(B38="",C38="",E38=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E38)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H38&lt;&gt;0,F38=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G38&lt;&gt;0,F38=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F38&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F38)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C38)*($E$5:$E$504=E38)*(($D$5:$D$504=D38)*(D38&lt;&gt;"")+($B$5:$B$504=B38)*(B38&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C38="Оплата",K38&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E38)&gt;0,ROUND(E38-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J38" s="5">
@@ -1633,7 +1633,7 @@
         <v/>
       </c>
       <c r="I39" s="6">
-        <f>IF(AND(B39="",C39="",D39="",E39="",F39=""),"",IF(OR(B39="",C39="",E39=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E39)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H39&lt;&gt;0,F39=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G39&lt;&gt;0,F39=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F39&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F39)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C39)*($E$5:$E$504=E39)*(($D$5:$D$504=D39)*(D39&lt;&gt;"")+($B$5:$B$504=B39)*(B39&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C39="Оплата",K39&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E39)&gt;0,ROUND(E39-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B39="",C39="",D39="",E39="",F39=""),"",IF(OR(B39="",C39="",E39=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E39)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H39&lt;&gt;0,F39=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G39&lt;&gt;0,F39=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F39&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F39)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C39)*($E$5:$E$504=E39)*(($D$5:$D$504=D39)*(D39&lt;&gt;"")+($B$5:$B$504=B39)*(B39&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C39="Оплата",K39&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E39)&gt;0,ROUND(E39-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J39" s="5">
@@ -1660,7 +1660,7 @@
         <v/>
       </c>
       <c r="I40" s="6">
-        <f>IF(AND(B40="",C40="",D40="",E40="",F40=""),"",IF(OR(B40="",C40="",E40=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E40)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H40&lt;&gt;0,F40=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G40&lt;&gt;0,F40=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F40&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F40)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C40)*($E$5:$E$504=E40)*(($D$5:$D$504=D40)*(D40&lt;&gt;"")+($B$5:$B$504=B40)*(B40&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C40="Оплата",K40&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E40)&gt;0,ROUND(E40-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B40="",C40="",D40="",E40="",F40=""),"",IF(OR(B40="",C40="",E40=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E40)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H40&lt;&gt;0,F40=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G40&lt;&gt;0,F40=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F40&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F40)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C40)*($E$5:$E$504=E40)*(($D$5:$D$504=D40)*(D40&lt;&gt;"")+($B$5:$B$504=B40)*(B40&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C40="Оплата",K40&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E40)&gt;0,ROUND(E40-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J40" s="5">
@@ -1687,7 +1687,7 @@
         <v/>
       </c>
       <c r="I41" s="6">
-        <f>IF(AND(B41="",C41="",D41="",E41="",F41=""),"",IF(OR(B41="",C41="",E41=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E41)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H41&lt;&gt;0,F41=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G41&lt;&gt;0,F41=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F41&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F41)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C41)*($E$5:$E$504=E41)*(($D$5:$D$504=D41)*(D41&lt;&gt;"")+($B$5:$B$504=B41)*(B41&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C41="Оплата",K41&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E41)&gt;0,ROUND(E41-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B41="",C41="",D41="",E41="",F41=""),"",IF(OR(B41="",C41="",E41=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E41)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H41&lt;&gt;0,F41=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G41&lt;&gt;0,F41=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F41&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F41)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C41)*($E$5:$E$504=E41)*(($D$5:$D$504=D41)*(D41&lt;&gt;"")+($B$5:$B$504=B41)*(B41&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C41="Оплата",K41&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E41)&gt;0,ROUND(E41-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J41" s="5">
@@ -1714,7 +1714,7 @@
         <v/>
       </c>
       <c r="I42" s="6">
-        <f>IF(AND(B42="",C42="",D42="",E42="",F42=""),"",IF(OR(B42="",C42="",E42=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E42)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H42&lt;&gt;0,F42=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G42&lt;&gt;0,F42=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F42&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F42)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C42)*($E$5:$E$504=E42)*(($D$5:$D$504=D42)*(D42&lt;&gt;"")+($B$5:$B$504=B42)*(B42&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C42="Оплата",K42&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E42)&gt;0,ROUND(E42-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B42="",C42="",D42="",E42="",F42=""),"",IF(OR(B42="",C42="",E42=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E42)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H42&lt;&gt;0,F42=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G42&lt;&gt;0,F42=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F42&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F42)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C42)*($E$5:$E$504=E42)*(($D$5:$D$504=D42)*(D42&lt;&gt;"")+($B$5:$B$504=B42)*(B42&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C42="Оплата",K42&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E42)&gt;0,ROUND(E42-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J42" s="5">
@@ -1741,7 +1741,7 @@
         <v/>
       </c>
       <c r="I43" s="6">
-        <f>IF(AND(B43="",C43="",D43="",E43="",F43=""),"",IF(OR(B43="",C43="",E43=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E43)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H43&lt;&gt;0,F43=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G43&lt;&gt;0,F43=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F43&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F43)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C43)*($E$5:$E$504=E43)*(($D$5:$D$504=D43)*(D43&lt;&gt;"")+($B$5:$B$504=B43)*(B43&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C43="Оплата",K43&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E43)&gt;0,ROUND(E43-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B43="",C43="",D43="",E43="",F43=""),"",IF(OR(B43="",C43="",E43=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E43)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H43&lt;&gt;0,F43=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G43&lt;&gt;0,F43=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F43&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F43)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C43)*($E$5:$E$504=E43)*(($D$5:$D$504=D43)*(D43&lt;&gt;"")+($B$5:$B$504=B43)*(B43&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C43="Оплата",K43&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E43)&gt;0,ROUND(E43-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J43" s="5">
@@ -1768,7 +1768,7 @@
         <v/>
       </c>
       <c r="I44" s="6">
-        <f>IF(AND(B44="",C44="",D44="",E44="",F44=""),"",IF(OR(B44="",C44="",E44=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E44)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H44&lt;&gt;0,F44=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G44&lt;&gt;0,F44=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F44&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F44)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C44)*($E$5:$E$504=E44)*(($D$5:$D$504=D44)*(D44&lt;&gt;"")+($B$5:$B$504=B44)*(B44&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C44="Оплата",K44&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E44)&gt;0,ROUND(E44-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B44="",C44="",D44="",E44="",F44=""),"",IF(OR(B44="",C44="",E44=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E44)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H44&lt;&gt;0,F44=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G44&lt;&gt;0,F44=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F44&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F44)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C44)*($E$5:$E$504=E44)*(($D$5:$D$504=D44)*(D44&lt;&gt;"")+($B$5:$B$504=B44)*(B44&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C44="Оплата",K44&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E44)&gt;0,ROUND(E44-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J44" s="5">
@@ -1795,7 +1795,7 @@
         <v/>
       </c>
       <c r="I45" s="6">
-        <f>IF(AND(B45="",C45="",D45="",E45="",F45=""),"",IF(OR(B45="",C45="",E45=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E45)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H45&lt;&gt;0,F45=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G45&lt;&gt;0,F45=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F45&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F45)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C45)*($E$5:$E$504=E45)*(($D$5:$D$504=D45)*(D45&lt;&gt;"")+($B$5:$B$504=B45)*(B45&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C45="Оплата",K45&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E45)&gt;0,ROUND(E45-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B45="",C45="",D45="",E45="",F45=""),"",IF(OR(B45="",C45="",E45=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E45)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H45&lt;&gt;0,F45=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G45&lt;&gt;0,F45=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F45&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F45)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C45)*($E$5:$E$504=E45)*(($D$5:$D$504=D45)*(D45&lt;&gt;"")+($B$5:$B$504=B45)*(B45&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C45="Оплата",K45&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E45)&gt;0,ROUND(E45-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J45" s="5">
@@ -1822,7 +1822,7 @@
         <v/>
       </c>
       <c r="I46" s="6">
-        <f>IF(AND(B46="",C46="",D46="",E46="",F46=""),"",IF(OR(B46="",C46="",E46=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E46)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H46&lt;&gt;0,F46=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G46&lt;&gt;0,F46=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F46&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F46)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C46)*($E$5:$E$504=E46)*(($D$5:$D$504=D46)*(D46&lt;&gt;"")+($B$5:$B$504=B46)*(B46&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C46="Оплата",K46&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E46)&gt;0,ROUND(E46-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B46="",C46="",D46="",E46="",F46=""),"",IF(OR(B46="",C46="",E46=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E46)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H46&lt;&gt;0,F46=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G46&lt;&gt;0,F46=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F46&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F46)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C46)*($E$5:$E$504=E46)*(($D$5:$D$504=D46)*(D46&lt;&gt;"")+($B$5:$B$504=B46)*(B46&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C46="Оплата",K46&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E46)&gt;0,ROUND(E46-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J46" s="5">
@@ -1849,7 +1849,7 @@
         <v/>
       </c>
       <c r="I47" s="6">
-        <f>IF(AND(B47="",C47="",D47="",E47="",F47=""),"",IF(OR(B47="",C47="",E47=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E47)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H47&lt;&gt;0,F47=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G47&lt;&gt;0,F47=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F47&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F47)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C47)*($E$5:$E$504=E47)*(($D$5:$D$504=D47)*(D47&lt;&gt;"")+($B$5:$B$504=B47)*(B47&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C47="Оплата",K47&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E47)&gt;0,ROUND(E47-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B47="",C47="",D47="",E47="",F47=""),"",IF(OR(B47="",C47="",E47=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E47)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H47&lt;&gt;0,F47=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G47&lt;&gt;0,F47=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F47&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F47)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C47)*($E$5:$E$504=E47)*(($D$5:$D$504=D47)*(D47&lt;&gt;"")+($B$5:$B$504=B47)*(B47&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C47="Оплата",K47&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E47)&gt;0,ROUND(E47-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J47" s="5">
@@ -1876,7 +1876,7 @@
         <v/>
       </c>
       <c r="I48" s="6">
-        <f>IF(AND(B48="",C48="",D48="",E48="",F48=""),"",IF(OR(B48="",C48="",E48=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E48)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H48&lt;&gt;0,F48=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G48&lt;&gt;0,F48=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F48&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F48)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C48)*($E$5:$E$504=E48)*(($D$5:$D$504=D48)*(D48&lt;&gt;"")+($B$5:$B$504=B48)*(B48&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C48="Оплата",K48&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E48)&gt;0,ROUND(E48-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B48="",C48="",D48="",E48="",F48=""),"",IF(OR(B48="",C48="",E48=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E48)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H48&lt;&gt;0,F48=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G48&lt;&gt;0,F48=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F48&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F48)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C48)*($E$5:$E$504=E48)*(($D$5:$D$504=D48)*(D48&lt;&gt;"")+($B$5:$B$504=B48)*(B48&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C48="Оплата",K48&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E48)&gt;0,ROUND(E48-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J48" s="5">
@@ -1903,7 +1903,7 @@
         <v/>
       </c>
       <c r="I49" s="6">
-        <f>IF(AND(B49="",C49="",D49="",E49="",F49=""),"",IF(OR(B49="",C49="",E49=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E49)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H49&lt;&gt;0,F49=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G49&lt;&gt;0,F49=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F49&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F49)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C49)*($E$5:$E$504=E49)*(($D$5:$D$504=D49)*(D49&lt;&gt;"")+($B$5:$B$504=B49)*(B49&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C49="Оплата",K49&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E49)&gt;0,ROUND(E49-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B49="",C49="",D49="",E49="",F49=""),"",IF(OR(B49="",C49="",E49=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E49)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H49&lt;&gt;0,F49=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G49&lt;&gt;0,F49=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F49&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F49)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C49)*($E$5:$E$504=E49)*(($D$5:$D$504=D49)*(D49&lt;&gt;"")+($B$5:$B$504=B49)*(B49&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C49="Оплата",K49&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E49)&gt;0,ROUND(E49-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J49" s="5">
@@ -1930,7 +1930,7 @@
         <v/>
       </c>
       <c r="I50" s="6">
-        <f>IF(AND(B50="",C50="",D50="",E50="",F50=""),"",IF(OR(B50="",C50="",E50=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E50)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H50&lt;&gt;0,F50=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G50&lt;&gt;0,F50=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F50&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F50)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C50)*($E$5:$E$504=E50)*(($D$5:$D$504=D50)*(D50&lt;&gt;"")+($B$5:$B$504=B50)*(B50&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C50="Оплата",K50&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E50)&gt;0,ROUND(E50-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B50="",C50="",D50="",E50="",F50=""),"",IF(OR(B50="",C50="",E50=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E50)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H50&lt;&gt;0,F50=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G50&lt;&gt;0,F50=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F50&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F50)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C50)*($E$5:$E$504=E50)*(($D$5:$D$504=D50)*(D50&lt;&gt;"")+($B$5:$B$504=B50)*(B50&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C50="Оплата",K50&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E50)&gt;0,ROUND(E50-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J50" s="5">
@@ -1957,7 +1957,7 @@
         <v/>
       </c>
       <c r="I51" s="6">
-        <f>IF(AND(B51="",C51="",D51="",E51="",F51=""),"",IF(OR(B51="",C51="",E51=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E51)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H51&lt;&gt;0,F51=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G51&lt;&gt;0,F51=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F51&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F51)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C51)*($E$5:$E$504=E51)*(($D$5:$D$504=D51)*(D51&lt;&gt;"")+($B$5:$B$504=B51)*(B51&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C51="Оплата",K51&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E51)&gt;0,ROUND(E51-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B51="",C51="",D51="",E51="",F51=""),"",IF(OR(B51="",C51="",E51=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E51)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H51&lt;&gt;0,F51=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G51&lt;&gt;0,F51=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F51&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F51)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C51)*($E$5:$E$504=E51)*(($D$5:$D$504=D51)*(D51&lt;&gt;"")+($B$5:$B$504=B51)*(B51&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C51="Оплата",K51&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E51)&gt;0,ROUND(E51-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J51" s="5">
@@ -1984,7 +1984,7 @@
         <v/>
       </c>
       <c r="I52" s="6">
-        <f>IF(AND(B52="",C52="",D52="",E52="",F52=""),"",IF(OR(B52="",C52="",E52=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E52)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H52&lt;&gt;0,F52=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G52&lt;&gt;0,F52=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F52&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F52)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C52)*($E$5:$E$504=E52)*(($D$5:$D$504=D52)*(D52&lt;&gt;"")+($B$5:$B$504=B52)*(B52&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C52="Оплата",K52&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E52)&gt;0,ROUND(E52-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B52="",C52="",D52="",E52="",F52=""),"",IF(OR(B52="",C52="",E52=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E52)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H52&lt;&gt;0,F52=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G52&lt;&gt;0,F52=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F52&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F52)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C52)*($E$5:$E$504=E52)*(($D$5:$D$504=D52)*(D52&lt;&gt;"")+($B$5:$B$504=B52)*(B52&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C52="Оплата",K52&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E52)&gt;0,ROUND(E52-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J52" s="5">
@@ -2011,7 +2011,7 @@
         <v/>
       </c>
       <c r="I53" s="6">
-        <f>IF(AND(B53="",C53="",D53="",E53="",F53=""),"",IF(OR(B53="",C53="",E53=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E53)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H53&lt;&gt;0,F53=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G53&lt;&gt;0,F53=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F53&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F53)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C53)*($E$5:$E$504=E53)*(($D$5:$D$504=D53)*(D53&lt;&gt;"")+($B$5:$B$504=B53)*(B53&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C53="Оплата",K53&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E53)&gt;0,ROUND(E53-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B53="",C53="",D53="",E53="",F53=""),"",IF(OR(B53="",C53="",E53=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E53)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H53&lt;&gt;0,F53=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G53&lt;&gt;0,F53=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F53&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F53)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C53)*($E$5:$E$504=E53)*(($D$5:$D$504=D53)*(D53&lt;&gt;"")+($B$5:$B$504=B53)*(B53&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C53="Оплата",K53&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E53)&gt;0,ROUND(E53-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J53" s="5">
@@ -2038,7 +2038,7 @@
         <v/>
       </c>
       <c r="I54" s="6">
-        <f>IF(AND(B54="",C54="",D54="",E54="",F54=""),"",IF(OR(B54="",C54="",E54=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E54)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H54&lt;&gt;0,F54=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G54&lt;&gt;0,F54=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F54&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F54)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C54)*($E$5:$E$504=E54)*(($D$5:$D$504=D54)*(D54&lt;&gt;"")+($B$5:$B$504=B54)*(B54&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C54="Оплата",K54&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E54)&gt;0,ROUND(E54-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B54="",C54="",D54="",E54="",F54=""),"",IF(OR(B54="",C54="",E54=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E54)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H54&lt;&gt;0,F54=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G54&lt;&gt;0,F54=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F54&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F54)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C54)*($E$5:$E$504=E54)*(($D$5:$D$504=D54)*(D54&lt;&gt;"")+($B$5:$B$504=B54)*(B54&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C54="Оплата",K54&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E54)&gt;0,ROUND(E54-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J54" s="5">
@@ -2065,7 +2065,7 @@
         <v/>
       </c>
       <c r="I55" s="6">
-        <f>IF(AND(B55="",C55="",D55="",E55="",F55=""),"",IF(OR(B55="",C55="",E55=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E55)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H55&lt;&gt;0,F55=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G55&lt;&gt;0,F55=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F55&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F55)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C55)*($E$5:$E$504=E55)*(($D$5:$D$504=D55)*(D55&lt;&gt;"")+($B$5:$B$504=B55)*(B55&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C55="Оплата",K55&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E55)&gt;0,ROUND(E55-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B55="",C55="",D55="",E55="",F55=""),"",IF(OR(B55="",C55="",E55=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E55)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H55&lt;&gt;0,F55=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G55&lt;&gt;0,F55=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F55&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F55)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C55)*($E$5:$E$504=E55)*(($D$5:$D$504=D55)*(D55&lt;&gt;"")+($B$5:$B$504=B55)*(B55&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C55="Оплата",K55&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E55)&gt;0,ROUND(E55-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J55" s="5">
@@ -2092,7 +2092,7 @@
         <v/>
       </c>
       <c r="I56" s="6">
-        <f>IF(AND(B56="",C56="",D56="",E56="",F56=""),"",IF(OR(B56="",C56="",E56=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E56)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H56&lt;&gt;0,F56=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G56&lt;&gt;0,F56=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F56&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F56)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C56)*($E$5:$E$504=E56)*(($D$5:$D$504=D56)*(D56&lt;&gt;"")+($B$5:$B$504=B56)*(B56&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C56="Оплата",K56&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E56)&gt;0,ROUND(E56-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B56="",C56="",D56="",E56="",F56=""),"",IF(OR(B56="",C56="",E56=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E56)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H56&lt;&gt;0,F56=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G56&lt;&gt;0,F56=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F56&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F56)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C56)*($E$5:$E$504=E56)*(($D$5:$D$504=D56)*(D56&lt;&gt;"")+($B$5:$B$504=B56)*(B56&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C56="Оплата",K56&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E56)&gt;0,ROUND(E56-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J56" s="5">
@@ -2119,7 +2119,7 @@
         <v/>
       </c>
       <c r="I57" s="6">
-        <f>IF(AND(B57="",C57="",D57="",E57="",F57=""),"",IF(OR(B57="",C57="",E57=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E57)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H57&lt;&gt;0,F57=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G57&lt;&gt;0,F57=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F57&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F57)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C57)*($E$5:$E$504=E57)*(($D$5:$D$504=D57)*(D57&lt;&gt;"")+($B$5:$B$504=B57)*(B57&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C57="Оплата",K57&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E57)&gt;0,ROUND(E57-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B57="",C57="",D57="",E57="",F57=""),"",IF(OR(B57="",C57="",E57=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E57)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H57&lt;&gt;0,F57=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G57&lt;&gt;0,F57=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F57&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F57)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C57)*($E$5:$E$504=E57)*(($D$5:$D$504=D57)*(D57&lt;&gt;"")+($B$5:$B$504=B57)*(B57&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C57="Оплата",K57&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E57)&gt;0,ROUND(E57-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J57" s="5">
@@ -2146,7 +2146,7 @@
         <v/>
       </c>
       <c r="I58" s="6">
-        <f>IF(AND(B58="",C58="",D58="",E58="",F58=""),"",IF(OR(B58="",C58="",E58=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E58)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H58&lt;&gt;0,F58=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G58&lt;&gt;0,F58=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F58&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F58)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C58)*($E$5:$E$504=E58)*(($D$5:$D$504=D58)*(D58&lt;&gt;"")+($B$5:$B$504=B58)*(B58&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C58="Оплата",K58&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E58)&gt;0,ROUND(E58-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B58="",C58="",D58="",E58="",F58=""),"",IF(OR(B58="",C58="",E58=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E58)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H58&lt;&gt;0,F58=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G58&lt;&gt;0,F58=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F58&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F58)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C58)*($E$5:$E$504=E58)*(($D$5:$D$504=D58)*(D58&lt;&gt;"")+($B$5:$B$504=B58)*(B58&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C58="Оплата",K58&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E58)&gt;0,ROUND(E58-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J58" s="5">
@@ -2173,7 +2173,7 @@
         <v/>
       </c>
       <c r="I59" s="6">
-        <f>IF(AND(B59="",C59="",D59="",E59="",F59=""),"",IF(OR(B59="",C59="",E59=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E59)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H59&lt;&gt;0,F59=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G59&lt;&gt;0,F59=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F59&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F59)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C59)*($E$5:$E$504=E59)*(($D$5:$D$504=D59)*(D59&lt;&gt;"")+($B$5:$B$504=B59)*(B59&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C59="Оплата",K59&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E59)&gt;0,ROUND(E59-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B59="",C59="",D59="",E59="",F59=""),"",IF(OR(B59="",C59="",E59=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E59)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H59&lt;&gt;0,F59=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G59&lt;&gt;0,F59=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F59&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F59)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C59)*($E$5:$E$504=E59)*(($D$5:$D$504=D59)*(D59&lt;&gt;"")+($B$5:$B$504=B59)*(B59&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C59="Оплата",K59&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E59)&gt;0,ROUND(E59-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J59" s="5">
@@ -2200,7 +2200,7 @@
         <v/>
       </c>
       <c r="I60" s="6">
-        <f>IF(AND(B60="",C60="",D60="",E60="",F60=""),"",IF(OR(B60="",C60="",E60=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E60)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H60&lt;&gt;0,F60=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G60&lt;&gt;0,F60=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F60&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F60)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C60)*($E$5:$E$504=E60)*(($D$5:$D$504=D60)*(D60&lt;&gt;"")+($B$5:$B$504=B60)*(B60&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C60="Оплата",K60&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E60)&gt;0,ROUND(E60-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B60="",C60="",D60="",E60="",F60=""),"",IF(OR(B60="",C60="",E60=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E60)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H60&lt;&gt;0,F60=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G60&lt;&gt;0,F60=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F60&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F60)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C60)*($E$5:$E$504=E60)*(($D$5:$D$504=D60)*(D60&lt;&gt;"")+($B$5:$B$504=B60)*(B60&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C60="Оплата",K60&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E60)&gt;0,ROUND(E60-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J60" s="5">
@@ -2227,7 +2227,7 @@
         <v/>
       </c>
       <c r="I61" s="6">
-        <f>IF(AND(B61="",C61="",D61="",E61="",F61=""),"",IF(OR(B61="",C61="",E61=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E61)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H61&lt;&gt;0,F61=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G61&lt;&gt;0,F61=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F61&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F61)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C61)*($E$5:$E$504=E61)*(($D$5:$D$504=D61)*(D61&lt;&gt;"")+($B$5:$B$504=B61)*(B61&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C61="Оплата",K61&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E61)&gt;0,ROUND(E61-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B61="",C61="",D61="",E61="",F61=""),"",IF(OR(B61="",C61="",E61=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E61)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H61&lt;&gt;0,F61=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G61&lt;&gt;0,F61=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F61&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F61)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C61)*($E$5:$E$504=E61)*(($D$5:$D$504=D61)*(D61&lt;&gt;"")+($B$5:$B$504=B61)*(B61&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C61="Оплата",K61&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E61)&gt;0,ROUND(E61-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J61" s="5">
@@ -2254,7 +2254,7 @@
         <v/>
       </c>
       <c r="I62" s="6">
-        <f>IF(AND(B62="",C62="",D62="",E62="",F62=""),"",IF(OR(B62="",C62="",E62=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E62)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H62&lt;&gt;0,F62=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G62&lt;&gt;0,F62=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F62&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F62)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C62)*($E$5:$E$504=E62)*(($D$5:$D$504=D62)*(D62&lt;&gt;"")+($B$5:$B$504=B62)*(B62&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C62="Оплата",K62&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E62)&gt;0,ROUND(E62-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B62="",C62="",D62="",E62="",F62=""),"",IF(OR(B62="",C62="",E62=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E62)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H62&lt;&gt;0,F62=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G62&lt;&gt;0,F62=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F62&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F62)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C62)*($E$5:$E$504=E62)*(($D$5:$D$504=D62)*(D62&lt;&gt;"")+($B$5:$B$504=B62)*(B62&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C62="Оплата",K62&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E62)&gt;0,ROUND(E62-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J62" s="5">
@@ -2281,7 +2281,7 @@
         <v/>
       </c>
       <c r="I63" s="6">
-        <f>IF(AND(B63="",C63="",D63="",E63="",F63=""),"",IF(OR(B63="",C63="",E63=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E63)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H63&lt;&gt;0,F63=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G63&lt;&gt;0,F63=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F63&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F63)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C63)*($E$5:$E$504=E63)*(($D$5:$D$504=D63)*(D63&lt;&gt;"")+($B$5:$B$504=B63)*(B63&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C63="Оплата",K63&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E63)&gt;0,ROUND(E63-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B63="",C63="",D63="",E63="",F63=""),"",IF(OR(B63="",C63="",E63=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E63)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H63&lt;&gt;0,F63=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G63&lt;&gt;0,F63=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F63&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F63)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C63)*($E$5:$E$504=E63)*(($D$5:$D$504=D63)*(D63&lt;&gt;"")+($B$5:$B$504=B63)*(B63&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C63="Оплата",K63&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E63)&gt;0,ROUND(E63-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J63" s="5">
@@ -2308,7 +2308,7 @@
         <v/>
       </c>
       <c r="I64" s="6">
-        <f>IF(AND(B64="",C64="",D64="",E64="",F64=""),"",IF(OR(B64="",C64="",E64=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E64)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H64&lt;&gt;0,F64=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G64&lt;&gt;0,F64=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F64&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F64)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C64)*($E$5:$E$504=E64)*(($D$5:$D$504=D64)*(D64&lt;&gt;"")+($B$5:$B$504=B64)*(B64&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C64="Оплата",K64&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E64)&gt;0,ROUND(E64-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B64="",C64="",D64="",E64="",F64=""),"",IF(OR(B64="",C64="",E64=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E64)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H64&lt;&gt;0,F64=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G64&lt;&gt;0,F64=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F64&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F64)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C64)*($E$5:$E$504=E64)*(($D$5:$D$504=D64)*(D64&lt;&gt;"")+($B$5:$B$504=B64)*(B64&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C64="Оплата",K64&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E64)&gt;0,ROUND(E64-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J64" s="5">
@@ -2335,7 +2335,7 @@
         <v/>
       </c>
       <c r="I65" s="6">
-        <f>IF(AND(B65="",C65="",D65="",E65="",F65=""),"",IF(OR(B65="",C65="",E65=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E65)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H65&lt;&gt;0,F65=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G65&lt;&gt;0,F65=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F65&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F65)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C65)*($E$5:$E$504=E65)*(($D$5:$D$504=D65)*(D65&lt;&gt;"")+($B$5:$B$504=B65)*(B65&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C65="Оплата",K65&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E65)&gt;0,ROUND(E65-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B65="",C65="",D65="",E65="",F65=""),"",IF(OR(B65="",C65="",E65=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E65)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H65&lt;&gt;0,F65=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G65&lt;&gt;0,F65=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F65&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F65)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C65)*($E$5:$E$504=E65)*(($D$5:$D$504=D65)*(D65&lt;&gt;"")+($B$5:$B$504=B65)*(B65&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C65="Оплата",K65&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E65)&gt;0,ROUND(E65-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J65" s="5">
@@ -2362,7 +2362,7 @@
         <v/>
       </c>
       <c r="I66" s="6">
-        <f>IF(AND(B66="",C66="",D66="",E66="",F66=""),"",IF(OR(B66="",C66="",E66=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E66)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H66&lt;&gt;0,F66=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G66&lt;&gt;0,F66=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F66&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F66)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C66)*($E$5:$E$504=E66)*(($D$5:$D$504=D66)*(D66&lt;&gt;"")+($B$5:$B$504=B66)*(B66&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C66="Оплата",K66&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E66)&gt;0,ROUND(E66-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B66="",C66="",D66="",E66="",F66=""),"",IF(OR(B66="",C66="",E66=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E66)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H66&lt;&gt;0,F66=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G66&lt;&gt;0,F66=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F66&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F66)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C66)*($E$5:$E$504=E66)*(($D$5:$D$504=D66)*(D66&lt;&gt;"")+($B$5:$B$504=B66)*(B66&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C66="Оплата",K66&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E66)&gt;0,ROUND(E66-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J66" s="5">
@@ -2389,7 +2389,7 @@
         <v/>
       </c>
       <c r="I67" s="6">
-        <f>IF(AND(B67="",C67="",D67="",E67="",F67=""),"",IF(OR(B67="",C67="",E67=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E67)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H67&lt;&gt;0,F67=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G67&lt;&gt;0,F67=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F67&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F67)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C67)*($E$5:$E$504=E67)*(($D$5:$D$504=D67)*(D67&lt;&gt;"")+($B$5:$B$504=B67)*(B67&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C67="Оплата",K67&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E67)&gt;0,ROUND(E67-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B67="",C67="",D67="",E67="",F67=""),"",IF(OR(B67="",C67="",E67=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E67)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H67&lt;&gt;0,F67=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G67&lt;&gt;0,F67=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F67&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F67)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C67)*($E$5:$E$504=E67)*(($D$5:$D$504=D67)*(D67&lt;&gt;"")+($B$5:$B$504=B67)*(B67&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C67="Оплата",K67&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E67)&gt;0,ROUND(E67-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J67" s="5">
@@ -2416,7 +2416,7 @@
         <v/>
       </c>
       <c r="I68" s="6">
-        <f>IF(AND(B68="",C68="",D68="",E68="",F68=""),"",IF(OR(B68="",C68="",E68=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E68)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H68&lt;&gt;0,F68=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G68&lt;&gt;0,F68=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F68&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F68)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C68)*($E$5:$E$504=E68)*(($D$5:$D$504=D68)*(D68&lt;&gt;"")+($B$5:$B$504=B68)*(B68&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C68="Оплата",K68&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E68)&gt;0,ROUND(E68-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B68="",C68="",D68="",E68="",F68=""),"",IF(OR(B68="",C68="",E68=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E68)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H68&lt;&gt;0,F68=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G68&lt;&gt;0,F68=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F68&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F68)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C68)*($E$5:$E$504=E68)*(($D$5:$D$504=D68)*(D68&lt;&gt;"")+($B$5:$B$504=B68)*(B68&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C68="Оплата",K68&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E68)&gt;0,ROUND(E68-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J68" s="5">
@@ -2443,7 +2443,7 @@
         <v/>
       </c>
       <c r="I69" s="6">
-        <f>IF(AND(B69="",C69="",D69="",E69="",F69=""),"",IF(OR(B69="",C69="",E69=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E69)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H69&lt;&gt;0,F69=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G69&lt;&gt;0,F69=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F69&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F69)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C69)*($E$5:$E$504=E69)*(($D$5:$D$504=D69)*(D69&lt;&gt;"")+($B$5:$B$504=B69)*(B69&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C69="Оплата",K69&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E69)&gt;0,ROUND(E69-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B69="",C69="",D69="",E69="",F69=""),"",IF(OR(B69="",C69="",E69=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E69)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H69&lt;&gt;0,F69=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G69&lt;&gt;0,F69=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F69&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F69)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C69)*($E$5:$E$504=E69)*(($D$5:$D$504=D69)*(D69&lt;&gt;"")+($B$5:$B$504=B69)*(B69&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C69="Оплата",K69&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E69)&gt;0,ROUND(E69-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J69" s="5">
@@ -2470,7 +2470,7 @@
         <v/>
       </c>
       <c r="I70" s="6">
-        <f>IF(AND(B70="",C70="",D70="",E70="",F70=""),"",IF(OR(B70="",C70="",E70=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E70)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H70&lt;&gt;0,F70=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G70&lt;&gt;0,F70=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F70&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F70)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C70)*($E$5:$E$504=E70)*(($D$5:$D$504=D70)*(D70&lt;&gt;"")+($B$5:$B$504=B70)*(B70&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C70="Оплата",K70&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E70)&gt;0,ROUND(E70-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B70="",C70="",D70="",E70="",F70=""),"",IF(OR(B70="",C70="",E70=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E70)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H70&lt;&gt;0,F70=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G70&lt;&gt;0,F70=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F70&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F70)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C70)*($E$5:$E$504=E70)*(($D$5:$D$504=D70)*(D70&lt;&gt;"")+($B$5:$B$504=B70)*(B70&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C70="Оплата",K70&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E70)&gt;0,ROUND(E70-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J70" s="5">
@@ -2497,7 +2497,7 @@
         <v/>
       </c>
       <c r="I71" s="6">
-        <f>IF(AND(B71="",C71="",D71="",E71="",F71=""),"",IF(OR(B71="",C71="",E71=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E71)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H71&lt;&gt;0,F71=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G71&lt;&gt;0,F71=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F71&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F71)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C71)*($E$5:$E$504=E71)*(($D$5:$D$504=D71)*(D71&lt;&gt;"")+($B$5:$B$504=B71)*(B71&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C71="Оплата",K71&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E71)&gt;0,ROUND(E71-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B71="",C71="",D71="",E71="",F71=""),"",IF(OR(B71="",C71="",E71=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E71)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H71&lt;&gt;0,F71=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G71&lt;&gt;0,F71=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F71&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F71)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C71)*($E$5:$E$504=E71)*(($D$5:$D$504=D71)*(D71&lt;&gt;"")+($B$5:$B$504=B71)*(B71&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C71="Оплата",K71&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E71)&gt;0,ROUND(E71-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J71" s="5">
@@ -2524,7 +2524,7 @@
         <v/>
       </c>
       <c r="I72" s="6">
-        <f>IF(AND(B72="",C72="",D72="",E72="",F72=""),"",IF(OR(B72="",C72="",E72=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E72)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H72&lt;&gt;0,F72=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G72&lt;&gt;0,F72=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F72&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F72)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C72)*($E$5:$E$504=E72)*(($D$5:$D$504=D72)*(D72&lt;&gt;"")+($B$5:$B$504=B72)*(B72&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C72="Оплата",K72&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E72)&gt;0,ROUND(E72-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B72="",C72="",D72="",E72="",F72=""),"",IF(OR(B72="",C72="",E72=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E72)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H72&lt;&gt;0,F72=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G72&lt;&gt;0,F72=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F72&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F72)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C72)*($E$5:$E$504=E72)*(($D$5:$D$504=D72)*(D72&lt;&gt;"")+($B$5:$B$504=B72)*(B72&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C72="Оплата",K72&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E72)&gt;0,ROUND(E72-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J72" s="5">
@@ -2551,7 +2551,7 @@
         <v/>
       </c>
       <c r="I73" s="6">
-        <f>IF(AND(B73="",C73="",D73="",E73="",F73=""),"",IF(OR(B73="",C73="",E73=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E73)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H73&lt;&gt;0,F73=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G73&lt;&gt;0,F73=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F73&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F73)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C73)*($E$5:$E$504=E73)*(($D$5:$D$504=D73)*(D73&lt;&gt;"")+($B$5:$B$504=B73)*(B73&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C73="Оплата",K73&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E73)&gt;0,ROUND(E73-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B73="",C73="",D73="",E73="",F73=""),"",IF(OR(B73="",C73="",E73=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E73)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H73&lt;&gt;0,F73=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G73&lt;&gt;0,F73=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F73&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F73)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C73)*($E$5:$E$504=E73)*(($D$5:$D$504=D73)*(D73&lt;&gt;"")+($B$5:$B$504=B73)*(B73&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C73="Оплата",K73&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E73)&gt;0,ROUND(E73-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J73" s="5">
@@ -2578,7 +2578,7 @@
         <v/>
       </c>
       <c r="I74" s="6">
-        <f>IF(AND(B74="",C74="",D74="",E74="",F74=""),"",IF(OR(B74="",C74="",E74=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E74)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H74&lt;&gt;0,F74=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G74&lt;&gt;0,F74=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F74&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F74)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C74)*($E$5:$E$504=E74)*(($D$5:$D$504=D74)*(D74&lt;&gt;"")+($B$5:$B$504=B74)*(B74&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C74="Оплата",K74&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E74)&gt;0,ROUND(E74-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B74="",C74="",D74="",E74="",F74=""),"",IF(OR(B74="",C74="",E74=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E74)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H74&lt;&gt;0,F74=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G74&lt;&gt;0,F74=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F74&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F74)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C74)*($E$5:$E$504=E74)*(($D$5:$D$504=D74)*(D74&lt;&gt;"")+($B$5:$B$504=B74)*(B74&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C74="Оплата",K74&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E74)&gt;0,ROUND(E74-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J74" s="5">
@@ -2605,7 +2605,7 @@
         <v/>
       </c>
       <c r="I75" s="6">
-        <f>IF(AND(B75="",C75="",D75="",E75="",F75=""),"",IF(OR(B75="",C75="",E75=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E75)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H75&lt;&gt;0,F75=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G75&lt;&gt;0,F75=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F75&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F75)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C75)*($E$5:$E$504=E75)*(($D$5:$D$504=D75)*(D75&lt;&gt;"")+($B$5:$B$504=B75)*(B75&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C75="Оплата",K75&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E75)&gt;0,ROUND(E75-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B75="",C75="",D75="",E75="",F75=""),"",IF(OR(B75="",C75="",E75=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E75)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H75&lt;&gt;0,F75=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G75&lt;&gt;0,F75=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F75&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F75)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C75)*($E$5:$E$504=E75)*(($D$5:$D$504=D75)*(D75&lt;&gt;"")+($B$5:$B$504=B75)*(B75&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C75="Оплата",K75&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E75)&gt;0,ROUND(E75-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J75" s="5">
@@ -2632,7 +2632,7 @@
         <v/>
       </c>
       <c r="I76" s="6">
-        <f>IF(AND(B76="",C76="",D76="",E76="",F76=""),"",IF(OR(B76="",C76="",E76=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E76)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H76&lt;&gt;0,F76=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G76&lt;&gt;0,F76=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F76&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F76)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C76)*($E$5:$E$504=E76)*(($D$5:$D$504=D76)*(D76&lt;&gt;"")+($B$5:$B$504=B76)*(B76&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C76="Оплата",K76&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E76)&gt;0,ROUND(E76-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B76="",C76="",D76="",E76="",F76=""),"",IF(OR(B76="",C76="",E76=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E76)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H76&lt;&gt;0,F76=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G76&lt;&gt;0,F76=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F76&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F76)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C76)*($E$5:$E$504=E76)*(($D$5:$D$504=D76)*(D76&lt;&gt;"")+($B$5:$B$504=B76)*(B76&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C76="Оплата",K76&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E76)&gt;0,ROUND(E76-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J76" s="5">
@@ -2659,7 +2659,7 @@
         <v/>
       </c>
       <c r="I77" s="6">
-        <f>IF(AND(B77="",C77="",D77="",E77="",F77=""),"",IF(OR(B77="",C77="",E77=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E77)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H77&lt;&gt;0,F77=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G77&lt;&gt;0,F77=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F77&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F77)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C77)*($E$5:$E$504=E77)*(($D$5:$D$504=D77)*(D77&lt;&gt;"")+($B$5:$B$504=B77)*(B77&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C77="Оплата",K77&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E77)&gt;0,ROUND(E77-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B77="",C77="",D77="",E77="",F77=""),"",IF(OR(B77="",C77="",E77=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E77)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H77&lt;&gt;0,F77=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G77&lt;&gt;0,F77=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F77&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F77)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C77)*($E$5:$E$504=E77)*(($D$5:$D$504=D77)*(D77&lt;&gt;"")+($B$5:$B$504=B77)*(B77&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C77="Оплата",K77&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E77)&gt;0,ROUND(E77-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J77" s="5">
@@ -2686,7 +2686,7 @@
         <v/>
       </c>
       <c r="I78" s="6">
-        <f>IF(AND(B78="",C78="",D78="",E78="",F78=""),"",IF(OR(B78="",C78="",E78=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E78)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H78&lt;&gt;0,F78=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G78&lt;&gt;0,F78=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F78&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F78)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C78)*($E$5:$E$504=E78)*(($D$5:$D$504=D78)*(D78&lt;&gt;"")+($B$5:$B$504=B78)*(B78&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C78="Оплата",K78&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E78)&gt;0,ROUND(E78-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B78="",C78="",D78="",E78="",F78=""),"",IF(OR(B78="",C78="",E78=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E78)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H78&lt;&gt;0,F78=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G78&lt;&gt;0,F78=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F78&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F78)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C78)*($E$5:$E$504=E78)*(($D$5:$D$504=D78)*(D78&lt;&gt;"")+($B$5:$B$504=B78)*(B78&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C78="Оплата",K78&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E78)&gt;0,ROUND(E78-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J78" s="5">
@@ -2713,7 +2713,7 @@
         <v/>
       </c>
       <c r="I79" s="6">
-        <f>IF(AND(B79="",C79="",D79="",E79="",F79=""),"",IF(OR(B79="",C79="",E79=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E79)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H79&lt;&gt;0,F79=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G79&lt;&gt;0,F79=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F79&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F79)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C79)*($E$5:$E$504=E79)*(($D$5:$D$504=D79)*(D79&lt;&gt;"")+($B$5:$B$504=B79)*(B79&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C79="Оплата",K79&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E79)&gt;0,ROUND(E79-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B79="",C79="",D79="",E79="",F79=""),"",IF(OR(B79="",C79="",E79=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E79)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H79&lt;&gt;0,F79=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G79&lt;&gt;0,F79=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F79&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F79)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C79)*($E$5:$E$504=E79)*(($D$5:$D$504=D79)*(D79&lt;&gt;"")+($B$5:$B$504=B79)*(B79&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C79="Оплата",K79&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E79)&gt;0,ROUND(E79-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J79" s="5">
@@ -2740,7 +2740,7 @@
         <v/>
       </c>
       <c r="I80" s="6">
-        <f>IF(AND(B80="",C80="",D80="",E80="",F80=""),"",IF(OR(B80="",C80="",E80=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E80)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H80&lt;&gt;0,F80=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G80&lt;&gt;0,F80=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F80&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F80)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C80)*($E$5:$E$504=E80)*(($D$5:$D$504=D80)*(D80&lt;&gt;"")+($B$5:$B$504=B80)*(B80&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C80="Оплата",K80&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E80)&gt;0,ROUND(E80-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B80="",C80="",D80="",E80="",F80=""),"",IF(OR(B80="",C80="",E80=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E80)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H80&lt;&gt;0,F80=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G80&lt;&gt;0,F80=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F80&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F80)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C80)*($E$5:$E$504=E80)*(($D$5:$D$504=D80)*(D80&lt;&gt;"")+($B$5:$B$504=B80)*(B80&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C80="Оплата",K80&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E80)&gt;0,ROUND(E80-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J80" s="5">
@@ -2767,7 +2767,7 @@
         <v/>
       </c>
       <c r="I81" s="6">
-        <f>IF(AND(B81="",C81="",D81="",E81="",F81=""),"",IF(OR(B81="",C81="",E81=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E81)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H81&lt;&gt;0,F81=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G81&lt;&gt;0,F81=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F81&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F81)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C81)*($E$5:$E$504=E81)*(($D$5:$D$504=D81)*(D81&lt;&gt;"")+($B$5:$B$504=B81)*(B81&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C81="Оплата",K81&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E81)&gt;0,ROUND(E81-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B81="",C81="",D81="",E81="",F81=""),"",IF(OR(B81="",C81="",E81=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E81)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H81&lt;&gt;0,F81=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G81&lt;&gt;0,F81=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F81&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F81)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C81)*($E$5:$E$504=E81)*(($D$5:$D$504=D81)*(D81&lt;&gt;"")+($B$5:$B$504=B81)*(B81&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C81="Оплата",K81&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E81)&gt;0,ROUND(E81-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J81" s="5">
@@ -2794,7 +2794,7 @@
         <v/>
       </c>
       <c r="I82" s="6">
-        <f>IF(AND(B82="",C82="",D82="",E82="",F82=""),"",IF(OR(B82="",C82="",E82=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E82)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H82&lt;&gt;0,F82=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G82&lt;&gt;0,F82=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F82&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F82)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C82)*($E$5:$E$504=E82)*(($D$5:$D$504=D82)*(D82&lt;&gt;"")+($B$5:$B$504=B82)*(B82&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C82="Оплата",K82&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E82)&gt;0,ROUND(E82-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B82="",C82="",D82="",E82="",F82=""),"",IF(OR(B82="",C82="",E82=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E82)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H82&lt;&gt;0,F82=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G82&lt;&gt;0,F82=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F82&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F82)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C82)*($E$5:$E$504=E82)*(($D$5:$D$504=D82)*(D82&lt;&gt;"")+($B$5:$B$504=B82)*(B82&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C82="Оплата",K82&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E82)&gt;0,ROUND(E82-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J82" s="5">
@@ -2821,7 +2821,7 @@
         <v/>
       </c>
       <c r="I83" s="6">
-        <f>IF(AND(B83="",C83="",D83="",E83="",F83=""),"",IF(OR(B83="",C83="",E83=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E83)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H83&lt;&gt;0,F83=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G83&lt;&gt;0,F83=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F83&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F83)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C83)*($E$5:$E$504=E83)*(($D$5:$D$504=D83)*(D83&lt;&gt;"")+($B$5:$B$504=B83)*(B83&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C83="Оплата",K83&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E83)&gt;0,ROUND(E83-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B83="",C83="",D83="",E83="",F83=""),"",IF(OR(B83="",C83="",E83=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E83)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H83&lt;&gt;0,F83=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G83&lt;&gt;0,F83=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F83&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F83)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C83)*($E$5:$E$504=E83)*(($D$5:$D$504=D83)*(D83&lt;&gt;"")+($B$5:$B$504=B83)*(B83&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C83="Оплата",K83&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E83)&gt;0,ROUND(E83-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J83" s="5">
@@ -2848,7 +2848,7 @@
         <v/>
       </c>
       <c r="I84" s="6">
-        <f>IF(AND(B84="",C84="",D84="",E84="",F84=""),"",IF(OR(B84="",C84="",E84=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E84)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H84&lt;&gt;0,F84=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G84&lt;&gt;0,F84=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F84&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F84)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C84)*($E$5:$E$504=E84)*(($D$5:$D$504=D84)*(D84&lt;&gt;"")+($B$5:$B$504=B84)*(B84&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C84="Оплата",K84&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E84)&gt;0,ROUND(E84-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B84="",C84="",D84="",E84="",F84=""),"",IF(OR(B84="",C84="",E84=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E84)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H84&lt;&gt;0,F84=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G84&lt;&gt;0,F84=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F84&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F84)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C84)*($E$5:$E$504=E84)*(($D$5:$D$504=D84)*(D84&lt;&gt;"")+($B$5:$B$504=B84)*(B84&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C84="Оплата",K84&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E84)&gt;0,ROUND(E84-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J84" s="5">
@@ -2875,7 +2875,7 @@
         <v/>
       </c>
       <c r="I85" s="6">
-        <f>IF(AND(B85="",C85="",D85="",E85="",F85=""),"",IF(OR(B85="",C85="",E85=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E85)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H85&lt;&gt;0,F85=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G85&lt;&gt;0,F85=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F85&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F85)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C85)*($E$5:$E$504=E85)*(($D$5:$D$504=D85)*(D85&lt;&gt;"")+($B$5:$B$504=B85)*(B85&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C85="Оплата",K85&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E85)&gt;0,ROUND(E85-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B85="",C85="",D85="",E85="",F85=""),"",IF(OR(B85="",C85="",E85=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E85)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H85&lt;&gt;0,F85=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G85&lt;&gt;0,F85=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F85&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F85)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C85)*($E$5:$E$504=E85)*(($D$5:$D$504=D85)*(D85&lt;&gt;"")+($B$5:$B$504=B85)*(B85&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C85="Оплата",K85&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E85)&gt;0,ROUND(E85-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J85" s="5">
@@ -2902,7 +2902,7 @@
         <v/>
       </c>
       <c r="I86" s="6">
-        <f>IF(AND(B86="",C86="",D86="",E86="",F86=""),"",IF(OR(B86="",C86="",E86=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E86)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H86&lt;&gt;0,F86=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G86&lt;&gt;0,F86=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F86&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F86)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C86)*($E$5:$E$504=E86)*(($D$5:$D$504=D86)*(D86&lt;&gt;"")+($B$5:$B$504=B86)*(B86&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C86="Оплата",K86&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E86)&gt;0,ROUND(E86-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B86="",C86="",D86="",E86="",F86=""),"",IF(OR(B86="",C86="",E86=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E86)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H86&lt;&gt;0,F86=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G86&lt;&gt;0,F86=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F86&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F86)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C86)*($E$5:$E$504=E86)*(($D$5:$D$504=D86)*(D86&lt;&gt;"")+($B$5:$B$504=B86)*(B86&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C86="Оплата",K86&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E86)&gt;0,ROUND(E86-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J86" s="5">
@@ -2929,7 +2929,7 @@
         <v/>
       </c>
       <c r="I87" s="6">
-        <f>IF(AND(B87="",C87="",D87="",E87="",F87=""),"",IF(OR(B87="",C87="",E87=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E87)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H87&lt;&gt;0,F87=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G87&lt;&gt;0,F87=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F87&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F87)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C87)*($E$5:$E$504=E87)*(($D$5:$D$504=D87)*(D87&lt;&gt;"")+($B$5:$B$504=B87)*(B87&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C87="Оплата",K87&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E87)&gt;0,ROUND(E87-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B87="",C87="",D87="",E87="",F87=""),"",IF(OR(B87="",C87="",E87=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E87)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H87&lt;&gt;0,F87=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G87&lt;&gt;0,F87=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F87&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F87)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C87)*($E$5:$E$504=E87)*(($D$5:$D$504=D87)*(D87&lt;&gt;"")+($B$5:$B$504=B87)*(B87&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C87="Оплата",K87&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E87)&gt;0,ROUND(E87-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J87" s="5">
@@ -2956,7 +2956,7 @@
         <v/>
       </c>
       <c r="I88" s="6">
-        <f>IF(AND(B88="",C88="",D88="",E88="",F88=""),"",IF(OR(B88="",C88="",E88=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E88)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H88&lt;&gt;0,F88=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G88&lt;&gt;0,F88=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F88&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F88)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C88)*($E$5:$E$504=E88)*(($D$5:$D$504=D88)*(D88&lt;&gt;"")+($B$5:$B$504=B88)*(B88&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C88="Оплата",K88&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E88)&gt;0,ROUND(E88-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B88="",C88="",D88="",E88="",F88=""),"",IF(OR(B88="",C88="",E88=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E88)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H88&lt;&gt;0,F88=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G88&lt;&gt;0,F88=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F88&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F88)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C88)*($E$5:$E$504=E88)*(($D$5:$D$504=D88)*(D88&lt;&gt;"")+($B$5:$B$504=B88)*(B88&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C88="Оплата",K88&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E88)&gt;0,ROUND(E88-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J88" s="5">
@@ -2983,7 +2983,7 @@
         <v/>
       </c>
       <c r="I89" s="6">
-        <f>IF(AND(B89="",C89="",D89="",E89="",F89=""),"",IF(OR(B89="",C89="",E89=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E89)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H89&lt;&gt;0,F89=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G89&lt;&gt;0,F89=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F89&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F89)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C89)*($E$5:$E$504=E89)*(($D$5:$D$504=D89)*(D89&lt;&gt;"")+($B$5:$B$504=B89)*(B89&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C89="Оплата",K89&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E89)&gt;0,ROUND(E89-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B89="",C89="",D89="",E89="",F89=""),"",IF(OR(B89="",C89="",E89=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E89)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H89&lt;&gt;0,F89=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G89&lt;&gt;0,F89=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F89&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F89)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C89)*($E$5:$E$504=E89)*(($D$5:$D$504=D89)*(D89&lt;&gt;"")+($B$5:$B$504=B89)*(B89&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C89="Оплата",K89&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E89)&gt;0,ROUND(E89-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J89" s="5">
@@ -3010,7 +3010,7 @@
         <v/>
       </c>
       <c r="I90" s="6">
-        <f>IF(AND(B90="",C90="",D90="",E90="",F90=""),"",IF(OR(B90="",C90="",E90=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E90)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H90&lt;&gt;0,F90=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G90&lt;&gt;0,F90=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F90&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F90)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C90)*($E$5:$E$504=E90)*(($D$5:$D$504=D90)*(D90&lt;&gt;"")+($B$5:$B$504=B90)*(B90&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C90="Оплата",K90&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E90)&gt;0,ROUND(E90-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B90="",C90="",D90="",E90="",F90=""),"",IF(OR(B90="",C90="",E90=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E90)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H90&lt;&gt;0,F90=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G90&lt;&gt;0,F90=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F90&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F90)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C90)*($E$5:$E$504=E90)*(($D$5:$D$504=D90)*(D90&lt;&gt;"")+($B$5:$B$504=B90)*(B90&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C90="Оплата",K90&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E90)&gt;0,ROUND(E90-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J90" s="5">
@@ -3037,7 +3037,7 @@
         <v/>
       </c>
       <c r="I91" s="6">
-        <f>IF(AND(B91="",C91="",D91="",E91="",F91=""),"",IF(OR(B91="",C91="",E91=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E91)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H91&lt;&gt;0,F91=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G91&lt;&gt;0,F91=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F91&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F91)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C91)*($E$5:$E$504=E91)*(($D$5:$D$504=D91)*(D91&lt;&gt;"")+($B$5:$B$504=B91)*(B91&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C91="Оплата",K91&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E91)&gt;0,ROUND(E91-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B91="",C91="",D91="",E91="",F91=""),"",IF(OR(B91="",C91="",E91=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E91)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H91&lt;&gt;0,F91=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G91&lt;&gt;0,F91=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F91&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F91)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C91)*($E$5:$E$504=E91)*(($D$5:$D$504=D91)*(D91&lt;&gt;"")+($B$5:$B$504=B91)*(B91&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C91="Оплата",K91&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E91)&gt;0,ROUND(E91-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J91" s="5">
@@ -3064,7 +3064,7 @@
         <v/>
       </c>
       <c r="I92" s="6">
-        <f>IF(AND(B92="",C92="",D92="",E92="",F92=""),"",IF(OR(B92="",C92="",E92=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E92)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H92&lt;&gt;0,F92=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G92&lt;&gt;0,F92=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F92&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F92)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C92)*($E$5:$E$504=E92)*(($D$5:$D$504=D92)*(D92&lt;&gt;"")+($B$5:$B$504=B92)*(B92&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C92="Оплата",K92&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E92)&gt;0,ROUND(E92-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B92="",C92="",D92="",E92="",F92=""),"",IF(OR(B92="",C92="",E92=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E92)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H92&lt;&gt;0,F92=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G92&lt;&gt;0,F92=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F92&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F92)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C92)*($E$5:$E$504=E92)*(($D$5:$D$504=D92)*(D92&lt;&gt;"")+($B$5:$B$504=B92)*(B92&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C92="Оплата",K92&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E92)&gt;0,ROUND(E92-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J92" s="5">
@@ -3091,7 +3091,7 @@
         <v/>
       </c>
       <c r="I93" s="6">
-        <f>IF(AND(B93="",C93="",D93="",E93="",F93=""),"",IF(OR(B93="",C93="",E93=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E93)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H93&lt;&gt;0,F93=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G93&lt;&gt;0,F93=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F93&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F93)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C93)*($E$5:$E$504=E93)*(($D$5:$D$504=D93)*(D93&lt;&gt;"")+($B$5:$B$504=B93)*(B93&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C93="Оплата",K93&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E93)&gt;0,ROUND(E93-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B93="",C93="",D93="",E93="",F93=""),"",IF(OR(B93="",C93="",E93=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E93)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H93&lt;&gt;0,F93=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G93&lt;&gt;0,F93=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F93&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F93)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C93)*($E$5:$E$504=E93)*(($D$5:$D$504=D93)*(D93&lt;&gt;"")+($B$5:$B$504=B93)*(B93&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C93="Оплата",K93&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E93)&gt;0,ROUND(E93-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J93" s="5">
@@ -3118,7 +3118,7 @@
         <v/>
       </c>
       <c r="I94" s="6">
-        <f>IF(AND(B94="",C94="",D94="",E94="",F94=""),"",IF(OR(B94="",C94="",E94=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E94)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H94&lt;&gt;0,F94=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G94&lt;&gt;0,F94=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F94&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F94)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C94)*($E$5:$E$504=E94)*(($D$5:$D$504=D94)*(D94&lt;&gt;"")+($B$5:$B$504=B94)*(B94&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C94="Оплата",K94&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E94)&gt;0,ROUND(E94-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B94="",C94="",D94="",E94="",F94=""),"",IF(OR(B94="",C94="",E94=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E94)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H94&lt;&gt;0,F94=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G94&lt;&gt;0,F94=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F94&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F94)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C94)*($E$5:$E$504=E94)*(($D$5:$D$504=D94)*(D94&lt;&gt;"")+($B$5:$B$504=B94)*(B94&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C94="Оплата",K94&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E94)&gt;0,ROUND(E94-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J94" s="5">
@@ -3145,7 +3145,7 @@
         <v/>
       </c>
       <c r="I95" s="6">
-        <f>IF(AND(B95="",C95="",D95="",E95="",F95=""),"",IF(OR(B95="",C95="",E95=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E95)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H95&lt;&gt;0,F95=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G95&lt;&gt;0,F95=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F95&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F95)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C95)*($E$5:$E$504=E95)*(($D$5:$D$504=D95)*(D95&lt;&gt;"")+($B$5:$B$504=B95)*(B95&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C95="Оплата",K95&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E95)&gt;0,ROUND(E95-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B95="",C95="",D95="",E95="",F95=""),"",IF(OR(B95="",C95="",E95=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E95)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H95&lt;&gt;0,F95=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G95&lt;&gt;0,F95=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F95&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F95)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C95)*($E$5:$E$504=E95)*(($D$5:$D$504=D95)*(D95&lt;&gt;"")+($B$5:$B$504=B95)*(B95&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C95="Оплата",K95&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E95)&gt;0,ROUND(E95-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J95" s="5">
@@ -3172,7 +3172,7 @@
         <v/>
       </c>
       <c r="I96" s="6">
-        <f>IF(AND(B96="",C96="",D96="",E96="",F96=""),"",IF(OR(B96="",C96="",E96=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E96)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H96&lt;&gt;0,F96=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G96&lt;&gt;0,F96=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F96&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F96)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C96)*($E$5:$E$504=E96)*(($D$5:$D$504=D96)*(D96&lt;&gt;"")+($B$5:$B$504=B96)*(B96&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C96="Оплата",K96&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E96)&gt;0,ROUND(E96-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B96="",C96="",D96="",E96="",F96=""),"",IF(OR(B96="",C96="",E96=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E96)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H96&lt;&gt;0,F96=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G96&lt;&gt;0,F96=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F96&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F96)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C96)*($E$5:$E$504=E96)*(($D$5:$D$504=D96)*(D96&lt;&gt;"")+($B$5:$B$504=B96)*(B96&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C96="Оплата",K96&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E96)&gt;0,ROUND(E96-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J96" s="5">
@@ -3199,7 +3199,7 @@
         <v/>
       </c>
       <c r="I97" s="6">
-        <f>IF(AND(B97="",C97="",D97="",E97="",F97=""),"",IF(OR(B97="",C97="",E97=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E97)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H97&lt;&gt;0,F97=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G97&lt;&gt;0,F97=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F97&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F97)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C97)*($E$5:$E$504=E97)*(($D$5:$D$504=D97)*(D97&lt;&gt;"")+($B$5:$B$504=B97)*(B97&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C97="Оплата",K97&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E97)&gt;0,ROUND(E97-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B97="",C97="",D97="",E97="",F97=""),"",IF(OR(B97="",C97="",E97=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E97)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H97&lt;&gt;0,F97=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G97&lt;&gt;0,F97=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F97&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F97)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C97)*($E$5:$E$504=E97)*(($D$5:$D$504=D97)*(D97&lt;&gt;"")+($B$5:$B$504=B97)*(B97&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C97="Оплата",K97&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E97)&gt;0,ROUND(E97-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J97" s="5">
@@ -3226,7 +3226,7 @@
         <v/>
       </c>
       <c r="I98" s="6">
-        <f>IF(AND(B98="",C98="",D98="",E98="",F98=""),"",IF(OR(B98="",C98="",E98=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E98)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H98&lt;&gt;0,F98=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G98&lt;&gt;0,F98=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F98&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F98)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C98)*($E$5:$E$504=E98)*(($D$5:$D$504=D98)*(D98&lt;&gt;"")+($B$5:$B$504=B98)*(B98&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C98="Оплата",K98&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E98)&gt;0,ROUND(E98-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B98="",C98="",D98="",E98="",F98=""),"",IF(OR(B98="",C98="",E98=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E98)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H98&lt;&gt;0,F98=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G98&lt;&gt;0,F98=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F98&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F98)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C98)*($E$5:$E$504=E98)*(($D$5:$D$504=D98)*(D98&lt;&gt;"")+($B$5:$B$504=B98)*(B98&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C98="Оплата",K98&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E98)&gt;0,ROUND(E98-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J98" s="5">
@@ -3253,7 +3253,7 @@
         <v/>
       </c>
       <c r="I99" s="6">
-        <f>IF(AND(B99="",C99="",D99="",E99="",F99=""),"",IF(OR(B99="",C99="",E99=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E99)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H99&lt;&gt;0,F99=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G99&lt;&gt;0,F99=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F99&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F99)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C99)*($E$5:$E$504=E99)*(($D$5:$D$504=D99)*(D99&lt;&gt;"")+($B$5:$B$504=B99)*(B99&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C99="Оплата",K99&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E99)&gt;0,ROUND(E99-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B99="",C99="",D99="",E99="",F99=""),"",IF(OR(B99="",C99="",E99=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E99)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H99&lt;&gt;0,F99=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G99&lt;&gt;0,F99=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F99&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F99)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C99)*($E$5:$E$504=E99)*(($D$5:$D$504=D99)*(D99&lt;&gt;"")+($B$5:$B$504=B99)*(B99&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C99="Оплата",K99&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E99)&gt;0,ROUND(E99-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J99" s="5">
@@ -3280,7 +3280,7 @@
         <v/>
       </c>
       <c r="I100" s="6">
-        <f>IF(AND(B100="",C100="",D100="",E100="",F100=""),"",IF(OR(B100="",C100="",E100=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E100)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H100&lt;&gt;0,F100=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G100&lt;&gt;0,F100=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F100&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F100)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C100)*($E$5:$E$504=E100)*(($D$5:$D$504=D100)*(D100&lt;&gt;"")+($B$5:$B$504=B100)*(B100&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C100="Оплата",K100&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E100)&gt;0,ROUND(E100-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B100="",C100="",D100="",E100="",F100=""),"",IF(OR(B100="",C100="",E100=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E100)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H100&lt;&gt;0,F100=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G100&lt;&gt;0,F100=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F100&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F100)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C100)*($E$5:$E$504=E100)*(($D$5:$D$504=D100)*(D100&lt;&gt;"")+($B$5:$B$504=B100)*(B100&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C100="Оплата",K100&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E100)&gt;0,ROUND(E100-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J100" s="5">
@@ -3307,7 +3307,7 @@
         <v/>
       </c>
       <c r="I101" s="6">
-        <f>IF(AND(B101="",C101="",D101="",E101="",F101=""),"",IF(OR(B101="",C101="",E101=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E101)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H101&lt;&gt;0,F101=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G101&lt;&gt;0,F101=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F101&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F101)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C101)*($E$5:$E$504=E101)*(($D$5:$D$504=D101)*(D101&lt;&gt;"")+($B$5:$B$504=B101)*(B101&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C101="Оплата",K101&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E101)&gt;0,ROUND(E101-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B101="",C101="",D101="",E101="",F101=""),"",IF(OR(B101="",C101="",E101=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E101)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H101&lt;&gt;0,F101=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G101&lt;&gt;0,F101=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F101&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F101)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C101)*($E$5:$E$504=E101)*(($D$5:$D$504=D101)*(D101&lt;&gt;"")+($B$5:$B$504=B101)*(B101&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C101="Оплата",K101&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E101)&gt;0,ROUND(E101-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J101" s="5">
@@ -3334,7 +3334,7 @@
         <v/>
       </c>
       <c r="I102" s="6">
-        <f>IF(AND(B102="",C102="",D102="",E102="",F102=""),"",IF(OR(B102="",C102="",E102=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E102)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H102&lt;&gt;0,F102=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G102&lt;&gt;0,F102=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F102&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F102)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C102)*($E$5:$E$504=E102)*(($D$5:$D$504=D102)*(D102&lt;&gt;"")+($B$5:$B$504=B102)*(B102&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C102="Оплата",K102&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E102)&gt;0,ROUND(E102-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B102="",C102="",D102="",E102="",F102=""),"",IF(OR(B102="",C102="",E102=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E102)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H102&lt;&gt;0,F102=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G102&lt;&gt;0,F102=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F102&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F102)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C102)*($E$5:$E$504=E102)*(($D$5:$D$504=D102)*(D102&lt;&gt;"")+($B$5:$B$504=B102)*(B102&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C102="Оплата",K102&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E102)&gt;0,ROUND(E102-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J102" s="5">
@@ -3361,7 +3361,7 @@
         <v/>
       </c>
       <c r="I103" s="6">
-        <f>IF(AND(B103="",C103="",D103="",E103="",F103=""),"",IF(OR(B103="",C103="",E103=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E103)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H103&lt;&gt;0,F103=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G103&lt;&gt;0,F103=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F103&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F103)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C103)*($E$5:$E$504=E103)*(($D$5:$D$504=D103)*(D103&lt;&gt;"")+($B$5:$B$504=B103)*(B103&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C103="Оплата",K103&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E103)&gt;0,ROUND(E103-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B103="",C103="",D103="",E103="",F103=""),"",IF(OR(B103="",C103="",E103=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E103)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H103&lt;&gt;0,F103=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G103&lt;&gt;0,F103=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F103&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F103)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C103)*($E$5:$E$504=E103)*(($D$5:$D$504=D103)*(D103&lt;&gt;"")+($B$5:$B$504=B103)*(B103&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C103="Оплата",K103&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E103)&gt;0,ROUND(E103-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J103" s="5">
@@ -3388,7 +3388,7 @@
         <v/>
       </c>
       <c r="I104" s="6">
-        <f>IF(AND(B104="",C104="",D104="",E104="",F104=""),"",IF(OR(B104="",C104="",E104=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E104)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H104&lt;&gt;0,F104=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G104&lt;&gt;0,F104=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F104&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F104)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C104)*($E$5:$E$504=E104)*(($D$5:$D$504=D104)*(D104&lt;&gt;"")+($B$5:$B$504=B104)*(B104&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C104="Оплата",K104&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E104)&gt;0,ROUND(E104-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B104="",C104="",D104="",E104="",F104=""),"",IF(OR(B104="",C104="",E104=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E104)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H104&lt;&gt;0,F104=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G104&lt;&gt;0,F104=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F104&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F104)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C104)*($E$5:$E$504=E104)*(($D$5:$D$504=D104)*(D104&lt;&gt;"")+($B$5:$B$504=B104)*(B104&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C104="Оплата",K104&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E104)&gt;0,ROUND(E104-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J104" s="5">
@@ -3415,7 +3415,7 @@
         <v/>
       </c>
       <c r="I105" s="6">
-        <f>IF(AND(B105="",C105="",D105="",E105="",F105=""),"",IF(OR(B105="",C105="",E105=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E105)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H105&lt;&gt;0,F105=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G105&lt;&gt;0,F105=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F105&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F105)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C105)*($E$5:$E$504=E105)*(($D$5:$D$504=D105)*(D105&lt;&gt;"")+($B$5:$B$504=B105)*(B105&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C105="Оплата",K105&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E105)&gt;0,ROUND(E105-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B105="",C105="",D105="",E105="",F105=""),"",IF(OR(B105="",C105="",E105=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E105)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H105&lt;&gt;0,F105=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G105&lt;&gt;0,F105=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F105&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F105)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C105)*($E$5:$E$504=E105)*(($D$5:$D$504=D105)*(D105&lt;&gt;"")+($B$5:$B$504=B105)*(B105&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C105="Оплата",K105&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E105)&gt;0,ROUND(E105-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J105" s="5">
@@ -3442,7 +3442,7 @@
         <v/>
       </c>
       <c r="I106" s="6">
-        <f>IF(AND(B106="",C106="",D106="",E106="",F106=""),"",IF(OR(B106="",C106="",E106=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E106)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H106&lt;&gt;0,F106=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G106&lt;&gt;0,F106=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F106&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F106)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C106)*($E$5:$E$504=E106)*(($D$5:$D$504=D106)*(D106&lt;&gt;"")+($B$5:$B$504=B106)*(B106&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C106="Оплата",K106&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E106)&gt;0,ROUND(E106-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B106="",C106="",D106="",E106="",F106=""),"",IF(OR(B106="",C106="",E106=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E106)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H106&lt;&gt;0,F106=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G106&lt;&gt;0,F106=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F106&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F106)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C106)*($E$5:$E$504=E106)*(($D$5:$D$504=D106)*(D106&lt;&gt;"")+($B$5:$B$504=B106)*(B106&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C106="Оплата",K106&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E106)&gt;0,ROUND(E106-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J106" s="5">
@@ -3469,7 +3469,7 @@
         <v/>
       </c>
       <c r="I107" s="6">
-        <f>IF(AND(B107="",C107="",D107="",E107="",F107=""),"",IF(OR(B107="",C107="",E107=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E107)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H107&lt;&gt;0,F107=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G107&lt;&gt;0,F107=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F107&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F107)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C107)*($E$5:$E$504=E107)*(($D$5:$D$504=D107)*(D107&lt;&gt;"")+($B$5:$B$504=B107)*(B107&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C107="Оплата",K107&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E107)&gt;0,ROUND(E107-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B107="",C107="",D107="",E107="",F107=""),"",IF(OR(B107="",C107="",E107=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E107)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H107&lt;&gt;0,F107=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G107&lt;&gt;0,F107=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F107&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F107)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C107)*($E$5:$E$504=E107)*(($D$5:$D$504=D107)*(D107&lt;&gt;"")+($B$5:$B$504=B107)*(B107&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C107="Оплата",K107&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E107)&gt;0,ROUND(E107-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J107" s="5">
@@ -3496,7 +3496,7 @@
         <v/>
       </c>
       <c r="I108" s="6">
-        <f>IF(AND(B108="",C108="",D108="",E108="",F108=""),"",IF(OR(B108="",C108="",E108=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E108)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H108&lt;&gt;0,F108=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G108&lt;&gt;0,F108=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F108&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F108)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C108)*($E$5:$E$504=E108)*(($D$5:$D$504=D108)*(D108&lt;&gt;"")+($B$5:$B$504=B108)*(B108&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C108="Оплата",K108&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E108)&gt;0,ROUND(E108-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B108="",C108="",D108="",E108="",F108=""),"",IF(OR(B108="",C108="",E108=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E108)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H108&lt;&gt;0,F108=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G108&lt;&gt;0,F108=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F108&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F108)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C108)*($E$5:$E$504=E108)*(($D$5:$D$504=D108)*(D108&lt;&gt;"")+($B$5:$B$504=B108)*(B108&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C108="Оплата",K108&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E108)&gt;0,ROUND(E108-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J108" s="5">
@@ -3523,7 +3523,7 @@
         <v/>
       </c>
       <c r="I109" s="6">
-        <f>IF(AND(B109="",C109="",D109="",E109="",F109=""),"",IF(OR(B109="",C109="",E109=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E109)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H109&lt;&gt;0,F109=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G109&lt;&gt;0,F109=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F109&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F109)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C109)*($E$5:$E$504=E109)*(($D$5:$D$504=D109)*(D109&lt;&gt;"")+($B$5:$B$504=B109)*(B109&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C109="Оплата",K109&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E109)&gt;0,ROUND(E109-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B109="",C109="",D109="",E109="",F109=""),"",IF(OR(B109="",C109="",E109=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E109)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H109&lt;&gt;0,F109=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G109&lt;&gt;0,F109=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F109&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F109)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C109)*($E$5:$E$504=E109)*(($D$5:$D$504=D109)*(D109&lt;&gt;"")+($B$5:$B$504=B109)*(B109&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C109="Оплата",K109&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E109)&gt;0,ROUND(E109-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J109" s="5">
@@ -3550,7 +3550,7 @@
         <v/>
       </c>
       <c r="I110" s="6">
-        <f>IF(AND(B110="",C110="",D110="",E110="",F110=""),"",IF(OR(B110="",C110="",E110=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E110)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H110&lt;&gt;0,F110=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G110&lt;&gt;0,F110=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F110&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F110)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C110)*($E$5:$E$504=E110)*(($D$5:$D$504=D110)*(D110&lt;&gt;"")+($B$5:$B$504=B110)*(B110&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C110="Оплата",K110&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E110)&gt;0,ROUND(E110-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B110="",C110="",D110="",E110="",F110=""),"",IF(OR(B110="",C110="",E110=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E110)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H110&lt;&gt;0,F110=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G110&lt;&gt;0,F110=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F110&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F110)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C110)*($E$5:$E$504=E110)*(($D$5:$D$504=D110)*(D110&lt;&gt;"")+($B$5:$B$504=B110)*(B110&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C110="Оплата",K110&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E110)&gt;0,ROUND(E110-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J110" s="5">
@@ -3577,7 +3577,7 @@
         <v/>
       </c>
       <c r="I111" s="6">
-        <f>IF(AND(B111="",C111="",D111="",E111="",F111=""),"",IF(OR(B111="",C111="",E111=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E111)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H111&lt;&gt;0,F111=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G111&lt;&gt;0,F111=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F111&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F111)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C111)*($E$5:$E$504=E111)*(($D$5:$D$504=D111)*(D111&lt;&gt;"")+($B$5:$B$504=B111)*(B111&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C111="Оплата",K111&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E111)&gt;0,ROUND(E111-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B111="",C111="",D111="",E111="",F111=""),"",IF(OR(B111="",C111="",E111=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E111)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H111&lt;&gt;0,F111=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G111&lt;&gt;0,F111=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F111&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F111)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C111)*($E$5:$E$504=E111)*(($D$5:$D$504=D111)*(D111&lt;&gt;"")+($B$5:$B$504=B111)*(B111&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C111="Оплата",K111&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E111)&gt;0,ROUND(E111-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J111" s="5">
@@ -3604,7 +3604,7 @@
         <v/>
       </c>
       <c r="I112" s="6">
-        <f>IF(AND(B112="",C112="",D112="",E112="",F112=""),"",IF(OR(B112="",C112="",E112=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E112)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H112&lt;&gt;0,F112=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G112&lt;&gt;0,F112=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F112&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F112)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C112)*($E$5:$E$504=E112)*(($D$5:$D$504=D112)*(D112&lt;&gt;"")+($B$5:$B$504=B112)*(B112&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C112="Оплата",K112&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E112)&gt;0,ROUND(E112-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B112="",C112="",D112="",E112="",F112=""),"",IF(OR(B112="",C112="",E112=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E112)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H112&lt;&gt;0,F112=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G112&lt;&gt;0,F112=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F112&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F112)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C112)*($E$5:$E$504=E112)*(($D$5:$D$504=D112)*(D112&lt;&gt;"")+($B$5:$B$504=B112)*(B112&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C112="Оплата",K112&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E112)&gt;0,ROUND(E112-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J112" s="5">
@@ -3631,7 +3631,7 @@
         <v/>
       </c>
       <c r="I113" s="6">
-        <f>IF(AND(B113="",C113="",D113="",E113="",F113=""),"",IF(OR(B113="",C113="",E113=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E113)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H113&lt;&gt;0,F113=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G113&lt;&gt;0,F113=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F113&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F113)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C113)*($E$5:$E$504=E113)*(($D$5:$D$504=D113)*(D113&lt;&gt;"")+($B$5:$B$504=B113)*(B113&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C113="Оплата",K113&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E113)&gt;0,ROUND(E113-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B113="",C113="",D113="",E113="",F113=""),"",IF(OR(B113="",C113="",E113=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E113)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H113&lt;&gt;0,F113=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G113&lt;&gt;0,F113=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F113&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F113)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C113)*($E$5:$E$504=E113)*(($D$5:$D$504=D113)*(D113&lt;&gt;"")+($B$5:$B$504=B113)*(B113&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C113="Оплата",K113&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E113)&gt;0,ROUND(E113-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J113" s="5">
@@ -3658,7 +3658,7 @@
         <v/>
       </c>
       <c r="I114" s="6">
-        <f>IF(AND(B114="",C114="",D114="",E114="",F114=""),"",IF(OR(B114="",C114="",E114=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E114)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H114&lt;&gt;0,F114=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G114&lt;&gt;0,F114=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F114&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F114)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C114)*($E$5:$E$504=E114)*(($D$5:$D$504=D114)*(D114&lt;&gt;"")+($B$5:$B$504=B114)*(B114&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C114="Оплата",K114&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E114)&gt;0,ROUND(E114-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B114="",C114="",D114="",E114="",F114=""),"",IF(OR(B114="",C114="",E114=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E114)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H114&lt;&gt;0,F114=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G114&lt;&gt;0,F114=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F114&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F114)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C114)*($E$5:$E$504=E114)*(($D$5:$D$504=D114)*(D114&lt;&gt;"")+($B$5:$B$504=B114)*(B114&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C114="Оплата",K114&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E114)&gt;0,ROUND(E114-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J114" s="5">
@@ -3685,7 +3685,7 @@
         <v/>
       </c>
       <c r="I115" s="6">
-        <f>IF(AND(B115="",C115="",D115="",E115="",F115=""),"",IF(OR(B115="",C115="",E115=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E115)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H115&lt;&gt;0,F115=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G115&lt;&gt;0,F115=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F115&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F115)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C115)*($E$5:$E$504=E115)*(($D$5:$D$504=D115)*(D115&lt;&gt;"")+($B$5:$B$504=B115)*(B115&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C115="Оплата",K115&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E115)&gt;0,ROUND(E115-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B115="",C115="",D115="",E115="",F115=""),"",IF(OR(B115="",C115="",E115=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E115)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H115&lt;&gt;0,F115=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G115&lt;&gt;0,F115=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F115&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F115)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C115)*($E$5:$E$504=E115)*(($D$5:$D$504=D115)*(D115&lt;&gt;"")+($B$5:$B$504=B115)*(B115&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C115="Оплата",K115&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E115)&gt;0,ROUND(E115-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J115" s="5">
@@ -3712,7 +3712,7 @@
         <v/>
       </c>
       <c r="I116" s="6">
-        <f>IF(AND(B116="",C116="",D116="",E116="",F116=""),"",IF(OR(B116="",C116="",E116=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E116)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H116&lt;&gt;0,F116=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G116&lt;&gt;0,F116=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F116&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F116)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C116)*($E$5:$E$504=E116)*(($D$5:$D$504=D116)*(D116&lt;&gt;"")+($B$5:$B$504=B116)*(B116&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C116="Оплата",K116&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E116)&gt;0,ROUND(E116-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B116="",C116="",D116="",E116="",F116=""),"",IF(OR(B116="",C116="",E116=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E116)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H116&lt;&gt;0,F116=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G116&lt;&gt;0,F116=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F116&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F116)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C116)*($E$5:$E$504=E116)*(($D$5:$D$504=D116)*(D116&lt;&gt;"")+($B$5:$B$504=B116)*(B116&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C116="Оплата",K116&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E116)&gt;0,ROUND(E116-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J116" s="5">
@@ -3739,7 +3739,7 @@
         <v/>
       </c>
       <c r="I117" s="6">
-        <f>IF(AND(B117="",C117="",D117="",E117="",F117=""),"",IF(OR(B117="",C117="",E117=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E117)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H117&lt;&gt;0,F117=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G117&lt;&gt;0,F117=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F117&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F117)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C117)*($E$5:$E$504=E117)*(($D$5:$D$504=D117)*(D117&lt;&gt;"")+($B$5:$B$504=B117)*(B117&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C117="Оплата",K117&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E117)&gt;0,ROUND(E117-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B117="",C117="",D117="",E117="",F117=""),"",IF(OR(B117="",C117="",E117=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E117)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H117&lt;&gt;0,F117=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G117&lt;&gt;0,F117=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F117&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F117)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C117)*($E$5:$E$504=E117)*(($D$5:$D$504=D117)*(D117&lt;&gt;"")+($B$5:$B$504=B117)*(B117&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C117="Оплата",K117&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E117)&gt;0,ROUND(E117-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J117" s="5">
@@ -3766,7 +3766,7 @@
         <v/>
       </c>
       <c r="I118" s="6">
-        <f>IF(AND(B118="",C118="",D118="",E118="",F118=""),"",IF(OR(B118="",C118="",E118=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E118)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H118&lt;&gt;0,F118=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G118&lt;&gt;0,F118=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F118&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F118)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C118)*($E$5:$E$504=E118)*(($D$5:$D$504=D118)*(D118&lt;&gt;"")+($B$5:$B$504=B118)*(B118&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C118="Оплата",K118&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E118)&gt;0,ROUND(E118-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B118="",C118="",D118="",E118="",F118=""),"",IF(OR(B118="",C118="",E118=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E118)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H118&lt;&gt;0,F118=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G118&lt;&gt;0,F118=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F118&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F118)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C118)*($E$5:$E$504=E118)*(($D$5:$D$504=D118)*(D118&lt;&gt;"")+($B$5:$B$504=B118)*(B118&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C118="Оплата",K118&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E118)&gt;0,ROUND(E118-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J118" s="5">
@@ -3793,7 +3793,7 @@
         <v/>
       </c>
       <c r="I119" s="6">
-        <f>IF(AND(B119="",C119="",D119="",E119="",F119=""),"",IF(OR(B119="",C119="",E119=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E119)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H119&lt;&gt;0,F119=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G119&lt;&gt;0,F119=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F119&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F119)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C119)*($E$5:$E$504=E119)*(($D$5:$D$504=D119)*(D119&lt;&gt;"")+($B$5:$B$504=B119)*(B119&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C119="Оплата",K119&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E119)&gt;0,ROUND(E119-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B119="",C119="",D119="",E119="",F119=""),"",IF(OR(B119="",C119="",E119=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E119)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H119&lt;&gt;0,F119=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G119&lt;&gt;0,F119=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F119&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F119)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C119)*($E$5:$E$504=E119)*(($D$5:$D$504=D119)*(D119&lt;&gt;"")+($B$5:$B$504=B119)*(B119&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C119="Оплата",K119&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E119)&gt;0,ROUND(E119-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J119" s="5">
@@ -3820,7 +3820,7 @@
         <v/>
       </c>
       <c r="I120" s="6">
-        <f>IF(AND(B120="",C120="",D120="",E120="",F120=""),"",IF(OR(B120="",C120="",E120=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E120)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H120&lt;&gt;0,F120=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G120&lt;&gt;0,F120=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F120&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F120)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C120)*($E$5:$E$504=E120)*(($D$5:$D$504=D120)*(D120&lt;&gt;"")+($B$5:$B$504=B120)*(B120&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C120="Оплата",K120&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E120)&gt;0,ROUND(E120-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B120="",C120="",D120="",E120="",F120=""),"",IF(OR(B120="",C120="",E120=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E120)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H120&lt;&gt;0,F120=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G120&lt;&gt;0,F120=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F120&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F120)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C120)*($E$5:$E$504=E120)*(($D$5:$D$504=D120)*(D120&lt;&gt;"")+($B$5:$B$504=B120)*(B120&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C120="Оплата",K120&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E120)&gt;0,ROUND(E120-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J120" s="5">
@@ -3847,7 +3847,7 @@
         <v/>
       </c>
       <c r="I121" s="6">
-        <f>IF(AND(B121="",C121="",D121="",E121="",F121=""),"",IF(OR(B121="",C121="",E121=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E121)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H121&lt;&gt;0,F121=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G121&lt;&gt;0,F121=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F121&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F121)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C121)*($E$5:$E$504=E121)*(($D$5:$D$504=D121)*(D121&lt;&gt;"")+($B$5:$B$504=B121)*(B121&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C121="Оплата",K121&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E121)&gt;0,ROUND(E121-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B121="",C121="",D121="",E121="",F121=""),"",IF(OR(B121="",C121="",E121=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E121)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H121&lt;&gt;0,F121=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G121&lt;&gt;0,F121=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F121&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F121)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C121)*($E$5:$E$504=E121)*(($D$5:$D$504=D121)*(D121&lt;&gt;"")+($B$5:$B$504=B121)*(B121&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C121="Оплата",K121&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E121)&gt;0,ROUND(E121-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J121" s="5">
@@ -3874,7 +3874,7 @@
         <v/>
       </c>
       <c r="I122" s="6">
-        <f>IF(AND(B122="",C122="",D122="",E122="",F122=""),"",IF(OR(B122="",C122="",E122=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E122)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H122&lt;&gt;0,F122=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G122&lt;&gt;0,F122=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F122&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F122)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C122)*($E$5:$E$504=E122)*(($D$5:$D$504=D122)*(D122&lt;&gt;"")+($B$5:$B$504=B122)*(B122&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C122="Оплата",K122&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E122)&gt;0,ROUND(E122-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B122="",C122="",D122="",E122="",F122=""),"",IF(OR(B122="",C122="",E122=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E122)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H122&lt;&gt;0,F122=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G122&lt;&gt;0,F122=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F122&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F122)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C122)*($E$5:$E$504=E122)*(($D$5:$D$504=D122)*(D122&lt;&gt;"")+($B$5:$B$504=B122)*(B122&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C122="Оплата",K122&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E122)&gt;0,ROUND(E122-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J122" s="5">
@@ -3901,7 +3901,7 @@
         <v/>
       </c>
       <c r="I123" s="6">
-        <f>IF(AND(B123="",C123="",D123="",E123="",F123=""),"",IF(OR(B123="",C123="",E123=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E123)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H123&lt;&gt;0,F123=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G123&lt;&gt;0,F123=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F123&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F123)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C123)*($E$5:$E$504=E123)*(($D$5:$D$504=D123)*(D123&lt;&gt;"")+($B$5:$B$504=B123)*(B123&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C123="Оплата",K123&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E123)&gt;0,ROUND(E123-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B123="",C123="",D123="",E123="",F123=""),"",IF(OR(B123="",C123="",E123=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E123)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H123&lt;&gt;0,F123=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G123&lt;&gt;0,F123=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F123&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F123)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C123)*($E$5:$E$504=E123)*(($D$5:$D$504=D123)*(D123&lt;&gt;"")+($B$5:$B$504=B123)*(B123&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C123="Оплата",K123&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E123)&gt;0,ROUND(E123-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J123" s="5">
@@ -3928,7 +3928,7 @@
         <v/>
       </c>
       <c r="I124" s="6">
-        <f>IF(AND(B124="",C124="",D124="",E124="",F124=""),"",IF(OR(B124="",C124="",E124=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E124)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H124&lt;&gt;0,F124=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G124&lt;&gt;0,F124=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F124&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F124)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C124)*($E$5:$E$504=E124)*(($D$5:$D$504=D124)*(D124&lt;&gt;"")+($B$5:$B$504=B124)*(B124&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C124="Оплата",K124&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E124)&gt;0,ROUND(E124-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B124="",C124="",D124="",E124="",F124=""),"",IF(OR(B124="",C124="",E124=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E124)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H124&lt;&gt;0,F124=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G124&lt;&gt;0,F124=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F124&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F124)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C124)*($E$5:$E$504=E124)*(($D$5:$D$504=D124)*(D124&lt;&gt;"")+($B$5:$B$504=B124)*(B124&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C124="Оплата",K124&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E124)&gt;0,ROUND(E124-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J124" s="5">
@@ -3955,7 +3955,7 @@
         <v/>
       </c>
       <c r="I125" s="6">
-        <f>IF(AND(B125="",C125="",D125="",E125="",F125=""),"",IF(OR(B125="",C125="",E125=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E125)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H125&lt;&gt;0,F125=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G125&lt;&gt;0,F125=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F125&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F125)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C125)*($E$5:$E$504=E125)*(($D$5:$D$504=D125)*(D125&lt;&gt;"")+($B$5:$B$504=B125)*(B125&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C125="Оплата",K125&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E125)&gt;0,ROUND(E125-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B125="",C125="",D125="",E125="",F125=""),"",IF(OR(B125="",C125="",E125=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E125)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H125&lt;&gt;0,F125=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G125&lt;&gt;0,F125=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F125&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F125)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C125)*($E$5:$E$504=E125)*(($D$5:$D$504=D125)*(D125&lt;&gt;"")+($B$5:$B$504=B125)*(B125&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C125="Оплата",K125&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E125)&gt;0,ROUND(E125-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J125" s="5">
@@ -3982,7 +3982,7 @@
         <v/>
       </c>
       <c r="I126" s="6">
-        <f>IF(AND(B126="",C126="",D126="",E126="",F126=""),"",IF(OR(B126="",C126="",E126=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E126)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H126&lt;&gt;0,F126=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G126&lt;&gt;0,F126=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F126&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F126)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C126)*($E$5:$E$504=E126)*(($D$5:$D$504=D126)*(D126&lt;&gt;"")+($B$5:$B$504=B126)*(B126&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C126="Оплата",K126&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E126)&gt;0,ROUND(E126-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B126="",C126="",D126="",E126="",F126=""),"",IF(OR(B126="",C126="",E126=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E126)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H126&lt;&gt;0,F126=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G126&lt;&gt;0,F126=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F126&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F126)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C126)*($E$5:$E$504=E126)*(($D$5:$D$504=D126)*(D126&lt;&gt;"")+($B$5:$B$504=B126)*(B126&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C126="Оплата",K126&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E126)&gt;0,ROUND(E126-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J126" s="5">
@@ -4009,7 +4009,7 @@
         <v/>
       </c>
       <c r="I127" s="6">
-        <f>IF(AND(B127="",C127="",D127="",E127="",F127=""),"",IF(OR(B127="",C127="",E127=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E127)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H127&lt;&gt;0,F127=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G127&lt;&gt;0,F127=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F127&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F127)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C127)*($E$5:$E$504=E127)*(($D$5:$D$504=D127)*(D127&lt;&gt;"")+($B$5:$B$504=B127)*(B127&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C127="Оплата",K127&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E127)&gt;0,ROUND(E127-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B127="",C127="",D127="",E127="",F127=""),"",IF(OR(B127="",C127="",E127=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E127)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H127&lt;&gt;0,F127=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G127&lt;&gt;0,F127=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F127&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F127)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C127)*($E$5:$E$504=E127)*(($D$5:$D$504=D127)*(D127&lt;&gt;"")+($B$5:$B$504=B127)*(B127&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C127="Оплата",K127&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E127)&gt;0,ROUND(E127-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J127" s="5">
@@ -4036,7 +4036,7 @@
         <v/>
       </c>
       <c r="I128" s="6">
-        <f>IF(AND(B128="",C128="",D128="",E128="",F128=""),"",IF(OR(B128="",C128="",E128=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E128)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H128&lt;&gt;0,F128=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G128&lt;&gt;0,F128=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F128&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F128)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C128)*($E$5:$E$504=E128)*(($D$5:$D$504=D128)*(D128&lt;&gt;"")+($B$5:$B$504=B128)*(B128&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C128="Оплата",K128&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E128)&gt;0,ROUND(E128-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B128="",C128="",D128="",E128="",F128=""),"",IF(OR(B128="",C128="",E128=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E128)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H128&lt;&gt;0,F128=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G128&lt;&gt;0,F128=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F128&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F128)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C128)*($E$5:$E$504=E128)*(($D$5:$D$504=D128)*(D128&lt;&gt;"")+($B$5:$B$504=B128)*(B128&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C128="Оплата",K128&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E128)&gt;0,ROUND(E128-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J128" s="5">
@@ -4063,7 +4063,7 @@
         <v/>
       </c>
       <c r="I129" s="6">
-        <f>IF(AND(B129="",C129="",D129="",E129="",F129=""),"",IF(OR(B129="",C129="",E129=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E129)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H129&lt;&gt;0,F129=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G129&lt;&gt;0,F129=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F129&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F129)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C129)*($E$5:$E$504=E129)*(($D$5:$D$504=D129)*(D129&lt;&gt;"")+($B$5:$B$504=B129)*(B129&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C129="Оплата",K129&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E129)&gt;0,ROUND(E129-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B129="",C129="",D129="",E129="",F129=""),"",IF(OR(B129="",C129="",E129=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E129)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H129&lt;&gt;0,F129=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G129&lt;&gt;0,F129=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F129&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F129)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C129)*($E$5:$E$504=E129)*(($D$5:$D$504=D129)*(D129&lt;&gt;"")+($B$5:$B$504=B129)*(B129&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C129="Оплата",K129&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E129)&gt;0,ROUND(E129-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J129" s="5">
@@ -4090,7 +4090,7 @@
         <v/>
       </c>
       <c r="I130" s="6">
-        <f>IF(AND(B130="",C130="",D130="",E130="",F130=""),"",IF(OR(B130="",C130="",E130=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E130)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H130&lt;&gt;0,F130=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G130&lt;&gt;0,F130=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F130&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F130)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C130)*($E$5:$E$504=E130)*(($D$5:$D$504=D130)*(D130&lt;&gt;"")+($B$5:$B$504=B130)*(B130&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C130="Оплата",K130&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E130)&gt;0,ROUND(E130-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B130="",C130="",D130="",E130="",F130=""),"",IF(OR(B130="",C130="",E130=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E130)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H130&lt;&gt;0,F130=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G130&lt;&gt;0,F130=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F130&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F130)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C130)*($E$5:$E$504=E130)*(($D$5:$D$504=D130)*(D130&lt;&gt;"")+($B$5:$B$504=B130)*(B130&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C130="Оплата",K130&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E130)&gt;0,ROUND(E130-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J130" s="5">
@@ -4117,7 +4117,7 @@
         <v/>
       </c>
       <c r="I131" s="6">
-        <f>IF(AND(B131="",C131="",D131="",E131="",F131=""),"",IF(OR(B131="",C131="",E131=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E131)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H131&lt;&gt;0,F131=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G131&lt;&gt;0,F131=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F131&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F131)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C131)*($E$5:$E$504=E131)*(($D$5:$D$504=D131)*(D131&lt;&gt;"")+($B$5:$B$504=B131)*(B131&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C131="Оплата",K131&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E131)&gt;0,ROUND(E131-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B131="",C131="",D131="",E131="",F131=""),"",IF(OR(B131="",C131="",E131=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E131)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H131&lt;&gt;0,F131=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G131&lt;&gt;0,F131=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F131&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F131)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C131)*($E$5:$E$504=E131)*(($D$5:$D$504=D131)*(D131&lt;&gt;"")+($B$5:$B$504=B131)*(B131&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C131="Оплата",K131&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E131)&gt;0,ROUND(E131-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J131" s="5">
@@ -4144,7 +4144,7 @@
         <v/>
       </c>
       <c r="I132" s="6">
-        <f>IF(AND(B132="",C132="",D132="",E132="",F132=""),"",IF(OR(B132="",C132="",E132=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E132)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H132&lt;&gt;0,F132=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G132&lt;&gt;0,F132=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F132&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F132)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C132)*($E$5:$E$504=E132)*(($D$5:$D$504=D132)*(D132&lt;&gt;"")+($B$5:$B$504=B132)*(B132&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C132="Оплата",K132&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E132)&gt;0,ROUND(E132-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B132="",C132="",D132="",E132="",F132=""),"",IF(OR(B132="",C132="",E132=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E132)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H132&lt;&gt;0,F132=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G132&lt;&gt;0,F132=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F132&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F132)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C132)*($E$5:$E$504=E132)*(($D$5:$D$504=D132)*(D132&lt;&gt;"")+($B$5:$B$504=B132)*(B132&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C132="Оплата",K132&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E132)&gt;0,ROUND(E132-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J132" s="5">
@@ -4171,7 +4171,7 @@
         <v/>
       </c>
       <c r="I133" s="6">
-        <f>IF(AND(B133="",C133="",D133="",E133="",F133=""),"",IF(OR(B133="",C133="",E133=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E133)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H133&lt;&gt;0,F133=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G133&lt;&gt;0,F133=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F133&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F133)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C133)*($E$5:$E$504=E133)*(($D$5:$D$504=D133)*(D133&lt;&gt;"")+($B$5:$B$504=B133)*(B133&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C133="Оплата",K133&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E133)&gt;0,ROUND(E133-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B133="",C133="",D133="",E133="",F133=""),"",IF(OR(B133="",C133="",E133=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E133)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H133&lt;&gt;0,F133=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G133&lt;&gt;0,F133=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F133&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F133)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C133)*($E$5:$E$504=E133)*(($D$5:$D$504=D133)*(D133&lt;&gt;"")+($B$5:$B$504=B133)*(B133&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C133="Оплата",K133&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E133)&gt;0,ROUND(E133-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J133" s="5">
@@ -4198,7 +4198,7 @@
         <v/>
       </c>
       <c r="I134" s="6">
-        <f>IF(AND(B134="",C134="",D134="",E134="",F134=""),"",IF(OR(B134="",C134="",E134=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E134)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H134&lt;&gt;0,F134=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G134&lt;&gt;0,F134=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F134&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F134)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C134)*($E$5:$E$504=E134)*(($D$5:$D$504=D134)*(D134&lt;&gt;"")+($B$5:$B$504=B134)*(B134&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C134="Оплата",K134&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E134)&gt;0,ROUND(E134-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B134="",C134="",D134="",E134="",F134=""),"",IF(OR(B134="",C134="",E134=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E134)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H134&lt;&gt;0,F134=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G134&lt;&gt;0,F134=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F134&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F134)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C134)*($E$5:$E$504=E134)*(($D$5:$D$504=D134)*(D134&lt;&gt;"")+($B$5:$B$504=B134)*(B134&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C134="Оплата",K134&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E134)&gt;0,ROUND(E134-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J134" s="5">
@@ -4225,7 +4225,7 @@
         <v/>
       </c>
       <c r="I135" s="6">
-        <f>IF(AND(B135="",C135="",D135="",E135="",F135=""),"",IF(OR(B135="",C135="",E135=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E135)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H135&lt;&gt;0,F135=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G135&lt;&gt;0,F135=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F135&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F135)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C135)*($E$5:$E$504=E135)*(($D$5:$D$504=D135)*(D135&lt;&gt;"")+($B$5:$B$504=B135)*(B135&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C135="Оплата",K135&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E135)&gt;0,ROUND(E135-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B135="",C135="",D135="",E135="",F135=""),"",IF(OR(B135="",C135="",E135=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E135)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H135&lt;&gt;0,F135=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G135&lt;&gt;0,F135=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F135&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F135)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C135)*($E$5:$E$504=E135)*(($D$5:$D$504=D135)*(D135&lt;&gt;"")+($B$5:$B$504=B135)*(B135&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C135="Оплата",K135&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E135)&gt;0,ROUND(E135-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J135" s="5">
@@ -4252,7 +4252,7 @@
         <v/>
       </c>
       <c r="I136" s="6">
-        <f>IF(AND(B136="",C136="",D136="",E136="",F136=""),"",IF(OR(B136="",C136="",E136=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E136)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H136&lt;&gt;0,F136=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G136&lt;&gt;0,F136=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F136&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F136)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C136)*($E$5:$E$504=E136)*(($D$5:$D$504=D136)*(D136&lt;&gt;"")+($B$5:$B$504=B136)*(B136&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C136="Оплата",K136&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E136)&gt;0,ROUND(E136-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B136="",C136="",D136="",E136="",F136=""),"",IF(OR(B136="",C136="",E136=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E136)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H136&lt;&gt;0,F136=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G136&lt;&gt;0,F136=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F136&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F136)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C136)*($E$5:$E$504=E136)*(($D$5:$D$504=D136)*(D136&lt;&gt;"")+($B$5:$B$504=B136)*(B136&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C136="Оплата",K136&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E136)&gt;0,ROUND(E136-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J136" s="5">
@@ -4279,7 +4279,7 @@
         <v/>
       </c>
       <c r="I137" s="6">
-        <f>IF(AND(B137="",C137="",D137="",E137="",F137=""),"",IF(OR(B137="",C137="",E137=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E137)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H137&lt;&gt;0,F137=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G137&lt;&gt;0,F137=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F137&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F137)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C137)*($E$5:$E$504=E137)*(($D$5:$D$504=D137)*(D137&lt;&gt;"")+($B$5:$B$504=B137)*(B137&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C137="Оплата",K137&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E137)&gt;0,ROUND(E137-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B137="",C137="",D137="",E137="",F137=""),"",IF(OR(B137="",C137="",E137=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E137)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H137&lt;&gt;0,F137=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G137&lt;&gt;0,F137=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F137&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F137)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C137)*($E$5:$E$504=E137)*(($D$5:$D$504=D137)*(D137&lt;&gt;"")+($B$5:$B$504=B137)*(B137&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C137="Оплата",K137&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E137)&gt;0,ROUND(E137-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J137" s="5">
@@ -4306,7 +4306,7 @@
         <v/>
       </c>
       <c r="I138" s="6">
-        <f>IF(AND(B138="",C138="",D138="",E138="",F138=""),"",IF(OR(B138="",C138="",E138=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E138)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H138&lt;&gt;0,F138=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G138&lt;&gt;0,F138=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F138&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F138)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C138)*($E$5:$E$504=E138)*(($D$5:$D$504=D138)*(D138&lt;&gt;"")+($B$5:$B$504=B138)*(B138&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C138="Оплата",K138&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E138)&gt;0,ROUND(E138-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B138="",C138="",D138="",E138="",F138=""),"",IF(OR(B138="",C138="",E138=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E138)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H138&lt;&gt;0,F138=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G138&lt;&gt;0,F138=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F138&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F138)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C138)*($E$5:$E$504=E138)*(($D$5:$D$504=D138)*(D138&lt;&gt;"")+($B$5:$B$504=B138)*(B138&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C138="Оплата",K138&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E138)&gt;0,ROUND(E138-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J138" s="5">
@@ -4333,7 +4333,7 @@
         <v/>
       </c>
       <c r="I139" s="6">
-        <f>IF(AND(B139="",C139="",D139="",E139="",F139=""),"",IF(OR(B139="",C139="",E139=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E139)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H139&lt;&gt;0,F139=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G139&lt;&gt;0,F139=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F139&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F139)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C139)*($E$5:$E$504=E139)*(($D$5:$D$504=D139)*(D139&lt;&gt;"")+($B$5:$B$504=B139)*(B139&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C139="Оплата",K139&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E139)&gt;0,ROUND(E139-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B139="",C139="",D139="",E139="",F139=""),"",IF(OR(B139="",C139="",E139=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E139)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H139&lt;&gt;0,F139=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G139&lt;&gt;0,F139=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F139&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F139)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C139)*($E$5:$E$504=E139)*(($D$5:$D$504=D139)*(D139&lt;&gt;"")+($B$5:$B$504=B139)*(B139&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C139="Оплата",K139&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E139)&gt;0,ROUND(E139-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J139" s="5">
@@ -4360,7 +4360,7 @@
         <v/>
       </c>
       <c r="I140" s="6">
-        <f>IF(AND(B140="",C140="",D140="",E140="",F140=""),"",IF(OR(B140="",C140="",E140=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E140)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H140&lt;&gt;0,F140=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G140&lt;&gt;0,F140=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F140&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F140)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C140)*($E$5:$E$504=E140)*(($D$5:$D$504=D140)*(D140&lt;&gt;"")+($B$5:$B$504=B140)*(B140&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C140="Оплата",K140&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E140)&gt;0,ROUND(E140-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B140="",C140="",D140="",E140="",F140=""),"",IF(OR(B140="",C140="",E140=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E140)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H140&lt;&gt;0,F140=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G140&lt;&gt;0,F140=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F140&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F140)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C140)*($E$5:$E$504=E140)*(($D$5:$D$504=D140)*(D140&lt;&gt;"")+($B$5:$B$504=B140)*(B140&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C140="Оплата",K140&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E140)&gt;0,ROUND(E140-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J140" s="5">
@@ -4387,7 +4387,7 @@
         <v/>
       </c>
       <c r="I141" s="6">
-        <f>IF(AND(B141="",C141="",D141="",E141="",F141=""),"",IF(OR(B141="",C141="",E141=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E141)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H141&lt;&gt;0,F141=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G141&lt;&gt;0,F141=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F141&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F141)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C141)*($E$5:$E$504=E141)*(($D$5:$D$504=D141)*(D141&lt;&gt;"")+($B$5:$B$504=B141)*(B141&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C141="Оплата",K141&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E141)&gt;0,ROUND(E141-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B141="",C141="",D141="",E141="",F141=""),"",IF(OR(B141="",C141="",E141=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E141)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H141&lt;&gt;0,F141=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G141&lt;&gt;0,F141=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F141&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F141)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C141)*($E$5:$E$504=E141)*(($D$5:$D$504=D141)*(D141&lt;&gt;"")+($B$5:$B$504=B141)*(B141&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C141="Оплата",K141&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E141)&gt;0,ROUND(E141-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J141" s="5">
@@ -4414,7 +4414,7 @@
         <v/>
       </c>
       <c r="I142" s="6">
-        <f>IF(AND(B142="",C142="",D142="",E142="",F142=""),"",IF(OR(B142="",C142="",E142=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E142)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H142&lt;&gt;0,F142=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G142&lt;&gt;0,F142=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F142&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F142)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C142)*($E$5:$E$504=E142)*(($D$5:$D$504=D142)*(D142&lt;&gt;"")+($B$5:$B$504=B142)*(B142&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C142="Оплата",K142&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E142)&gt;0,ROUND(E142-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B142="",C142="",D142="",E142="",F142=""),"",IF(OR(B142="",C142="",E142=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E142)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H142&lt;&gt;0,F142=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G142&lt;&gt;0,F142=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F142&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F142)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C142)*($E$5:$E$504=E142)*(($D$5:$D$504=D142)*(D142&lt;&gt;"")+($B$5:$B$504=B142)*(B142&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C142="Оплата",K142&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E142)&gt;0,ROUND(E142-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J142" s="5">
@@ -4441,7 +4441,7 @@
         <v/>
       </c>
       <c r="I143" s="6">
-        <f>IF(AND(B143="",C143="",D143="",E143="",F143=""),"",IF(OR(B143="",C143="",E143=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E143)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H143&lt;&gt;0,F143=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G143&lt;&gt;0,F143=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F143&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F143)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C143)*($E$5:$E$504=E143)*(($D$5:$D$504=D143)*(D143&lt;&gt;"")+($B$5:$B$504=B143)*(B143&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C143="Оплата",K143&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E143)&gt;0,ROUND(E143-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B143="",C143="",D143="",E143="",F143=""),"",IF(OR(B143="",C143="",E143=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E143)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H143&lt;&gt;0,F143=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G143&lt;&gt;0,F143=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F143&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F143)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C143)*($E$5:$E$504=E143)*(($D$5:$D$504=D143)*(D143&lt;&gt;"")+($B$5:$B$504=B143)*(B143&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C143="Оплата",K143&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E143)&gt;0,ROUND(E143-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J143" s="5">
@@ -4468,7 +4468,7 @@
         <v/>
       </c>
       <c r="I144" s="6">
-        <f>IF(AND(B144="",C144="",D144="",E144="",F144=""),"",IF(OR(B144="",C144="",E144=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E144)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H144&lt;&gt;0,F144=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G144&lt;&gt;0,F144=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F144&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F144)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C144)*($E$5:$E$504=E144)*(($D$5:$D$504=D144)*(D144&lt;&gt;"")+($B$5:$B$504=B144)*(B144&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C144="Оплата",K144&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E144)&gt;0,ROUND(E144-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B144="",C144="",D144="",E144="",F144=""),"",IF(OR(B144="",C144="",E144=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E144)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H144&lt;&gt;0,F144=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G144&lt;&gt;0,F144=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F144&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F144)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C144)*($E$5:$E$504=E144)*(($D$5:$D$504=D144)*(D144&lt;&gt;"")+($B$5:$B$504=B144)*(B144&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C144="Оплата",K144&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E144)&gt;0,ROUND(E144-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J144" s="5">
@@ -4495,7 +4495,7 @@
         <v/>
       </c>
       <c r="I145" s="6">
-        <f>IF(AND(B145="",C145="",D145="",E145="",F145=""),"",IF(OR(B145="",C145="",E145=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E145)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H145&lt;&gt;0,F145=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G145&lt;&gt;0,F145=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F145&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F145)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C145)*($E$5:$E$504=E145)*(($D$5:$D$504=D145)*(D145&lt;&gt;"")+($B$5:$B$504=B145)*(B145&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C145="Оплата",K145&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E145)&gt;0,ROUND(E145-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B145="",C145="",D145="",E145="",F145=""),"",IF(OR(B145="",C145="",E145=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E145)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H145&lt;&gt;0,F145=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G145&lt;&gt;0,F145=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F145&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F145)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C145)*($E$5:$E$504=E145)*(($D$5:$D$504=D145)*(D145&lt;&gt;"")+($B$5:$B$504=B145)*(B145&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C145="Оплата",K145&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E145)&gt;0,ROUND(E145-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J145" s="5">
@@ -4522,7 +4522,7 @@
         <v/>
       </c>
       <c r="I146" s="6">
-        <f>IF(AND(B146="",C146="",D146="",E146="",F146=""),"",IF(OR(B146="",C146="",E146=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E146)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H146&lt;&gt;0,F146=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G146&lt;&gt;0,F146=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F146&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F146)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C146)*($E$5:$E$504=E146)*(($D$5:$D$504=D146)*(D146&lt;&gt;"")+($B$5:$B$504=B146)*(B146&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C146="Оплата",K146&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E146)&gt;0,ROUND(E146-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B146="",C146="",D146="",E146="",F146=""),"",IF(OR(B146="",C146="",E146=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E146)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H146&lt;&gt;0,F146=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G146&lt;&gt;0,F146=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F146&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F146)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C146)*($E$5:$E$504=E146)*(($D$5:$D$504=D146)*(D146&lt;&gt;"")+($B$5:$B$504=B146)*(B146&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C146="Оплата",K146&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E146)&gt;0,ROUND(E146-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J146" s="5">
@@ -4549,7 +4549,7 @@
         <v/>
       </c>
       <c r="I147" s="6">
-        <f>IF(AND(B147="",C147="",D147="",E147="",F147=""),"",IF(OR(B147="",C147="",E147=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E147)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H147&lt;&gt;0,F147=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G147&lt;&gt;0,F147=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F147&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F147)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C147)*($E$5:$E$504=E147)*(($D$5:$D$504=D147)*(D147&lt;&gt;"")+($B$5:$B$504=B147)*(B147&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C147="Оплата",K147&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E147)&gt;0,ROUND(E147-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B147="",C147="",D147="",E147="",F147=""),"",IF(OR(B147="",C147="",E147=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E147)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H147&lt;&gt;0,F147=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G147&lt;&gt;0,F147=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F147&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F147)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C147)*($E$5:$E$504=E147)*(($D$5:$D$504=D147)*(D147&lt;&gt;"")+($B$5:$B$504=B147)*(B147&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C147="Оплата",K147&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E147)&gt;0,ROUND(E147-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J147" s="5">
@@ -4576,7 +4576,7 @@
         <v/>
       </c>
       <c r="I148" s="6">
-        <f>IF(AND(B148="",C148="",D148="",E148="",F148=""),"",IF(OR(B148="",C148="",E148=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E148)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H148&lt;&gt;0,F148=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G148&lt;&gt;0,F148=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F148&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F148)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C148)*($E$5:$E$504=E148)*(($D$5:$D$504=D148)*(D148&lt;&gt;"")+($B$5:$B$504=B148)*(B148&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C148="Оплата",K148&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E148)&gt;0,ROUND(E148-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B148="",C148="",D148="",E148="",F148=""),"",IF(OR(B148="",C148="",E148=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E148)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H148&lt;&gt;0,F148=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G148&lt;&gt;0,F148=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F148&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F148)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C148)*($E$5:$E$504=E148)*(($D$5:$D$504=D148)*(D148&lt;&gt;"")+($B$5:$B$504=B148)*(B148&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C148="Оплата",K148&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E148)&gt;0,ROUND(E148-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J148" s="5">
@@ -4603,7 +4603,7 @@
         <v/>
       </c>
       <c r="I149" s="6">
-        <f>IF(AND(B149="",C149="",D149="",E149="",F149=""),"",IF(OR(B149="",C149="",E149=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E149)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H149&lt;&gt;0,F149=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G149&lt;&gt;0,F149=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F149&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F149)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C149)*($E$5:$E$504=E149)*(($D$5:$D$504=D149)*(D149&lt;&gt;"")+($B$5:$B$504=B149)*(B149&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C149="Оплата",K149&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E149)&gt;0,ROUND(E149-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B149="",C149="",D149="",E149="",F149=""),"",IF(OR(B149="",C149="",E149=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E149)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H149&lt;&gt;0,F149=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G149&lt;&gt;0,F149=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F149&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F149)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C149)*($E$5:$E$504=E149)*(($D$5:$D$504=D149)*(D149&lt;&gt;"")+($B$5:$B$504=B149)*(B149&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C149="Оплата",K149&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E149)&gt;0,ROUND(E149-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J149" s="5">
@@ -4630,7 +4630,7 @@
         <v/>
       </c>
       <c r="I150" s="6">
-        <f>IF(AND(B150="",C150="",D150="",E150="",F150=""),"",IF(OR(B150="",C150="",E150=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E150)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H150&lt;&gt;0,F150=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G150&lt;&gt;0,F150=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F150&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F150)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C150)*($E$5:$E$504=E150)*(($D$5:$D$504=D150)*(D150&lt;&gt;"")+($B$5:$B$504=B150)*(B150&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C150="Оплата",K150&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E150)&gt;0,ROUND(E150-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B150="",C150="",D150="",E150="",F150=""),"",IF(OR(B150="",C150="",E150=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E150)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H150&lt;&gt;0,F150=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G150&lt;&gt;0,F150=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F150&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F150)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C150)*($E$5:$E$504=E150)*(($D$5:$D$504=D150)*(D150&lt;&gt;"")+($B$5:$B$504=B150)*(B150&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C150="Оплата",K150&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E150)&gt;0,ROUND(E150-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J150" s="5">
@@ -4657,7 +4657,7 @@
         <v/>
       </c>
       <c r="I151" s="6">
-        <f>IF(AND(B151="",C151="",D151="",E151="",F151=""),"",IF(OR(B151="",C151="",E151=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E151)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H151&lt;&gt;0,F151=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G151&lt;&gt;0,F151=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F151&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F151)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C151)*($E$5:$E$504=E151)*(($D$5:$D$504=D151)*(D151&lt;&gt;"")+($B$5:$B$504=B151)*(B151&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C151="Оплата",K151&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E151)&gt;0,ROUND(E151-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B151="",C151="",D151="",E151="",F151=""),"",IF(OR(B151="",C151="",E151=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E151)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H151&lt;&gt;0,F151=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G151&lt;&gt;0,F151=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F151&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F151)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C151)*($E$5:$E$504=E151)*(($D$5:$D$504=D151)*(D151&lt;&gt;"")+($B$5:$B$504=B151)*(B151&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C151="Оплата",K151&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E151)&gt;0,ROUND(E151-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J151" s="5">
@@ -4684,7 +4684,7 @@
         <v/>
       </c>
       <c r="I152" s="6">
-        <f>IF(AND(B152="",C152="",D152="",E152="",F152=""),"",IF(OR(B152="",C152="",E152=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E152)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H152&lt;&gt;0,F152=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G152&lt;&gt;0,F152=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F152&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F152)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C152)*($E$5:$E$504=E152)*(($D$5:$D$504=D152)*(D152&lt;&gt;"")+($B$5:$B$504=B152)*(B152&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C152="Оплата",K152&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E152)&gt;0,ROUND(E152-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B152="",C152="",D152="",E152="",F152=""),"",IF(OR(B152="",C152="",E152=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E152)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H152&lt;&gt;0,F152=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G152&lt;&gt;0,F152=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F152&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F152)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C152)*($E$5:$E$504=E152)*(($D$5:$D$504=D152)*(D152&lt;&gt;"")+($B$5:$B$504=B152)*(B152&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C152="Оплата",K152&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E152)&gt;0,ROUND(E152-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J152" s="5">
@@ -4711,7 +4711,7 @@
         <v/>
       </c>
       <c r="I153" s="6">
-        <f>IF(AND(B153="",C153="",D153="",E153="",F153=""),"",IF(OR(B153="",C153="",E153=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E153)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H153&lt;&gt;0,F153=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G153&lt;&gt;0,F153=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F153&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F153)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C153)*($E$5:$E$504=E153)*(($D$5:$D$504=D153)*(D153&lt;&gt;"")+($B$5:$B$504=B153)*(B153&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C153="Оплата",K153&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E153)&gt;0,ROUND(E153-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B153="",C153="",D153="",E153="",F153=""),"",IF(OR(B153="",C153="",E153=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E153)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H153&lt;&gt;0,F153=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G153&lt;&gt;0,F153=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F153&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F153)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C153)*($E$5:$E$504=E153)*(($D$5:$D$504=D153)*(D153&lt;&gt;"")+($B$5:$B$504=B153)*(B153&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C153="Оплата",K153&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E153)&gt;0,ROUND(E153-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J153" s="5">
@@ -4738,7 +4738,7 @@
         <v/>
       </c>
       <c r="I154" s="6">
-        <f>IF(AND(B154="",C154="",D154="",E154="",F154=""),"",IF(OR(B154="",C154="",E154=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E154)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H154&lt;&gt;0,F154=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G154&lt;&gt;0,F154=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F154&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F154)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C154)*($E$5:$E$504=E154)*(($D$5:$D$504=D154)*(D154&lt;&gt;"")+($B$5:$B$504=B154)*(B154&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C154="Оплата",K154&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E154)&gt;0,ROUND(E154-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B154="",C154="",D154="",E154="",F154=""),"",IF(OR(B154="",C154="",E154=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E154)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H154&lt;&gt;0,F154=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G154&lt;&gt;0,F154=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F154&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F154)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C154)*($E$5:$E$504=E154)*(($D$5:$D$504=D154)*(D154&lt;&gt;"")+($B$5:$B$504=B154)*(B154&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C154="Оплата",K154&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E154)&gt;0,ROUND(E154-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J154" s="5">
@@ -4765,7 +4765,7 @@
         <v/>
       </c>
       <c r="I155" s="6">
-        <f>IF(AND(B155="",C155="",D155="",E155="",F155=""),"",IF(OR(B155="",C155="",E155=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E155)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H155&lt;&gt;0,F155=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G155&lt;&gt;0,F155=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F155&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F155)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C155)*($E$5:$E$504=E155)*(($D$5:$D$504=D155)*(D155&lt;&gt;"")+($B$5:$B$504=B155)*(B155&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C155="Оплата",K155&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E155)&gt;0,ROUND(E155-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B155="",C155="",D155="",E155="",F155=""),"",IF(OR(B155="",C155="",E155=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E155)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H155&lt;&gt;0,F155=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G155&lt;&gt;0,F155=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F155&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F155)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C155)*($E$5:$E$504=E155)*(($D$5:$D$504=D155)*(D155&lt;&gt;"")+($B$5:$B$504=B155)*(B155&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C155="Оплата",K155&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E155)&gt;0,ROUND(E155-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J155" s="5">
@@ -4792,7 +4792,7 @@
         <v/>
       </c>
       <c r="I156" s="6">
-        <f>IF(AND(B156="",C156="",D156="",E156="",F156=""),"",IF(OR(B156="",C156="",E156=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E156)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H156&lt;&gt;0,F156=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G156&lt;&gt;0,F156=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F156&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F156)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C156)*($E$5:$E$504=E156)*(($D$5:$D$504=D156)*(D156&lt;&gt;"")+($B$5:$B$504=B156)*(B156&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C156="Оплата",K156&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E156)&gt;0,ROUND(E156-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B156="",C156="",D156="",E156="",F156=""),"",IF(OR(B156="",C156="",E156=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E156)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H156&lt;&gt;0,F156=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G156&lt;&gt;0,F156=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F156&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F156)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C156)*($E$5:$E$504=E156)*(($D$5:$D$504=D156)*(D156&lt;&gt;"")+($B$5:$B$504=B156)*(B156&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C156="Оплата",K156&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E156)&gt;0,ROUND(E156-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J156" s="5">
@@ -4819,7 +4819,7 @@
         <v/>
       </c>
       <c r="I157" s="6">
-        <f>IF(AND(B157="",C157="",D157="",E157="",F157=""),"",IF(OR(B157="",C157="",E157=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E157)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H157&lt;&gt;0,F157=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G157&lt;&gt;0,F157=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F157&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F157)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C157)*($E$5:$E$504=E157)*(($D$5:$D$504=D157)*(D157&lt;&gt;"")+($B$5:$B$504=B157)*(B157&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C157="Оплата",K157&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E157)&gt;0,ROUND(E157-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B157="",C157="",D157="",E157="",F157=""),"",IF(OR(B157="",C157="",E157=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E157)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H157&lt;&gt;0,F157=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G157&lt;&gt;0,F157=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F157&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F157)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C157)*($E$5:$E$504=E157)*(($D$5:$D$504=D157)*(D157&lt;&gt;"")+($B$5:$B$504=B157)*(B157&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C157="Оплата",K157&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E157)&gt;0,ROUND(E157-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J157" s="5">
@@ -4846,7 +4846,7 @@
         <v/>
       </c>
       <c r="I158" s="6">
-        <f>IF(AND(B158="",C158="",D158="",E158="",F158=""),"",IF(OR(B158="",C158="",E158=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E158)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H158&lt;&gt;0,F158=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G158&lt;&gt;0,F158=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F158&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F158)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C158)*($E$5:$E$504=E158)*(($D$5:$D$504=D158)*(D158&lt;&gt;"")+($B$5:$B$504=B158)*(B158&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C158="Оплата",K158&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E158)&gt;0,ROUND(E158-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B158="",C158="",D158="",E158="",F158=""),"",IF(OR(B158="",C158="",E158=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E158)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H158&lt;&gt;0,F158=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G158&lt;&gt;0,F158=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F158&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F158)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C158)*($E$5:$E$504=E158)*(($D$5:$D$504=D158)*(D158&lt;&gt;"")+($B$5:$B$504=B158)*(B158&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C158="Оплата",K158&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E158)&gt;0,ROUND(E158-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J158" s="5">
@@ -4873,7 +4873,7 @@
         <v/>
       </c>
       <c r="I159" s="6">
-        <f>IF(AND(B159="",C159="",D159="",E159="",F159=""),"",IF(OR(B159="",C159="",E159=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E159)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H159&lt;&gt;0,F159=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G159&lt;&gt;0,F159=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F159&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F159)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C159)*($E$5:$E$504=E159)*(($D$5:$D$504=D159)*(D159&lt;&gt;"")+($B$5:$B$504=B159)*(B159&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C159="Оплата",K159&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E159)&gt;0,ROUND(E159-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B159="",C159="",D159="",E159="",F159=""),"",IF(OR(B159="",C159="",E159=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E159)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H159&lt;&gt;0,F159=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G159&lt;&gt;0,F159=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F159&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F159)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C159)*($E$5:$E$504=E159)*(($D$5:$D$504=D159)*(D159&lt;&gt;"")+($B$5:$B$504=B159)*(B159&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C159="Оплата",K159&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E159)&gt;0,ROUND(E159-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J159" s="5">
@@ -4900,7 +4900,7 @@
         <v/>
       </c>
       <c r="I160" s="6">
-        <f>IF(AND(B160="",C160="",D160="",E160="",F160=""),"",IF(OR(B160="",C160="",E160=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E160)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H160&lt;&gt;0,F160=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G160&lt;&gt;0,F160=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F160&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F160)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C160)*($E$5:$E$504=E160)*(($D$5:$D$504=D160)*(D160&lt;&gt;"")+($B$5:$B$504=B160)*(B160&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C160="Оплата",K160&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E160)&gt;0,ROUND(E160-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B160="",C160="",D160="",E160="",F160=""),"",IF(OR(B160="",C160="",E160=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E160)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H160&lt;&gt;0,F160=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G160&lt;&gt;0,F160=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F160&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F160)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C160)*($E$5:$E$504=E160)*(($D$5:$D$504=D160)*(D160&lt;&gt;"")+($B$5:$B$504=B160)*(B160&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C160="Оплата",K160&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E160)&gt;0,ROUND(E160-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J160" s="5">
@@ -4927,7 +4927,7 @@
         <v/>
       </c>
       <c r="I161" s="6">
-        <f>IF(AND(B161="",C161="",D161="",E161="",F161=""),"",IF(OR(B161="",C161="",E161=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E161)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H161&lt;&gt;0,F161=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G161&lt;&gt;0,F161=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F161&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F161)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C161)*($E$5:$E$504=E161)*(($D$5:$D$504=D161)*(D161&lt;&gt;"")+($B$5:$B$504=B161)*(B161&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C161="Оплата",K161&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E161)&gt;0,ROUND(E161-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B161="",C161="",D161="",E161="",F161=""),"",IF(OR(B161="",C161="",E161=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E161)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H161&lt;&gt;0,F161=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G161&lt;&gt;0,F161=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F161&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F161)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C161)*($E$5:$E$504=E161)*(($D$5:$D$504=D161)*(D161&lt;&gt;"")+($B$5:$B$504=B161)*(B161&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C161="Оплата",K161&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E161)&gt;0,ROUND(E161-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J161" s="5">
@@ -4954,7 +4954,7 @@
         <v/>
       </c>
       <c r="I162" s="6">
-        <f>IF(AND(B162="",C162="",D162="",E162="",F162=""),"",IF(OR(B162="",C162="",E162=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E162)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H162&lt;&gt;0,F162=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G162&lt;&gt;0,F162=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F162&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F162)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C162)*($E$5:$E$504=E162)*(($D$5:$D$504=D162)*(D162&lt;&gt;"")+($B$5:$B$504=B162)*(B162&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C162="Оплата",K162&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E162)&gt;0,ROUND(E162-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B162="",C162="",D162="",E162="",F162=""),"",IF(OR(B162="",C162="",E162=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E162)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H162&lt;&gt;0,F162=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G162&lt;&gt;0,F162=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F162&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F162)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C162)*($E$5:$E$504=E162)*(($D$5:$D$504=D162)*(D162&lt;&gt;"")+($B$5:$B$504=B162)*(B162&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C162="Оплата",K162&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E162)&gt;0,ROUND(E162-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J162" s="5">
@@ -4981,7 +4981,7 @@
         <v/>
       </c>
       <c r="I163" s="6">
-        <f>IF(AND(B163="",C163="",D163="",E163="",F163=""),"",IF(OR(B163="",C163="",E163=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E163)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H163&lt;&gt;0,F163=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G163&lt;&gt;0,F163=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F163&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F163)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C163)*($E$5:$E$504=E163)*(($D$5:$D$504=D163)*(D163&lt;&gt;"")+($B$5:$B$504=B163)*(B163&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C163="Оплата",K163&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E163)&gt;0,ROUND(E163-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B163="",C163="",D163="",E163="",F163=""),"",IF(OR(B163="",C163="",E163=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E163)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H163&lt;&gt;0,F163=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G163&lt;&gt;0,F163=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F163&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F163)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C163)*($E$5:$E$504=E163)*(($D$5:$D$504=D163)*(D163&lt;&gt;"")+($B$5:$B$504=B163)*(B163&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C163="Оплата",K163&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E163)&gt;0,ROUND(E163-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J163" s="5">
@@ -5008,7 +5008,7 @@
         <v/>
       </c>
       <c r="I164" s="6">
-        <f>IF(AND(B164="",C164="",D164="",E164="",F164=""),"",IF(OR(B164="",C164="",E164=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E164)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H164&lt;&gt;0,F164=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G164&lt;&gt;0,F164=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F164&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F164)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C164)*($E$5:$E$504=E164)*(($D$5:$D$504=D164)*(D164&lt;&gt;"")+($B$5:$B$504=B164)*(B164&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C164="Оплата",K164&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E164)&gt;0,ROUND(E164-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B164="",C164="",D164="",E164="",F164=""),"",IF(OR(B164="",C164="",E164=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E164)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H164&lt;&gt;0,F164=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G164&lt;&gt;0,F164=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F164&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F164)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C164)*($E$5:$E$504=E164)*(($D$5:$D$504=D164)*(D164&lt;&gt;"")+($B$5:$B$504=B164)*(B164&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C164="Оплата",K164&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E164)&gt;0,ROUND(E164-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J164" s="5">
@@ -5035,7 +5035,7 @@
         <v/>
       </c>
       <c r="I165" s="6">
-        <f>IF(AND(B165="",C165="",D165="",E165="",F165=""),"",IF(OR(B165="",C165="",E165=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E165)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H165&lt;&gt;0,F165=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G165&lt;&gt;0,F165=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F165&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F165)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C165)*($E$5:$E$504=E165)*(($D$5:$D$504=D165)*(D165&lt;&gt;"")+($B$5:$B$504=B165)*(B165&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C165="Оплата",K165&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E165)&gt;0,ROUND(E165-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B165="",C165="",D165="",E165="",F165=""),"",IF(OR(B165="",C165="",E165=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E165)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H165&lt;&gt;0,F165=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G165&lt;&gt;0,F165=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F165&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F165)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C165)*($E$5:$E$504=E165)*(($D$5:$D$504=D165)*(D165&lt;&gt;"")+($B$5:$B$504=B165)*(B165&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C165="Оплата",K165&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E165)&gt;0,ROUND(E165-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J165" s="5">
@@ -5062,7 +5062,7 @@
         <v/>
       </c>
       <c r="I166" s="6">
-        <f>IF(AND(B166="",C166="",D166="",E166="",F166=""),"",IF(OR(B166="",C166="",E166=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E166)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H166&lt;&gt;0,F166=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G166&lt;&gt;0,F166=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F166&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F166)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C166)*($E$5:$E$504=E166)*(($D$5:$D$504=D166)*(D166&lt;&gt;"")+($B$5:$B$504=B166)*(B166&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C166="Оплата",K166&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E166)&gt;0,ROUND(E166-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B166="",C166="",D166="",E166="",F166=""),"",IF(OR(B166="",C166="",E166=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E166)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H166&lt;&gt;0,F166=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G166&lt;&gt;0,F166=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F166&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F166)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C166)*($E$5:$E$504=E166)*(($D$5:$D$504=D166)*(D166&lt;&gt;"")+($B$5:$B$504=B166)*(B166&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C166="Оплата",K166&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E166)&gt;0,ROUND(E166-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J166" s="5">
@@ -5089,7 +5089,7 @@
         <v/>
       </c>
       <c r="I167" s="6">
-        <f>IF(AND(B167="",C167="",D167="",E167="",F167=""),"",IF(OR(B167="",C167="",E167=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E167)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H167&lt;&gt;0,F167=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G167&lt;&gt;0,F167=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F167&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F167)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C167)*($E$5:$E$504=E167)*(($D$5:$D$504=D167)*(D167&lt;&gt;"")+($B$5:$B$504=B167)*(B167&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C167="Оплата",K167&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E167)&gt;0,ROUND(E167-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B167="",C167="",D167="",E167="",F167=""),"",IF(OR(B167="",C167="",E167=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E167)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H167&lt;&gt;0,F167=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G167&lt;&gt;0,F167=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F167&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F167)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C167)*($E$5:$E$504=E167)*(($D$5:$D$504=D167)*(D167&lt;&gt;"")+($B$5:$B$504=B167)*(B167&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C167="Оплата",K167&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E167)&gt;0,ROUND(E167-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J167" s="5">
@@ -5116,7 +5116,7 @@
         <v/>
       </c>
       <c r="I168" s="6">
-        <f>IF(AND(B168="",C168="",D168="",E168="",F168=""),"",IF(OR(B168="",C168="",E168=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E168)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H168&lt;&gt;0,F168=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G168&lt;&gt;0,F168=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F168&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F168)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C168)*($E$5:$E$504=E168)*(($D$5:$D$504=D168)*(D168&lt;&gt;"")+($B$5:$B$504=B168)*(B168&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C168="Оплата",K168&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E168)&gt;0,ROUND(E168-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B168="",C168="",D168="",E168="",F168=""),"",IF(OR(B168="",C168="",E168=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E168)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H168&lt;&gt;0,F168=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G168&lt;&gt;0,F168=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F168&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F168)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C168)*($E$5:$E$504=E168)*(($D$5:$D$504=D168)*(D168&lt;&gt;"")+($B$5:$B$504=B168)*(B168&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C168="Оплата",K168&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E168)&gt;0,ROUND(E168-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J168" s="5">
@@ -5143,7 +5143,7 @@
         <v/>
       </c>
       <c r="I169" s="6">
-        <f>IF(AND(B169="",C169="",D169="",E169="",F169=""),"",IF(OR(B169="",C169="",E169=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E169)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H169&lt;&gt;0,F169=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G169&lt;&gt;0,F169=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F169&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F169)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C169)*($E$5:$E$504=E169)*(($D$5:$D$504=D169)*(D169&lt;&gt;"")+($B$5:$B$504=B169)*(B169&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C169="Оплата",K169&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E169)&gt;0,ROUND(E169-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B169="",C169="",D169="",E169="",F169=""),"",IF(OR(B169="",C169="",E169=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E169)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H169&lt;&gt;0,F169=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G169&lt;&gt;0,F169=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F169&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F169)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C169)*($E$5:$E$504=E169)*(($D$5:$D$504=D169)*(D169&lt;&gt;"")+($B$5:$B$504=B169)*(B169&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C169="Оплата",K169&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E169)&gt;0,ROUND(E169-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J169" s="5">
@@ -5170,7 +5170,7 @@
         <v/>
       </c>
       <c r="I170" s="6">
-        <f>IF(AND(B170="",C170="",D170="",E170="",F170=""),"",IF(OR(B170="",C170="",E170=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E170)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H170&lt;&gt;0,F170=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G170&lt;&gt;0,F170=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F170&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F170)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C170)*($E$5:$E$504=E170)*(($D$5:$D$504=D170)*(D170&lt;&gt;"")+($B$5:$B$504=B170)*(B170&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C170="Оплата",K170&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E170)&gt;0,ROUND(E170-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B170="",C170="",D170="",E170="",F170=""),"",IF(OR(B170="",C170="",E170=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E170)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H170&lt;&gt;0,F170=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G170&lt;&gt;0,F170=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F170&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F170)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C170)*($E$5:$E$504=E170)*(($D$5:$D$504=D170)*(D170&lt;&gt;"")+($B$5:$B$504=B170)*(B170&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C170="Оплата",K170&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E170)&gt;0,ROUND(E170-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J170" s="5">
@@ -5197,7 +5197,7 @@
         <v/>
       </c>
       <c r="I171" s="6">
-        <f>IF(AND(B171="",C171="",D171="",E171="",F171=""),"",IF(OR(B171="",C171="",E171=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E171)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H171&lt;&gt;0,F171=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G171&lt;&gt;0,F171=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F171&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F171)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C171)*($E$5:$E$504=E171)*(($D$5:$D$504=D171)*(D171&lt;&gt;"")+($B$5:$B$504=B171)*(B171&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C171="Оплата",K171&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E171)&gt;0,ROUND(E171-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B171="",C171="",D171="",E171="",F171=""),"",IF(OR(B171="",C171="",E171=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E171)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H171&lt;&gt;0,F171=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G171&lt;&gt;0,F171=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F171&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F171)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C171)*($E$5:$E$504=E171)*(($D$5:$D$504=D171)*(D171&lt;&gt;"")+($B$5:$B$504=B171)*(B171&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C171="Оплата",K171&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E171)&gt;0,ROUND(E171-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J171" s="5">
@@ -5224,7 +5224,7 @@
         <v/>
       </c>
       <c r="I172" s="6">
-        <f>IF(AND(B172="",C172="",D172="",E172="",F172=""),"",IF(OR(B172="",C172="",E172=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E172)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H172&lt;&gt;0,F172=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G172&lt;&gt;0,F172=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F172&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F172)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C172)*($E$5:$E$504=E172)*(($D$5:$D$504=D172)*(D172&lt;&gt;"")+($B$5:$B$504=B172)*(B172&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C172="Оплата",K172&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E172)&gt;0,ROUND(E172-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B172="",C172="",D172="",E172="",F172=""),"",IF(OR(B172="",C172="",E172=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E172)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H172&lt;&gt;0,F172=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G172&lt;&gt;0,F172=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F172&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F172)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C172)*($E$5:$E$504=E172)*(($D$5:$D$504=D172)*(D172&lt;&gt;"")+($B$5:$B$504=B172)*(B172&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C172="Оплата",K172&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E172)&gt;0,ROUND(E172-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J172" s="5">
@@ -5251,7 +5251,7 @@
         <v/>
       </c>
       <c r="I173" s="6">
-        <f>IF(AND(B173="",C173="",D173="",E173="",F173=""),"",IF(OR(B173="",C173="",E173=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E173)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H173&lt;&gt;0,F173=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G173&lt;&gt;0,F173=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F173&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F173)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C173)*($E$5:$E$504=E173)*(($D$5:$D$504=D173)*(D173&lt;&gt;"")+($B$5:$B$504=B173)*(B173&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C173="Оплата",K173&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E173)&gt;0,ROUND(E173-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B173="",C173="",D173="",E173="",F173=""),"",IF(OR(B173="",C173="",E173=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E173)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H173&lt;&gt;0,F173=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G173&lt;&gt;0,F173=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F173&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F173)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C173)*($E$5:$E$504=E173)*(($D$5:$D$504=D173)*(D173&lt;&gt;"")+($B$5:$B$504=B173)*(B173&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C173="Оплата",K173&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E173)&gt;0,ROUND(E173-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J173" s="5">
@@ -5278,7 +5278,7 @@
         <v/>
       </c>
       <c r="I174" s="6">
-        <f>IF(AND(B174="",C174="",D174="",E174="",F174=""),"",IF(OR(B174="",C174="",E174=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E174)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H174&lt;&gt;0,F174=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G174&lt;&gt;0,F174=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F174&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F174)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C174)*($E$5:$E$504=E174)*(($D$5:$D$504=D174)*(D174&lt;&gt;"")+($B$5:$B$504=B174)*(B174&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C174="Оплата",K174&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E174)&gt;0,ROUND(E174-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B174="",C174="",D174="",E174="",F174=""),"",IF(OR(B174="",C174="",E174=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E174)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H174&lt;&gt;0,F174=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G174&lt;&gt;0,F174=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F174&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F174)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C174)*($E$5:$E$504=E174)*(($D$5:$D$504=D174)*(D174&lt;&gt;"")+($B$5:$B$504=B174)*(B174&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C174="Оплата",K174&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E174)&gt;0,ROUND(E174-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J174" s="5">
@@ -5305,7 +5305,7 @@
         <v/>
       </c>
       <c r="I175" s="6">
-        <f>IF(AND(B175="",C175="",D175="",E175="",F175=""),"",IF(OR(B175="",C175="",E175=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E175)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H175&lt;&gt;0,F175=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G175&lt;&gt;0,F175=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F175&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F175)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C175)*($E$5:$E$504=E175)*(($D$5:$D$504=D175)*(D175&lt;&gt;"")+($B$5:$B$504=B175)*(B175&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C175="Оплата",K175&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E175)&gt;0,ROUND(E175-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B175="",C175="",D175="",E175="",F175=""),"",IF(OR(B175="",C175="",E175=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E175)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H175&lt;&gt;0,F175=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G175&lt;&gt;0,F175=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F175&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F175)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C175)*($E$5:$E$504=E175)*(($D$5:$D$504=D175)*(D175&lt;&gt;"")+($B$5:$B$504=B175)*(B175&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C175="Оплата",K175&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E175)&gt;0,ROUND(E175-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J175" s="5">
@@ -5332,7 +5332,7 @@
         <v/>
       </c>
       <c r="I176" s="6">
-        <f>IF(AND(B176="",C176="",D176="",E176="",F176=""),"",IF(OR(B176="",C176="",E176=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E176)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H176&lt;&gt;0,F176=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G176&lt;&gt;0,F176=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F176&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F176)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C176)*($E$5:$E$504=E176)*(($D$5:$D$504=D176)*(D176&lt;&gt;"")+($B$5:$B$504=B176)*(B176&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C176="Оплата",K176&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E176)&gt;0,ROUND(E176-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B176="",C176="",D176="",E176="",F176=""),"",IF(OR(B176="",C176="",E176=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E176)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H176&lt;&gt;0,F176=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G176&lt;&gt;0,F176=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F176&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F176)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C176)*($E$5:$E$504=E176)*(($D$5:$D$504=D176)*(D176&lt;&gt;"")+($B$5:$B$504=B176)*(B176&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C176="Оплата",K176&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E176)&gt;0,ROUND(E176-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J176" s="5">
@@ -5359,7 +5359,7 @@
         <v/>
       </c>
       <c r="I177" s="6">
-        <f>IF(AND(B177="",C177="",D177="",E177="",F177=""),"",IF(OR(B177="",C177="",E177=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E177)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H177&lt;&gt;0,F177=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G177&lt;&gt;0,F177=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F177&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F177)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C177)*($E$5:$E$504=E177)*(($D$5:$D$504=D177)*(D177&lt;&gt;"")+($B$5:$B$504=B177)*(B177&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C177="Оплата",K177&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E177)&gt;0,ROUND(E177-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B177="",C177="",D177="",E177="",F177=""),"",IF(OR(B177="",C177="",E177=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E177)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H177&lt;&gt;0,F177=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G177&lt;&gt;0,F177=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F177&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F177)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C177)*($E$5:$E$504=E177)*(($D$5:$D$504=D177)*(D177&lt;&gt;"")+($B$5:$B$504=B177)*(B177&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C177="Оплата",K177&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E177)&gt;0,ROUND(E177-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J177" s="5">
@@ -5386,7 +5386,7 @@
         <v/>
       </c>
       <c r="I178" s="6">
-        <f>IF(AND(B178="",C178="",D178="",E178="",F178=""),"",IF(OR(B178="",C178="",E178=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E178)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H178&lt;&gt;0,F178=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G178&lt;&gt;0,F178=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F178&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F178)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C178)*($E$5:$E$504=E178)*(($D$5:$D$504=D178)*(D178&lt;&gt;"")+($B$5:$B$504=B178)*(B178&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C178="Оплата",K178&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E178)&gt;0,ROUND(E178-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B178="",C178="",D178="",E178="",F178=""),"",IF(OR(B178="",C178="",E178=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E178)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H178&lt;&gt;0,F178=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G178&lt;&gt;0,F178=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F178&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F178)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C178)*($E$5:$E$504=E178)*(($D$5:$D$504=D178)*(D178&lt;&gt;"")+($B$5:$B$504=B178)*(B178&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C178="Оплата",K178&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E178)&gt;0,ROUND(E178-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J178" s="5">
@@ -5413,7 +5413,7 @@
         <v/>
       </c>
       <c r="I179" s="6">
-        <f>IF(AND(B179="",C179="",D179="",E179="",F179=""),"",IF(OR(B179="",C179="",E179=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E179)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H179&lt;&gt;0,F179=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G179&lt;&gt;0,F179=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F179&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F179)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C179)*($E$5:$E$504=E179)*(($D$5:$D$504=D179)*(D179&lt;&gt;"")+($B$5:$B$504=B179)*(B179&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C179="Оплата",K179&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E179)&gt;0,ROUND(E179-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B179="",C179="",D179="",E179="",F179=""),"",IF(OR(B179="",C179="",E179=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E179)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H179&lt;&gt;0,F179=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G179&lt;&gt;0,F179=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F179&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F179)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C179)*($E$5:$E$504=E179)*(($D$5:$D$504=D179)*(D179&lt;&gt;"")+($B$5:$B$504=B179)*(B179&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C179="Оплата",K179&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E179)&gt;0,ROUND(E179-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J179" s="5">
@@ -5440,7 +5440,7 @@
         <v/>
       </c>
       <c r="I180" s="6">
-        <f>IF(AND(B180="",C180="",D180="",E180="",F180=""),"",IF(OR(B180="",C180="",E180=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E180)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H180&lt;&gt;0,F180=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G180&lt;&gt;0,F180=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F180&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F180)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C180)*($E$5:$E$504=E180)*(($D$5:$D$504=D180)*(D180&lt;&gt;"")+($B$5:$B$504=B180)*(B180&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C180="Оплата",K180&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E180)&gt;0,ROUND(E180-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B180="",C180="",D180="",E180="",F180=""),"",IF(OR(B180="",C180="",E180=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E180)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H180&lt;&gt;0,F180=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G180&lt;&gt;0,F180=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F180&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F180)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C180)*($E$5:$E$504=E180)*(($D$5:$D$504=D180)*(D180&lt;&gt;"")+($B$5:$B$504=B180)*(B180&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C180="Оплата",K180&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E180)&gt;0,ROUND(E180-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J180" s="5">
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="I181" s="6">
-        <f>IF(AND(B181="",C181="",D181="",E181="",F181=""),"",IF(OR(B181="",C181="",E181=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E181)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H181&lt;&gt;0,F181=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G181&lt;&gt;0,F181=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F181&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F181)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C181)*($E$5:$E$504=E181)*(($D$5:$D$504=D181)*(D181&lt;&gt;"")+($B$5:$B$504=B181)*(B181&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C181="Оплата",K181&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E181)&gt;0,ROUND(E181-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B181="",C181="",D181="",E181="",F181=""),"",IF(OR(B181="",C181="",E181=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E181)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H181&lt;&gt;0,F181=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G181&lt;&gt;0,F181=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F181&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F181)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C181)*($E$5:$E$504=E181)*(($D$5:$D$504=D181)*(D181&lt;&gt;"")+($B$5:$B$504=B181)*(B181&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C181="Оплата",K181&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E181)&gt;0,ROUND(E181-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J181" s="5">
@@ -5494,7 +5494,7 @@
         <v/>
       </c>
       <c r="I182" s="6">
-        <f>IF(AND(B182="",C182="",D182="",E182="",F182=""),"",IF(OR(B182="",C182="",E182=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E182)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H182&lt;&gt;0,F182=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G182&lt;&gt;0,F182=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F182&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F182)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C182)*($E$5:$E$504=E182)*(($D$5:$D$504=D182)*(D182&lt;&gt;"")+($B$5:$B$504=B182)*(B182&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C182="Оплата",K182&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E182)&gt;0,ROUND(E182-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B182="",C182="",D182="",E182="",F182=""),"",IF(OR(B182="",C182="",E182=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E182)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H182&lt;&gt;0,F182=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G182&lt;&gt;0,F182=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F182&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F182)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C182)*($E$5:$E$504=E182)*(($D$5:$D$504=D182)*(D182&lt;&gt;"")+($B$5:$B$504=B182)*(B182&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C182="Оплата",K182&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E182)&gt;0,ROUND(E182-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J182" s="5">
@@ -5521,7 +5521,7 @@
         <v/>
       </c>
       <c r="I183" s="6">
-        <f>IF(AND(B183="",C183="",D183="",E183="",F183=""),"",IF(OR(B183="",C183="",E183=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E183)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H183&lt;&gt;0,F183=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G183&lt;&gt;0,F183=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F183&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F183)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C183)*($E$5:$E$504=E183)*(($D$5:$D$504=D183)*(D183&lt;&gt;"")+($B$5:$B$504=B183)*(B183&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C183="Оплата",K183&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E183)&gt;0,ROUND(E183-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B183="",C183="",D183="",E183="",F183=""),"",IF(OR(B183="",C183="",E183=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E183)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H183&lt;&gt;0,F183=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G183&lt;&gt;0,F183=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F183&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F183)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C183)*($E$5:$E$504=E183)*(($D$5:$D$504=D183)*(D183&lt;&gt;"")+($B$5:$B$504=B183)*(B183&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C183="Оплата",K183&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E183)&gt;0,ROUND(E183-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J183" s="5">
@@ -5548,7 +5548,7 @@
         <v/>
       </c>
       <c r="I184" s="6">
-        <f>IF(AND(B184="",C184="",D184="",E184="",F184=""),"",IF(OR(B184="",C184="",E184=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E184)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H184&lt;&gt;0,F184=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G184&lt;&gt;0,F184=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F184&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F184)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C184)*($E$5:$E$504=E184)*(($D$5:$D$504=D184)*(D184&lt;&gt;"")+($B$5:$B$504=B184)*(B184&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C184="Оплата",K184&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E184)&gt;0,ROUND(E184-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B184="",C184="",D184="",E184="",F184=""),"",IF(OR(B184="",C184="",E184=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E184)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H184&lt;&gt;0,F184=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G184&lt;&gt;0,F184=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F184&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F184)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C184)*($E$5:$E$504=E184)*(($D$5:$D$504=D184)*(D184&lt;&gt;"")+($B$5:$B$504=B184)*(B184&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C184="Оплата",K184&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E184)&gt;0,ROUND(E184-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J184" s="5">
@@ -5575,7 +5575,7 @@
         <v/>
       </c>
       <c r="I185" s="6">
-        <f>IF(AND(B185="",C185="",D185="",E185="",F185=""),"",IF(OR(B185="",C185="",E185=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E185)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H185&lt;&gt;0,F185=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G185&lt;&gt;0,F185=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F185&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F185)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C185)*($E$5:$E$504=E185)*(($D$5:$D$504=D185)*(D185&lt;&gt;"")+($B$5:$B$504=B185)*(B185&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C185="Оплата",K185&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E185)&gt;0,ROUND(E185-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B185="",C185="",D185="",E185="",F185=""),"",IF(OR(B185="",C185="",E185=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E185)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H185&lt;&gt;0,F185=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G185&lt;&gt;0,F185=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F185&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F185)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C185)*($E$5:$E$504=E185)*(($D$5:$D$504=D185)*(D185&lt;&gt;"")+($B$5:$B$504=B185)*(B185&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C185="Оплата",K185&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E185)&gt;0,ROUND(E185-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J185" s="5">
@@ -5602,7 +5602,7 @@
         <v/>
       </c>
       <c r="I186" s="6">
-        <f>IF(AND(B186="",C186="",D186="",E186="",F186=""),"",IF(OR(B186="",C186="",E186=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E186)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H186&lt;&gt;0,F186=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G186&lt;&gt;0,F186=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F186&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F186)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C186)*($E$5:$E$504=E186)*(($D$5:$D$504=D186)*(D186&lt;&gt;"")+($B$5:$B$504=B186)*(B186&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C186="Оплата",K186&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E186)&gt;0,ROUND(E186-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B186="",C186="",D186="",E186="",F186=""),"",IF(OR(B186="",C186="",E186=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E186)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H186&lt;&gt;0,F186=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G186&lt;&gt;0,F186=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F186&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F186)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C186)*($E$5:$E$504=E186)*(($D$5:$D$504=D186)*(D186&lt;&gt;"")+($B$5:$B$504=B186)*(B186&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C186="Оплата",K186&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E186)&gt;0,ROUND(E186-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J186" s="5">
@@ -5629,7 +5629,7 @@
         <v/>
       </c>
       <c r="I187" s="6">
-        <f>IF(AND(B187="",C187="",D187="",E187="",F187=""),"",IF(OR(B187="",C187="",E187=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E187)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H187&lt;&gt;0,F187=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G187&lt;&gt;0,F187=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F187&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F187)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C187)*($E$5:$E$504=E187)*(($D$5:$D$504=D187)*(D187&lt;&gt;"")+($B$5:$B$504=B187)*(B187&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C187="Оплата",K187&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E187)&gt;0,ROUND(E187-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B187="",C187="",D187="",E187="",F187=""),"",IF(OR(B187="",C187="",E187=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E187)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H187&lt;&gt;0,F187=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G187&lt;&gt;0,F187=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F187&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F187)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C187)*($E$5:$E$504=E187)*(($D$5:$D$504=D187)*(D187&lt;&gt;"")+($B$5:$B$504=B187)*(B187&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C187="Оплата",K187&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E187)&gt;0,ROUND(E187-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J187" s="5">
@@ -5656,7 +5656,7 @@
         <v/>
       </c>
       <c r="I188" s="6">
-        <f>IF(AND(B188="",C188="",D188="",E188="",F188=""),"",IF(OR(B188="",C188="",E188=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E188)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H188&lt;&gt;0,F188=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G188&lt;&gt;0,F188=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F188&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F188)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C188)*($E$5:$E$504=E188)*(($D$5:$D$504=D188)*(D188&lt;&gt;"")+($B$5:$B$504=B188)*(B188&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C188="Оплата",K188&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E188)&gt;0,ROUND(E188-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B188="",C188="",D188="",E188="",F188=""),"",IF(OR(B188="",C188="",E188=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E188)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H188&lt;&gt;0,F188=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G188&lt;&gt;0,F188=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F188&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F188)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C188)*($E$5:$E$504=E188)*(($D$5:$D$504=D188)*(D188&lt;&gt;"")+($B$5:$B$504=B188)*(B188&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C188="Оплата",K188&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E188)&gt;0,ROUND(E188-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J188" s="5">
@@ -5683,7 +5683,7 @@
         <v/>
       </c>
       <c r="I189" s="6">
-        <f>IF(AND(B189="",C189="",D189="",E189="",F189=""),"",IF(OR(B189="",C189="",E189=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E189)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H189&lt;&gt;0,F189=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G189&lt;&gt;0,F189=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F189&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F189)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C189)*($E$5:$E$504=E189)*(($D$5:$D$504=D189)*(D189&lt;&gt;"")+($B$5:$B$504=B189)*(B189&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C189="Оплата",K189&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E189)&gt;0,ROUND(E189-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B189="",C189="",D189="",E189="",F189=""),"",IF(OR(B189="",C189="",E189=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E189)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H189&lt;&gt;0,F189=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G189&lt;&gt;0,F189=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F189&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F189)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C189)*($E$5:$E$504=E189)*(($D$5:$D$504=D189)*(D189&lt;&gt;"")+($B$5:$B$504=B189)*(B189&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C189="Оплата",K189&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E189)&gt;0,ROUND(E189-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J189" s="5">
@@ -5710,7 +5710,7 @@
         <v/>
       </c>
       <c r="I190" s="6">
-        <f>IF(AND(B190="",C190="",D190="",E190="",F190=""),"",IF(OR(B190="",C190="",E190=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E190)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H190&lt;&gt;0,F190=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G190&lt;&gt;0,F190=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F190&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F190)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C190)*($E$5:$E$504=E190)*(($D$5:$D$504=D190)*(D190&lt;&gt;"")+($B$5:$B$504=B190)*(B190&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C190="Оплата",K190&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E190)&gt;0,ROUND(E190-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B190="",C190="",D190="",E190="",F190=""),"",IF(OR(B190="",C190="",E190=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E190)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H190&lt;&gt;0,F190=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G190&lt;&gt;0,F190=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F190&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F190)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C190)*($E$5:$E$504=E190)*(($D$5:$D$504=D190)*(D190&lt;&gt;"")+($B$5:$B$504=B190)*(B190&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C190="Оплата",K190&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E190)&gt;0,ROUND(E190-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J190" s="5">
@@ -5737,7 +5737,7 @@
         <v/>
       </c>
       <c r="I191" s="6">
-        <f>IF(AND(B191="",C191="",D191="",E191="",F191=""),"",IF(OR(B191="",C191="",E191=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E191)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H191&lt;&gt;0,F191=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G191&lt;&gt;0,F191=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F191&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F191)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C191)*($E$5:$E$504=E191)*(($D$5:$D$504=D191)*(D191&lt;&gt;"")+($B$5:$B$504=B191)*(B191&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C191="Оплата",K191&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E191)&gt;0,ROUND(E191-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B191="",C191="",D191="",E191="",F191=""),"",IF(OR(B191="",C191="",E191=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E191)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H191&lt;&gt;0,F191=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G191&lt;&gt;0,F191=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F191&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F191)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C191)*($E$5:$E$504=E191)*(($D$5:$D$504=D191)*(D191&lt;&gt;"")+($B$5:$B$504=B191)*(B191&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C191="Оплата",K191&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E191)&gt;0,ROUND(E191-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J191" s="5">
@@ -5764,7 +5764,7 @@
         <v/>
       </c>
       <c r="I192" s="6">
-        <f>IF(AND(B192="",C192="",D192="",E192="",F192=""),"",IF(OR(B192="",C192="",E192=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E192)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H192&lt;&gt;0,F192=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G192&lt;&gt;0,F192=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F192&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F192)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C192)*($E$5:$E$504=E192)*(($D$5:$D$504=D192)*(D192&lt;&gt;"")+($B$5:$B$504=B192)*(B192&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C192="Оплата",K192&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E192)&gt;0,ROUND(E192-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B192="",C192="",D192="",E192="",F192=""),"",IF(OR(B192="",C192="",E192=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E192)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H192&lt;&gt;0,F192=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G192&lt;&gt;0,F192=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F192&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F192)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C192)*($E$5:$E$504=E192)*(($D$5:$D$504=D192)*(D192&lt;&gt;"")+($B$5:$B$504=B192)*(B192&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C192="Оплата",K192&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E192)&gt;0,ROUND(E192-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J192" s="5">
@@ -5791,7 +5791,7 @@
         <v/>
       </c>
       <c r="I193" s="6">
-        <f>IF(AND(B193="",C193="",D193="",E193="",F193=""),"",IF(OR(B193="",C193="",E193=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E193)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H193&lt;&gt;0,F193=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G193&lt;&gt;0,F193=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F193&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F193)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C193)*($E$5:$E$504=E193)*(($D$5:$D$504=D193)*(D193&lt;&gt;"")+($B$5:$B$504=B193)*(B193&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C193="Оплата",K193&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E193)&gt;0,ROUND(E193-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B193="",C193="",D193="",E193="",F193=""),"",IF(OR(B193="",C193="",E193=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E193)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H193&lt;&gt;0,F193=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G193&lt;&gt;0,F193=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F193&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F193)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C193)*($E$5:$E$504=E193)*(($D$5:$D$504=D193)*(D193&lt;&gt;"")+($B$5:$B$504=B193)*(B193&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C193="Оплата",K193&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E193)&gt;0,ROUND(E193-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J193" s="5">
@@ -5818,7 +5818,7 @@
         <v/>
       </c>
       <c r="I194" s="6">
-        <f>IF(AND(B194="",C194="",D194="",E194="",F194=""),"",IF(OR(B194="",C194="",E194=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E194)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H194&lt;&gt;0,F194=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G194&lt;&gt;0,F194=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F194&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F194)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C194)*($E$5:$E$504=E194)*(($D$5:$D$504=D194)*(D194&lt;&gt;"")+($B$5:$B$504=B194)*(B194&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C194="Оплата",K194&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E194)&gt;0,ROUND(E194-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B194="",C194="",D194="",E194="",F194=""),"",IF(OR(B194="",C194="",E194=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E194)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H194&lt;&gt;0,F194=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G194&lt;&gt;0,F194=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F194&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F194)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C194)*($E$5:$E$504=E194)*(($D$5:$D$504=D194)*(D194&lt;&gt;"")+($B$5:$B$504=B194)*(B194&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C194="Оплата",K194&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E194)&gt;0,ROUND(E194-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J194" s="5">
@@ -5845,7 +5845,7 @@
         <v/>
       </c>
       <c r="I195" s="6">
-        <f>IF(AND(B195="",C195="",D195="",E195="",F195=""),"",IF(OR(B195="",C195="",E195=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E195)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H195&lt;&gt;0,F195=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G195&lt;&gt;0,F195=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F195&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F195)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C195)*($E$5:$E$504=E195)*(($D$5:$D$504=D195)*(D195&lt;&gt;"")+($B$5:$B$504=B195)*(B195&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C195="Оплата",K195&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E195)&gt;0,ROUND(E195-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B195="",C195="",D195="",E195="",F195=""),"",IF(OR(B195="",C195="",E195=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E195)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H195&lt;&gt;0,F195=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G195&lt;&gt;0,F195=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F195&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F195)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C195)*($E$5:$E$504=E195)*(($D$5:$D$504=D195)*(D195&lt;&gt;"")+($B$5:$B$504=B195)*(B195&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C195="Оплата",K195&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E195)&gt;0,ROUND(E195-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J195" s="5">
@@ -5872,7 +5872,7 @@
         <v/>
       </c>
       <c r="I196" s="6">
-        <f>IF(AND(B196="",C196="",D196="",E196="",F196=""),"",IF(OR(B196="",C196="",E196=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E196)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H196&lt;&gt;0,F196=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G196&lt;&gt;0,F196=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F196&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F196)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C196)*($E$5:$E$504=E196)*(($D$5:$D$504=D196)*(D196&lt;&gt;"")+($B$5:$B$504=B196)*(B196&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C196="Оплата",K196&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E196)&gt;0,ROUND(E196-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B196="",C196="",D196="",E196="",F196=""),"",IF(OR(B196="",C196="",E196=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E196)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H196&lt;&gt;0,F196=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G196&lt;&gt;0,F196=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F196&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F196)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C196)*($E$5:$E$504=E196)*(($D$5:$D$504=D196)*(D196&lt;&gt;"")+($B$5:$B$504=B196)*(B196&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C196="Оплата",K196&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E196)&gt;0,ROUND(E196-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J196" s="5">
@@ -5899,7 +5899,7 @@
         <v/>
       </c>
       <c r="I197" s="6">
-        <f>IF(AND(B197="",C197="",D197="",E197="",F197=""),"",IF(OR(B197="",C197="",E197=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E197)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H197&lt;&gt;0,F197=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G197&lt;&gt;0,F197=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F197&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F197)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C197)*($E$5:$E$504=E197)*(($D$5:$D$504=D197)*(D197&lt;&gt;"")+($B$5:$B$504=B197)*(B197&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C197="Оплата",K197&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E197)&gt;0,ROUND(E197-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B197="",C197="",D197="",E197="",F197=""),"",IF(OR(B197="",C197="",E197=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E197)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H197&lt;&gt;0,F197=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G197&lt;&gt;0,F197=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F197&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F197)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C197)*($E$5:$E$504=E197)*(($D$5:$D$504=D197)*(D197&lt;&gt;"")+($B$5:$B$504=B197)*(B197&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C197="Оплата",K197&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E197)&gt;0,ROUND(E197-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J197" s="5">
@@ -5926,7 +5926,7 @@
         <v/>
       </c>
       <c r="I198" s="6">
-        <f>IF(AND(B198="",C198="",D198="",E198="",F198=""),"",IF(OR(B198="",C198="",E198=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E198)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H198&lt;&gt;0,F198=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G198&lt;&gt;0,F198=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F198&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F198)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C198)*($E$5:$E$504=E198)*(($D$5:$D$504=D198)*(D198&lt;&gt;"")+($B$5:$B$504=B198)*(B198&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C198="Оплата",K198&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E198)&gt;0,ROUND(E198-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B198="",C198="",D198="",E198="",F198=""),"",IF(OR(B198="",C198="",E198=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E198)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H198&lt;&gt;0,F198=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G198&lt;&gt;0,F198=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F198&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F198)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C198)*($E$5:$E$504=E198)*(($D$5:$D$504=D198)*(D198&lt;&gt;"")+($B$5:$B$504=B198)*(B198&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C198="Оплата",K198&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E198)&gt;0,ROUND(E198-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J198" s="5">
@@ -5953,7 +5953,7 @@
         <v/>
       </c>
       <c r="I199" s="6">
-        <f>IF(AND(B199="",C199="",D199="",E199="",F199=""),"",IF(OR(B199="",C199="",E199=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E199)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H199&lt;&gt;0,F199=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G199&lt;&gt;0,F199=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F199&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F199)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C199)*($E$5:$E$504=E199)*(($D$5:$D$504=D199)*(D199&lt;&gt;"")+($B$5:$B$504=B199)*(B199&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C199="Оплата",K199&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E199)&gt;0,ROUND(E199-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B199="",C199="",D199="",E199="",F199=""),"",IF(OR(B199="",C199="",E199=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E199)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H199&lt;&gt;0,F199=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G199&lt;&gt;0,F199=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F199&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F199)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C199)*($E$5:$E$504=E199)*(($D$5:$D$504=D199)*(D199&lt;&gt;"")+($B$5:$B$504=B199)*(B199&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C199="Оплата",K199&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E199)&gt;0,ROUND(E199-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J199" s="5">
@@ -5980,7 +5980,7 @@
         <v/>
       </c>
       <c r="I200" s="6">
-        <f>IF(AND(B200="",C200="",D200="",E200="",F200=""),"",IF(OR(B200="",C200="",E200=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E200)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H200&lt;&gt;0,F200=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G200&lt;&gt;0,F200=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F200&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F200)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C200)*($E$5:$E$504=E200)*(($D$5:$D$504=D200)*(D200&lt;&gt;"")+($B$5:$B$504=B200)*(B200&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C200="Оплата",K200&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E200)&gt;0,ROUND(E200-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B200="",C200="",D200="",E200="",F200=""),"",IF(OR(B200="",C200="",E200=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E200)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H200&lt;&gt;0,F200=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G200&lt;&gt;0,F200=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F200&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F200)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C200)*($E$5:$E$504=E200)*(($D$5:$D$504=D200)*(D200&lt;&gt;"")+($B$5:$B$504=B200)*(B200&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C200="Оплата",K200&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E200)&gt;0,ROUND(E200-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J200" s="5">
@@ -6007,7 +6007,7 @@
         <v/>
       </c>
       <c r="I201" s="6">
-        <f>IF(AND(B201="",C201="",D201="",E201="",F201=""),"",IF(OR(B201="",C201="",E201=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E201)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H201&lt;&gt;0,F201=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G201&lt;&gt;0,F201=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F201&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F201)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C201)*($E$5:$E$504=E201)*(($D$5:$D$504=D201)*(D201&lt;&gt;"")+($B$5:$B$504=B201)*(B201&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C201="Оплата",K201&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E201)&gt;0,ROUND(E201-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B201="",C201="",D201="",E201="",F201=""),"",IF(OR(B201="",C201="",E201=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E201)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H201&lt;&gt;0,F201=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G201&lt;&gt;0,F201=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F201&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F201)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C201)*($E$5:$E$504=E201)*(($D$5:$D$504=D201)*(D201&lt;&gt;"")+($B$5:$B$504=B201)*(B201&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C201="Оплата",K201&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E201)&gt;0,ROUND(E201-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J201" s="5">
@@ -6034,7 +6034,7 @@
         <v/>
       </c>
       <c r="I202" s="6">
-        <f>IF(AND(B202="",C202="",D202="",E202="",F202=""),"",IF(OR(B202="",C202="",E202=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E202)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H202&lt;&gt;0,F202=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G202&lt;&gt;0,F202=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F202&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F202)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C202)*($E$5:$E$504=E202)*(($D$5:$D$504=D202)*(D202&lt;&gt;"")+($B$5:$B$504=B202)*(B202&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C202="Оплата",K202&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E202)&gt;0,ROUND(E202-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B202="",C202="",D202="",E202="",F202=""),"",IF(OR(B202="",C202="",E202=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E202)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H202&lt;&gt;0,F202=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G202&lt;&gt;0,F202=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F202&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F202)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C202)*($E$5:$E$504=E202)*(($D$5:$D$504=D202)*(D202&lt;&gt;"")+($B$5:$B$504=B202)*(B202&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C202="Оплата",K202&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E202)&gt;0,ROUND(E202-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J202" s="5">
@@ -6061,7 +6061,7 @@
         <v/>
       </c>
       <c r="I203" s="6">
-        <f>IF(AND(B203="",C203="",D203="",E203="",F203=""),"",IF(OR(B203="",C203="",E203=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E203)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H203&lt;&gt;0,F203=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G203&lt;&gt;0,F203=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F203&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F203)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C203)*($E$5:$E$504=E203)*(($D$5:$D$504=D203)*(D203&lt;&gt;"")+($B$5:$B$504=B203)*(B203&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C203="Оплата",K203&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E203)&gt;0,ROUND(E203-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B203="",C203="",D203="",E203="",F203=""),"",IF(OR(B203="",C203="",E203=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E203)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H203&lt;&gt;0,F203=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G203&lt;&gt;0,F203=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F203&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F203)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C203)*($E$5:$E$504=E203)*(($D$5:$D$504=D203)*(D203&lt;&gt;"")+($B$5:$B$504=B203)*(B203&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C203="Оплата",K203&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E203)&gt;0,ROUND(E203-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J203" s="5">
@@ -6088,7 +6088,7 @@
         <v/>
       </c>
       <c r="I204" s="6">
-        <f>IF(AND(B204="",C204="",D204="",E204="",F204=""),"",IF(OR(B204="",C204="",E204=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E204)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H204&lt;&gt;0,F204=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G204&lt;&gt;0,F204=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F204&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F204)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C204)*($E$5:$E$504=E204)*(($D$5:$D$504=D204)*(D204&lt;&gt;"")+($B$5:$B$504=B204)*(B204&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C204="Оплата",K204&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E204)&gt;0,ROUND(E204-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B204="",C204="",D204="",E204="",F204=""),"",IF(OR(B204="",C204="",E204=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E204)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H204&lt;&gt;0,F204=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G204&lt;&gt;0,F204=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F204&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F204)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C204)*($E$5:$E$504=E204)*(($D$5:$D$504=D204)*(D204&lt;&gt;"")+($B$5:$B$504=B204)*(B204&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C204="Оплата",K204&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E204)&gt;0,ROUND(E204-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J204" s="5">
@@ -6115,7 +6115,7 @@
         <v/>
       </c>
       <c r="I205" s="6">
-        <f>IF(AND(B205="",C205="",D205="",E205="",F205=""),"",IF(OR(B205="",C205="",E205=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E205)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H205&lt;&gt;0,F205=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G205&lt;&gt;0,F205=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F205&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F205)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C205)*($E$5:$E$504=E205)*(($D$5:$D$504=D205)*(D205&lt;&gt;"")+($B$5:$B$504=B205)*(B205&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C205="Оплата",K205&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E205)&gt;0,ROUND(E205-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B205="",C205="",D205="",E205="",F205=""),"",IF(OR(B205="",C205="",E205=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E205)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H205&lt;&gt;0,F205=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G205&lt;&gt;0,F205=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F205&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F205)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C205)*($E$5:$E$504=E205)*(($D$5:$D$504=D205)*(D205&lt;&gt;"")+($B$5:$B$504=B205)*(B205&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C205="Оплата",K205&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E205)&gt;0,ROUND(E205-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J205" s="5">
@@ -6142,7 +6142,7 @@
         <v/>
       </c>
       <c r="I206" s="6">
-        <f>IF(AND(B206="",C206="",D206="",E206="",F206=""),"",IF(OR(B206="",C206="",E206=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E206)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H206&lt;&gt;0,F206=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G206&lt;&gt;0,F206=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F206&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F206)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C206)*($E$5:$E$504=E206)*(($D$5:$D$504=D206)*(D206&lt;&gt;"")+($B$5:$B$504=B206)*(B206&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C206="Оплата",K206&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E206)&gt;0,ROUND(E206-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B206="",C206="",D206="",E206="",F206=""),"",IF(OR(B206="",C206="",E206=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E206)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H206&lt;&gt;0,F206=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G206&lt;&gt;0,F206=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F206&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F206)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C206)*($E$5:$E$504=E206)*(($D$5:$D$504=D206)*(D206&lt;&gt;"")+($B$5:$B$504=B206)*(B206&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C206="Оплата",K206&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E206)&gt;0,ROUND(E206-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J206" s="5">
@@ -6169,7 +6169,7 @@
         <v/>
       </c>
       <c r="I207" s="6">
-        <f>IF(AND(B207="",C207="",D207="",E207="",F207=""),"",IF(OR(B207="",C207="",E207=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E207)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H207&lt;&gt;0,F207=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G207&lt;&gt;0,F207=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F207&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F207)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C207)*($E$5:$E$504=E207)*(($D$5:$D$504=D207)*(D207&lt;&gt;"")+($B$5:$B$504=B207)*(B207&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C207="Оплата",K207&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E207)&gt;0,ROUND(E207-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B207="",C207="",D207="",E207="",F207=""),"",IF(OR(B207="",C207="",E207=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E207)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H207&lt;&gt;0,F207=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G207&lt;&gt;0,F207=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F207&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F207)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C207)*($E$5:$E$504=E207)*(($D$5:$D$504=D207)*(D207&lt;&gt;"")+($B$5:$B$504=B207)*(B207&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C207="Оплата",K207&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E207)&gt;0,ROUND(E207-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J207" s="5">
@@ -6196,7 +6196,7 @@
         <v/>
       </c>
       <c r="I208" s="6">
-        <f>IF(AND(B208="",C208="",D208="",E208="",F208=""),"",IF(OR(B208="",C208="",E208=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E208)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H208&lt;&gt;0,F208=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G208&lt;&gt;0,F208=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F208&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F208)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C208)*($E$5:$E$504=E208)*(($D$5:$D$504=D208)*(D208&lt;&gt;"")+($B$5:$B$504=B208)*(B208&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C208="Оплата",K208&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E208)&gt;0,ROUND(E208-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B208="",C208="",D208="",E208="",F208=""),"",IF(OR(B208="",C208="",E208=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E208)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H208&lt;&gt;0,F208=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G208&lt;&gt;0,F208=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F208&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F208)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C208)*($E$5:$E$504=E208)*(($D$5:$D$504=D208)*(D208&lt;&gt;"")+($B$5:$B$504=B208)*(B208&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C208="Оплата",K208&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E208)&gt;0,ROUND(E208-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J208" s="5">
@@ -6223,7 +6223,7 @@
         <v/>
       </c>
       <c r="I209" s="6">
-        <f>IF(AND(B209="",C209="",D209="",E209="",F209=""),"",IF(OR(B209="",C209="",E209=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E209)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H209&lt;&gt;0,F209=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G209&lt;&gt;0,F209=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F209&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F209)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C209)*($E$5:$E$504=E209)*(($D$5:$D$504=D209)*(D209&lt;&gt;"")+($B$5:$B$504=B209)*(B209&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C209="Оплата",K209&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E209)&gt;0,ROUND(E209-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B209="",C209="",D209="",E209="",F209=""),"",IF(OR(B209="",C209="",E209=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E209)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H209&lt;&gt;0,F209=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G209&lt;&gt;0,F209=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F209&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F209)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C209)*($E$5:$E$504=E209)*(($D$5:$D$504=D209)*(D209&lt;&gt;"")+($B$5:$B$504=B209)*(B209&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C209="Оплата",K209&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E209)&gt;0,ROUND(E209-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J209" s="5">
@@ -6250,7 +6250,7 @@
         <v/>
       </c>
       <c r="I210" s="6">
-        <f>IF(AND(B210="",C210="",D210="",E210="",F210=""),"",IF(OR(B210="",C210="",E210=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E210)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H210&lt;&gt;0,F210=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G210&lt;&gt;0,F210=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F210&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F210)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C210)*($E$5:$E$504=E210)*(($D$5:$D$504=D210)*(D210&lt;&gt;"")+($B$5:$B$504=B210)*(B210&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C210="Оплата",K210&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E210)&gt;0,ROUND(E210-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B210="",C210="",D210="",E210="",F210=""),"",IF(OR(B210="",C210="",E210=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E210)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H210&lt;&gt;0,F210=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G210&lt;&gt;0,F210=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F210&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F210)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C210)*($E$5:$E$504=E210)*(($D$5:$D$504=D210)*(D210&lt;&gt;"")+($B$5:$B$504=B210)*(B210&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C210="Оплата",K210&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E210)&gt;0,ROUND(E210-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J210" s="5">
@@ -6277,7 +6277,7 @@
         <v/>
       </c>
       <c r="I211" s="6">
-        <f>IF(AND(B211="",C211="",D211="",E211="",F211=""),"",IF(OR(B211="",C211="",E211=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E211)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H211&lt;&gt;0,F211=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G211&lt;&gt;0,F211=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F211&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F211)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C211)*($E$5:$E$504=E211)*(($D$5:$D$504=D211)*(D211&lt;&gt;"")+($B$5:$B$504=B211)*(B211&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C211="Оплата",K211&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E211)&gt;0,ROUND(E211-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B211="",C211="",D211="",E211="",F211=""),"",IF(OR(B211="",C211="",E211=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E211)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H211&lt;&gt;0,F211=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G211&lt;&gt;0,F211=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F211&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F211)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C211)*($E$5:$E$504=E211)*(($D$5:$D$504=D211)*(D211&lt;&gt;"")+($B$5:$B$504=B211)*(B211&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C211="Оплата",K211&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E211)&gt;0,ROUND(E211-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J211" s="5">
@@ -6304,7 +6304,7 @@
         <v/>
       </c>
       <c r="I212" s="6">
-        <f>IF(AND(B212="",C212="",D212="",E212="",F212=""),"",IF(OR(B212="",C212="",E212=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E212)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H212&lt;&gt;0,F212=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G212&lt;&gt;0,F212=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F212&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F212)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C212)*($E$5:$E$504=E212)*(($D$5:$D$504=D212)*(D212&lt;&gt;"")+($B$5:$B$504=B212)*(B212&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C212="Оплата",K212&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E212)&gt;0,ROUND(E212-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B212="",C212="",D212="",E212="",F212=""),"",IF(OR(B212="",C212="",E212=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E212)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H212&lt;&gt;0,F212=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G212&lt;&gt;0,F212=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F212&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F212)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C212)*($E$5:$E$504=E212)*(($D$5:$D$504=D212)*(D212&lt;&gt;"")+($B$5:$B$504=B212)*(B212&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C212="Оплата",K212&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E212)&gt;0,ROUND(E212-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J212" s="5">
@@ -6331,7 +6331,7 @@
         <v/>
       </c>
       <c r="I213" s="6">
-        <f>IF(AND(B213="",C213="",D213="",E213="",F213=""),"",IF(OR(B213="",C213="",E213=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E213)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H213&lt;&gt;0,F213=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G213&lt;&gt;0,F213=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F213&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F213)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C213)*($E$5:$E$504=E213)*(($D$5:$D$504=D213)*(D213&lt;&gt;"")+($B$5:$B$504=B213)*(B213&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C213="Оплата",K213&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E213)&gt;0,ROUND(E213-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B213="",C213="",D213="",E213="",F213=""),"",IF(OR(B213="",C213="",E213=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E213)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H213&lt;&gt;0,F213=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G213&lt;&gt;0,F213=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F213&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F213)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C213)*($E$5:$E$504=E213)*(($D$5:$D$504=D213)*(D213&lt;&gt;"")+($B$5:$B$504=B213)*(B213&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C213="Оплата",K213&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E213)&gt;0,ROUND(E213-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J213" s="5">
@@ -6358,7 +6358,7 @@
         <v/>
       </c>
       <c r="I214" s="6">
-        <f>IF(AND(B214="",C214="",D214="",E214="",F214=""),"",IF(OR(B214="",C214="",E214=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E214)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H214&lt;&gt;0,F214=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G214&lt;&gt;0,F214=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F214&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F214)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C214)*($E$5:$E$504=E214)*(($D$5:$D$504=D214)*(D214&lt;&gt;"")+($B$5:$B$504=B214)*(B214&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C214="Оплата",K214&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E214)&gt;0,ROUND(E214-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B214="",C214="",D214="",E214="",F214=""),"",IF(OR(B214="",C214="",E214=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E214)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H214&lt;&gt;0,F214=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G214&lt;&gt;0,F214=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F214&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F214)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C214)*($E$5:$E$504=E214)*(($D$5:$D$504=D214)*(D214&lt;&gt;"")+($B$5:$B$504=B214)*(B214&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C214="Оплата",K214&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E214)&gt;0,ROUND(E214-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J214" s="5">
@@ -6385,7 +6385,7 @@
         <v/>
       </c>
       <c r="I215" s="6">
-        <f>IF(AND(B215="",C215="",D215="",E215="",F215=""),"",IF(OR(B215="",C215="",E215=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E215)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H215&lt;&gt;0,F215=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G215&lt;&gt;0,F215=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F215&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F215)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C215)*($E$5:$E$504=E215)*(($D$5:$D$504=D215)*(D215&lt;&gt;"")+($B$5:$B$504=B215)*(B215&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C215="Оплата",K215&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E215)&gt;0,ROUND(E215-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B215="",C215="",D215="",E215="",F215=""),"",IF(OR(B215="",C215="",E215=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E215)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H215&lt;&gt;0,F215=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G215&lt;&gt;0,F215=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F215&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F215)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C215)*($E$5:$E$504=E215)*(($D$5:$D$504=D215)*(D215&lt;&gt;"")+($B$5:$B$504=B215)*(B215&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C215="Оплата",K215&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E215)&gt;0,ROUND(E215-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J215" s="5">
@@ -6412,7 +6412,7 @@
         <v/>
       </c>
       <c r="I216" s="6">
-        <f>IF(AND(B216="",C216="",D216="",E216="",F216=""),"",IF(OR(B216="",C216="",E216=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E216)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H216&lt;&gt;0,F216=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G216&lt;&gt;0,F216=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F216&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F216)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C216)*($E$5:$E$504=E216)*(($D$5:$D$504=D216)*(D216&lt;&gt;"")+($B$5:$B$504=B216)*(B216&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C216="Оплата",K216&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E216)&gt;0,ROUND(E216-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B216="",C216="",D216="",E216="",F216=""),"",IF(OR(B216="",C216="",E216=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E216)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H216&lt;&gt;0,F216=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G216&lt;&gt;0,F216=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F216&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F216)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C216)*($E$5:$E$504=E216)*(($D$5:$D$504=D216)*(D216&lt;&gt;"")+($B$5:$B$504=B216)*(B216&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C216="Оплата",K216&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E216)&gt;0,ROUND(E216-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J216" s="5">
@@ -6439,7 +6439,7 @@
         <v/>
       </c>
       <c r="I217" s="6">
-        <f>IF(AND(B217="",C217="",D217="",E217="",F217=""),"",IF(OR(B217="",C217="",E217=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E217)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H217&lt;&gt;0,F217=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G217&lt;&gt;0,F217=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F217&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F217)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C217)*($E$5:$E$504=E217)*(($D$5:$D$504=D217)*(D217&lt;&gt;"")+($B$5:$B$504=B217)*(B217&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C217="Оплата",K217&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E217)&gt;0,ROUND(E217-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B217="",C217="",D217="",E217="",F217=""),"",IF(OR(B217="",C217="",E217=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E217)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H217&lt;&gt;0,F217=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G217&lt;&gt;0,F217=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F217&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F217)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C217)*($E$5:$E$504=E217)*(($D$5:$D$504=D217)*(D217&lt;&gt;"")+($B$5:$B$504=B217)*(B217&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C217="Оплата",K217&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E217)&gt;0,ROUND(E217-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J217" s="5">
@@ -6466,7 +6466,7 @@
         <v/>
       </c>
       <c r="I218" s="6">
-        <f>IF(AND(B218="",C218="",D218="",E218="",F218=""),"",IF(OR(B218="",C218="",E218=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E218)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H218&lt;&gt;0,F218=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G218&lt;&gt;0,F218=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F218&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F218)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C218)*($E$5:$E$504=E218)*(($D$5:$D$504=D218)*(D218&lt;&gt;"")+($B$5:$B$504=B218)*(B218&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C218="Оплата",K218&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E218)&gt;0,ROUND(E218-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B218="",C218="",D218="",E218="",F218=""),"",IF(OR(B218="",C218="",E218=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E218)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H218&lt;&gt;0,F218=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G218&lt;&gt;0,F218=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F218&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F218)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C218)*($E$5:$E$504=E218)*(($D$5:$D$504=D218)*(D218&lt;&gt;"")+($B$5:$B$504=B218)*(B218&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C218="Оплата",K218&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E218)&gt;0,ROUND(E218-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J218" s="5">
@@ -6493,7 +6493,7 @@
         <v/>
       </c>
       <c r="I219" s="6">
-        <f>IF(AND(B219="",C219="",D219="",E219="",F219=""),"",IF(OR(B219="",C219="",E219=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E219)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H219&lt;&gt;0,F219=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G219&lt;&gt;0,F219=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F219&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F219)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C219)*($E$5:$E$504=E219)*(($D$5:$D$504=D219)*(D219&lt;&gt;"")+($B$5:$B$504=B219)*(B219&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C219="Оплата",K219&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E219)&gt;0,ROUND(E219-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B219="",C219="",D219="",E219="",F219=""),"",IF(OR(B219="",C219="",E219=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E219)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H219&lt;&gt;0,F219=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G219&lt;&gt;0,F219=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F219&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F219)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C219)*($E$5:$E$504=E219)*(($D$5:$D$504=D219)*(D219&lt;&gt;"")+($B$5:$B$504=B219)*(B219&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C219="Оплата",K219&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E219)&gt;0,ROUND(E219-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J219" s="5">
@@ -6520,7 +6520,7 @@
         <v/>
       </c>
       <c r="I220" s="6">
-        <f>IF(AND(B220="",C220="",D220="",E220="",F220=""),"",IF(OR(B220="",C220="",E220=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E220)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H220&lt;&gt;0,F220=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G220&lt;&gt;0,F220=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F220&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F220)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C220)*($E$5:$E$504=E220)*(($D$5:$D$504=D220)*(D220&lt;&gt;"")+($B$5:$B$504=B220)*(B220&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C220="Оплата",K220&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E220)&gt;0,ROUND(E220-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B220="",C220="",D220="",E220="",F220=""),"",IF(OR(B220="",C220="",E220=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E220)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H220&lt;&gt;0,F220=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G220&lt;&gt;0,F220=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F220&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F220)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C220)*($E$5:$E$504=E220)*(($D$5:$D$504=D220)*(D220&lt;&gt;"")+($B$5:$B$504=B220)*(B220&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C220="Оплата",K220&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E220)&gt;0,ROUND(E220-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J220" s="5">
@@ -6547,7 +6547,7 @@
         <v/>
       </c>
       <c r="I221" s="6">
-        <f>IF(AND(B221="",C221="",D221="",E221="",F221=""),"",IF(OR(B221="",C221="",E221=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E221)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H221&lt;&gt;0,F221=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G221&lt;&gt;0,F221=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F221&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F221)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C221)*($E$5:$E$504=E221)*(($D$5:$D$504=D221)*(D221&lt;&gt;"")+($B$5:$B$504=B221)*(B221&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C221="Оплата",K221&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E221)&gt;0,ROUND(E221-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B221="",C221="",D221="",E221="",F221=""),"",IF(OR(B221="",C221="",E221=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E221)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H221&lt;&gt;0,F221=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G221&lt;&gt;0,F221=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F221&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F221)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C221)*($E$5:$E$504=E221)*(($D$5:$D$504=D221)*(D221&lt;&gt;"")+($B$5:$B$504=B221)*(B221&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C221="Оплата",K221&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E221)&gt;0,ROUND(E221-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J221" s="5">
@@ -6574,7 +6574,7 @@
         <v/>
       </c>
       <c r="I222" s="6">
-        <f>IF(AND(B222="",C222="",D222="",E222="",F222=""),"",IF(OR(B222="",C222="",E222=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E222)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H222&lt;&gt;0,F222=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G222&lt;&gt;0,F222=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F222&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F222)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C222)*($E$5:$E$504=E222)*(($D$5:$D$504=D222)*(D222&lt;&gt;"")+($B$5:$B$504=B222)*(B222&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C222="Оплата",K222&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E222)&gt;0,ROUND(E222-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B222="",C222="",D222="",E222="",F222=""),"",IF(OR(B222="",C222="",E222=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E222)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H222&lt;&gt;0,F222=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G222&lt;&gt;0,F222=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F222&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F222)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C222)*($E$5:$E$504=E222)*(($D$5:$D$504=D222)*(D222&lt;&gt;"")+($B$5:$B$504=B222)*(B222&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C222="Оплата",K222&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E222)&gt;0,ROUND(E222-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J222" s="5">
@@ -6601,7 +6601,7 @@
         <v/>
       </c>
       <c r="I223" s="6">
-        <f>IF(AND(B223="",C223="",D223="",E223="",F223=""),"",IF(OR(B223="",C223="",E223=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E223)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H223&lt;&gt;0,F223=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G223&lt;&gt;0,F223=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F223&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F223)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C223)*($E$5:$E$504=E223)*(($D$5:$D$504=D223)*(D223&lt;&gt;"")+($B$5:$B$504=B223)*(B223&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C223="Оплата",K223&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E223)&gt;0,ROUND(E223-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B223="",C223="",D223="",E223="",F223=""),"",IF(OR(B223="",C223="",E223=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E223)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H223&lt;&gt;0,F223=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G223&lt;&gt;0,F223=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F223&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F223)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C223)*($E$5:$E$504=E223)*(($D$5:$D$504=D223)*(D223&lt;&gt;"")+($B$5:$B$504=B223)*(B223&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C223="Оплата",K223&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E223)&gt;0,ROUND(E223-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J223" s="5">
@@ -6628,7 +6628,7 @@
         <v/>
       </c>
       <c r="I224" s="6">
-        <f>IF(AND(B224="",C224="",D224="",E224="",F224=""),"",IF(OR(B224="",C224="",E224=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E224)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H224&lt;&gt;0,F224=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G224&lt;&gt;0,F224=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F224&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F224)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C224)*($E$5:$E$504=E224)*(($D$5:$D$504=D224)*(D224&lt;&gt;"")+($B$5:$B$504=B224)*(B224&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C224="Оплата",K224&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E224)&gt;0,ROUND(E224-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B224="",C224="",D224="",E224="",F224=""),"",IF(OR(B224="",C224="",E224=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E224)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H224&lt;&gt;0,F224=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G224&lt;&gt;0,F224=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F224&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F224)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C224)*($E$5:$E$504=E224)*(($D$5:$D$504=D224)*(D224&lt;&gt;"")+($B$5:$B$504=B224)*(B224&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C224="Оплата",K224&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E224)&gt;0,ROUND(E224-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J224" s="5">
@@ -6655,7 +6655,7 @@
         <v/>
       </c>
       <c r="I225" s="6">
-        <f>IF(AND(B225="",C225="",D225="",E225="",F225=""),"",IF(OR(B225="",C225="",E225=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E225)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H225&lt;&gt;0,F225=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G225&lt;&gt;0,F225=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F225&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F225)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C225)*($E$5:$E$504=E225)*(($D$5:$D$504=D225)*(D225&lt;&gt;"")+($B$5:$B$504=B225)*(B225&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C225="Оплата",K225&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E225)&gt;0,ROUND(E225-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B225="",C225="",D225="",E225="",F225=""),"",IF(OR(B225="",C225="",E225=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E225)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H225&lt;&gt;0,F225=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G225&lt;&gt;0,F225=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F225&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F225)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C225)*($E$5:$E$504=E225)*(($D$5:$D$504=D225)*(D225&lt;&gt;"")+($B$5:$B$504=B225)*(B225&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C225="Оплата",K225&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E225)&gt;0,ROUND(E225-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J225" s="5">
@@ -6682,7 +6682,7 @@
         <v/>
       </c>
       <c r="I226" s="6">
-        <f>IF(AND(B226="",C226="",D226="",E226="",F226=""),"",IF(OR(B226="",C226="",E226=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E226)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H226&lt;&gt;0,F226=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G226&lt;&gt;0,F226=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F226&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F226)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C226)*($E$5:$E$504=E226)*(($D$5:$D$504=D226)*(D226&lt;&gt;"")+($B$5:$B$504=B226)*(B226&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C226="Оплата",K226&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E226)&gt;0,ROUND(E226-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B226="",C226="",D226="",E226="",F226=""),"",IF(OR(B226="",C226="",E226=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E226)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H226&lt;&gt;0,F226=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G226&lt;&gt;0,F226=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F226&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F226)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C226)*($E$5:$E$504=E226)*(($D$5:$D$504=D226)*(D226&lt;&gt;"")+($B$5:$B$504=B226)*(B226&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C226="Оплата",K226&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E226)&gt;0,ROUND(E226-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J226" s="5">
@@ -6709,7 +6709,7 @@
         <v/>
       </c>
       <c r="I227" s="6">
-        <f>IF(AND(B227="",C227="",D227="",E227="",F227=""),"",IF(OR(B227="",C227="",E227=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E227)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H227&lt;&gt;0,F227=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G227&lt;&gt;0,F227=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F227&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F227)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C227)*($E$5:$E$504=E227)*(($D$5:$D$504=D227)*(D227&lt;&gt;"")+($B$5:$B$504=B227)*(B227&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C227="Оплата",K227&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E227)&gt;0,ROUND(E227-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B227="",C227="",D227="",E227="",F227=""),"",IF(OR(B227="",C227="",E227=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E227)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H227&lt;&gt;0,F227=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G227&lt;&gt;0,F227=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F227&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F227)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C227)*($E$5:$E$504=E227)*(($D$5:$D$504=D227)*(D227&lt;&gt;"")+($B$5:$B$504=B227)*(B227&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C227="Оплата",K227&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E227)&gt;0,ROUND(E227-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J227" s="5">
@@ -6736,7 +6736,7 @@
         <v/>
       </c>
       <c r="I228" s="6">
-        <f>IF(AND(B228="",C228="",D228="",E228="",F228=""),"",IF(OR(B228="",C228="",E228=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E228)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H228&lt;&gt;0,F228=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G228&lt;&gt;0,F228=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F228&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F228)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C228)*($E$5:$E$504=E228)*(($D$5:$D$504=D228)*(D228&lt;&gt;"")+($B$5:$B$504=B228)*(B228&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C228="Оплата",K228&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E228)&gt;0,ROUND(E228-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B228="",C228="",D228="",E228="",F228=""),"",IF(OR(B228="",C228="",E228=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E228)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H228&lt;&gt;0,F228=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G228&lt;&gt;0,F228=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F228&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F228)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C228)*($E$5:$E$504=E228)*(($D$5:$D$504=D228)*(D228&lt;&gt;"")+($B$5:$B$504=B228)*(B228&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C228="Оплата",K228&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E228)&gt;0,ROUND(E228-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J228" s="5">
@@ -6763,7 +6763,7 @@
         <v/>
       </c>
       <c r="I229" s="6">
-        <f>IF(AND(B229="",C229="",D229="",E229="",F229=""),"",IF(OR(B229="",C229="",E229=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E229)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H229&lt;&gt;0,F229=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G229&lt;&gt;0,F229=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F229&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F229)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C229)*($E$5:$E$504=E229)*(($D$5:$D$504=D229)*(D229&lt;&gt;"")+($B$5:$B$504=B229)*(B229&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C229="Оплата",K229&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E229)&gt;0,ROUND(E229-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B229="",C229="",D229="",E229="",F229=""),"",IF(OR(B229="",C229="",E229=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E229)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H229&lt;&gt;0,F229=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G229&lt;&gt;0,F229=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F229&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F229)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C229)*($E$5:$E$504=E229)*(($D$5:$D$504=D229)*(D229&lt;&gt;"")+($B$5:$B$504=B229)*(B229&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C229="Оплата",K229&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E229)&gt;0,ROUND(E229-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J229" s="5">
@@ -6790,7 +6790,7 @@
         <v/>
       </c>
       <c r="I230" s="6">
-        <f>IF(AND(B230="",C230="",D230="",E230="",F230=""),"",IF(OR(B230="",C230="",E230=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E230)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H230&lt;&gt;0,F230=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G230&lt;&gt;0,F230=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F230&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F230)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C230)*($E$5:$E$504=E230)*(($D$5:$D$504=D230)*(D230&lt;&gt;"")+($B$5:$B$504=B230)*(B230&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C230="Оплата",K230&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E230)&gt;0,ROUND(E230-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B230="",C230="",D230="",E230="",F230=""),"",IF(OR(B230="",C230="",E230=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E230)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H230&lt;&gt;0,F230=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G230&lt;&gt;0,F230=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F230&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F230)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C230)*($E$5:$E$504=E230)*(($D$5:$D$504=D230)*(D230&lt;&gt;"")+($B$5:$B$504=B230)*(B230&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C230="Оплата",K230&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E230)&gt;0,ROUND(E230-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J230" s="5">
@@ -6817,7 +6817,7 @@
         <v/>
       </c>
       <c r="I231" s="6">
-        <f>IF(AND(B231="",C231="",D231="",E231="",F231=""),"",IF(OR(B231="",C231="",E231=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E231)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H231&lt;&gt;0,F231=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G231&lt;&gt;0,F231=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F231&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F231)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C231)*($E$5:$E$504=E231)*(($D$5:$D$504=D231)*(D231&lt;&gt;"")+($B$5:$B$504=B231)*(B231&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C231="Оплата",K231&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E231)&gt;0,ROUND(E231-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B231="",C231="",D231="",E231="",F231=""),"",IF(OR(B231="",C231="",E231=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E231)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H231&lt;&gt;0,F231=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G231&lt;&gt;0,F231=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F231&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F231)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C231)*($E$5:$E$504=E231)*(($D$5:$D$504=D231)*(D231&lt;&gt;"")+($B$5:$B$504=B231)*(B231&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C231="Оплата",K231&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E231)&gt;0,ROUND(E231-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J231" s="5">
@@ -6844,7 +6844,7 @@
         <v/>
       </c>
       <c r="I232" s="6">
-        <f>IF(AND(B232="",C232="",D232="",E232="",F232=""),"",IF(OR(B232="",C232="",E232=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E232)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H232&lt;&gt;0,F232=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G232&lt;&gt;0,F232=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F232&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F232)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C232)*($E$5:$E$504=E232)*(($D$5:$D$504=D232)*(D232&lt;&gt;"")+($B$5:$B$504=B232)*(B232&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C232="Оплата",K232&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E232)&gt;0,ROUND(E232-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B232="",C232="",D232="",E232="",F232=""),"",IF(OR(B232="",C232="",E232=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E232)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H232&lt;&gt;0,F232=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G232&lt;&gt;0,F232=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F232&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F232)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C232)*($E$5:$E$504=E232)*(($D$5:$D$504=D232)*(D232&lt;&gt;"")+($B$5:$B$504=B232)*(B232&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C232="Оплата",K232&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E232)&gt;0,ROUND(E232-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J232" s="5">
@@ -6871,7 +6871,7 @@
         <v/>
       </c>
       <c r="I233" s="6">
-        <f>IF(AND(B233="",C233="",D233="",E233="",F233=""),"",IF(OR(B233="",C233="",E233=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E233)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H233&lt;&gt;0,F233=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G233&lt;&gt;0,F233=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F233&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F233)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C233)*($E$5:$E$504=E233)*(($D$5:$D$504=D233)*(D233&lt;&gt;"")+($B$5:$B$504=B233)*(B233&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C233="Оплата",K233&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E233)&gt;0,ROUND(E233-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B233="",C233="",D233="",E233="",F233=""),"",IF(OR(B233="",C233="",E233=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E233)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H233&lt;&gt;0,F233=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G233&lt;&gt;0,F233=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F233&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F233)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C233)*($E$5:$E$504=E233)*(($D$5:$D$504=D233)*(D233&lt;&gt;"")+($B$5:$B$504=B233)*(B233&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C233="Оплата",K233&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E233)&gt;0,ROUND(E233-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J233" s="5">
@@ -6898,7 +6898,7 @@
         <v/>
       </c>
       <c r="I234" s="6">
-        <f>IF(AND(B234="",C234="",D234="",E234="",F234=""),"",IF(OR(B234="",C234="",E234=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E234)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H234&lt;&gt;0,F234=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G234&lt;&gt;0,F234=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F234&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F234)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C234)*($E$5:$E$504=E234)*(($D$5:$D$504=D234)*(D234&lt;&gt;"")+($B$5:$B$504=B234)*(B234&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C234="Оплата",K234&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E234)&gt;0,ROUND(E234-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B234="",C234="",D234="",E234="",F234=""),"",IF(OR(B234="",C234="",E234=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E234)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H234&lt;&gt;0,F234=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G234&lt;&gt;0,F234=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F234&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F234)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C234)*($E$5:$E$504=E234)*(($D$5:$D$504=D234)*(D234&lt;&gt;"")+($B$5:$B$504=B234)*(B234&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C234="Оплата",K234&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E234)&gt;0,ROUND(E234-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J234" s="5">
@@ -6925,7 +6925,7 @@
         <v/>
       </c>
       <c r="I235" s="6">
-        <f>IF(AND(B235="",C235="",D235="",E235="",F235=""),"",IF(OR(B235="",C235="",E235=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E235)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H235&lt;&gt;0,F235=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G235&lt;&gt;0,F235=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F235&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F235)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C235)*($E$5:$E$504=E235)*(($D$5:$D$504=D235)*(D235&lt;&gt;"")+($B$5:$B$504=B235)*(B235&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C235="Оплата",K235&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E235)&gt;0,ROUND(E235-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B235="",C235="",D235="",E235="",F235=""),"",IF(OR(B235="",C235="",E235=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E235)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H235&lt;&gt;0,F235=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G235&lt;&gt;0,F235=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F235&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F235)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C235)*($E$5:$E$504=E235)*(($D$5:$D$504=D235)*(D235&lt;&gt;"")+($B$5:$B$504=B235)*(B235&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C235="Оплата",K235&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E235)&gt;0,ROUND(E235-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J235" s="5">
@@ -6952,7 +6952,7 @@
         <v/>
       </c>
       <c r="I236" s="6">
-        <f>IF(AND(B236="",C236="",D236="",E236="",F236=""),"",IF(OR(B236="",C236="",E236=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E236)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H236&lt;&gt;0,F236=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G236&lt;&gt;0,F236=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F236&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F236)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C236)*($E$5:$E$504=E236)*(($D$5:$D$504=D236)*(D236&lt;&gt;"")+($B$5:$B$504=B236)*(B236&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C236="Оплата",K236&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E236)&gt;0,ROUND(E236-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B236="",C236="",D236="",E236="",F236=""),"",IF(OR(B236="",C236="",E236=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E236)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H236&lt;&gt;0,F236=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G236&lt;&gt;0,F236=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F236&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F236)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C236)*($E$5:$E$504=E236)*(($D$5:$D$504=D236)*(D236&lt;&gt;"")+($B$5:$B$504=B236)*(B236&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C236="Оплата",K236&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E236)&gt;0,ROUND(E236-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J236" s="5">
@@ -6979,7 +6979,7 @@
         <v/>
       </c>
       <c r="I237" s="6">
-        <f>IF(AND(B237="",C237="",D237="",E237="",F237=""),"",IF(OR(B237="",C237="",E237=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E237)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H237&lt;&gt;0,F237=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G237&lt;&gt;0,F237=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F237&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F237)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C237)*($E$5:$E$504=E237)*(($D$5:$D$504=D237)*(D237&lt;&gt;"")+($B$5:$B$504=B237)*(B237&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C237="Оплата",K237&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E237)&gt;0,ROUND(E237-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B237="",C237="",D237="",E237="",F237=""),"",IF(OR(B237="",C237="",E237=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E237)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H237&lt;&gt;0,F237=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G237&lt;&gt;0,F237=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F237&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F237)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C237)*($E$5:$E$504=E237)*(($D$5:$D$504=D237)*(D237&lt;&gt;"")+($B$5:$B$504=B237)*(B237&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C237="Оплата",K237&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E237)&gt;0,ROUND(E237-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J237" s="5">
@@ -7006,7 +7006,7 @@
         <v/>
       </c>
       <c r="I238" s="6">
-        <f>IF(AND(B238="",C238="",D238="",E238="",F238=""),"",IF(OR(B238="",C238="",E238=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E238)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H238&lt;&gt;0,F238=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G238&lt;&gt;0,F238=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F238&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F238)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C238)*($E$5:$E$504=E238)*(($D$5:$D$504=D238)*(D238&lt;&gt;"")+($B$5:$B$504=B238)*(B238&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C238="Оплата",K238&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E238)&gt;0,ROUND(E238-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B238="",C238="",D238="",E238="",F238=""),"",IF(OR(B238="",C238="",E238=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E238)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H238&lt;&gt;0,F238=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G238&lt;&gt;0,F238=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F238&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F238)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C238)*($E$5:$E$504=E238)*(($D$5:$D$504=D238)*(D238&lt;&gt;"")+($B$5:$B$504=B238)*(B238&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C238="Оплата",K238&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E238)&gt;0,ROUND(E238-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J238" s="5">
@@ -7033,7 +7033,7 @@
         <v/>
       </c>
       <c r="I239" s="6">
-        <f>IF(AND(B239="",C239="",D239="",E239="",F239=""),"",IF(OR(B239="",C239="",E239=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E239)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H239&lt;&gt;0,F239=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G239&lt;&gt;0,F239=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F239&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F239)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C239)*($E$5:$E$504=E239)*(($D$5:$D$504=D239)*(D239&lt;&gt;"")+($B$5:$B$504=B239)*(B239&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C239="Оплата",K239&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E239)&gt;0,ROUND(E239-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B239="",C239="",D239="",E239="",F239=""),"",IF(OR(B239="",C239="",E239=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E239)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H239&lt;&gt;0,F239=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G239&lt;&gt;0,F239=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F239&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F239)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C239)*($E$5:$E$504=E239)*(($D$5:$D$504=D239)*(D239&lt;&gt;"")+($B$5:$B$504=B239)*(B239&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C239="Оплата",K239&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E239)&gt;0,ROUND(E239-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J239" s="5">
@@ -7060,7 +7060,7 @@
         <v/>
       </c>
       <c r="I240" s="6">
-        <f>IF(AND(B240="",C240="",D240="",E240="",F240=""),"",IF(OR(B240="",C240="",E240=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E240)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H240&lt;&gt;0,F240=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G240&lt;&gt;0,F240=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F240&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F240)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C240)*($E$5:$E$504=E240)*(($D$5:$D$504=D240)*(D240&lt;&gt;"")+($B$5:$B$504=B240)*(B240&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C240="Оплата",K240&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E240)&gt;0,ROUND(E240-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B240="",C240="",D240="",E240="",F240=""),"",IF(OR(B240="",C240="",E240=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E240)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H240&lt;&gt;0,F240=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G240&lt;&gt;0,F240=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F240&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F240)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C240)*($E$5:$E$504=E240)*(($D$5:$D$504=D240)*(D240&lt;&gt;"")+($B$5:$B$504=B240)*(B240&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C240="Оплата",K240&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E240)&gt;0,ROUND(E240-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J240" s="5">
@@ -7087,7 +7087,7 @@
         <v/>
       </c>
       <c r="I241" s="6">
-        <f>IF(AND(B241="",C241="",D241="",E241="",F241=""),"",IF(OR(B241="",C241="",E241=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E241)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H241&lt;&gt;0,F241=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G241&lt;&gt;0,F241=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F241&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F241)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C241)*($E$5:$E$504=E241)*(($D$5:$D$504=D241)*(D241&lt;&gt;"")+($B$5:$B$504=B241)*(B241&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C241="Оплата",K241&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E241)&gt;0,ROUND(E241-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B241="",C241="",D241="",E241="",F241=""),"",IF(OR(B241="",C241="",E241=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E241)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H241&lt;&gt;0,F241=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G241&lt;&gt;0,F241=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F241&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F241)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C241)*($E$5:$E$504=E241)*(($D$5:$D$504=D241)*(D241&lt;&gt;"")+($B$5:$B$504=B241)*(B241&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C241="Оплата",K241&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E241)&gt;0,ROUND(E241-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J241" s="5">
@@ -7114,7 +7114,7 @@
         <v/>
       </c>
       <c r="I242" s="6">
-        <f>IF(AND(B242="",C242="",D242="",E242="",F242=""),"",IF(OR(B242="",C242="",E242=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E242)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H242&lt;&gt;0,F242=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G242&lt;&gt;0,F242=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F242&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F242)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C242)*($E$5:$E$504=E242)*(($D$5:$D$504=D242)*(D242&lt;&gt;"")+($B$5:$B$504=B242)*(B242&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C242="Оплата",K242&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E242)&gt;0,ROUND(E242-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B242="",C242="",D242="",E242="",F242=""),"",IF(OR(B242="",C242="",E242=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E242)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H242&lt;&gt;0,F242=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G242&lt;&gt;0,F242=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F242&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F242)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C242)*($E$5:$E$504=E242)*(($D$5:$D$504=D242)*(D242&lt;&gt;"")+($B$5:$B$504=B242)*(B242&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C242="Оплата",K242&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E242)&gt;0,ROUND(E242-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J242" s="5">
@@ -7141,7 +7141,7 @@
         <v/>
       </c>
       <c r="I243" s="6">
-        <f>IF(AND(B243="",C243="",D243="",E243="",F243=""),"",IF(OR(B243="",C243="",E243=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E243)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H243&lt;&gt;0,F243=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G243&lt;&gt;0,F243=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F243&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F243)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C243)*($E$5:$E$504=E243)*(($D$5:$D$504=D243)*(D243&lt;&gt;"")+($B$5:$B$504=B243)*(B243&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C243="Оплата",K243&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E243)&gt;0,ROUND(E243-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B243="",C243="",D243="",E243="",F243=""),"",IF(OR(B243="",C243="",E243=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E243)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H243&lt;&gt;0,F243=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G243&lt;&gt;0,F243=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F243&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F243)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C243)*($E$5:$E$504=E243)*(($D$5:$D$504=D243)*(D243&lt;&gt;"")+($B$5:$B$504=B243)*(B243&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C243="Оплата",K243&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E243)&gt;0,ROUND(E243-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J243" s="5">
@@ -7168,7 +7168,7 @@
         <v/>
       </c>
       <c r="I244" s="6">
-        <f>IF(AND(B244="",C244="",D244="",E244="",F244=""),"",IF(OR(B244="",C244="",E244=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E244)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H244&lt;&gt;0,F244=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G244&lt;&gt;0,F244=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F244&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F244)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C244)*($E$5:$E$504=E244)*(($D$5:$D$504=D244)*(D244&lt;&gt;"")+($B$5:$B$504=B244)*(B244&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C244="Оплата",K244&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E244)&gt;0,ROUND(E244-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B244="",C244="",D244="",E244="",F244=""),"",IF(OR(B244="",C244="",E244=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E244)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H244&lt;&gt;0,F244=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G244&lt;&gt;0,F244=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F244&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F244)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C244)*($E$5:$E$504=E244)*(($D$5:$D$504=D244)*(D244&lt;&gt;"")+($B$5:$B$504=B244)*(B244&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C244="Оплата",K244&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E244)&gt;0,ROUND(E244-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J244" s="5">
@@ -7195,7 +7195,7 @@
         <v/>
       </c>
       <c r="I245" s="6">
-        <f>IF(AND(B245="",C245="",D245="",E245="",F245=""),"",IF(OR(B245="",C245="",E245=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E245)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H245&lt;&gt;0,F245=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G245&lt;&gt;0,F245=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F245&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F245)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C245)*($E$5:$E$504=E245)*(($D$5:$D$504=D245)*(D245&lt;&gt;"")+($B$5:$B$504=B245)*(B245&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C245="Оплата",K245&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E245)&gt;0,ROUND(E245-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B245="",C245="",D245="",E245="",F245=""),"",IF(OR(B245="",C245="",E245=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E245)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H245&lt;&gt;0,F245=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G245&lt;&gt;0,F245=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F245&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F245)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C245)*($E$5:$E$504=E245)*(($D$5:$D$504=D245)*(D245&lt;&gt;"")+($B$5:$B$504=B245)*(B245&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C245="Оплата",K245&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E245)&gt;0,ROUND(E245-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J245" s="5">
@@ -7222,7 +7222,7 @@
         <v/>
       </c>
       <c r="I246" s="6">
-        <f>IF(AND(B246="",C246="",D246="",E246="",F246=""),"",IF(OR(B246="",C246="",E246=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E246)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H246&lt;&gt;0,F246=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G246&lt;&gt;0,F246=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F246&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F246)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C246)*($E$5:$E$504=E246)*(($D$5:$D$504=D246)*(D246&lt;&gt;"")+($B$5:$B$504=B246)*(B246&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C246="Оплата",K246&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E246)&gt;0,ROUND(E246-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B246="",C246="",D246="",E246="",F246=""),"",IF(OR(B246="",C246="",E246=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E246)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H246&lt;&gt;0,F246=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G246&lt;&gt;0,F246=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F246&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F246)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C246)*($E$5:$E$504=E246)*(($D$5:$D$504=D246)*(D246&lt;&gt;"")+($B$5:$B$504=B246)*(B246&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C246="Оплата",K246&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E246)&gt;0,ROUND(E246-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J246" s="5">
@@ -7249,7 +7249,7 @@
         <v/>
       </c>
       <c r="I247" s="6">
-        <f>IF(AND(B247="",C247="",D247="",E247="",F247=""),"",IF(OR(B247="",C247="",E247=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E247)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H247&lt;&gt;0,F247=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G247&lt;&gt;0,F247=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F247&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F247)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C247)*($E$5:$E$504=E247)*(($D$5:$D$504=D247)*(D247&lt;&gt;"")+($B$5:$B$504=B247)*(B247&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C247="Оплата",K247&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E247)&gt;0,ROUND(E247-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B247="",C247="",D247="",E247="",F247=""),"",IF(OR(B247="",C247="",E247=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E247)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H247&lt;&gt;0,F247=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G247&lt;&gt;0,F247=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F247&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F247)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C247)*($E$5:$E$504=E247)*(($D$5:$D$504=D247)*(D247&lt;&gt;"")+($B$5:$B$504=B247)*(B247&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C247="Оплата",K247&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E247)&gt;0,ROUND(E247-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J247" s="5">
@@ -7276,7 +7276,7 @@
         <v/>
       </c>
       <c r="I248" s="6">
-        <f>IF(AND(B248="",C248="",D248="",E248="",F248=""),"",IF(OR(B248="",C248="",E248=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E248)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H248&lt;&gt;0,F248=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G248&lt;&gt;0,F248=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F248&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F248)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C248)*($E$5:$E$504=E248)*(($D$5:$D$504=D248)*(D248&lt;&gt;"")+($B$5:$B$504=B248)*(B248&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C248="Оплата",K248&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E248)&gt;0,ROUND(E248-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B248="",C248="",D248="",E248="",F248=""),"",IF(OR(B248="",C248="",E248=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E248)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H248&lt;&gt;0,F248=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G248&lt;&gt;0,F248=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F248&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F248)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C248)*($E$5:$E$504=E248)*(($D$5:$D$504=D248)*(D248&lt;&gt;"")+($B$5:$B$504=B248)*(B248&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C248="Оплата",K248&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E248)&gt;0,ROUND(E248-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J248" s="5">
@@ -7303,7 +7303,7 @@
         <v/>
       </c>
       <c r="I249" s="6">
-        <f>IF(AND(B249="",C249="",D249="",E249="",F249=""),"",IF(OR(B249="",C249="",E249=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E249)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H249&lt;&gt;0,F249=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G249&lt;&gt;0,F249=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F249&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F249)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C249)*($E$5:$E$504=E249)*(($D$5:$D$504=D249)*(D249&lt;&gt;"")+($B$5:$B$504=B249)*(B249&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C249="Оплата",K249&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E249)&gt;0,ROUND(E249-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B249="",C249="",D249="",E249="",F249=""),"",IF(OR(B249="",C249="",E249=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E249)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H249&lt;&gt;0,F249=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G249&lt;&gt;0,F249=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F249&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F249)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C249)*($E$5:$E$504=E249)*(($D$5:$D$504=D249)*(D249&lt;&gt;"")+($B$5:$B$504=B249)*(B249&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C249="Оплата",K249&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E249)&gt;0,ROUND(E249-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J249" s="5">
@@ -7330,7 +7330,7 @@
         <v/>
       </c>
       <c r="I250" s="6">
-        <f>IF(AND(B250="",C250="",D250="",E250="",F250=""),"",IF(OR(B250="",C250="",E250=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E250)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H250&lt;&gt;0,F250=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G250&lt;&gt;0,F250=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F250&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F250)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C250)*($E$5:$E$504=E250)*(($D$5:$D$504=D250)*(D250&lt;&gt;"")+($B$5:$B$504=B250)*(B250&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C250="Оплата",K250&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E250)&gt;0,ROUND(E250-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B250="",C250="",D250="",E250="",F250=""),"",IF(OR(B250="",C250="",E250=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E250)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H250&lt;&gt;0,F250=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G250&lt;&gt;0,F250=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F250&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F250)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C250)*($E$5:$E$504=E250)*(($D$5:$D$504=D250)*(D250&lt;&gt;"")+($B$5:$B$504=B250)*(B250&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C250="Оплата",K250&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E250)&gt;0,ROUND(E250-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J250" s="5">
@@ -7357,7 +7357,7 @@
         <v/>
       </c>
       <c r="I251" s="6">
-        <f>IF(AND(B251="",C251="",D251="",E251="",F251=""),"",IF(OR(B251="",C251="",E251=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E251)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H251&lt;&gt;0,F251=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G251&lt;&gt;0,F251=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F251&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F251)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C251)*($E$5:$E$504=E251)*(($D$5:$D$504=D251)*(D251&lt;&gt;"")+($B$5:$B$504=B251)*(B251&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C251="Оплата",K251&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E251)&gt;0,ROUND(E251-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B251="",C251="",D251="",E251="",F251=""),"",IF(OR(B251="",C251="",E251=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E251)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H251&lt;&gt;0,F251=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G251&lt;&gt;0,F251=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F251&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F251)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C251)*($E$5:$E$504=E251)*(($D$5:$D$504=D251)*(D251&lt;&gt;"")+($B$5:$B$504=B251)*(B251&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C251="Оплата",K251&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E251)&gt;0,ROUND(E251-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J251" s="5">
@@ -7384,7 +7384,7 @@
         <v/>
       </c>
       <c r="I252" s="6">
-        <f>IF(AND(B252="",C252="",D252="",E252="",F252=""),"",IF(OR(B252="",C252="",E252=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E252)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H252&lt;&gt;0,F252=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G252&lt;&gt;0,F252=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F252&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F252)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C252)*($E$5:$E$504=E252)*(($D$5:$D$504=D252)*(D252&lt;&gt;"")+($B$5:$B$504=B252)*(B252&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C252="Оплата",K252&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E252)&gt;0,ROUND(E252-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B252="",C252="",D252="",E252="",F252=""),"",IF(OR(B252="",C252="",E252=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E252)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H252&lt;&gt;0,F252=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G252&lt;&gt;0,F252=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F252&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F252)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C252)*($E$5:$E$504=E252)*(($D$5:$D$504=D252)*(D252&lt;&gt;"")+($B$5:$B$504=B252)*(B252&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C252="Оплата",K252&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E252)&gt;0,ROUND(E252-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J252" s="5">
@@ -7411,7 +7411,7 @@
         <v/>
       </c>
       <c r="I253" s="6">
-        <f>IF(AND(B253="",C253="",D253="",E253="",F253=""),"",IF(OR(B253="",C253="",E253=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E253)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H253&lt;&gt;0,F253=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G253&lt;&gt;0,F253=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F253&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F253)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C253)*($E$5:$E$504=E253)*(($D$5:$D$504=D253)*(D253&lt;&gt;"")+($B$5:$B$504=B253)*(B253&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C253="Оплата",K253&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E253)&gt;0,ROUND(E253-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B253="",C253="",D253="",E253="",F253=""),"",IF(OR(B253="",C253="",E253=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E253)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H253&lt;&gt;0,F253=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G253&lt;&gt;0,F253=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F253&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F253)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C253)*($E$5:$E$504=E253)*(($D$5:$D$504=D253)*(D253&lt;&gt;"")+($B$5:$B$504=B253)*(B253&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C253="Оплата",K253&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E253)&gt;0,ROUND(E253-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J253" s="5">
@@ -7438,7 +7438,7 @@
         <v/>
       </c>
       <c r="I254" s="6">
-        <f>IF(AND(B254="",C254="",D254="",E254="",F254=""),"",IF(OR(B254="",C254="",E254=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E254)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H254&lt;&gt;0,F254=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G254&lt;&gt;0,F254=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F254&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F254)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C254)*($E$5:$E$504=E254)*(($D$5:$D$504=D254)*(D254&lt;&gt;"")+($B$5:$B$504=B254)*(B254&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C254="Оплата",K254&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E254)&gt;0,ROUND(E254-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B254="",C254="",D254="",E254="",F254=""),"",IF(OR(B254="",C254="",E254=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E254)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H254&lt;&gt;0,F254=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G254&lt;&gt;0,F254=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F254&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F254)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C254)*($E$5:$E$504=E254)*(($D$5:$D$504=D254)*(D254&lt;&gt;"")+($B$5:$B$504=B254)*(B254&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C254="Оплата",K254&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E254)&gt;0,ROUND(E254-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J254" s="5">
@@ -7465,7 +7465,7 @@
         <v/>
       </c>
       <c r="I255" s="6">
-        <f>IF(AND(B255="",C255="",D255="",E255="",F255=""),"",IF(OR(B255="",C255="",E255=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E255)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H255&lt;&gt;0,F255=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G255&lt;&gt;0,F255=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F255&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F255)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C255)*($E$5:$E$504=E255)*(($D$5:$D$504=D255)*(D255&lt;&gt;"")+($B$5:$B$504=B255)*(B255&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C255="Оплата",K255&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E255)&gt;0,ROUND(E255-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B255="",C255="",D255="",E255="",F255=""),"",IF(OR(B255="",C255="",E255=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E255)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H255&lt;&gt;0,F255=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G255&lt;&gt;0,F255=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F255&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F255)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C255)*($E$5:$E$504=E255)*(($D$5:$D$504=D255)*(D255&lt;&gt;"")+($B$5:$B$504=B255)*(B255&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C255="Оплата",K255&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E255)&gt;0,ROUND(E255-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J255" s="5">
@@ -7492,7 +7492,7 @@
         <v/>
       </c>
       <c r="I256" s="6">
-        <f>IF(AND(B256="",C256="",D256="",E256="",F256=""),"",IF(OR(B256="",C256="",E256=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E256)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H256&lt;&gt;0,F256=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G256&lt;&gt;0,F256=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F256&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F256)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C256)*($E$5:$E$504=E256)*(($D$5:$D$504=D256)*(D256&lt;&gt;"")+($B$5:$B$504=B256)*(B256&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C256="Оплата",K256&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E256)&gt;0,ROUND(E256-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B256="",C256="",D256="",E256="",F256=""),"",IF(OR(B256="",C256="",E256=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E256)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H256&lt;&gt;0,F256=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G256&lt;&gt;0,F256=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F256&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F256)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C256)*($E$5:$E$504=E256)*(($D$5:$D$504=D256)*(D256&lt;&gt;"")+($B$5:$B$504=B256)*(B256&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C256="Оплата",K256&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E256)&gt;0,ROUND(E256-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J256" s="5">
@@ -7519,7 +7519,7 @@
         <v/>
       </c>
       <c r="I257" s="6">
-        <f>IF(AND(B257="",C257="",D257="",E257="",F257=""),"",IF(OR(B257="",C257="",E257=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E257)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H257&lt;&gt;0,F257=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G257&lt;&gt;0,F257=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F257&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F257)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C257)*($E$5:$E$504=E257)*(($D$5:$D$504=D257)*(D257&lt;&gt;"")+($B$5:$B$504=B257)*(B257&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C257="Оплата",K257&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E257)&gt;0,ROUND(E257-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B257="",C257="",D257="",E257="",F257=""),"",IF(OR(B257="",C257="",E257=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E257)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H257&lt;&gt;0,F257=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G257&lt;&gt;0,F257=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F257&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F257)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C257)*($E$5:$E$504=E257)*(($D$5:$D$504=D257)*(D257&lt;&gt;"")+($B$5:$B$504=B257)*(B257&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C257="Оплата",K257&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E257)&gt;0,ROUND(E257-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J257" s="5">
@@ -7546,7 +7546,7 @@
         <v/>
       </c>
       <c r="I258" s="6">
-        <f>IF(AND(B258="",C258="",D258="",E258="",F258=""),"",IF(OR(B258="",C258="",E258=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E258)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H258&lt;&gt;0,F258=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G258&lt;&gt;0,F258=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F258&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F258)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C258)*($E$5:$E$504=E258)*(($D$5:$D$504=D258)*(D258&lt;&gt;"")+($B$5:$B$504=B258)*(B258&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C258="Оплата",K258&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E258)&gt;0,ROUND(E258-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B258="",C258="",D258="",E258="",F258=""),"",IF(OR(B258="",C258="",E258=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E258)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H258&lt;&gt;0,F258=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G258&lt;&gt;0,F258=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F258&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F258)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C258)*($E$5:$E$504=E258)*(($D$5:$D$504=D258)*(D258&lt;&gt;"")+($B$5:$B$504=B258)*(B258&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C258="Оплата",K258&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E258)&gt;0,ROUND(E258-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J258" s="5">
@@ -7573,7 +7573,7 @@
         <v/>
       </c>
       <c r="I259" s="6">
-        <f>IF(AND(B259="",C259="",D259="",E259="",F259=""),"",IF(OR(B259="",C259="",E259=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E259)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H259&lt;&gt;0,F259=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G259&lt;&gt;0,F259=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F259&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F259)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C259)*($E$5:$E$504=E259)*(($D$5:$D$504=D259)*(D259&lt;&gt;"")+($B$5:$B$504=B259)*(B259&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C259="Оплата",K259&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E259)&gt;0,ROUND(E259-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B259="",C259="",D259="",E259="",F259=""),"",IF(OR(B259="",C259="",E259=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E259)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H259&lt;&gt;0,F259=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G259&lt;&gt;0,F259=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F259&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F259)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C259)*($E$5:$E$504=E259)*(($D$5:$D$504=D259)*(D259&lt;&gt;"")+($B$5:$B$504=B259)*(B259&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C259="Оплата",K259&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E259)&gt;0,ROUND(E259-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J259" s="5">
@@ -7600,7 +7600,7 @@
         <v/>
       </c>
       <c r="I260" s="6">
-        <f>IF(AND(B260="",C260="",D260="",E260="",F260=""),"",IF(OR(B260="",C260="",E260=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E260)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H260&lt;&gt;0,F260=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G260&lt;&gt;0,F260=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F260&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F260)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C260)*($E$5:$E$504=E260)*(($D$5:$D$504=D260)*(D260&lt;&gt;"")+($B$5:$B$504=B260)*(B260&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C260="Оплата",K260&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E260)&gt;0,ROUND(E260-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B260="",C260="",D260="",E260="",F260=""),"",IF(OR(B260="",C260="",E260=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E260)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H260&lt;&gt;0,F260=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G260&lt;&gt;0,F260=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F260&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F260)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C260)*($E$5:$E$504=E260)*(($D$5:$D$504=D260)*(D260&lt;&gt;"")+($B$5:$B$504=B260)*(B260&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C260="Оплата",K260&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E260)&gt;0,ROUND(E260-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J260" s="5">
@@ -7627,7 +7627,7 @@
         <v/>
       </c>
       <c r="I261" s="6">
-        <f>IF(AND(B261="",C261="",D261="",E261="",F261=""),"",IF(OR(B261="",C261="",E261=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E261)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H261&lt;&gt;0,F261=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G261&lt;&gt;0,F261=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F261&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F261)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C261)*($E$5:$E$504=E261)*(($D$5:$D$504=D261)*(D261&lt;&gt;"")+($B$5:$B$504=B261)*(B261&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C261="Оплата",K261&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E261)&gt;0,ROUND(E261-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B261="",C261="",D261="",E261="",F261=""),"",IF(OR(B261="",C261="",E261=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E261)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H261&lt;&gt;0,F261=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G261&lt;&gt;0,F261=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F261&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F261)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C261)*($E$5:$E$504=E261)*(($D$5:$D$504=D261)*(D261&lt;&gt;"")+($B$5:$B$504=B261)*(B261&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C261="Оплата",K261&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E261)&gt;0,ROUND(E261-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J261" s="5">
@@ -7654,7 +7654,7 @@
         <v/>
       </c>
       <c r="I262" s="6">
-        <f>IF(AND(B262="",C262="",D262="",E262="",F262=""),"",IF(OR(B262="",C262="",E262=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E262)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H262&lt;&gt;0,F262=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G262&lt;&gt;0,F262=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F262&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F262)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C262)*($E$5:$E$504=E262)*(($D$5:$D$504=D262)*(D262&lt;&gt;"")+($B$5:$B$504=B262)*(B262&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C262="Оплата",K262&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E262)&gt;0,ROUND(E262-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B262="",C262="",D262="",E262="",F262=""),"",IF(OR(B262="",C262="",E262=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E262)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H262&lt;&gt;0,F262=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G262&lt;&gt;0,F262=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F262&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F262)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C262)*($E$5:$E$504=E262)*(($D$5:$D$504=D262)*(D262&lt;&gt;"")+($B$5:$B$504=B262)*(B262&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C262="Оплата",K262&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E262)&gt;0,ROUND(E262-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J262" s="5">
@@ -7681,7 +7681,7 @@
         <v/>
       </c>
       <c r="I263" s="6">
-        <f>IF(AND(B263="",C263="",D263="",E263="",F263=""),"",IF(OR(B263="",C263="",E263=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E263)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H263&lt;&gt;0,F263=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G263&lt;&gt;0,F263=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F263&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F263)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C263)*($E$5:$E$504=E263)*(($D$5:$D$504=D263)*(D263&lt;&gt;"")+($B$5:$B$504=B263)*(B263&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C263="Оплата",K263&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E263)&gt;0,ROUND(E263-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B263="",C263="",D263="",E263="",F263=""),"",IF(OR(B263="",C263="",E263=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E263)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H263&lt;&gt;0,F263=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G263&lt;&gt;0,F263=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F263&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F263)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C263)*($E$5:$E$504=E263)*(($D$5:$D$504=D263)*(D263&lt;&gt;"")+($B$5:$B$504=B263)*(B263&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C263="Оплата",K263&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E263)&gt;0,ROUND(E263-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J263" s="5">
@@ -7708,7 +7708,7 @@
         <v/>
       </c>
       <c r="I264" s="6">
-        <f>IF(AND(B264="",C264="",D264="",E264="",F264=""),"",IF(OR(B264="",C264="",E264=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E264)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H264&lt;&gt;0,F264=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G264&lt;&gt;0,F264=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F264&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F264)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C264)*($E$5:$E$504=E264)*(($D$5:$D$504=D264)*(D264&lt;&gt;"")+($B$5:$B$504=B264)*(B264&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C264="Оплата",K264&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E264)&gt;0,ROUND(E264-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B264="",C264="",D264="",E264="",F264=""),"",IF(OR(B264="",C264="",E264=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E264)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H264&lt;&gt;0,F264=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G264&lt;&gt;0,F264=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F264&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F264)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C264)*($E$5:$E$504=E264)*(($D$5:$D$504=D264)*(D264&lt;&gt;"")+($B$5:$B$504=B264)*(B264&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C264="Оплата",K264&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E264)&gt;0,ROUND(E264-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J264" s="5">
@@ -7735,7 +7735,7 @@
         <v/>
       </c>
       <c r="I265" s="6">
-        <f>IF(AND(B265="",C265="",D265="",E265="",F265=""),"",IF(OR(B265="",C265="",E265=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E265)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H265&lt;&gt;0,F265=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G265&lt;&gt;0,F265=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F265&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F265)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C265)*($E$5:$E$504=E265)*(($D$5:$D$504=D265)*(D265&lt;&gt;"")+($B$5:$B$504=B265)*(B265&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C265="Оплата",K265&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E265)&gt;0,ROUND(E265-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B265="",C265="",D265="",E265="",F265=""),"",IF(OR(B265="",C265="",E265=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E265)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H265&lt;&gt;0,F265=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G265&lt;&gt;0,F265=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F265&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F265)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C265)*($E$5:$E$504=E265)*(($D$5:$D$504=D265)*(D265&lt;&gt;"")+($B$5:$B$504=B265)*(B265&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C265="Оплата",K265&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E265)&gt;0,ROUND(E265-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J265" s="5">
@@ -7762,7 +7762,7 @@
         <v/>
       </c>
       <c r="I266" s="6">
-        <f>IF(AND(B266="",C266="",D266="",E266="",F266=""),"",IF(OR(B266="",C266="",E266=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E266)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H266&lt;&gt;0,F266=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G266&lt;&gt;0,F266=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F266&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F266)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C266)*($E$5:$E$504=E266)*(($D$5:$D$504=D266)*(D266&lt;&gt;"")+($B$5:$B$504=B266)*(B266&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C266="Оплата",K266&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E266)&gt;0,ROUND(E266-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B266="",C266="",D266="",E266="",F266=""),"",IF(OR(B266="",C266="",E266=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E266)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H266&lt;&gt;0,F266=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G266&lt;&gt;0,F266=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F266&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F266)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C266)*($E$5:$E$504=E266)*(($D$5:$D$504=D266)*(D266&lt;&gt;"")+($B$5:$B$504=B266)*(B266&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C266="Оплата",K266&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E266)&gt;0,ROUND(E266-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J266" s="5">
@@ -7789,7 +7789,7 @@
         <v/>
       </c>
       <c r="I267" s="6">
-        <f>IF(AND(B267="",C267="",D267="",E267="",F267=""),"",IF(OR(B267="",C267="",E267=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E267)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H267&lt;&gt;0,F267=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G267&lt;&gt;0,F267=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F267&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F267)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C267)*($E$5:$E$504=E267)*(($D$5:$D$504=D267)*(D267&lt;&gt;"")+($B$5:$B$504=B267)*(B267&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C267="Оплата",K267&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E267)&gt;0,ROUND(E267-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B267="",C267="",D267="",E267="",F267=""),"",IF(OR(B267="",C267="",E267=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E267)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H267&lt;&gt;0,F267=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G267&lt;&gt;0,F267=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F267&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F267)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C267)*($E$5:$E$504=E267)*(($D$5:$D$504=D267)*(D267&lt;&gt;"")+($B$5:$B$504=B267)*(B267&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C267="Оплата",K267&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E267)&gt;0,ROUND(E267-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J267" s="5">
@@ -7816,7 +7816,7 @@
         <v/>
       </c>
       <c r="I268" s="6">
-        <f>IF(AND(B268="",C268="",D268="",E268="",F268=""),"",IF(OR(B268="",C268="",E268=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E268)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H268&lt;&gt;0,F268=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G268&lt;&gt;0,F268=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F268&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F268)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C268)*($E$5:$E$504=E268)*(($D$5:$D$504=D268)*(D268&lt;&gt;"")+($B$5:$B$504=B268)*(B268&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C268="Оплата",K268&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E268)&gt;0,ROUND(E268-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B268="",C268="",D268="",E268="",F268=""),"",IF(OR(B268="",C268="",E268=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E268)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H268&lt;&gt;0,F268=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G268&lt;&gt;0,F268=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F268&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F268)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C268)*($E$5:$E$504=E268)*(($D$5:$D$504=D268)*(D268&lt;&gt;"")+($B$5:$B$504=B268)*(B268&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C268="Оплата",K268&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E268)&gt;0,ROUND(E268-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J268" s="5">
@@ -7843,7 +7843,7 @@
         <v/>
       </c>
       <c r="I269" s="6">
-        <f>IF(AND(B269="",C269="",D269="",E269="",F269=""),"",IF(OR(B269="",C269="",E269=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E269)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H269&lt;&gt;0,F269=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G269&lt;&gt;0,F269=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F269&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F269)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C269)*($E$5:$E$504=E269)*(($D$5:$D$504=D269)*(D269&lt;&gt;"")+($B$5:$B$504=B269)*(B269&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C269="Оплата",K269&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E269)&gt;0,ROUND(E269-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B269="",C269="",D269="",E269="",F269=""),"",IF(OR(B269="",C269="",E269=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E269)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H269&lt;&gt;0,F269=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G269&lt;&gt;0,F269=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F269&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F269)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C269)*($E$5:$E$504=E269)*(($D$5:$D$504=D269)*(D269&lt;&gt;"")+($B$5:$B$504=B269)*(B269&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C269="Оплата",K269&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E269)&gt;0,ROUND(E269-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J269" s="5">
@@ -7870,7 +7870,7 @@
         <v/>
       </c>
       <c r="I270" s="6">
-        <f>IF(AND(B270="",C270="",D270="",E270="",F270=""),"",IF(OR(B270="",C270="",E270=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E270)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H270&lt;&gt;0,F270=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G270&lt;&gt;0,F270=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F270&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F270)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C270)*($E$5:$E$504=E270)*(($D$5:$D$504=D270)*(D270&lt;&gt;"")+($B$5:$B$504=B270)*(B270&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C270="Оплата",K270&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E270)&gt;0,ROUND(E270-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B270="",C270="",D270="",E270="",F270=""),"",IF(OR(B270="",C270="",E270=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E270)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H270&lt;&gt;0,F270=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G270&lt;&gt;0,F270=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F270&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F270)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C270)*($E$5:$E$504=E270)*(($D$5:$D$504=D270)*(D270&lt;&gt;"")+($B$5:$B$504=B270)*(B270&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C270="Оплата",K270&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E270)&gt;0,ROUND(E270-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J270" s="5">
@@ -7897,7 +7897,7 @@
         <v/>
       </c>
       <c r="I271" s="6">
-        <f>IF(AND(B271="",C271="",D271="",E271="",F271=""),"",IF(OR(B271="",C271="",E271=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E271)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H271&lt;&gt;0,F271=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G271&lt;&gt;0,F271=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F271&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F271)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C271)*($E$5:$E$504=E271)*(($D$5:$D$504=D271)*(D271&lt;&gt;"")+($B$5:$B$504=B271)*(B271&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C271="Оплата",K271&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E271)&gt;0,ROUND(E271-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B271="",C271="",D271="",E271="",F271=""),"",IF(OR(B271="",C271="",E271=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E271)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H271&lt;&gt;0,F271=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G271&lt;&gt;0,F271=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F271&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F271)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C271)*($E$5:$E$504=E271)*(($D$5:$D$504=D271)*(D271&lt;&gt;"")+($B$5:$B$504=B271)*(B271&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C271="Оплата",K271&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E271)&gt;0,ROUND(E271-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J271" s="5">
@@ -7924,7 +7924,7 @@
         <v/>
       </c>
       <c r="I272" s="6">
-        <f>IF(AND(B272="",C272="",D272="",E272="",F272=""),"",IF(OR(B272="",C272="",E272=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E272)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H272&lt;&gt;0,F272=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G272&lt;&gt;0,F272=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F272&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F272)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C272)*($E$5:$E$504=E272)*(($D$5:$D$504=D272)*(D272&lt;&gt;"")+($B$5:$B$504=B272)*(B272&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C272="Оплата",K272&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E272)&gt;0,ROUND(E272-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B272="",C272="",D272="",E272="",F272=""),"",IF(OR(B272="",C272="",E272=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E272)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H272&lt;&gt;0,F272=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G272&lt;&gt;0,F272=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F272&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F272)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C272)*($E$5:$E$504=E272)*(($D$5:$D$504=D272)*(D272&lt;&gt;"")+($B$5:$B$504=B272)*(B272&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C272="Оплата",K272&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E272)&gt;0,ROUND(E272-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J272" s="5">
@@ -7951,7 +7951,7 @@
         <v/>
       </c>
       <c r="I273" s="6">
-        <f>IF(AND(B273="",C273="",D273="",E273="",F273=""),"",IF(OR(B273="",C273="",E273=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E273)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H273&lt;&gt;0,F273=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G273&lt;&gt;0,F273=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F273&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F273)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C273)*($E$5:$E$504=E273)*(($D$5:$D$504=D273)*(D273&lt;&gt;"")+($B$5:$B$504=B273)*(B273&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C273="Оплата",K273&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E273)&gt;0,ROUND(E273-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B273="",C273="",D273="",E273="",F273=""),"",IF(OR(B273="",C273="",E273=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E273)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H273&lt;&gt;0,F273=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G273&lt;&gt;0,F273=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F273&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F273)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C273)*($E$5:$E$504=E273)*(($D$5:$D$504=D273)*(D273&lt;&gt;"")+($B$5:$B$504=B273)*(B273&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C273="Оплата",K273&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E273)&gt;0,ROUND(E273-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J273" s="5">
@@ -7978,7 +7978,7 @@
         <v/>
       </c>
       <c r="I274" s="6">
-        <f>IF(AND(B274="",C274="",D274="",E274="",F274=""),"",IF(OR(B274="",C274="",E274=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E274)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H274&lt;&gt;0,F274=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G274&lt;&gt;0,F274=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F274&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F274)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C274)*($E$5:$E$504=E274)*(($D$5:$D$504=D274)*(D274&lt;&gt;"")+($B$5:$B$504=B274)*(B274&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C274="Оплата",K274&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E274)&gt;0,ROUND(E274-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B274="",C274="",D274="",E274="",F274=""),"",IF(OR(B274="",C274="",E274=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E274)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H274&lt;&gt;0,F274=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G274&lt;&gt;0,F274=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F274&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F274)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C274)*($E$5:$E$504=E274)*(($D$5:$D$504=D274)*(D274&lt;&gt;"")+($B$5:$B$504=B274)*(B274&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C274="Оплата",K274&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E274)&gt;0,ROUND(E274-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J274" s="5">
@@ -8005,7 +8005,7 @@
         <v/>
       </c>
       <c r="I275" s="6">
-        <f>IF(AND(B275="",C275="",D275="",E275="",F275=""),"",IF(OR(B275="",C275="",E275=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E275)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H275&lt;&gt;0,F275=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G275&lt;&gt;0,F275=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F275&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F275)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C275)*($E$5:$E$504=E275)*(($D$5:$D$504=D275)*(D275&lt;&gt;"")+($B$5:$B$504=B275)*(B275&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C275="Оплата",K275&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E275)&gt;0,ROUND(E275-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B275="",C275="",D275="",E275="",F275=""),"",IF(OR(B275="",C275="",E275=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E275)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H275&lt;&gt;0,F275=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G275&lt;&gt;0,F275=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F275&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F275)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C275)*($E$5:$E$504=E275)*(($D$5:$D$504=D275)*(D275&lt;&gt;"")+($B$5:$B$504=B275)*(B275&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C275="Оплата",K275&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E275)&gt;0,ROUND(E275-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J275" s="5">
@@ -8032,7 +8032,7 @@
         <v/>
       </c>
       <c r="I276" s="6">
-        <f>IF(AND(B276="",C276="",D276="",E276="",F276=""),"",IF(OR(B276="",C276="",E276=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E276)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H276&lt;&gt;0,F276=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G276&lt;&gt;0,F276=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F276&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F276)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C276)*($E$5:$E$504=E276)*(($D$5:$D$504=D276)*(D276&lt;&gt;"")+($B$5:$B$504=B276)*(B276&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C276="Оплата",K276&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E276)&gt;0,ROUND(E276-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B276="",C276="",D276="",E276="",F276=""),"",IF(OR(B276="",C276="",E276=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E276)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H276&lt;&gt;0,F276=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G276&lt;&gt;0,F276=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F276&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F276)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C276)*($E$5:$E$504=E276)*(($D$5:$D$504=D276)*(D276&lt;&gt;"")+($B$5:$B$504=B276)*(B276&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C276="Оплата",K276&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E276)&gt;0,ROUND(E276-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J276" s="5">
@@ -8059,7 +8059,7 @@
         <v/>
       </c>
       <c r="I277" s="6">
-        <f>IF(AND(B277="",C277="",D277="",E277="",F277=""),"",IF(OR(B277="",C277="",E277=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E277)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H277&lt;&gt;0,F277=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G277&lt;&gt;0,F277=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F277&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F277)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C277)*($E$5:$E$504=E277)*(($D$5:$D$504=D277)*(D277&lt;&gt;"")+($B$5:$B$504=B277)*(B277&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C277="Оплата",K277&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E277)&gt;0,ROUND(E277-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B277="",C277="",D277="",E277="",F277=""),"",IF(OR(B277="",C277="",E277=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E277)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H277&lt;&gt;0,F277=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G277&lt;&gt;0,F277=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F277&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F277)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C277)*($E$5:$E$504=E277)*(($D$5:$D$504=D277)*(D277&lt;&gt;"")+($B$5:$B$504=B277)*(B277&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C277="Оплата",K277&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E277)&gt;0,ROUND(E277-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J277" s="5">
@@ -8086,7 +8086,7 @@
         <v/>
       </c>
       <c r="I278" s="6">
-        <f>IF(AND(B278="",C278="",D278="",E278="",F278=""),"",IF(OR(B278="",C278="",E278=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E278)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H278&lt;&gt;0,F278=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G278&lt;&gt;0,F278=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F278&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F278)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C278)*($E$5:$E$504=E278)*(($D$5:$D$504=D278)*(D278&lt;&gt;"")+($B$5:$B$504=B278)*(B278&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C278="Оплата",K278&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E278)&gt;0,ROUND(E278-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B278="",C278="",D278="",E278="",F278=""),"",IF(OR(B278="",C278="",E278=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E278)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H278&lt;&gt;0,F278=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G278&lt;&gt;0,F278=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F278&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F278)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C278)*($E$5:$E$504=E278)*(($D$5:$D$504=D278)*(D278&lt;&gt;"")+($B$5:$B$504=B278)*(B278&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C278="Оплата",K278&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E278)&gt;0,ROUND(E278-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J278" s="5">
@@ -8113,7 +8113,7 @@
         <v/>
       </c>
       <c r="I279" s="6">
-        <f>IF(AND(B279="",C279="",D279="",E279="",F279=""),"",IF(OR(B279="",C279="",E279=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E279)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H279&lt;&gt;0,F279=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G279&lt;&gt;0,F279=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F279&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F279)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C279)*($E$5:$E$504=E279)*(($D$5:$D$504=D279)*(D279&lt;&gt;"")+($B$5:$B$504=B279)*(B279&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C279="Оплата",K279&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E279)&gt;0,ROUND(E279-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B279="",C279="",D279="",E279="",F279=""),"",IF(OR(B279="",C279="",E279=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E279)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H279&lt;&gt;0,F279=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G279&lt;&gt;0,F279=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F279&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F279)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C279)*($E$5:$E$504=E279)*(($D$5:$D$504=D279)*(D279&lt;&gt;"")+($B$5:$B$504=B279)*(B279&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C279="Оплата",K279&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E279)&gt;0,ROUND(E279-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J279" s="5">
@@ -8140,7 +8140,7 @@
         <v/>
       </c>
       <c r="I280" s="6">
-        <f>IF(AND(B280="",C280="",D280="",E280="",F280=""),"",IF(OR(B280="",C280="",E280=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E280)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H280&lt;&gt;0,F280=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G280&lt;&gt;0,F280=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F280&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F280)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C280)*($E$5:$E$504=E280)*(($D$5:$D$504=D280)*(D280&lt;&gt;"")+($B$5:$B$504=B280)*(B280&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C280="Оплата",K280&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E280)&gt;0,ROUND(E280-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B280="",C280="",D280="",E280="",F280=""),"",IF(OR(B280="",C280="",E280=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E280)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H280&lt;&gt;0,F280=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G280&lt;&gt;0,F280=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F280&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F280)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C280)*($E$5:$E$504=E280)*(($D$5:$D$504=D280)*(D280&lt;&gt;"")+($B$5:$B$504=B280)*(B280&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C280="Оплата",K280&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E280)&gt;0,ROUND(E280-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J280" s="5">
@@ -8167,7 +8167,7 @@
         <v/>
       </c>
       <c r="I281" s="6">
-        <f>IF(AND(B281="",C281="",D281="",E281="",F281=""),"",IF(OR(B281="",C281="",E281=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E281)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H281&lt;&gt;0,F281=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G281&lt;&gt;0,F281=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F281&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F281)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C281)*($E$5:$E$504=E281)*(($D$5:$D$504=D281)*(D281&lt;&gt;"")+($B$5:$B$504=B281)*(B281&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C281="Оплата",K281&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E281)&gt;0,ROUND(E281-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B281="",C281="",D281="",E281="",F281=""),"",IF(OR(B281="",C281="",E281=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E281)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H281&lt;&gt;0,F281=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G281&lt;&gt;0,F281=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F281&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F281)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C281)*($E$5:$E$504=E281)*(($D$5:$D$504=D281)*(D281&lt;&gt;"")+($B$5:$B$504=B281)*(B281&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C281="Оплата",K281&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E281)&gt;0,ROUND(E281-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J281" s="5">
@@ -8194,7 +8194,7 @@
         <v/>
       </c>
       <c r="I282" s="6">
-        <f>IF(AND(B282="",C282="",D282="",E282="",F282=""),"",IF(OR(B282="",C282="",E282=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E282)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H282&lt;&gt;0,F282=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G282&lt;&gt;0,F282=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F282&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F282)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C282)*($E$5:$E$504=E282)*(($D$5:$D$504=D282)*(D282&lt;&gt;"")+($B$5:$B$504=B282)*(B282&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C282="Оплата",K282&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E282)&gt;0,ROUND(E282-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B282="",C282="",D282="",E282="",F282=""),"",IF(OR(B282="",C282="",E282=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E282)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H282&lt;&gt;0,F282=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G282&lt;&gt;0,F282=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F282&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F282)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C282)*($E$5:$E$504=E282)*(($D$5:$D$504=D282)*(D282&lt;&gt;"")+($B$5:$B$504=B282)*(B282&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C282="Оплата",K282&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E282)&gt;0,ROUND(E282-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J282" s="5">
@@ -8221,7 +8221,7 @@
         <v/>
       </c>
       <c r="I283" s="6">
-        <f>IF(AND(B283="",C283="",D283="",E283="",F283=""),"",IF(OR(B283="",C283="",E283=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E283)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H283&lt;&gt;0,F283=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G283&lt;&gt;0,F283=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F283&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F283)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C283)*($E$5:$E$504=E283)*(($D$5:$D$504=D283)*(D283&lt;&gt;"")+($B$5:$B$504=B283)*(B283&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C283="Оплата",K283&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E283)&gt;0,ROUND(E283-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B283="",C283="",D283="",E283="",F283=""),"",IF(OR(B283="",C283="",E283=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E283)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H283&lt;&gt;0,F283=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G283&lt;&gt;0,F283=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F283&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F283)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C283)*($E$5:$E$504=E283)*(($D$5:$D$504=D283)*(D283&lt;&gt;"")+($B$5:$B$504=B283)*(B283&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C283="Оплата",K283&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E283)&gt;0,ROUND(E283-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J283" s="5">
@@ -8248,7 +8248,7 @@
         <v/>
       </c>
       <c r="I284" s="6">
-        <f>IF(AND(B284="",C284="",D284="",E284="",F284=""),"",IF(OR(B284="",C284="",E284=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E284)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H284&lt;&gt;0,F284=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G284&lt;&gt;0,F284=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F284&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F284)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C284)*($E$5:$E$504=E284)*(($D$5:$D$504=D284)*(D284&lt;&gt;"")+($B$5:$B$504=B284)*(B284&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C284="Оплата",K284&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E284)&gt;0,ROUND(E284-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B284="",C284="",D284="",E284="",F284=""),"",IF(OR(B284="",C284="",E284=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E284)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H284&lt;&gt;0,F284=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G284&lt;&gt;0,F284=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F284&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F284)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C284)*($E$5:$E$504=E284)*(($D$5:$D$504=D284)*(D284&lt;&gt;"")+($B$5:$B$504=B284)*(B284&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C284="Оплата",K284&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E284)&gt;0,ROUND(E284-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J284" s="5">
@@ -8275,7 +8275,7 @@
         <v/>
       </c>
       <c r="I285" s="6">
-        <f>IF(AND(B285="",C285="",D285="",E285="",F285=""),"",IF(OR(B285="",C285="",E285=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E285)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H285&lt;&gt;0,F285=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G285&lt;&gt;0,F285=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F285&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F285)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C285)*($E$5:$E$504=E285)*(($D$5:$D$504=D285)*(D285&lt;&gt;"")+($B$5:$B$504=B285)*(B285&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C285="Оплата",K285&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E285)&gt;0,ROUND(E285-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B285="",C285="",D285="",E285="",F285=""),"",IF(OR(B285="",C285="",E285=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E285)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H285&lt;&gt;0,F285=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G285&lt;&gt;0,F285=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F285&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F285)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C285)*($E$5:$E$504=E285)*(($D$5:$D$504=D285)*(D285&lt;&gt;"")+($B$5:$B$504=B285)*(B285&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C285="Оплата",K285&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E285)&gt;0,ROUND(E285-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J285" s="5">
@@ -8302,7 +8302,7 @@
         <v/>
       </c>
       <c r="I286" s="6">
-        <f>IF(AND(B286="",C286="",D286="",E286="",F286=""),"",IF(OR(B286="",C286="",E286=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E286)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H286&lt;&gt;0,F286=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G286&lt;&gt;0,F286=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F286&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F286)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C286)*($E$5:$E$504=E286)*(($D$5:$D$504=D286)*(D286&lt;&gt;"")+($B$5:$B$504=B286)*(B286&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C286="Оплата",K286&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E286)&gt;0,ROUND(E286-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B286="",C286="",D286="",E286="",F286=""),"",IF(OR(B286="",C286="",E286=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E286)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H286&lt;&gt;0,F286=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G286&lt;&gt;0,F286=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F286&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F286)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C286)*($E$5:$E$504=E286)*(($D$5:$D$504=D286)*(D286&lt;&gt;"")+($B$5:$B$504=B286)*(B286&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C286="Оплата",K286&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E286)&gt;0,ROUND(E286-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J286" s="5">
@@ -8329,7 +8329,7 @@
         <v/>
       </c>
       <c r="I287" s="6">
-        <f>IF(AND(B287="",C287="",D287="",E287="",F287=""),"",IF(OR(B287="",C287="",E287=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E287)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H287&lt;&gt;0,F287=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G287&lt;&gt;0,F287=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F287&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F287)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C287)*($E$5:$E$504=E287)*(($D$5:$D$504=D287)*(D287&lt;&gt;"")+($B$5:$B$504=B287)*(B287&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C287="Оплата",K287&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E287)&gt;0,ROUND(E287-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B287="",C287="",D287="",E287="",F287=""),"",IF(OR(B287="",C287="",E287=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E287)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H287&lt;&gt;0,F287=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G287&lt;&gt;0,F287=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F287&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F287)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C287)*($E$5:$E$504=E287)*(($D$5:$D$504=D287)*(D287&lt;&gt;"")+($B$5:$B$504=B287)*(B287&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C287="Оплата",K287&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E287)&gt;0,ROUND(E287-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J287" s="5">
@@ -8356,7 +8356,7 @@
         <v/>
       </c>
       <c r="I288" s="6">
-        <f>IF(AND(B288="",C288="",D288="",E288="",F288=""),"",IF(OR(B288="",C288="",E288=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E288)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H288&lt;&gt;0,F288=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G288&lt;&gt;0,F288=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F288&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F288)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C288)*($E$5:$E$504=E288)*(($D$5:$D$504=D288)*(D288&lt;&gt;"")+($B$5:$B$504=B288)*(B288&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C288="Оплата",K288&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E288)&gt;0,ROUND(E288-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B288="",C288="",D288="",E288="",F288=""),"",IF(OR(B288="",C288="",E288=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E288)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H288&lt;&gt;0,F288=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G288&lt;&gt;0,F288=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F288&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F288)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C288)*($E$5:$E$504=E288)*(($D$5:$D$504=D288)*(D288&lt;&gt;"")+($B$5:$B$504=B288)*(B288&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C288="Оплата",K288&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E288)&gt;0,ROUND(E288-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J288" s="5">
@@ -8383,7 +8383,7 @@
         <v/>
       </c>
       <c r="I289" s="6">
-        <f>IF(AND(B289="",C289="",D289="",E289="",F289=""),"",IF(OR(B289="",C289="",E289=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E289)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H289&lt;&gt;0,F289=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G289&lt;&gt;0,F289=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F289&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F289)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C289)*($E$5:$E$504=E289)*(($D$5:$D$504=D289)*(D289&lt;&gt;"")+($B$5:$B$504=B289)*(B289&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C289="Оплата",K289&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E289)&gt;0,ROUND(E289-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B289="",C289="",D289="",E289="",F289=""),"",IF(OR(B289="",C289="",E289=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E289)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H289&lt;&gt;0,F289=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G289&lt;&gt;0,F289=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F289&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F289)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C289)*($E$5:$E$504=E289)*(($D$5:$D$504=D289)*(D289&lt;&gt;"")+($B$5:$B$504=B289)*(B289&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C289="Оплата",K289&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E289)&gt;0,ROUND(E289-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J289" s="5">
@@ -8410,7 +8410,7 @@
         <v/>
       </c>
       <c r="I290" s="6">
-        <f>IF(AND(B290="",C290="",D290="",E290="",F290=""),"",IF(OR(B290="",C290="",E290=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E290)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H290&lt;&gt;0,F290=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G290&lt;&gt;0,F290=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F290&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F290)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C290)*($E$5:$E$504=E290)*(($D$5:$D$504=D290)*(D290&lt;&gt;"")+($B$5:$B$504=B290)*(B290&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C290="Оплата",K290&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E290)&gt;0,ROUND(E290-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B290="",C290="",D290="",E290="",F290=""),"",IF(OR(B290="",C290="",E290=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E290)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H290&lt;&gt;0,F290=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G290&lt;&gt;0,F290=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F290&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F290)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C290)*($E$5:$E$504=E290)*(($D$5:$D$504=D290)*(D290&lt;&gt;"")+($B$5:$B$504=B290)*(B290&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C290="Оплата",K290&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E290)&gt;0,ROUND(E290-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J290" s="5">
@@ -8437,7 +8437,7 @@
         <v/>
       </c>
       <c r="I291" s="6">
-        <f>IF(AND(B291="",C291="",D291="",E291="",F291=""),"",IF(OR(B291="",C291="",E291=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E291)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H291&lt;&gt;0,F291=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G291&lt;&gt;0,F291=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F291&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F291)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C291)*($E$5:$E$504=E291)*(($D$5:$D$504=D291)*(D291&lt;&gt;"")+($B$5:$B$504=B291)*(B291&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C291="Оплата",K291&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E291)&gt;0,ROUND(E291-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B291="",C291="",D291="",E291="",F291=""),"",IF(OR(B291="",C291="",E291=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E291)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H291&lt;&gt;0,F291=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G291&lt;&gt;0,F291=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F291&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F291)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C291)*($E$5:$E$504=E291)*(($D$5:$D$504=D291)*(D291&lt;&gt;"")+($B$5:$B$504=B291)*(B291&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C291="Оплата",K291&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E291)&gt;0,ROUND(E291-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J291" s="5">
@@ -8464,7 +8464,7 @@
         <v/>
       </c>
       <c r="I292" s="6">
-        <f>IF(AND(B292="",C292="",D292="",E292="",F292=""),"",IF(OR(B292="",C292="",E292=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E292)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H292&lt;&gt;0,F292=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G292&lt;&gt;0,F292=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F292&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F292)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C292)*($E$5:$E$504=E292)*(($D$5:$D$504=D292)*(D292&lt;&gt;"")+($B$5:$B$504=B292)*(B292&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C292="Оплата",K292&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E292)&gt;0,ROUND(E292-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B292="",C292="",D292="",E292="",F292=""),"",IF(OR(B292="",C292="",E292=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E292)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H292&lt;&gt;0,F292=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G292&lt;&gt;0,F292=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F292&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F292)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C292)*($E$5:$E$504=E292)*(($D$5:$D$504=D292)*(D292&lt;&gt;"")+($B$5:$B$504=B292)*(B292&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C292="Оплата",K292&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E292)&gt;0,ROUND(E292-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J292" s="5">
@@ -8491,7 +8491,7 @@
         <v/>
       </c>
       <c r="I293" s="6">
-        <f>IF(AND(B293="",C293="",D293="",E293="",F293=""),"",IF(OR(B293="",C293="",E293=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E293)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H293&lt;&gt;0,F293=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G293&lt;&gt;0,F293=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F293&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F293)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C293)*($E$5:$E$504=E293)*(($D$5:$D$504=D293)*(D293&lt;&gt;"")+($B$5:$B$504=B293)*(B293&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C293="Оплата",K293&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E293)&gt;0,ROUND(E293-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B293="",C293="",D293="",E293="",F293=""),"",IF(OR(B293="",C293="",E293=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E293)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H293&lt;&gt;0,F293=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G293&lt;&gt;0,F293=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F293&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F293)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C293)*($E$5:$E$504=E293)*(($D$5:$D$504=D293)*(D293&lt;&gt;"")+($B$5:$B$504=B293)*(B293&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C293="Оплата",K293&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E293)&gt;0,ROUND(E293-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J293" s="5">
@@ -8518,7 +8518,7 @@
         <v/>
       </c>
       <c r="I294" s="6">
-        <f>IF(AND(B294="",C294="",D294="",E294="",F294=""),"",IF(OR(B294="",C294="",E294=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E294)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H294&lt;&gt;0,F294=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G294&lt;&gt;0,F294=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F294&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F294)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C294)*($E$5:$E$504=E294)*(($D$5:$D$504=D294)*(D294&lt;&gt;"")+($B$5:$B$504=B294)*(B294&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C294="Оплата",K294&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E294)&gt;0,ROUND(E294-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B294="",C294="",D294="",E294="",F294=""),"",IF(OR(B294="",C294="",E294=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E294)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H294&lt;&gt;0,F294=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G294&lt;&gt;0,F294=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F294&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F294)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C294)*($E$5:$E$504=E294)*(($D$5:$D$504=D294)*(D294&lt;&gt;"")+($B$5:$B$504=B294)*(B294&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C294="Оплата",K294&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E294)&gt;0,ROUND(E294-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J294" s="5">
@@ -8545,7 +8545,7 @@
         <v/>
       </c>
       <c r="I295" s="6">
-        <f>IF(AND(B295="",C295="",D295="",E295="",F295=""),"",IF(OR(B295="",C295="",E295=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E295)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H295&lt;&gt;0,F295=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G295&lt;&gt;0,F295=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F295&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F295)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C295)*($E$5:$E$504=E295)*(($D$5:$D$504=D295)*(D295&lt;&gt;"")+($B$5:$B$504=B295)*(B295&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C295="Оплата",K295&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E295)&gt;0,ROUND(E295-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B295="",C295="",D295="",E295="",F295=""),"",IF(OR(B295="",C295="",E295=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E295)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H295&lt;&gt;0,F295=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G295&lt;&gt;0,F295=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F295&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F295)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C295)*($E$5:$E$504=E295)*(($D$5:$D$504=D295)*(D295&lt;&gt;"")+($B$5:$B$504=B295)*(B295&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C295="Оплата",K295&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E295)&gt;0,ROUND(E295-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J295" s="5">
@@ -8572,7 +8572,7 @@
         <v/>
       </c>
       <c r="I296" s="6">
-        <f>IF(AND(B296="",C296="",D296="",E296="",F296=""),"",IF(OR(B296="",C296="",E296=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E296)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H296&lt;&gt;0,F296=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G296&lt;&gt;0,F296=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F296&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F296)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C296)*($E$5:$E$504=E296)*(($D$5:$D$504=D296)*(D296&lt;&gt;"")+($B$5:$B$504=B296)*(B296&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C296="Оплата",K296&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E296)&gt;0,ROUND(E296-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B296="",C296="",D296="",E296="",F296=""),"",IF(OR(B296="",C296="",E296=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E296)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H296&lt;&gt;0,F296=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G296&lt;&gt;0,F296=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F296&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F296)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C296)*($E$5:$E$504=E296)*(($D$5:$D$504=D296)*(D296&lt;&gt;"")+($B$5:$B$504=B296)*(B296&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C296="Оплата",K296&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E296)&gt;0,ROUND(E296-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J296" s="5">
@@ -8599,7 +8599,7 @@
         <v/>
       </c>
       <c r="I297" s="6">
-        <f>IF(AND(B297="",C297="",D297="",E297="",F297=""),"",IF(OR(B297="",C297="",E297=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E297)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H297&lt;&gt;0,F297=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G297&lt;&gt;0,F297=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F297&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F297)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C297)*($E$5:$E$504=E297)*(($D$5:$D$504=D297)*(D297&lt;&gt;"")+($B$5:$B$504=B297)*(B297&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C297="Оплата",K297&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E297)&gt;0,ROUND(E297-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B297="",C297="",D297="",E297="",F297=""),"",IF(OR(B297="",C297="",E297=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E297)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H297&lt;&gt;0,F297=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G297&lt;&gt;0,F297=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F297&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F297)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C297)*($E$5:$E$504=E297)*(($D$5:$D$504=D297)*(D297&lt;&gt;"")+($B$5:$B$504=B297)*(B297&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C297="Оплата",K297&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E297)&gt;0,ROUND(E297-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J297" s="5">
@@ -8626,7 +8626,7 @@
         <v/>
       </c>
       <c r="I298" s="6">
-        <f>IF(AND(B298="",C298="",D298="",E298="",F298=""),"",IF(OR(B298="",C298="",E298=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E298)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H298&lt;&gt;0,F298=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G298&lt;&gt;0,F298=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F298&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F298)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C298)*($E$5:$E$504=E298)*(($D$5:$D$504=D298)*(D298&lt;&gt;"")+($B$5:$B$504=B298)*(B298&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C298="Оплата",K298&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E298)&gt;0,ROUND(E298-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B298="",C298="",D298="",E298="",F298=""),"",IF(OR(B298="",C298="",E298=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E298)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H298&lt;&gt;0,F298=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G298&lt;&gt;0,F298=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F298&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F298)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C298)*($E$5:$E$504=E298)*(($D$5:$D$504=D298)*(D298&lt;&gt;"")+($B$5:$B$504=B298)*(B298&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C298="Оплата",K298&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E298)&gt;0,ROUND(E298-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J298" s="5">
@@ -8653,7 +8653,7 @@
         <v/>
       </c>
       <c r="I299" s="6">
-        <f>IF(AND(B299="",C299="",D299="",E299="",F299=""),"",IF(OR(B299="",C299="",E299=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E299)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H299&lt;&gt;0,F299=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G299&lt;&gt;0,F299=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F299&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F299)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C299)*($E$5:$E$504=E299)*(($D$5:$D$504=D299)*(D299&lt;&gt;"")+($B$5:$B$504=B299)*(B299&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C299="Оплата",K299&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E299)&gt;0,ROUND(E299-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B299="",C299="",D299="",E299="",F299=""),"",IF(OR(B299="",C299="",E299=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E299)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H299&lt;&gt;0,F299=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G299&lt;&gt;0,F299=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F299&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F299)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C299)*($E$5:$E$504=E299)*(($D$5:$D$504=D299)*(D299&lt;&gt;"")+($B$5:$B$504=B299)*(B299&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C299="Оплата",K299&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E299)&gt;0,ROUND(E299-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J299" s="5">
@@ -8680,7 +8680,7 @@
         <v/>
       </c>
       <c r="I300" s="6">
-        <f>IF(AND(B300="",C300="",D300="",E300="",F300=""),"",IF(OR(B300="",C300="",E300=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E300)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H300&lt;&gt;0,F300=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G300&lt;&gt;0,F300=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F300&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F300)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C300)*($E$5:$E$504=E300)*(($D$5:$D$504=D300)*(D300&lt;&gt;"")+($B$5:$B$504=B300)*(B300&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C300="Оплата",K300&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E300)&gt;0,ROUND(E300-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B300="",C300="",D300="",E300="",F300=""),"",IF(OR(B300="",C300="",E300=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E300)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H300&lt;&gt;0,F300=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G300&lt;&gt;0,F300=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F300&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F300)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C300)*($E$5:$E$504=E300)*(($D$5:$D$504=D300)*(D300&lt;&gt;"")+($B$5:$B$504=B300)*(B300&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C300="Оплата",K300&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E300)&gt;0,ROUND(E300-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J300" s="5">
@@ -8707,7 +8707,7 @@
         <v/>
       </c>
       <c r="I301" s="6">
-        <f>IF(AND(B301="",C301="",D301="",E301="",F301=""),"",IF(OR(B301="",C301="",E301=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E301)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H301&lt;&gt;0,F301=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G301&lt;&gt;0,F301=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F301&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F301)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C301)*($E$5:$E$504=E301)*(($D$5:$D$504=D301)*(D301&lt;&gt;"")+($B$5:$B$504=B301)*(B301&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C301="Оплата",K301&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E301)&gt;0,ROUND(E301-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B301="",C301="",D301="",E301="",F301=""),"",IF(OR(B301="",C301="",E301=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E301)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H301&lt;&gt;0,F301=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G301&lt;&gt;0,F301=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F301&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F301)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C301)*($E$5:$E$504=E301)*(($D$5:$D$504=D301)*(D301&lt;&gt;"")+($B$5:$B$504=B301)*(B301&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C301="Оплата",K301&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E301)&gt;0,ROUND(E301-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J301" s="5">
@@ -8734,7 +8734,7 @@
         <v/>
       </c>
       <c r="I302" s="6">
-        <f>IF(AND(B302="",C302="",D302="",E302="",F302=""),"",IF(OR(B302="",C302="",E302=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E302)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H302&lt;&gt;0,F302=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G302&lt;&gt;0,F302=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F302&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F302)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C302)*($E$5:$E$504=E302)*(($D$5:$D$504=D302)*(D302&lt;&gt;"")+($B$5:$B$504=B302)*(B302&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C302="Оплата",K302&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E302)&gt;0,ROUND(E302-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B302="",C302="",D302="",E302="",F302=""),"",IF(OR(B302="",C302="",E302=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E302)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H302&lt;&gt;0,F302=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G302&lt;&gt;0,F302=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F302&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F302)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C302)*($E$5:$E$504=E302)*(($D$5:$D$504=D302)*(D302&lt;&gt;"")+($B$5:$B$504=B302)*(B302&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C302="Оплата",K302&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E302)&gt;0,ROUND(E302-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J302" s="5">
@@ -8761,7 +8761,7 @@
         <v/>
       </c>
       <c r="I303" s="6">
-        <f>IF(AND(B303="",C303="",D303="",E303="",F303=""),"",IF(OR(B303="",C303="",E303=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E303)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H303&lt;&gt;0,F303=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G303&lt;&gt;0,F303=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F303&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F303)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C303)*($E$5:$E$504=E303)*(($D$5:$D$504=D303)*(D303&lt;&gt;"")+($B$5:$B$504=B303)*(B303&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C303="Оплата",K303&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E303)&gt;0,ROUND(E303-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B303="",C303="",D303="",E303="",F303=""),"",IF(OR(B303="",C303="",E303=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E303)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H303&lt;&gt;0,F303=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G303&lt;&gt;0,F303=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F303&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F303)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C303)*($E$5:$E$504=E303)*(($D$5:$D$504=D303)*(D303&lt;&gt;"")+($B$5:$B$504=B303)*(B303&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C303="Оплата",K303&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E303)&gt;0,ROUND(E303-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J303" s="5">
@@ -8788,7 +8788,7 @@
         <v/>
       </c>
       <c r="I304" s="6">
-        <f>IF(AND(B304="",C304="",D304="",E304="",F304=""),"",IF(OR(B304="",C304="",E304=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E304)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H304&lt;&gt;0,F304=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G304&lt;&gt;0,F304=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F304&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F304)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C304)*($E$5:$E$504=E304)*(($D$5:$D$504=D304)*(D304&lt;&gt;"")+($B$5:$B$504=B304)*(B304&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C304="Оплата",K304&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E304)&gt;0,ROUND(E304-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B304="",C304="",D304="",E304="",F304=""),"",IF(OR(B304="",C304="",E304=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E304)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H304&lt;&gt;0,F304=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G304&lt;&gt;0,F304=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F304&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F304)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C304)*($E$5:$E$504=E304)*(($D$5:$D$504=D304)*(D304&lt;&gt;"")+($B$5:$B$504=B304)*(B304&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C304="Оплата",K304&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E304)&gt;0,ROUND(E304-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J304" s="5">
@@ -8815,7 +8815,7 @@
         <v/>
       </c>
       <c r="I305" s="6">
-        <f>IF(AND(B305="",C305="",D305="",E305="",F305=""),"",IF(OR(B305="",C305="",E305=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E305)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H305&lt;&gt;0,F305=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G305&lt;&gt;0,F305=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F305&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F305)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C305)*($E$5:$E$504=E305)*(($D$5:$D$504=D305)*(D305&lt;&gt;"")+($B$5:$B$504=B305)*(B305&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C305="Оплата",K305&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E305)&gt;0,ROUND(E305-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B305="",C305="",D305="",E305="",F305=""),"",IF(OR(B305="",C305="",E305=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E305)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H305&lt;&gt;0,F305=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G305&lt;&gt;0,F305=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F305&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F305)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C305)*($E$5:$E$504=E305)*(($D$5:$D$504=D305)*(D305&lt;&gt;"")+($B$5:$B$504=B305)*(B305&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C305="Оплата",K305&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E305)&gt;0,ROUND(E305-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J305" s="5">
@@ -8842,7 +8842,7 @@
         <v/>
       </c>
       <c r="I306" s="6">
-        <f>IF(AND(B306="",C306="",D306="",E306="",F306=""),"",IF(OR(B306="",C306="",E306=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E306)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H306&lt;&gt;0,F306=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G306&lt;&gt;0,F306=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F306&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F306)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C306)*($E$5:$E$504=E306)*(($D$5:$D$504=D306)*(D306&lt;&gt;"")+($B$5:$B$504=B306)*(B306&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C306="Оплата",K306&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E306)&gt;0,ROUND(E306-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B306="",C306="",D306="",E306="",F306=""),"",IF(OR(B306="",C306="",E306=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E306)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H306&lt;&gt;0,F306=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G306&lt;&gt;0,F306=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F306&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F306)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C306)*($E$5:$E$504=E306)*(($D$5:$D$504=D306)*(D306&lt;&gt;"")+($B$5:$B$504=B306)*(B306&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C306="Оплата",K306&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E306)&gt;0,ROUND(E306-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J306" s="5">
@@ -8869,7 +8869,7 @@
         <v/>
       </c>
       <c r="I307" s="6">
-        <f>IF(AND(B307="",C307="",D307="",E307="",F307=""),"",IF(OR(B307="",C307="",E307=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E307)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H307&lt;&gt;0,F307=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G307&lt;&gt;0,F307=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F307&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F307)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C307)*($E$5:$E$504=E307)*(($D$5:$D$504=D307)*(D307&lt;&gt;"")+($B$5:$B$504=B307)*(B307&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C307="Оплата",K307&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E307)&gt;0,ROUND(E307-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B307="",C307="",D307="",E307="",F307=""),"",IF(OR(B307="",C307="",E307=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E307)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H307&lt;&gt;0,F307=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G307&lt;&gt;0,F307=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F307&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F307)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C307)*($E$5:$E$504=E307)*(($D$5:$D$504=D307)*(D307&lt;&gt;"")+($B$5:$B$504=B307)*(B307&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C307="Оплата",K307&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E307)&gt;0,ROUND(E307-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J307" s="5">
@@ -8896,7 +8896,7 @@
         <v/>
       </c>
       <c r="I308" s="6">
-        <f>IF(AND(B308="",C308="",D308="",E308="",F308=""),"",IF(OR(B308="",C308="",E308=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E308)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H308&lt;&gt;0,F308=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G308&lt;&gt;0,F308=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F308&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F308)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C308)*($E$5:$E$504=E308)*(($D$5:$D$504=D308)*(D308&lt;&gt;"")+($B$5:$B$504=B308)*(B308&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C308="Оплата",K308&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E308)&gt;0,ROUND(E308-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B308="",C308="",D308="",E308="",F308=""),"",IF(OR(B308="",C308="",E308=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E308)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H308&lt;&gt;0,F308=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G308&lt;&gt;0,F308=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F308&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F308)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C308)*($E$5:$E$504=E308)*(($D$5:$D$504=D308)*(D308&lt;&gt;"")+($B$5:$B$504=B308)*(B308&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C308="Оплата",K308&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E308)&gt;0,ROUND(E308-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J308" s="5">
@@ -8923,7 +8923,7 @@
         <v/>
       </c>
       <c r="I309" s="6">
-        <f>IF(AND(B309="",C309="",D309="",E309="",F309=""),"",IF(OR(B309="",C309="",E309=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E309)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H309&lt;&gt;0,F309=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G309&lt;&gt;0,F309=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F309&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F309)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C309)*($E$5:$E$504=E309)*(($D$5:$D$504=D309)*(D309&lt;&gt;"")+($B$5:$B$504=B309)*(B309&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C309="Оплата",K309&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E309)&gt;0,ROUND(E309-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B309="",C309="",D309="",E309="",F309=""),"",IF(OR(B309="",C309="",E309=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E309)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H309&lt;&gt;0,F309=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G309&lt;&gt;0,F309=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F309&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F309)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C309)*($E$5:$E$504=E309)*(($D$5:$D$504=D309)*(D309&lt;&gt;"")+($B$5:$B$504=B309)*(B309&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C309="Оплата",K309&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E309)&gt;0,ROUND(E309-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J309" s="5">
@@ -8950,7 +8950,7 @@
         <v/>
       </c>
       <c r="I310" s="6">
-        <f>IF(AND(B310="",C310="",D310="",E310="",F310=""),"",IF(OR(B310="",C310="",E310=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E310)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H310&lt;&gt;0,F310=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G310&lt;&gt;0,F310=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F310&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F310)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C310)*($E$5:$E$504=E310)*(($D$5:$D$504=D310)*(D310&lt;&gt;"")+($B$5:$B$504=B310)*(B310&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C310="Оплата",K310&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E310)&gt;0,ROUND(E310-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B310="",C310="",D310="",E310="",F310=""),"",IF(OR(B310="",C310="",E310=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E310)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H310&lt;&gt;0,F310=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G310&lt;&gt;0,F310=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F310&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F310)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C310)*($E$5:$E$504=E310)*(($D$5:$D$504=D310)*(D310&lt;&gt;"")+($B$5:$B$504=B310)*(B310&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C310="Оплата",K310&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E310)&gt;0,ROUND(E310-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J310" s="5">
@@ -8977,7 +8977,7 @@
         <v/>
       </c>
       <c r="I311" s="6">
-        <f>IF(AND(B311="",C311="",D311="",E311="",F311=""),"",IF(OR(B311="",C311="",E311=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E311)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H311&lt;&gt;0,F311=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G311&lt;&gt;0,F311=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F311&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F311)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C311)*($E$5:$E$504=E311)*(($D$5:$D$504=D311)*(D311&lt;&gt;"")+($B$5:$B$504=B311)*(B311&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C311="Оплата",K311&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E311)&gt;0,ROUND(E311-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B311="",C311="",D311="",E311="",F311=""),"",IF(OR(B311="",C311="",E311=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E311)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H311&lt;&gt;0,F311=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G311&lt;&gt;0,F311=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F311&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F311)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C311)*($E$5:$E$504=E311)*(($D$5:$D$504=D311)*(D311&lt;&gt;"")+($B$5:$B$504=B311)*(B311&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C311="Оплата",K311&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E311)&gt;0,ROUND(E311-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J311" s="5">
@@ -9004,7 +9004,7 @@
         <v/>
       </c>
       <c r="I312" s="6">
-        <f>IF(AND(B312="",C312="",D312="",E312="",F312=""),"",IF(OR(B312="",C312="",E312=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E312)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H312&lt;&gt;0,F312=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G312&lt;&gt;0,F312=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F312&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F312)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C312)*($E$5:$E$504=E312)*(($D$5:$D$504=D312)*(D312&lt;&gt;"")+($B$5:$B$504=B312)*(B312&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C312="Оплата",K312&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E312)&gt;0,ROUND(E312-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B312="",C312="",D312="",E312="",F312=""),"",IF(OR(B312="",C312="",E312=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E312)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H312&lt;&gt;0,F312=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G312&lt;&gt;0,F312=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F312&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F312)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C312)*($E$5:$E$504=E312)*(($D$5:$D$504=D312)*(D312&lt;&gt;"")+($B$5:$B$504=B312)*(B312&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C312="Оплата",K312&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E312)&gt;0,ROUND(E312-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J312" s="5">
@@ -9031,7 +9031,7 @@
         <v/>
       </c>
       <c r="I313" s="6">
-        <f>IF(AND(B313="",C313="",D313="",E313="",F313=""),"",IF(OR(B313="",C313="",E313=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E313)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H313&lt;&gt;0,F313=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G313&lt;&gt;0,F313=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F313&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F313)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C313)*($E$5:$E$504=E313)*(($D$5:$D$504=D313)*(D313&lt;&gt;"")+($B$5:$B$504=B313)*(B313&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C313="Оплата",K313&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E313)&gt;0,ROUND(E313-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B313="",C313="",D313="",E313="",F313=""),"",IF(OR(B313="",C313="",E313=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E313)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H313&lt;&gt;0,F313=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G313&lt;&gt;0,F313=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F313&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F313)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C313)*($E$5:$E$504=E313)*(($D$5:$D$504=D313)*(D313&lt;&gt;"")+($B$5:$B$504=B313)*(B313&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C313="Оплата",K313&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E313)&gt;0,ROUND(E313-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J313" s="5">
@@ -9058,7 +9058,7 @@
         <v/>
       </c>
       <c r="I314" s="6">
-        <f>IF(AND(B314="",C314="",D314="",E314="",F314=""),"",IF(OR(B314="",C314="",E314=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E314)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H314&lt;&gt;0,F314=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G314&lt;&gt;0,F314=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F314&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F314)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C314)*($E$5:$E$504=E314)*(($D$5:$D$504=D314)*(D314&lt;&gt;"")+($B$5:$B$504=B314)*(B314&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C314="Оплата",K314&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E314)&gt;0,ROUND(E314-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B314="",C314="",D314="",E314="",F314=""),"",IF(OR(B314="",C314="",E314=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E314)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H314&lt;&gt;0,F314=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G314&lt;&gt;0,F314=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F314&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F314)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C314)*($E$5:$E$504=E314)*(($D$5:$D$504=D314)*(D314&lt;&gt;"")+($B$5:$B$504=B314)*(B314&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C314="Оплата",K314&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E314)&gt;0,ROUND(E314-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J314" s="5">
@@ -9085,7 +9085,7 @@
         <v/>
       </c>
       <c r="I315" s="6">
-        <f>IF(AND(B315="",C315="",D315="",E315="",F315=""),"",IF(OR(B315="",C315="",E315=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E315)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H315&lt;&gt;0,F315=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G315&lt;&gt;0,F315=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F315&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F315)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C315)*($E$5:$E$504=E315)*(($D$5:$D$504=D315)*(D315&lt;&gt;"")+($B$5:$B$504=B315)*(B315&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C315="Оплата",K315&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E315)&gt;0,ROUND(E315-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B315="",C315="",D315="",E315="",F315=""),"",IF(OR(B315="",C315="",E315=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E315)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H315&lt;&gt;0,F315=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G315&lt;&gt;0,F315=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F315&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F315)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C315)*($E$5:$E$504=E315)*(($D$5:$D$504=D315)*(D315&lt;&gt;"")+($B$5:$B$504=B315)*(B315&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C315="Оплата",K315&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E315)&gt;0,ROUND(E315-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J315" s="5">
@@ -9112,7 +9112,7 @@
         <v/>
       </c>
       <c r="I316" s="6">
-        <f>IF(AND(B316="",C316="",D316="",E316="",F316=""),"",IF(OR(B316="",C316="",E316=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E316)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H316&lt;&gt;0,F316=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G316&lt;&gt;0,F316=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F316&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F316)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C316)*($E$5:$E$504=E316)*(($D$5:$D$504=D316)*(D316&lt;&gt;"")+($B$5:$B$504=B316)*(B316&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C316="Оплата",K316&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E316)&gt;0,ROUND(E316-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B316="",C316="",D316="",E316="",F316=""),"",IF(OR(B316="",C316="",E316=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E316)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H316&lt;&gt;0,F316=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G316&lt;&gt;0,F316=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F316&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F316)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C316)*($E$5:$E$504=E316)*(($D$5:$D$504=D316)*(D316&lt;&gt;"")+($B$5:$B$504=B316)*(B316&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C316="Оплата",K316&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E316)&gt;0,ROUND(E316-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J316" s="5">
@@ -9139,7 +9139,7 @@
         <v/>
       </c>
       <c r="I317" s="6">
-        <f>IF(AND(B317="",C317="",D317="",E317="",F317=""),"",IF(OR(B317="",C317="",E317=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E317)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H317&lt;&gt;0,F317=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G317&lt;&gt;0,F317=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F317&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F317)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C317)*($E$5:$E$504=E317)*(($D$5:$D$504=D317)*(D317&lt;&gt;"")+($B$5:$B$504=B317)*(B317&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C317="Оплата",K317&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E317)&gt;0,ROUND(E317-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B317="",C317="",D317="",E317="",F317=""),"",IF(OR(B317="",C317="",E317=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E317)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H317&lt;&gt;0,F317=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G317&lt;&gt;0,F317=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F317&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F317)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C317)*($E$5:$E$504=E317)*(($D$5:$D$504=D317)*(D317&lt;&gt;"")+($B$5:$B$504=B317)*(B317&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C317="Оплата",K317&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E317)&gt;0,ROUND(E317-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J317" s="5">
@@ -9166,7 +9166,7 @@
         <v/>
       </c>
       <c r="I318" s="6">
-        <f>IF(AND(B318="",C318="",D318="",E318="",F318=""),"",IF(OR(B318="",C318="",E318=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E318)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H318&lt;&gt;0,F318=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G318&lt;&gt;0,F318=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F318&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F318)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C318)*($E$5:$E$504=E318)*(($D$5:$D$504=D318)*(D318&lt;&gt;"")+($B$5:$B$504=B318)*(B318&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C318="Оплата",K318&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E318)&gt;0,ROUND(E318-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B318="",C318="",D318="",E318="",F318=""),"",IF(OR(B318="",C318="",E318=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E318)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H318&lt;&gt;0,F318=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G318&lt;&gt;0,F318=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F318&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F318)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C318)*($E$5:$E$504=E318)*(($D$5:$D$504=D318)*(D318&lt;&gt;"")+($B$5:$B$504=B318)*(B318&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C318="Оплата",K318&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E318)&gt;0,ROUND(E318-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J318" s="5">
@@ -9193,7 +9193,7 @@
         <v/>
       </c>
       <c r="I319" s="6">
-        <f>IF(AND(B319="",C319="",D319="",E319="",F319=""),"",IF(OR(B319="",C319="",E319=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E319)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H319&lt;&gt;0,F319=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G319&lt;&gt;0,F319=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F319&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F319)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C319)*($E$5:$E$504=E319)*(($D$5:$D$504=D319)*(D319&lt;&gt;"")+($B$5:$B$504=B319)*(B319&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C319="Оплата",K319&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E319)&gt;0,ROUND(E319-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B319="",C319="",D319="",E319="",F319=""),"",IF(OR(B319="",C319="",E319=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E319)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H319&lt;&gt;0,F319=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G319&lt;&gt;0,F319=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F319&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F319)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C319)*($E$5:$E$504=E319)*(($D$5:$D$504=D319)*(D319&lt;&gt;"")+($B$5:$B$504=B319)*(B319&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C319="Оплата",K319&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E319)&gt;0,ROUND(E319-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J319" s="5">
@@ -9220,7 +9220,7 @@
         <v/>
       </c>
       <c r="I320" s="6">
-        <f>IF(AND(B320="",C320="",D320="",E320="",F320=""),"",IF(OR(B320="",C320="",E320=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E320)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H320&lt;&gt;0,F320=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G320&lt;&gt;0,F320=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F320&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F320)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C320)*($E$5:$E$504=E320)*(($D$5:$D$504=D320)*(D320&lt;&gt;"")+($B$5:$B$504=B320)*(B320&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C320="Оплата",K320&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E320)&gt;0,ROUND(E320-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B320="",C320="",D320="",E320="",F320=""),"",IF(OR(B320="",C320="",E320=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E320)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H320&lt;&gt;0,F320=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G320&lt;&gt;0,F320=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F320&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F320)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C320)*($E$5:$E$504=E320)*(($D$5:$D$504=D320)*(D320&lt;&gt;"")+($B$5:$B$504=B320)*(B320&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C320="Оплата",K320&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E320)&gt;0,ROUND(E320-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J320" s="5">
@@ -9247,7 +9247,7 @@
         <v/>
       </c>
       <c r="I321" s="6">
-        <f>IF(AND(B321="",C321="",D321="",E321="",F321=""),"",IF(OR(B321="",C321="",E321=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E321)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H321&lt;&gt;0,F321=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G321&lt;&gt;0,F321=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F321&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F321)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C321)*($E$5:$E$504=E321)*(($D$5:$D$504=D321)*(D321&lt;&gt;"")+($B$5:$B$504=B321)*(B321&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C321="Оплата",K321&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E321)&gt;0,ROUND(E321-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B321="",C321="",D321="",E321="",F321=""),"",IF(OR(B321="",C321="",E321=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E321)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H321&lt;&gt;0,F321=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G321&lt;&gt;0,F321=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F321&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F321)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C321)*($E$5:$E$504=E321)*(($D$5:$D$504=D321)*(D321&lt;&gt;"")+($B$5:$B$504=B321)*(B321&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C321="Оплата",K321&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E321)&gt;0,ROUND(E321-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J321" s="5">
@@ -9274,7 +9274,7 @@
         <v/>
       </c>
       <c r="I322" s="6">
-        <f>IF(AND(B322="",C322="",D322="",E322="",F322=""),"",IF(OR(B322="",C322="",E322=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E322)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H322&lt;&gt;0,F322=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G322&lt;&gt;0,F322=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F322&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F322)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C322)*($E$5:$E$504=E322)*(($D$5:$D$504=D322)*(D322&lt;&gt;"")+($B$5:$B$504=B322)*(B322&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C322="Оплата",K322&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E322)&gt;0,ROUND(E322-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B322="",C322="",D322="",E322="",F322=""),"",IF(OR(B322="",C322="",E322=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E322)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H322&lt;&gt;0,F322=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G322&lt;&gt;0,F322=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F322&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F322)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C322)*($E$5:$E$504=E322)*(($D$5:$D$504=D322)*(D322&lt;&gt;"")+($B$5:$B$504=B322)*(B322&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C322="Оплата",K322&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E322)&gt;0,ROUND(E322-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J322" s="5">
@@ -9301,7 +9301,7 @@
         <v/>
       </c>
       <c r="I323" s="6">
-        <f>IF(AND(B323="",C323="",D323="",E323="",F323=""),"",IF(OR(B323="",C323="",E323=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E323)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H323&lt;&gt;0,F323=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G323&lt;&gt;0,F323=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F323&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F323)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C323)*($E$5:$E$504=E323)*(($D$5:$D$504=D323)*(D323&lt;&gt;"")+($B$5:$B$504=B323)*(B323&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C323="Оплата",K323&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E323)&gt;0,ROUND(E323-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B323="",C323="",D323="",E323="",F323=""),"",IF(OR(B323="",C323="",E323=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E323)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H323&lt;&gt;0,F323=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G323&lt;&gt;0,F323=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F323&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F323)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C323)*($E$5:$E$504=E323)*(($D$5:$D$504=D323)*(D323&lt;&gt;"")+($B$5:$B$504=B323)*(B323&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C323="Оплата",K323&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E323)&gt;0,ROUND(E323-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J323" s="5">
@@ -9328,7 +9328,7 @@
         <v/>
       </c>
       <c r="I324" s="6">
-        <f>IF(AND(B324="",C324="",D324="",E324="",F324=""),"",IF(OR(B324="",C324="",E324=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E324)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H324&lt;&gt;0,F324=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G324&lt;&gt;0,F324=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F324&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F324)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C324)*($E$5:$E$504=E324)*(($D$5:$D$504=D324)*(D324&lt;&gt;"")+($B$5:$B$504=B324)*(B324&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C324="Оплата",K324&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E324)&gt;0,ROUND(E324-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B324="",C324="",D324="",E324="",F324=""),"",IF(OR(B324="",C324="",E324=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E324)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H324&lt;&gt;0,F324=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G324&lt;&gt;0,F324=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F324&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F324)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C324)*($E$5:$E$504=E324)*(($D$5:$D$504=D324)*(D324&lt;&gt;"")+($B$5:$B$504=B324)*(B324&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C324="Оплата",K324&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E324)&gt;0,ROUND(E324-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J324" s="5">
@@ -9355,7 +9355,7 @@
         <v/>
       </c>
       <c r="I325" s="6">
-        <f>IF(AND(B325="",C325="",D325="",E325="",F325=""),"",IF(OR(B325="",C325="",E325=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E325)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H325&lt;&gt;0,F325=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G325&lt;&gt;0,F325=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F325&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F325)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C325)*($E$5:$E$504=E325)*(($D$5:$D$504=D325)*(D325&lt;&gt;"")+($B$5:$B$504=B325)*(B325&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C325="Оплата",K325&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E325)&gt;0,ROUND(E325-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B325="",C325="",D325="",E325="",F325=""),"",IF(OR(B325="",C325="",E325=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E325)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H325&lt;&gt;0,F325=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G325&lt;&gt;0,F325=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F325&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F325)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C325)*($E$5:$E$504=E325)*(($D$5:$D$504=D325)*(D325&lt;&gt;"")+($B$5:$B$504=B325)*(B325&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C325="Оплата",K325&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E325)&gt;0,ROUND(E325-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J325" s="5">
@@ -9382,7 +9382,7 @@
         <v/>
       </c>
       <c r="I326" s="6">
-        <f>IF(AND(B326="",C326="",D326="",E326="",F326=""),"",IF(OR(B326="",C326="",E326=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E326)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H326&lt;&gt;0,F326=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G326&lt;&gt;0,F326=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F326&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F326)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C326)*($E$5:$E$504=E326)*(($D$5:$D$504=D326)*(D326&lt;&gt;"")+($B$5:$B$504=B326)*(B326&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C326="Оплата",K326&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E326)&gt;0,ROUND(E326-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B326="",C326="",D326="",E326="",F326=""),"",IF(OR(B326="",C326="",E326=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E326)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H326&lt;&gt;0,F326=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G326&lt;&gt;0,F326=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F326&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F326)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C326)*($E$5:$E$504=E326)*(($D$5:$D$504=D326)*(D326&lt;&gt;"")+($B$5:$B$504=B326)*(B326&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C326="Оплата",K326&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E326)&gt;0,ROUND(E326-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J326" s="5">
@@ -9409,7 +9409,7 @@
         <v/>
       </c>
       <c r="I327" s="6">
-        <f>IF(AND(B327="",C327="",D327="",E327="",F327=""),"",IF(OR(B327="",C327="",E327=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E327)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H327&lt;&gt;0,F327=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G327&lt;&gt;0,F327=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F327&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F327)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C327)*($E$5:$E$504=E327)*(($D$5:$D$504=D327)*(D327&lt;&gt;"")+($B$5:$B$504=B327)*(B327&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C327="Оплата",K327&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E327)&gt;0,ROUND(E327-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B327="",C327="",D327="",E327="",F327=""),"",IF(OR(B327="",C327="",E327=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E327)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H327&lt;&gt;0,F327=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G327&lt;&gt;0,F327=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F327&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F327)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C327)*($E$5:$E$504=E327)*(($D$5:$D$504=D327)*(D327&lt;&gt;"")+($B$5:$B$504=B327)*(B327&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C327="Оплата",K327&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E327)&gt;0,ROUND(E327-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J327" s="5">
@@ -9436,7 +9436,7 @@
         <v/>
       </c>
       <c r="I328" s="6">
-        <f>IF(AND(B328="",C328="",D328="",E328="",F328=""),"",IF(OR(B328="",C328="",E328=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E328)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H328&lt;&gt;0,F328=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G328&lt;&gt;0,F328=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F328&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F328)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C328)*($E$5:$E$504=E328)*(($D$5:$D$504=D328)*(D328&lt;&gt;"")+($B$5:$B$504=B328)*(B328&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C328="Оплата",K328&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E328)&gt;0,ROUND(E328-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B328="",C328="",D328="",E328="",F328=""),"",IF(OR(B328="",C328="",E328=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E328)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H328&lt;&gt;0,F328=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G328&lt;&gt;0,F328=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F328&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F328)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C328)*($E$5:$E$504=E328)*(($D$5:$D$504=D328)*(D328&lt;&gt;"")+($B$5:$B$504=B328)*(B328&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C328="Оплата",K328&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E328)&gt;0,ROUND(E328-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J328" s="5">
@@ -9463,7 +9463,7 @@
         <v/>
       </c>
       <c r="I329" s="6">
-        <f>IF(AND(B329="",C329="",D329="",E329="",F329=""),"",IF(OR(B329="",C329="",E329=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E329)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H329&lt;&gt;0,F329=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G329&lt;&gt;0,F329=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F329&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F329)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C329)*($E$5:$E$504=E329)*(($D$5:$D$504=D329)*(D329&lt;&gt;"")+($B$5:$B$504=B329)*(B329&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C329="Оплата",K329&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E329)&gt;0,ROUND(E329-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B329="",C329="",D329="",E329="",F329=""),"",IF(OR(B329="",C329="",E329=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E329)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H329&lt;&gt;0,F329=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G329&lt;&gt;0,F329=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F329&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F329)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C329)*($E$5:$E$504=E329)*(($D$5:$D$504=D329)*(D329&lt;&gt;"")+($B$5:$B$504=B329)*(B329&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C329="Оплата",K329&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E329)&gt;0,ROUND(E329-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J329" s="5">
@@ -9490,7 +9490,7 @@
         <v/>
       </c>
       <c r="I330" s="6">
-        <f>IF(AND(B330="",C330="",D330="",E330="",F330=""),"",IF(OR(B330="",C330="",E330=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E330)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H330&lt;&gt;0,F330=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G330&lt;&gt;0,F330=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F330&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F330)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C330)*($E$5:$E$504=E330)*(($D$5:$D$504=D330)*(D330&lt;&gt;"")+($B$5:$B$504=B330)*(B330&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C330="Оплата",K330&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E330)&gt;0,ROUND(E330-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B330="",C330="",D330="",E330="",F330=""),"",IF(OR(B330="",C330="",E330=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E330)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H330&lt;&gt;0,F330=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G330&lt;&gt;0,F330=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F330&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F330)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C330)*($E$5:$E$504=E330)*(($D$5:$D$504=D330)*(D330&lt;&gt;"")+($B$5:$B$504=B330)*(B330&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C330="Оплата",K330&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E330)&gt;0,ROUND(E330-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J330" s="5">
@@ -9517,7 +9517,7 @@
         <v/>
       </c>
       <c r="I331" s="6">
-        <f>IF(AND(B331="",C331="",D331="",E331="",F331=""),"",IF(OR(B331="",C331="",E331=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E331)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H331&lt;&gt;0,F331=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G331&lt;&gt;0,F331=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F331&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F331)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C331)*($E$5:$E$504=E331)*(($D$5:$D$504=D331)*(D331&lt;&gt;"")+($B$5:$B$504=B331)*(B331&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C331="Оплата",K331&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E331)&gt;0,ROUND(E331-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B331="",C331="",D331="",E331="",F331=""),"",IF(OR(B331="",C331="",E331=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E331)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H331&lt;&gt;0,F331=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G331&lt;&gt;0,F331=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F331&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F331)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C331)*($E$5:$E$504=E331)*(($D$5:$D$504=D331)*(D331&lt;&gt;"")+($B$5:$B$504=B331)*(B331&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C331="Оплата",K331&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E331)&gt;0,ROUND(E331-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J331" s="5">
@@ -9544,7 +9544,7 @@
         <v/>
       </c>
       <c r="I332" s="6">
-        <f>IF(AND(B332="",C332="",D332="",E332="",F332=""),"",IF(OR(B332="",C332="",E332=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E332)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H332&lt;&gt;0,F332=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G332&lt;&gt;0,F332=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F332&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F332)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C332)*($E$5:$E$504=E332)*(($D$5:$D$504=D332)*(D332&lt;&gt;"")+($B$5:$B$504=B332)*(B332&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C332="Оплата",K332&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E332)&gt;0,ROUND(E332-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B332="",C332="",D332="",E332="",F332=""),"",IF(OR(B332="",C332="",E332=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E332)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H332&lt;&gt;0,F332=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G332&lt;&gt;0,F332=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F332&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F332)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C332)*($E$5:$E$504=E332)*(($D$5:$D$504=D332)*(D332&lt;&gt;"")+($B$5:$B$504=B332)*(B332&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C332="Оплата",K332&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E332)&gt;0,ROUND(E332-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J332" s="5">
@@ -9571,7 +9571,7 @@
         <v/>
       </c>
       <c r="I333" s="6">
-        <f>IF(AND(B333="",C333="",D333="",E333="",F333=""),"",IF(OR(B333="",C333="",E333=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E333)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H333&lt;&gt;0,F333=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G333&lt;&gt;0,F333=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F333&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F333)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C333)*($E$5:$E$504=E333)*(($D$5:$D$504=D333)*(D333&lt;&gt;"")+($B$5:$B$504=B333)*(B333&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C333="Оплата",K333&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E333)&gt;0,ROUND(E333-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B333="",C333="",D333="",E333="",F333=""),"",IF(OR(B333="",C333="",E333=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E333)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H333&lt;&gt;0,F333=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G333&lt;&gt;0,F333=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F333&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F333)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C333)*($E$5:$E$504=E333)*(($D$5:$D$504=D333)*(D333&lt;&gt;"")+($B$5:$B$504=B333)*(B333&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C333="Оплата",K333&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E333)&gt;0,ROUND(E333-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J333" s="5">
@@ -9598,7 +9598,7 @@
         <v/>
       </c>
       <c r="I334" s="6">
-        <f>IF(AND(B334="",C334="",D334="",E334="",F334=""),"",IF(OR(B334="",C334="",E334=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E334)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H334&lt;&gt;0,F334=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G334&lt;&gt;0,F334=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F334&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F334)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C334)*($E$5:$E$504=E334)*(($D$5:$D$504=D334)*(D334&lt;&gt;"")+($B$5:$B$504=B334)*(B334&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C334="Оплата",K334&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E334)&gt;0,ROUND(E334-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B334="",C334="",D334="",E334="",F334=""),"",IF(OR(B334="",C334="",E334=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E334)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H334&lt;&gt;0,F334=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G334&lt;&gt;0,F334=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F334&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F334)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C334)*($E$5:$E$504=E334)*(($D$5:$D$504=D334)*(D334&lt;&gt;"")+($B$5:$B$504=B334)*(B334&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C334="Оплата",K334&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E334)&gt;0,ROUND(E334-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J334" s="5">
@@ -9625,7 +9625,7 @@
         <v/>
       </c>
       <c r="I335" s="6">
-        <f>IF(AND(B335="",C335="",D335="",E335="",F335=""),"",IF(OR(B335="",C335="",E335=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E335)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H335&lt;&gt;0,F335=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G335&lt;&gt;0,F335=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F335&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F335)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C335)*($E$5:$E$504=E335)*(($D$5:$D$504=D335)*(D335&lt;&gt;"")+($B$5:$B$504=B335)*(B335&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C335="Оплата",K335&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E335)&gt;0,ROUND(E335-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B335="",C335="",D335="",E335="",F335=""),"",IF(OR(B335="",C335="",E335=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E335)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H335&lt;&gt;0,F335=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G335&lt;&gt;0,F335=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F335&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F335)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C335)*($E$5:$E$504=E335)*(($D$5:$D$504=D335)*(D335&lt;&gt;"")+($B$5:$B$504=B335)*(B335&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C335="Оплата",K335&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E335)&gt;0,ROUND(E335-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J335" s="5">
@@ -9652,7 +9652,7 @@
         <v/>
       </c>
       <c r="I336" s="6">
-        <f>IF(AND(B336="",C336="",D336="",E336="",F336=""),"",IF(OR(B336="",C336="",E336=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E336)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H336&lt;&gt;0,F336=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G336&lt;&gt;0,F336=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F336&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F336)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C336)*($E$5:$E$504=E336)*(($D$5:$D$504=D336)*(D336&lt;&gt;"")+($B$5:$B$504=B336)*(B336&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C336="Оплата",K336&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E336)&gt;0,ROUND(E336-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B336="",C336="",D336="",E336="",F336=""),"",IF(OR(B336="",C336="",E336=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E336)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H336&lt;&gt;0,F336=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G336&lt;&gt;0,F336=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F336&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F336)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C336)*($E$5:$E$504=E336)*(($D$5:$D$504=D336)*(D336&lt;&gt;"")+($B$5:$B$504=B336)*(B336&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C336="Оплата",K336&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E336)&gt;0,ROUND(E336-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J336" s="5">
@@ -9679,7 +9679,7 @@
         <v/>
       </c>
       <c r="I337" s="6">
-        <f>IF(AND(B337="",C337="",D337="",E337="",F337=""),"",IF(OR(B337="",C337="",E337=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E337)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H337&lt;&gt;0,F337=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G337&lt;&gt;0,F337=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F337&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F337)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C337)*($E$5:$E$504=E337)*(($D$5:$D$504=D337)*(D337&lt;&gt;"")+($B$5:$B$504=B337)*(B337&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C337="Оплата",K337&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E337)&gt;0,ROUND(E337-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B337="",C337="",D337="",E337="",F337=""),"",IF(OR(B337="",C337="",E337=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E337)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H337&lt;&gt;0,F337=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G337&lt;&gt;0,F337=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F337&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F337)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C337)*($E$5:$E$504=E337)*(($D$5:$D$504=D337)*(D337&lt;&gt;"")+($B$5:$B$504=B337)*(B337&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C337="Оплата",K337&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E337)&gt;0,ROUND(E337-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J337" s="5">
@@ -9706,7 +9706,7 @@
         <v/>
       </c>
       <c r="I338" s="6">
-        <f>IF(AND(B338="",C338="",D338="",E338="",F338=""),"",IF(OR(B338="",C338="",E338=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E338)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H338&lt;&gt;0,F338=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G338&lt;&gt;0,F338=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F338&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F338)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C338)*($E$5:$E$504=E338)*(($D$5:$D$504=D338)*(D338&lt;&gt;"")+($B$5:$B$504=B338)*(B338&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C338="Оплата",K338&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E338)&gt;0,ROUND(E338-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B338="",C338="",D338="",E338="",F338=""),"",IF(OR(B338="",C338="",E338=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E338)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H338&lt;&gt;0,F338=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G338&lt;&gt;0,F338=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F338&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F338)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C338)*($E$5:$E$504=E338)*(($D$5:$D$504=D338)*(D338&lt;&gt;"")+($B$5:$B$504=B338)*(B338&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C338="Оплата",K338&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E338)&gt;0,ROUND(E338-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J338" s="5">
@@ -9733,7 +9733,7 @@
         <v/>
       </c>
       <c r="I339" s="6">
-        <f>IF(AND(B339="",C339="",D339="",E339="",F339=""),"",IF(OR(B339="",C339="",E339=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E339)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H339&lt;&gt;0,F339=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G339&lt;&gt;0,F339=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F339&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F339)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C339)*($E$5:$E$504=E339)*(($D$5:$D$504=D339)*(D339&lt;&gt;"")+($B$5:$B$504=B339)*(B339&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C339="Оплата",K339&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E339)&gt;0,ROUND(E339-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B339="",C339="",D339="",E339="",F339=""),"",IF(OR(B339="",C339="",E339=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E339)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H339&lt;&gt;0,F339=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G339&lt;&gt;0,F339=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F339&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F339)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C339)*($E$5:$E$504=E339)*(($D$5:$D$504=D339)*(D339&lt;&gt;"")+($B$5:$B$504=B339)*(B339&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C339="Оплата",K339&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E339)&gt;0,ROUND(E339-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J339" s="5">
@@ -9760,7 +9760,7 @@
         <v/>
       </c>
       <c r="I340" s="6">
-        <f>IF(AND(B340="",C340="",D340="",E340="",F340=""),"",IF(OR(B340="",C340="",E340=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E340)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H340&lt;&gt;0,F340=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G340&lt;&gt;0,F340=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F340&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F340)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C340)*($E$5:$E$504=E340)*(($D$5:$D$504=D340)*(D340&lt;&gt;"")+($B$5:$B$504=B340)*(B340&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C340="Оплата",K340&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E340)&gt;0,ROUND(E340-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B340="",C340="",D340="",E340="",F340=""),"",IF(OR(B340="",C340="",E340=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E340)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H340&lt;&gt;0,F340=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G340&lt;&gt;0,F340=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F340&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F340)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C340)*($E$5:$E$504=E340)*(($D$5:$D$504=D340)*(D340&lt;&gt;"")+($B$5:$B$504=B340)*(B340&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C340="Оплата",K340&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E340)&gt;0,ROUND(E340-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J340" s="5">
@@ -9787,7 +9787,7 @@
         <v/>
       </c>
       <c r="I341" s="6">
-        <f>IF(AND(B341="",C341="",D341="",E341="",F341=""),"",IF(OR(B341="",C341="",E341=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E341)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H341&lt;&gt;0,F341=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G341&lt;&gt;0,F341=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F341&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F341)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C341)*($E$5:$E$504=E341)*(($D$5:$D$504=D341)*(D341&lt;&gt;"")+($B$5:$B$504=B341)*(B341&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C341="Оплата",K341&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E341)&gt;0,ROUND(E341-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B341="",C341="",D341="",E341="",F341=""),"",IF(OR(B341="",C341="",E341=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E341)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H341&lt;&gt;0,F341=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G341&lt;&gt;0,F341=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F341&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F341)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C341)*($E$5:$E$504=E341)*(($D$5:$D$504=D341)*(D341&lt;&gt;"")+($B$5:$B$504=B341)*(B341&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C341="Оплата",K341&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E341)&gt;0,ROUND(E341-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J341" s="5">
@@ -9814,7 +9814,7 @@
         <v/>
       </c>
       <c r="I342" s="6">
-        <f>IF(AND(B342="",C342="",D342="",E342="",F342=""),"",IF(OR(B342="",C342="",E342=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E342)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H342&lt;&gt;0,F342=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G342&lt;&gt;0,F342=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F342&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F342)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C342)*($E$5:$E$504=E342)*(($D$5:$D$504=D342)*(D342&lt;&gt;"")+($B$5:$B$504=B342)*(B342&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C342="Оплата",K342&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E342)&gt;0,ROUND(E342-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B342="",C342="",D342="",E342="",F342=""),"",IF(OR(B342="",C342="",E342=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E342)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H342&lt;&gt;0,F342=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G342&lt;&gt;0,F342=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F342&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F342)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C342)*($E$5:$E$504=E342)*(($D$5:$D$504=D342)*(D342&lt;&gt;"")+($B$5:$B$504=B342)*(B342&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C342="Оплата",K342&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E342)&gt;0,ROUND(E342-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J342" s="5">
@@ -9841,7 +9841,7 @@
         <v/>
       </c>
       <c r="I343" s="6">
-        <f>IF(AND(B343="",C343="",D343="",E343="",F343=""),"",IF(OR(B343="",C343="",E343=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E343)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H343&lt;&gt;0,F343=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G343&lt;&gt;0,F343=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F343&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F343)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C343)*($E$5:$E$504=E343)*(($D$5:$D$504=D343)*(D343&lt;&gt;"")+($B$5:$B$504=B343)*(B343&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C343="Оплата",K343&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E343)&gt;0,ROUND(E343-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B343="",C343="",D343="",E343="",F343=""),"",IF(OR(B343="",C343="",E343=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E343)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H343&lt;&gt;0,F343=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G343&lt;&gt;0,F343=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F343&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F343)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C343)*($E$5:$E$504=E343)*(($D$5:$D$504=D343)*(D343&lt;&gt;"")+($B$5:$B$504=B343)*(B343&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C343="Оплата",K343&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E343)&gt;0,ROUND(E343-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J343" s="5">
@@ -9868,7 +9868,7 @@
         <v/>
       </c>
       <c r="I344" s="6">
-        <f>IF(AND(B344="",C344="",D344="",E344="",F344=""),"",IF(OR(B344="",C344="",E344=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E344)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H344&lt;&gt;0,F344=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G344&lt;&gt;0,F344=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F344&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F344)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C344)*($E$5:$E$504=E344)*(($D$5:$D$504=D344)*(D344&lt;&gt;"")+($B$5:$B$504=B344)*(B344&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C344="Оплата",K344&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E344)&gt;0,ROUND(E344-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B344="",C344="",D344="",E344="",F344=""),"",IF(OR(B344="",C344="",E344=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E344)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H344&lt;&gt;0,F344=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G344&lt;&gt;0,F344=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F344&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F344)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C344)*($E$5:$E$504=E344)*(($D$5:$D$504=D344)*(D344&lt;&gt;"")+($B$5:$B$504=B344)*(B344&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C344="Оплата",K344&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E344)&gt;0,ROUND(E344-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J344" s="5">
@@ -9895,7 +9895,7 @@
         <v/>
       </c>
       <c r="I345" s="6">
-        <f>IF(AND(B345="",C345="",D345="",E345="",F345=""),"",IF(OR(B345="",C345="",E345=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E345)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H345&lt;&gt;0,F345=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G345&lt;&gt;0,F345=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F345&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F345)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C345)*($E$5:$E$504=E345)*(($D$5:$D$504=D345)*(D345&lt;&gt;"")+($B$5:$B$504=B345)*(B345&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C345="Оплата",K345&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E345)&gt;0,ROUND(E345-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B345="",C345="",D345="",E345="",F345=""),"",IF(OR(B345="",C345="",E345=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E345)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H345&lt;&gt;0,F345=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G345&lt;&gt;0,F345=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F345&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F345)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C345)*($E$5:$E$504=E345)*(($D$5:$D$504=D345)*(D345&lt;&gt;"")+($B$5:$B$504=B345)*(B345&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C345="Оплата",K345&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E345)&gt;0,ROUND(E345-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J345" s="5">
@@ -9922,7 +9922,7 @@
         <v/>
       </c>
       <c r="I346" s="6">
-        <f>IF(AND(B346="",C346="",D346="",E346="",F346=""),"",IF(OR(B346="",C346="",E346=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E346)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H346&lt;&gt;0,F346=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G346&lt;&gt;0,F346=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F346&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F346)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C346)*($E$5:$E$504=E346)*(($D$5:$D$504=D346)*(D346&lt;&gt;"")+($B$5:$B$504=B346)*(B346&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C346="Оплата",K346&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E346)&gt;0,ROUND(E346-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B346="",C346="",D346="",E346="",F346=""),"",IF(OR(B346="",C346="",E346=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E346)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H346&lt;&gt;0,F346=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G346&lt;&gt;0,F346=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F346&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F346)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C346)*($E$5:$E$504=E346)*(($D$5:$D$504=D346)*(D346&lt;&gt;"")+($B$5:$B$504=B346)*(B346&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C346="Оплата",K346&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E346)&gt;0,ROUND(E346-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J346" s="5">
@@ -9949,7 +9949,7 @@
         <v/>
       </c>
       <c r="I347" s="6">
-        <f>IF(AND(B347="",C347="",D347="",E347="",F347=""),"",IF(OR(B347="",C347="",E347=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E347)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H347&lt;&gt;0,F347=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G347&lt;&gt;0,F347=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F347&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F347)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C347)*($E$5:$E$504=E347)*(($D$5:$D$504=D347)*(D347&lt;&gt;"")+($B$5:$B$504=B347)*(B347&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C347="Оплата",K347&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E347)&gt;0,ROUND(E347-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B347="",C347="",D347="",E347="",F347=""),"",IF(OR(B347="",C347="",E347=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E347)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H347&lt;&gt;0,F347=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G347&lt;&gt;0,F347=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F347&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F347)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C347)*($E$5:$E$504=E347)*(($D$5:$D$504=D347)*(D347&lt;&gt;"")+($B$5:$B$504=B347)*(B347&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C347="Оплата",K347&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E347)&gt;0,ROUND(E347-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J347" s="5">
@@ -9976,7 +9976,7 @@
         <v/>
       </c>
       <c r="I348" s="6">
-        <f>IF(AND(B348="",C348="",D348="",E348="",F348=""),"",IF(OR(B348="",C348="",E348=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E348)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H348&lt;&gt;0,F348=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G348&lt;&gt;0,F348=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F348&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F348)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C348)*($E$5:$E$504=E348)*(($D$5:$D$504=D348)*(D348&lt;&gt;"")+($B$5:$B$504=B348)*(B348&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C348="Оплата",K348&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E348)&gt;0,ROUND(E348-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B348="",C348="",D348="",E348="",F348=""),"",IF(OR(B348="",C348="",E348=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E348)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H348&lt;&gt;0,F348=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G348&lt;&gt;0,F348=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F348&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F348)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C348)*($E$5:$E$504=E348)*(($D$5:$D$504=D348)*(D348&lt;&gt;"")+($B$5:$B$504=B348)*(B348&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C348="Оплата",K348&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E348)&gt;0,ROUND(E348-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J348" s="5">
@@ -10003,7 +10003,7 @@
         <v/>
       </c>
       <c r="I349" s="6">
-        <f>IF(AND(B349="",C349="",D349="",E349="",F349=""),"",IF(OR(B349="",C349="",E349=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E349)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H349&lt;&gt;0,F349=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G349&lt;&gt;0,F349=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F349&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F349)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C349)*($E$5:$E$504=E349)*(($D$5:$D$504=D349)*(D349&lt;&gt;"")+($B$5:$B$504=B349)*(B349&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C349="Оплата",K349&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E349)&gt;0,ROUND(E349-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B349="",C349="",D349="",E349="",F349=""),"",IF(OR(B349="",C349="",E349=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E349)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H349&lt;&gt;0,F349=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G349&lt;&gt;0,F349=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F349&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F349)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C349)*($E$5:$E$504=E349)*(($D$5:$D$504=D349)*(D349&lt;&gt;"")+($B$5:$B$504=B349)*(B349&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C349="Оплата",K349&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E349)&gt;0,ROUND(E349-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J349" s="5">
@@ -10030,7 +10030,7 @@
         <v/>
       </c>
       <c r="I350" s="6">
-        <f>IF(AND(B350="",C350="",D350="",E350="",F350=""),"",IF(OR(B350="",C350="",E350=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E350)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H350&lt;&gt;0,F350=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G350&lt;&gt;0,F350=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F350&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F350)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C350)*($E$5:$E$504=E350)*(($D$5:$D$504=D350)*(D350&lt;&gt;"")+($B$5:$B$504=B350)*(B350&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C350="Оплата",K350&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E350)&gt;0,ROUND(E350-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B350="",C350="",D350="",E350="",F350=""),"",IF(OR(B350="",C350="",E350=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E350)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H350&lt;&gt;0,F350=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G350&lt;&gt;0,F350=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F350&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F350)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C350)*($E$5:$E$504=E350)*(($D$5:$D$504=D350)*(D350&lt;&gt;"")+($B$5:$B$504=B350)*(B350&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C350="Оплата",K350&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E350)&gt;0,ROUND(E350-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J350" s="5">
@@ -10057,7 +10057,7 @@
         <v/>
       </c>
       <c r="I351" s="6">
-        <f>IF(AND(B351="",C351="",D351="",E351="",F351=""),"",IF(OR(B351="",C351="",E351=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E351)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H351&lt;&gt;0,F351=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G351&lt;&gt;0,F351=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F351&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F351)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C351)*($E$5:$E$504=E351)*(($D$5:$D$504=D351)*(D351&lt;&gt;"")+($B$5:$B$504=B351)*(B351&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C351="Оплата",K351&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E351)&gt;0,ROUND(E351-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B351="",C351="",D351="",E351="",F351=""),"",IF(OR(B351="",C351="",E351=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E351)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H351&lt;&gt;0,F351=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G351&lt;&gt;0,F351=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F351&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F351)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C351)*($E$5:$E$504=E351)*(($D$5:$D$504=D351)*(D351&lt;&gt;"")+($B$5:$B$504=B351)*(B351&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C351="Оплата",K351&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E351)&gt;0,ROUND(E351-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J351" s="5">
@@ -10084,7 +10084,7 @@
         <v/>
       </c>
       <c r="I352" s="6">
-        <f>IF(AND(B352="",C352="",D352="",E352="",F352=""),"",IF(OR(B352="",C352="",E352=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E352)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H352&lt;&gt;0,F352=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G352&lt;&gt;0,F352=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F352&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F352)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C352)*($E$5:$E$504=E352)*(($D$5:$D$504=D352)*(D352&lt;&gt;"")+($B$5:$B$504=B352)*(B352&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C352="Оплата",K352&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E352)&gt;0,ROUND(E352-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B352="",C352="",D352="",E352="",F352=""),"",IF(OR(B352="",C352="",E352=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E352)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H352&lt;&gt;0,F352=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G352&lt;&gt;0,F352=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F352&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F352)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C352)*($E$5:$E$504=E352)*(($D$5:$D$504=D352)*(D352&lt;&gt;"")+($B$5:$B$504=B352)*(B352&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C352="Оплата",K352&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E352)&gt;0,ROUND(E352-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J352" s="5">
@@ -10111,7 +10111,7 @@
         <v/>
       </c>
       <c r="I353" s="6">
-        <f>IF(AND(B353="",C353="",D353="",E353="",F353=""),"",IF(OR(B353="",C353="",E353=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E353)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H353&lt;&gt;0,F353=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G353&lt;&gt;0,F353=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F353&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F353)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C353)*($E$5:$E$504=E353)*(($D$5:$D$504=D353)*(D353&lt;&gt;"")+($B$5:$B$504=B353)*(B353&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C353="Оплата",K353&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E353)&gt;0,ROUND(E353-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B353="",C353="",D353="",E353="",F353=""),"",IF(OR(B353="",C353="",E353=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E353)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H353&lt;&gt;0,F353=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G353&lt;&gt;0,F353=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F353&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F353)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C353)*($E$5:$E$504=E353)*(($D$5:$D$504=D353)*(D353&lt;&gt;"")+($B$5:$B$504=B353)*(B353&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C353="Оплата",K353&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E353)&gt;0,ROUND(E353-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J353" s="5">
@@ -10138,7 +10138,7 @@
         <v/>
       </c>
       <c r="I354" s="6">
-        <f>IF(AND(B354="",C354="",D354="",E354="",F354=""),"",IF(OR(B354="",C354="",E354=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E354)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H354&lt;&gt;0,F354=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G354&lt;&gt;0,F354=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F354&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F354)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C354)*($E$5:$E$504=E354)*(($D$5:$D$504=D354)*(D354&lt;&gt;"")+($B$5:$B$504=B354)*(B354&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C354="Оплата",K354&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E354)&gt;0,ROUND(E354-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B354="",C354="",D354="",E354="",F354=""),"",IF(OR(B354="",C354="",E354=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E354)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H354&lt;&gt;0,F354=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G354&lt;&gt;0,F354=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F354&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F354)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C354)*($E$5:$E$504=E354)*(($D$5:$D$504=D354)*(D354&lt;&gt;"")+($B$5:$B$504=B354)*(B354&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C354="Оплата",K354&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E354)&gt;0,ROUND(E354-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J354" s="5">
@@ -10165,7 +10165,7 @@
         <v/>
       </c>
       <c r="I355" s="6">
-        <f>IF(AND(B355="",C355="",D355="",E355="",F355=""),"",IF(OR(B355="",C355="",E355=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E355)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H355&lt;&gt;0,F355=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G355&lt;&gt;0,F355=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F355&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F355)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C355)*($E$5:$E$504=E355)*(($D$5:$D$504=D355)*(D355&lt;&gt;"")+($B$5:$B$504=B355)*(B355&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C355="Оплата",K355&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E355)&gt;0,ROUND(E355-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B355="",C355="",D355="",E355="",F355=""),"",IF(OR(B355="",C355="",E355=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E355)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H355&lt;&gt;0,F355=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G355&lt;&gt;0,F355=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F355&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F355)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C355)*($E$5:$E$504=E355)*(($D$5:$D$504=D355)*(D355&lt;&gt;"")+($B$5:$B$504=B355)*(B355&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C355="Оплата",K355&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E355)&gt;0,ROUND(E355-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J355" s="5">
@@ -10192,7 +10192,7 @@
         <v/>
       </c>
       <c r="I356" s="6">
-        <f>IF(AND(B356="",C356="",D356="",E356="",F356=""),"",IF(OR(B356="",C356="",E356=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E356)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H356&lt;&gt;0,F356=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G356&lt;&gt;0,F356=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F356&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F356)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C356)*($E$5:$E$504=E356)*(($D$5:$D$504=D356)*(D356&lt;&gt;"")+($B$5:$B$504=B356)*(B356&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C356="Оплата",K356&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E356)&gt;0,ROUND(E356-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B356="",C356="",D356="",E356="",F356=""),"",IF(OR(B356="",C356="",E356=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E356)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H356&lt;&gt;0,F356=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G356&lt;&gt;0,F356=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F356&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F356)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C356)*($E$5:$E$504=E356)*(($D$5:$D$504=D356)*(D356&lt;&gt;"")+($B$5:$B$504=B356)*(B356&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C356="Оплата",K356&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E356)&gt;0,ROUND(E356-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J356" s="5">
@@ -10219,7 +10219,7 @@
         <v/>
       </c>
       <c r="I357" s="6">
-        <f>IF(AND(B357="",C357="",D357="",E357="",F357=""),"",IF(OR(B357="",C357="",E357=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E357)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H357&lt;&gt;0,F357=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G357&lt;&gt;0,F357=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F357&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F357)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C357)*($E$5:$E$504=E357)*(($D$5:$D$504=D357)*(D357&lt;&gt;"")+($B$5:$B$504=B357)*(B357&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C357="Оплата",K357&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E357)&gt;0,ROUND(E357-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B357="",C357="",D357="",E357="",F357=""),"",IF(OR(B357="",C357="",E357=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E357)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H357&lt;&gt;0,F357=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G357&lt;&gt;0,F357=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F357&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F357)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C357)*($E$5:$E$504=E357)*(($D$5:$D$504=D357)*(D357&lt;&gt;"")+($B$5:$B$504=B357)*(B357&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C357="Оплата",K357&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E357)&gt;0,ROUND(E357-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J357" s="5">
@@ -10246,7 +10246,7 @@
         <v/>
       </c>
       <c r="I358" s="6">
-        <f>IF(AND(B358="",C358="",D358="",E358="",F358=""),"",IF(OR(B358="",C358="",E358=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E358)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H358&lt;&gt;0,F358=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G358&lt;&gt;0,F358=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F358&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F358)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C358)*($E$5:$E$504=E358)*(($D$5:$D$504=D358)*(D358&lt;&gt;"")+($B$5:$B$504=B358)*(B358&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C358="Оплата",K358&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E358)&gt;0,ROUND(E358-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B358="",C358="",D358="",E358="",F358=""),"",IF(OR(B358="",C358="",E358=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E358)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H358&lt;&gt;0,F358=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G358&lt;&gt;0,F358=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F358&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F358)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C358)*($E$5:$E$504=E358)*(($D$5:$D$504=D358)*(D358&lt;&gt;"")+($B$5:$B$504=B358)*(B358&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C358="Оплата",K358&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E358)&gt;0,ROUND(E358-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J358" s="5">
@@ -10273,7 +10273,7 @@
         <v/>
       </c>
       <c r="I359" s="6">
-        <f>IF(AND(B359="",C359="",D359="",E359="",F359=""),"",IF(OR(B359="",C359="",E359=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E359)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H359&lt;&gt;0,F359=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G359&lt;&gt;0,F359=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F359&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F359)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C359)*($E$5:$E$504=E359)*(($D$5:$D$504=D359)*(D359&lt;&gt;"")+($B$5:$B$504=B359)*(B359&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C359="Оплата",K359&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E359)&gt;0,ROUND(E359-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B359="",C359="",D359="",E359="",F359=""),"",IF(OR(B359="",C359="",E359=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E359)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H359&lt;&gt;0,F359=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G359&lt;&gt;0,F359=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F359&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F359)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C359)*($E$5:$E$504=E359)*(($D$5:$D$504=D359)*(D359&lt;&gt;"")+($B$5:$B$504=B359)*(B359&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C359="Оплата",K359&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E359)&gt;0,ROUND(E359-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J359" s="5">
@@ -10300,7 +10300,7 @@
         <v/>
       </c>
       <c r="I360" s="6">
-        <f>IF(AND(B360="",C360="",D360="",E360="",F360=""),"",IF(OR(B360="",C360="",E360=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E360)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H360&lt;&gt;0,F360=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G360&lt;&gt;0,F360=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F360&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F360)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C360)*($E$5:$E$504=E360)*(($D$5:$D$504=D360)*(D360&lt;&gt;"")+($B$5:$B$504=B360)*(B360&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C360="Оплата",K360&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E360)&gt;0,ROUND(E360-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B360="",C360="",D360="",E360="",F360=""),"",IF(OR(B360="",C360="",E360=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E360)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H360&lt;&gt;0,F360=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G360&lt;&gt;0,F360=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F360&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F360)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C360)*($E$5:$E$504=E360)*(($D$5:$D$504=D360)*(D360&lt;&gt;"")+($B$5:$B$504=B360)*(B360&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C360="Оплата",K360&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E360)&gt;0,ROUND(E360-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J360" s="5">
@@ -10327,7 +10327,7 @@
         <v/>
       </c>
       <c r="I361" s="6">
-        <f>IF(AND(B361="",C361="",D361="",E361="",F361=""),"",IF(OR(B361="",C361="",E361=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E361)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H361&lt;&gt;0,F361=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G361&lt;&gt;0,F361=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F361&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F361)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C361)*($E$5:$E$504=E361)*(($D$5:$D$504=D361)*(D361&lt;&gt;"")+($B$5:$B$504=B361)*(B361&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C361="Оплата",K361&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E361)&gt;0,ROUND(E361-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B361="",C361="",D361="",E361="",F361=""),"",IF(OR(B361="",C361="",E361=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E361)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H361&lt;&gt;0,F361=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G361&lt;&gt;0,F361=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F361&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F361)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C361)*($E$5:$E$504=E361)*(($D$5:$D$504=D361)*(D361&lt;&gt;"")+($B$5:$B$504=B361)*(B361&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C361="Оплата",K361&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E361)&gt;0,ROUND(E361-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J361" s="5">
@@ -10354,7 +10354,7 @@
         <v/>
       </c>
       <c r="I362" s="6">
-        <f>IF(AND(B362="",C362="",D362="",E362="",F362=""),"",IF(OR(B362="",C362="",E362=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E362)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H362&lt;&gt;0,F362=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G362&lt;&gt;0,F362=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F362&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F362)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C362)*($E$5:$E$504=E362)*(($D$5:$D$504=D362)*(D362&lt;&gt;"")+($B$5:$B$504=B362)*(B362&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C362="Оплата",K362&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E362)&gt;0,ROUND(E362-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B362="",C362="",D362="",E362="",F362=""),"",IF(OR(B362="",C362="",E362=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E362)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H362&lt;&gt;0,F362=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G362&lt;&gt;0,F362=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F362&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F362)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C362)*($E$5:$E$504=E362)*(($D$5:$D$504=D362)*(D362&lt;&gt;"")+($B$5:$B$504=B362)*(B362&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C362="Оплата",K362&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E362)&gt;0,ROUND(E362-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J362" s="5">
@@ -10381,7 +10381,7 @@
         <v/>
       </c>
       <c r="I363" s="6">
-        <f>IF(AND(B363="",C363="",D363="",E363="",F363=""),"",IF(OR(B363="",C363="",E363=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E363)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H363&lt;&gt;0,F363=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G363&lt;&gt;0,F363=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F363&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F363)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C363)*($E$5:$E$504=E363)*(($D$5:$D$504=D363)*(D363&lt;&gt;"")+($B$5:$B$504=B363)*(B363&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C363="Оплата",K363&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E363)&gt;0,ROUND(E363-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B363="",C363="",D363="",E363="",F363=""),"",IF(OR(B363="",C363="",E363=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E363)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H363&lt;&gt;0,F363=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G363&lt;&gt;0,F363=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F363&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F363)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C363)*($E$5:$E$504=E363)*(($D$5:$D$504=D363)*(D363&lt;&gt;"")+($B$5:$B$504=B363)*(B363&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C363="Оплата",K363&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E363)&gt;0,ROUND(E363-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J363" s="5">
@@ -10408,7 +10408,7 @@
         <v/>
       </c>
       <c r="I364" s="6">
-        <f>IF(AND(B364="",C364="",D364="",E364="",F364=""),"",IF(OR(B364="",C364="",E364=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E364)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H364&lt;&gt;0,F364=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G364&lt;&gt;0,F364=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F364&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F364)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C364)*($E$5:$E$504=E364)*(($D$5:$D$504=D364)*(D364&lt;&gt;"")+($B$5:$B$504=B364)*(B364&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C364="Оплата",K364&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E364)&gt;0,ROUND(E364-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B364="",C364="",D364="",E364="",F364=""),"",IF(OR(B364="",C364="",E364=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E364)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H364&lt;&gt;0,F364=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G364&lt;&gt;0,F364=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F364&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F364)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C364)*($E$5:$E$504=E364)*(($D$5:$D$504=D364)*(D364&lt;&gt;"")+($B$5:$B$504=B364)*(B364&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C364="Оплата",K364&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E364)&gt;0,ROUND(E364-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J364" s="5">
@@ -10435,7 +10435,7 @@
         <v/>
       </c>
       <c r="I365" s="6">
-        <f>IF(AND(B365="",C365="",D365="",E365="",F365=""),"",IF(OR(B365="",C365="",E365=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E365)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H365&lt;&gt;0,F365=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G365&lt;&gt;0,F365=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F365&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F365)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C365)*($E$5:$E$504=E365)*(($D$5:$D$504=D365)*(D365&lt;&gt;"")+($B$5:$B$504=B365)*(B365&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C365="Оплата",K365&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E365)&gt;0,ROUND(E365-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B365="",C365="",D365="",E365="",F365=""),"",IF(OR(B365="",C365="",E365=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E365)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H365&lt;&gt;0,F365=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G365&lt;&gt;0,F365=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F365&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F365)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C365)*($E$5:$E$504=E365)*(($D$5:$D$504=D365)*(D365&lt;&gt;"")+($B$5:$B$504=B365)*(B365&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C365="Оплата",K365&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E365)&gt;0,ROUND(E365-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J365" s="5">
@@ -10462,7 +10462,7 @@
         <v/>
       </c>
       <c r="I366" s="6">
-        <f>IF(AND(B366="",C366="",D366="",E366="",F366=""),"",IF(OR(B366="",C366="",E366=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E366)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H366&lt;&gt;0,F366=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G366&lt;&gt;0,F366=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F366&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F366)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C366)*($E$5:$E$504=E366)*(($D$5:$D$504=D366)*(D366&lt;&gt;"")+($B$5:$B$504=B366)*(B366&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C366="Оплата",K366&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E366)&gt;0,ROUND(E366-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B366="",C366="",D366="",E366="",F366=""),"",IF(OR(B366="",C366="",E366=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E366)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H366&lt;&gt;0,F366=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G366&lt;&gt;0,F366=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F366&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F366)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C366)*($E$5:$E$504=E366)*(($D$5:$D$504=D366)*(D366&lt;&gt;"")+($B$5:$B$504=B366)*(B366&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C366="Оплата",K366&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E366)&gt;0,ROUND(E366-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J366" s="5">
@@ -10489,7 +10489,7 @@
         <v/>
       </c>
       <c r="I367" s="6">
-        <f>IF(AND(B367="",C367="",D367="",E367="",F367=""),"",IF(OR(B367="",C367="",E367=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E367)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H367&lt;&gt;0,F367=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G367&lt;&gt;0,F367=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F367&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F367)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C367)*($E$5:$E$504=E367)*(($D$5:$D$504=D367)*(D367&lt;&gt;"")+($B$5:$B$504=B367)*(B367&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C367="Оплата",K367&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E367)&gt;0,ROUND(E367-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B367="",C367="",D367="",E367="",F367=""),"",IF(OR(B367="",C367="",E367=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E367)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H367&lt;&gt;0,F367=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G367&lt;&gt;0,F367=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F367&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F367)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C367)*($E$5:$E$504=E367)*(($D$5:$D$504=D367)*(D367&lt;&gt;"")+($B$5:$B$504=B367)*(B367&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C367="Оплата",K367&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E367)&gt;0,ROUND(E367-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J367" s="5">
@@ -10516,7 +10516,7 @@
         <v/>
       </c>
       <c r="I368" s="6">
-        <f>IF(AND(B368="",C368="",D368="",E368="",F368=""),"",IF(OR(B368="",C368="",E368=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E368)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H368&lt;&gt;0,F368=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G368&lt;&gt;0,F368=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F368&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F368)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C368)*($E$5:$E$504=E368)*(($D$5:$D$504=D368)*(D368&lt;&gt;"")+($B$5:$B$504=B368)*(B368&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C368="Оплата",K368&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E368)&gt;0,ROUND(E368-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B368="",C368="",D368="",E368="",F368=""),"",IF(OR(B368="",C368="",E368=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E368)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H368&lt;&gt;0,F368=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G368&lt;&gt;0,F368=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F368&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F368)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C368)*($E$5:$E$504=E368)*(($D$5:$D$504=D368)*(D368&lt;&gt;"")+($B$5:$B$504=B368)*(B368&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C368="Оплата",K368&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E368)&gt;0,ROUND(E368-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J368" s="5">
@@ -10543,7 +10543,7 @@
         <v/>
       </c>
       <c r="I369" s="6">
-        <f>IF(AND(B369="",C369="",D369="",E369="",F369=""),"",IF(OR(B369="",C369="",E369=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E369)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H369&lt;&gt;0,F369=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G369&lt;&gt;0,F369=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F369&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F369)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C369)*($E$5:$E$504=E369)*(($D$5:$D$504=D369)*(D369&lt;&gt;"")+($B$5:$B$504=B369)*(B369&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C369="Оплата",K369&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E369)&gt;0,ROUND(E369-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B369="",C369="",D369="",E369="",F369=""),"",IF(OR(B369="",C369="",E369=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E369)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H369&lt;&gt;0,F369=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G369&lt;&gt;0,F369=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F369&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F369)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C369)*($E$5:$E$504=E369)*(($D$5:$D$504=D369)*(D369&lt;&gt;"")+($B$5:$B$504=B369)*(B369&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C369="Оплата",K369&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E369)&gt;0,ROUND(E369-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J369" s="5">
@@ -10570,7 +10570,7 @@
         <v/>
       </c>
       <c r="I370" s="6">
-        <f>IF(AND(B370="",C370="",D370="",E370="",F370=""),"",IF(OR(B370="",C370="",E370=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E370)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H370&lt;&gt;0,F370=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G370&lt;&gt;0,F370=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F370&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F370)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C370)*($E$5:$E$504=E370)*(($D$5:$D$504=D370)*(D370&lt;&gt;"")+($B$5:$B$504=B370)*(B370&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C370="Оплата",K370&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E370)&gt;0,ROUND(E370-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B370="",C370="",D370="",E370="",F370=""),"",IF(OR(B370="",C370="",E370=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E370)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H370&lt;&gt;0,F370=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G370&lt;&gt;0,F370=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F370&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F370)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C370)*($E$5:$E$504=E370)*(($D$5:$D$504=D370)*(D370&lt;&gt;"")+($B$5:$B$504=B370)*(B370&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C370="Оплата",K370&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E370)&gt;0,ROUND(E370-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J370" s="5">
@@ -10597,7 +10597,7 @@
         <v/>
       </c>
       <c r="I371" s="6">
-        <f>IF(AND(B371="",C371="",D371="",E371="",F371=""),"",IF(OR(B371="",C371="",E371=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E371)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H371&lt;&gt;0,F371=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G371&lt;&gt;0,F371=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F371&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F371)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C371)*($E$5:$E$504=E371)*(($D$5:$D$504=D371)*(D371&lt;&gt;"")+($B$5:$B$504=B371)*(B371&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C371="Оплата",K371&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E371)&gt;0,ROUND(E371-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B371="",C371="",D371="",E371="",F371=""),"",IF(OR(B371="",C371="",E371=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E371)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H371&lt;&gt;0,F371=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G371&lt;&gt;0,F371=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F371&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F371)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C371)*($E$5:$E$504=E371)*(($D$5:$D$504=D371)*(D371&lt;&gt;"")+($B$5:$B$504=B371)*(B371&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C371="Оплата",K371&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E371)&gt;0,ROUND(E371-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J371" s="5">
@@ -10624,7 +10624,7 @@
         <v/>
       </c>
       <c r="I372" s="6">
-        <f>IF(AND(B372="",C372="",D372="",E372="",F372=""),"",IF(OR(B372="",C372="",E372=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E372)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H372&lt;&gt;0,F372=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G372&lt;&gt;0,F372=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F372&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F372)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C372)*($E$5:$E$504=E372)*(($D$5:$D$504=D372)*(D372&lt;&gt;"")+($B$5:$B$504=B372)*(B372&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C372="Оплата",K372&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E372)&gt;0,ROUND(E372-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B372="",C372="",D372="",E372="",F372=""),"",IF(OR(B372="",C372="",E372=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E372)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H372&lt;&gt;0,F372=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G372&lt;&gt;0,F372=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F372&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F372)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C372)*($E$5:$E$504=E372)*(($D$5:$D$504=D372)*(D372&lt;&gt;"")+($B$5:$B$504=B372)*(B372&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C372="Оплата",K372&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E372)&gt;0,ROUND(E372-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J372" s="5">
@@ -10651,7 +10651,7 @@
         <v/>
       </c>
       <c r="I373" s="6">
-        <f>IF(AND(B373="",C373="",D373="",E373="",F373=""),"",IF(OR(B373="",C373="",E373=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E373)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H373&lt;&gt;0,F373=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G373&lt;&gt;0,F373=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F373&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F373)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C373)*($E$5:$E$504=E373)*(($D$5:$D$504=D373)*(D373&lt;&gt;"")+($B$5:$B$504=B373)*(B373&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C373="Оплата",K373&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E373)&gt;0,ROUND(E373-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B373="",C373="",D373="",E373="",F373=""),"",IF(OR(B373="",C373="",E373=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E373)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H373&lt;&gt;0,F373=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G373&lt;&gt;0,F373=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F373&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F373)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C373)*($E$5:$E$504=E373)*(($D$5:$D$504=D373)*(D373&lt;&gt;"")+($B$5:$B$504=B373)*(B373&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C373="Оплата",K373&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E373)&gt;0,ROUND(E373-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J373" s="5">
@@ -10678,7 +10678,7 @@
         <v/>
       </c>
       <c r="I374" s="6">
-        <f>IF(AND(B374="",C374="",D374="",E374="",F374=""),"",IF(OR(B374="",C374="",E374=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E374)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H374&lt;&gt;0,F374=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G374&lt;&gt;0,F374=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F374&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F374)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C374)*($E$5:$E$504=E374)*(($D$5:$D$504=D374)*(D374&lt;&gt;"")+($B$5:$B$504=B374)*(B374&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C374="Оплата",K374&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E374)&gt;0,ROUND(E374-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B374="",C374="",D374="",E374="",F374=""),"",IF(OR(B374="",C374="",E374=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E374)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H374&lt;&gt;0,F374=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G374&lt;&gt;0,F374=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F374&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F374)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C374)*($E$5:$E$504=E374)*(($D$5:$D$504=D374)*(D374&lt;&gt;"")+($B$5:$B$504=B374)*(B374&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C374="Оплата",K374&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E374)&gt;0,ROUND(E374-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J374" s="5">
@@ -10705,7 +10705,7 @@
         <v/>
       </c>
       <c r="I375" s="6">
-        <f>IF(AND(B375="",C375="",D375="",E375="",F375=""),"",IF(OR(B375="",C375="",E375=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E375)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H375&lt;&gt;0,F375=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G375&lt;&gt;0,F375=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F375&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F375)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C375)*($E$5:$E$504=E375)*(($D$5:$D$504=D375)*(D375&lt;&gt;"")+($B$5:$B$504=B375)*(B375&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C375="Оплата",K375&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E375)&gt;0,ROUND(E375-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B375="",C375="",D375="",E375="",F375=""),"",IF(OR(B375="",C375="",E375=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E375)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H375&lt;&gt;0,F375=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G375&lt;&gt;0,F375=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F375&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F375)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C375)*($E$5:$E$504=E375)*(($D$5:$D$504=D375)*(D375&lt;&gt;"")+($B$5:$B$504=B375)*(B375&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C375="Оплата",K375&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E375)&gt;0,ROUND(E375-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J375" s="5">
@@ -10732,7 +10732,7 @@
         <v/>
       </c>
       <c r="I376" s="6">
-        <f>IF(AND(B376="",C376="",D376="",E376="",F376=""),"",IF(OR(B376="",C376="",E376=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E376)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H376&lt;&gt;0,F376=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G376&lt;&gt;0,F376=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F376&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F376)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C376)*($E$5:$E$504=E376)*(($D$5:$D$504=D376)*(D376&lt;&gt;"")+($B$5:$B$504=B376)*(B376&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C376="Оплата",K376&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E376)&gt;0,ROUND(E376-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B376="",C376="",D376="",E376="",F376=""),"",IF(OR(B376="",C376="",E376=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E376)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H376&lt;&gt;0,F376=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G376&lt;&gt;0,F376=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F376&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F376)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C376)*($E$5:$E$504=E376)*(($D$5:$D$504=D376)*(D376&lt;&gt;"")+($B$5:$B$504=B376)*(B376&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C376="Оплата",K376&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E376)&gt;0,ROUND(E376-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J376" s="5">
@@ -10759,7 +10759,7 @@
         <v/>
       </c>
       <c r="I377" s="6">
-        <f>IF(AND(B377="",C377="",D377="",E377="",F377=""),"",IF(OR(B377="",C377="",E377=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E377)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H377&lt;&gt;0,F377=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G377&lt;&gt;0,F377=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F377&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F377)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C377)*($E$5:$E$504=E377)*(($D$5:$D$504=D377)*(D377&lt;&gt;"")+($B$5:$B$504=B377)*(B377&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C377="Оплата",K377&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E377)&gt;0,ROUND(E377-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B377="",C377="",D377="",E377="",F377=""),"",IF(OR(B377="",C377="",E377=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E377)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H377&lt;&gt;0,F377=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G377&lt;&gt;0,F377=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F377&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F377)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C377)*($E$5:$E$504=E377)*(($D$5:$D$504=D377)*(D377&lt;&gt;"")+($B$5:$B$504=B377)*(B377&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C377="Оплата",K377&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E377)&gt;0,ROUND(E377-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J377" s="5">
@@ -10786,7 +10786,7 @@
         <v/>
       </c>
       <c r="I378" s="6">
-        <f>IF(AND(B378="",C378="",D378="",E378="",F378=""),"",IF(OR(B378="",C378="",E378=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E378)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H378&lt;&gt;0,F378=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G378&lt;&gt;0,F378=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F378&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F378)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C378)*($E$5:$E$504=E378)*(($D$5:$D$504=D378)*(D378&lt;&gt;"")+($B$5:$B$504=B378)*(B378&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C378="Оплата",K378&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E378)&gt;0,ROUND(E378-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B378="",C378="",D378="",E378="",F378=""),"",IF(OR(B378="",C378="",E378=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E378)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H378&lt;&gt;0,F378=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G378&lt;&gt;0,F378=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F378&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F378)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C378)*($E$5:$E$504=E378)*(($D$5:$D$504=D378)*(D378&lt;&gt;"")+($B$5:$B$504=B378)*(B378&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C378="Оплата",K378&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E378)&gt;0,ROUND(E378-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J378" s="5">
@@ -10813,7 +10813,7 @@
         <v/>
       </c>
       <c r="I379" s="6">
-        <f>IF(AND(B379="",C379="",D379="",E379="",F379=""),"",IF(OR(B379="",C379="",E379=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E379)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H379&lt;&gt;0,F379=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G379&lt;&gt;0,F379=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F379&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F379)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C379)*($E$5:$E$504=E379)*(($D$5:$D$504=D379)*(D379&lt;&gt;"")+($B$5:$B$504=B379)*(B379&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C379="Оплата",K379&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E379)&gt;0,ROUND(E379-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B379="",C379="",D379="",E379="",F379=""),"",IF(OR(B379="",C379="",E379=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E379)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H379&lt;&gt;0,F379=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G379&lt;&gt;0,F379=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F379&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F379)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C379)*($E$5:$E$504=E379)*(($D$5:$D$504=D379)*(D379&lt;&gt;"")+($B$5:$B$504=B379)*(B379&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C379="Оплата",K379&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E379)&gt;0,ROUND(E379-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J379" s="5">
@@ -10840,7 +10840,7 @@
         <v/>
       </c>
       <c r="I380" s="6">
-        <f>IF(AND(B380="",C380="",D380="",E380="",F380=""),"",IF(OR(B380="",C380="",E380=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E380)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H380&lt;&gt;0,F380=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G380&lt;&gt;0,F380=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F380&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F380)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C380)*($E$5:$E$504=E380)*(($D$5:$D$504=D380)*(D380&lt;&gt;"")+($B$5:$B$504=B380)*(B380&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C380="Оплата",K380&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E380)&gt;0,ROUND(E380-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B380="",C380="",D380="",E380="",F380=""),"",IF(OR(B380="",C380="",E380=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E380)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H380&lt;&gt;0,F380=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G380&lt;&gt;0,F380=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F380&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F380)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C380)*($E$5:$E$504=E380)*(($D$5:$D$504=D380)*(D380&lt;&gt;"")+($B$5:$B$504=B380)*(B380&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C380="Оплата",K380&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E380)&gt;0,ROUND(E380-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J380" s="5">
@@ -10867,7 +10867,7 @@
         <v/>
       </c>
       <c r="I381" s="6">
-        <f>IF(AND(B381="",C381="",D381="",E381="",F381=""),"",IF(OR(B381="",C381="",E381=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E381)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H381&lt;&gt;0,F381=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G381&lt;&gt;0,F381=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F381&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F381)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C381)*($E$5:$E$504=E381)*(($D$5:$D$504=D381)*(D381&lt;&gt;"")+($B$5:$B$504=B381)*(B381&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C381="Оплата",K381&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E381)&gt;0,ROUND(E381-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B381="",C381="",D381="",E381="",F381=""),"",IF(OR(B381="",C381="",E381=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E381)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H381&lt;&gt;0,F381=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G381&lt;&gt;0,F381=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F381&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F381)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C381)*($E$5:$E$504=E381)*(($D$5:$D$504=D381)*(D381&lt;&gt;"")+($B$5:$B$504=B381)*(B381&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C381="Оплата",K381&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E381)&gt;0,ROUND(E381-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J381" s="5">
@@ -10894,7 +10894,7 @@
         <v/>
       </c>
       <c r="I382" s="6">
-        <f>IF(AND(B382="",C382="",D382="",E382="",F382=""),"",IF(OR(B382="",C382="",E382=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E382)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H382&lt;&gt;0,F382=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G382&lt;&gt;0,F382=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F382&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F382)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C382)*($E$5:$E$504=E382)*(($D$5:$D$504=D382)*(D382&lt;&gt;"")+($B$5:$B$504=B382)*(B382&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C382="Оплата",K382&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E382)&gt;0,ROUND(E382-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B382="",C382="",D382="",E382="",F382=""),"",IF(OR(B382="",C382="",E382=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E382)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H382&lt;&gt;0,F382=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G382&lt;&gt;0,F382=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F382&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F382)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C382)*($E$5:$E$504=E382)*(($D$5:$D$504=D382)*(D382&lt;&gt;"")+($B$5:$B$504=B382)*(B382&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C382="Оплата",K382&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E382)&gt;0,ROUND(E382-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J382" s="5">
@@ -10921,7 +10921,7 @@
         <v/>
       </c>
       <c r="I383" s="6">
-        <f>IF(AND(B383="",C383="",D383="",E383="",F383=""),"",IF(OR(B383="",C383="",E383=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E383)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H383&lt;&gt;0,F383=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G383&lt;&gt;0,F383=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F383&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F383)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C383)*($E$5:$E$504=E383)*(($D$5:$D$504=D383)*(D383&lt;&gt;"")+($B$5:$B$504=B383)*(B383&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C383="Оплата",K383&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E383)&gt;0,ROUND(E383-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B383="",C383="",D383="",E383="",F383=""),"",IF(OR(B383="",C383="",E383=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E383)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H383&lt;&gt;0,F383=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G383&lt;&gt;0,F383=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F383&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F383)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C383)*($E$5:$E$504=E383)*(($D$5:$D$504=D383)*(D383&lt;&gt;"")+($B$5:$B$504=B383)*(B383&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C383="Оплата",K383&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E383)&gt;0,ROUND(E383-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J383" s="5">
@@ -10948,7 +10948,7 @@
         <v/>
       </c>
       <c r="I384" s="6">
-        <f>IF(AND(B384="",C384="",D384="",E384="",F384=""),"",IF(OR(B384="",C384="",E384=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E384)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H384&lt;&gt;0,F384=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G384&lt;&gt;0,F384=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F384&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F384)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C384)*($E$5:$E$504=E384)*(($D$5:$D$504=D384)*(D384&lt;&gt;"")+($B$5:$B$504=B384)*(B384&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C384="Оплата",K384&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E384)&gt;0,ROUND(E384-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B384="",C384="",D384="",E384="",F384=""),"",IF(OR(B384="",C384="",E384=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E384)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H384&lt;&gt;0,F384=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G384&lt;&gt;0,F384=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F384&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F384)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C384)*($E$5:$E$504=E384)*(($D$5:$D$504=D384)*(D384&lt;&gt;"")+($B$5:$B$504=B384)*(B384&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C384="Оплата",K384&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E384)&gt;0,ROUND(E384-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J384" s="5">
@@ -10975,7 +10975,7 @@
         <v/>
       </c>
       <c r="I385" s="6">
-        <f>IF(AND(B385="",C385="",D385="",E385="",F385=""),"",IF(OR(B385="",C385="",E385=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E385)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H385&lt;&gt;0,F385=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G385&lt;&gt;0,F385=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F385&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F385)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C385)*($E$5:$E$504=E385)*(($D$5:$D$504=D385)*(D385&lt;&gt;"")+($B$5:$B$504=B385)*(B385&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C385="Оплата",K385&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E385)&gt;0,ROUND(E385-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B385="",C385="",D385="",E385="",F385=""),"",IF(OR(B385="",C385="",E385=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E385)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H385&lt;&gt;0,F385=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G385&lt;&gt;0,F385=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F385&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F385)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C385)*($E$5:$E$504=E385)*(($D$5:$D$504=D385)*(D385&lt;&gt;"")+($B$5:$B$504=B385)*(B385&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C385="Оплата",K385&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E385)&gt;0,ROUND(E385-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J385" s="5">
@@ -11002,7 +11002,7 @@
         <v/>
       </c>
       <c r="I386" s="6">
-        <f>IF(AND(B386="",C386="",D386="",E386="",F386=""),"",IF(OR(B386="",C386="",E386=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E386)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H386&lt;&gt;0,F386=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G386&lt;&gt;0,F386=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F386&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F386)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C386)*($E$5:$E$504=E386)*(($D$5:$D$504=D386)*(D386&lt;&gt;"")+($B$5:$B$504=B386)*(B386&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C386="Оплата",K386&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E386)&gt;0,ROUND(E386-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B386="",C386="",D386="",E386="",F386=""),"",IF(OR(B386="",C386="",E386=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E386)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H386&lt;&gt;0,F386=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G386&lt;&gt;0,F386=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F386&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F386)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C386)*($E$5:$E$504=E386)*(($D$5:$D$504=D386)*(D386&lt;&gt;"")+($B$5:$B$504=B386)*(B386&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C386="Оплата",K386&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E386)&gt;0,ROUND(E386-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J386" s="5">
@@ -11029,7 +11029,7 @@
         <v/>
       </c>
       <c r="I387" s="6">
-        <f>IF(AND(B387="",C387="",D387="",E387="",F387=""),"",IF(OR(B387="",C387="",E387=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E387)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H387&lt;&gt;0,F387=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G387&lt;&gt;0,F387=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F387&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F387)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C387)*($E$5:$E$504=E387)*(($D$5:$D$504=D387)*(D387&lt;&gt;"")+($B$5:$B$504=B387)*(B387&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C387="Оплата",K387&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E387)&gt;0,ROUND(E387-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B387="",C387="",D387="",E387="",F387=""),"",IF(OR(B387="",C387="",E387=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E387)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H387&lt;&gt;0,F387=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G387&lt;&gt;0,F387=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F387&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F387)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C387)*($E$5:$E$504=E387)*(($D$5:$D$504=D387)*(D387&lt;&gt;"")+($B$5:$B$504=B387)*(B387&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C387="Оплата",K387&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E387)&gt;0,ROUND(E387-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J387" s="5">
@@ -11056,7 +11056,7 @@
         <v/>
       </c>
       <c r="I388" s="6">
-        <f>IF(AND(B388="",C388="",D388="",E388="",F388=""),"",IF(OR(B388="",C388="",E388=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E388)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H388&lt;&gt;0,F388=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G388&lt;&gt;0,F388=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F388&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F388)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C388)*($E$5:$E$504=E388)*(($D$5:$D$504=D388)*(D388&lt;&gt;"")+($B$5:$B$504=B388)*(B388&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C388="Оплата",K388&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E388)&gt;0,ROUND(E388-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B388="",C388="",D388="",E388="",F388=""),"",IF(OR(B388="",C388="",E388=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E388)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H388&lt;&gt;0,F388=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G388&lt;&gt;0,F388=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F388&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F388)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C388)*($E$5:$E$504=E388)*(($D$5:$D$504=D388)*(D388&lt;&gt;"")+($B$5:$B$504=B388)*(B388&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C388="Оплата",K388&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E388)&gt;0,ROUND(E388-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J388" s="5">
@@ -11083,7 +11083,7 @@
         <v/>
       </c>
       <c r="I389" s="6">
-        <f>IF(AND(B389="",C389="",D389="",E389="",F389=""),"",IF(OR(B389="",C389="",E389=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E389)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H389&lt;&gt;0,F389=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G389&lt;&gt;0,F389=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F389&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F389)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C389)*($E$5:$E$504=E389)*(($D$5:$D$504=D389)*(D389&lt;&gt;"")+($B$5:$B$504=B389)*(B389&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C389="Оплата",K389&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E389)&gt;0,ROUND(E389-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B389="",C389="",D389="",E389="",F389=""),"",IF(OR(B389="",C389="",E389=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E389)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H389&lt;&gt;0,F389=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G389&lt;&gt;0,F389=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F389&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F389)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C389)*($E$5:$E$504=E389)*(($D$5:$D$504=D389)*(D389&lt;&gt;"")+($B$5:$B$504=B389)*(B389&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C389="Оплата",K389&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E389)&gt;0,ROUND(E389-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J389" s="5">
@@ -11110,7 +11110,7 @@
         <v/>
       </c>
       <c r="I390" s="6">
-        <f>IF(AND(B390="",C390="",D390="",E390="",F390=""),"",IF(OR(B390="",C390="",E390=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E390)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H390&lt;&gt;0,F390=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G390&lt;&gt;0,F390=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F390&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F390)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C390)*($E$5:$E$504=E390)*(($D$5:$D$504=D390)*(D390&lt;&gt;"")+($B$5:$B$504=B390)*(B390&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C390="Оплата",K390&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E390)&gt;0,ROUND(E390-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B390="",C390="",D390="",E390="",F390=""),"",IF(OR(B390="",C390="",E390=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E390)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H390&lt;&gt;0,F390=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G390&lt;&gt;0,F390=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F390&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F390)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C390)*($E$5:$E$504=E390)*(($D$5:$D$504=D390)*(D390&lt;&gt;"")+($B$5:$B$504=B390)*(B390&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C390="Оплата",K390&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E390)&gt;0,ROUND(E390-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J390" s="5">
@@ -11137,7 +11137,7 @@
         <v/>
       </c>
       <c r="I391" s="6">
-        <f>IF(AND(B391="",C391="",D391="",E391="",F391=""),"",IF(OR(B391="",C391="",E391=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E391)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H391&lt;&gt;0,F391=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G391&lt;&gt;0,F391=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F391&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F391)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C391)*($E$5:$E$504=E391)*(($D$5:$D$504=D391)*(D391&lt;&gt;"")+($B$5:$B$504=B391)*(B391&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C391="Оплата",K391&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E391)&gt;0,ROUND(E391-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B391="",C391="",D391="",E391="",F391=""),"",IF(OR(B391="",C391="",E391=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E391)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H391&lt;&gt;0,F391=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G391&lt;&gt;0,F391=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F391&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F391)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C391)*($E$5:$E$504=E391)*(($D$5:$D$504=D391)*(D391&lt;&gt;"")+($B$5:$B$504=B391)*(B391&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C391="Оплата",K391&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E391)&gt;0,ROUND(E391-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J391" s="5">
@@ -11164,7 +11164,7 @@
         <v/>
       </c>
       <c r="I392" s="6">
-        <f>IF(AND(B392="",C392="",D392="",E392="",F392=""),"",IF(OR(B392="",C392="",E392=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E392)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H392&lt;&gt;0,F392=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G392&lt;&gt;0,F392=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F392&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F392)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C392)*($E$5:$E$504=E392)*(($D$5:$D$504=D392)*(D392&lt;&gt;"")+($B$5:$B$504=B392)*(B392&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C392="Оплата",K392&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E392)&gt;0,ROUND(E392-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B392="",C392="",D392="",E392="",F392=""),"",IF(OR(B392="",C392="",E392=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E392)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H392&lt;&gt;0,F392=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G392&lt;&gt;0,F392=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F392&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F392)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C392)*($E$5:$E$504=E392)*(($D$5:$D$504=D392)*(D392&lt;&gt;"")+($B$5:$B$504=B392)*(B392&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C392="Оплата",K392&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E392)&gt;0,ROUND(E392-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J392" s="5">
@@ -11191,7 +11191,7 @@
         <v/>
       </c>
       <c r="I393" s="6">
-        <f>IF(AND(B393="",C393="",D393="",E393="",F393=""),"",IF(OR(B393="",C393="",E393=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E393)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H393&lt;&gt;0,F393=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G393&lt;&gt;0,F393=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F393&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F393)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C393)*($E$5:$E$504=E393)*(($D$5:$D$504=D393)*(D393&lt;&gt;"")+($B$5:$B$504=B393)*(B393&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C393="Оплата",K393&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E393)&gt;0,ROUND(E393-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B393="",C393="",D393="",E393="",F393=""),"",IF(OR(B393="",C393="",E393=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E393)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H393&lt;&gt;0,F393=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G393&lt;&gt;0,F393=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F393&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F393)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C393)*($E$5:$E$504=E393)*(($D$5:$D$504=D393)*(D393&lt;&gt;"")+($B$5:$B$504=B393)*(B393&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C393="Оплата",K393&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E393)&gt;0,ROUND(E393-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J393" s="5">
@@ -11218,7 +11218,7 @@
         <v/>
       </c>
       <c r="I394" s="6">
-        <f>IF(AND(B394="",C394="",D394="",E394="",F394=""),"",IF(OR(B394="",C394="",E394=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E394)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H394&lt;&gt;0,F394=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G394&lt;&gt;0,F394=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F394&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F394)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C394)*($E$5:$E$504=E394)*(($D$5:$D$504=D394)*(D394&lt;&gt;"")+($B$5:$B$504=B394)*(B394&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C394="Оплата",K394&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E394)&gt;0,ROUND(E394-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B394="",C394="",D394="",E394="",F394=""),"",IF(OR(B394="",C394="",E394=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E394)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H394&lt;&gt;0,F394=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G394&lt;&gt;0,F394=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F394&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F394)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C394)*($E$5:$E$504=E394)*(($D$5:$D$504=D394)*(D394&lt;&gt;"")+($B$5:$B$504=B394)*(B394&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C394="Оплата",K394&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E394)&gt;0,ROUND(E394-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J394" s="5">
@@ -11245,7 +11245,7 @@
         <v/>
       </c>
       <c r="I395" s="6">
-        <f>IF(AND(B395="",C395="",D395="",E395="",F395=""),"",IF(OR(B395="",C395="",E395=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E395)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H395&lt;&gt;0,F395=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G395&lt;&gt;0,F395=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F395&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F395)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C395)*($E$5:$E$504=E395)*(($D$5:$D$504=D395)*(D395&lt;&gt;"")+($B$5:$B$504=B395)*(B395&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C395="Оплата",K395&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E395)&gt;0,ROUND(E395-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B395="",C395="",D395="",E395="",F395=""),"",IF(OR(B395="",C395="",E395=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E395)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H395&lt;&gt;0,F395=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G395&lt;&gt;0,F395=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F395&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F395)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C395)*($E$5:$E$504=E395)*(($D$5:$D$504=D395)*(D395&lt;&gt;"")+($B$5:$B$504=B395)*(B395&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C395="Оплата",K395&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E395)&gt;0,ROUND(E395-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J395" s="5">
@@ -11272,7 +11272,7 @@
         <v/>
       </c>
       <c r="I396" s="6">
-        <f>IF(AND(B396="",C396="",D396="",E396="",F396=""),"",IF(OR(B396="",C396="",E396=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E396)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H396&lt;&gt;0,F396=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G396&lt;&gt;0,F396=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F396&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F396)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C396)*($E$5:$E$504=E396)*(($D$5:$D$504=D396)*(D396&lt;&gt;"")+($B$5:$B$504=B396)*(B396&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C396="Оплата",K396&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E396)&gt;0,ROUND(E396-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B396="",C396="",D396="",E396="",F396=""),"",IF(OR(B396="",C396="",E396=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E396)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H396&lt;&gt;0,F396=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G396&lt;&gt;0,F396=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F396&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F396)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C396)*($E$5:$E$504=E396)*(($D$5:$D$504=D396)*(D396&lt;&gt;"")+($B$5:$B$504=B396)*(B396&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C396="Оплата",K396&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E396)&gt;0,ROUND(E396-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J396" s="5">
@@ -11299,7 +11299,7 @@
         <v/>
       </c>
       <c r="I397" s="6">
-        <f>IF(AND(B397="",C397="",D397="",E397="",F397=""),"",IF(OR(B397="",C397="",E397=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E397)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H397&lt;&gt;0,F397=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G397&lt;&gt;0,F397=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F397&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F397)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C397)*($E$5:$E$504=E397)*(($D$5:$D$504=D397)*(D397&lt;&gt;"")+($B$5:$B$504=B397)*(B397&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C397="Оплата",K397&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E397)&gt;0,ROUND(E397-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B397="",C397="",D397="",E397="",F397=""),"",IF(OR(B397="",C397="",E397=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E397)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H397&lt;&gt;0,F397=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G397&lt;&gt;0,F397=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F397&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F397)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C397)*($E$5:$E$504=E397)*(($D$5:$D$504=D397)*(D397&lt;&gt;"")+($B$5:$B$504=B397)*(B397&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C397="Оплата",K397&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E397)&gt;0,ROUND(E397-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J397" s="5">
@@ -11326,7 +11326,7 @@
         <v/>
       </c>
       <c r="I398" s="6">
-        <f>IF(AND(B398="",C398="",D398="",E398="",F398=""),"",IF(OR(B398="",C398="",E398=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E398)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H398&lt;&gt;0,F398=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G398&lt;&gt;0,F398=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F398&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F398)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C398)*($E$5:$E$504=E398)*(($D$5:$D$504=D398)*(D398&lt;&gt;"")+($B$5:$B$504=B398)*(B398&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C398="Оплата",K398&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E398)&gt;0,ROUND(E398-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B398="",C398="",D398="",E398="",F398=""),"",IF(OR(B398="",C398="",E398=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E398)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H398&lt;&gt;0,F398=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G398&lt;&gt;0,F398=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F398&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F398)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C398)*($E$5:$E$504=E398)*(($D$5:$D$504=D398)*(D398&lt;&gt;"")+($B$5:$B$504=B398)*(B398&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C398="Оплата",K398&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E398)&gt;0,ROUND(E398-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J398" s="5">
@@ -11353,7 +11353,7 @@
         <v/>
       </c>
       <c r="I399" s="6">
-        <f>IF(AND(B399="",C399="",D399="",E399="",F399=""),"",IF(OR(B399="",C399="",E399=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E399)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H399&lt;&gt;0,F399=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G399&lt;&gt;0,F399=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F399&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F399)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C399)*($E$5:$E$504=E399)*(($D$5:$D$504=D399)*(D399&lt;&gt;"")+($B$5:$B$504=B399)*(B399&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C399="Оплата",K399&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E399)&gt;0,ROUND(E399-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B399="",C399="",D399="",E399="",F399=""),"",IF(OR(B399="",C399="",E399=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E399)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H399&lt;&gt;0,F399=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G399&lt;&gt;0,F399=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F399&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F399)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C399)*($E$5:$E$504=E399)*(($D$5:$D$504=D399)*(D399&lt;&gt;"")+($B$5:$B$504=B399)*(B399&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C399="Оплата",K399&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E399)&gt;0,ROUND(E399-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J399" s="5">
@@ -11380,7 +11380,7 @@
         <v/>
       </c>
       <c r="I400" s="6">
-        <f>IF(AND(B400="",C400="",D400="",E400="",F400=""),"",IF(OR(B400="",C400="",E400=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E400)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H400&lt;&gt;0,F400=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G400&lt;&gt;0,F400=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F400&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F400)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C400)*($E$5:$E$504=E400)*(($D$5:$D$504=D400)*(D400&lt;&gt;"")+($B$5:$B$504=B400)*(B400&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C400="Оплата",K400&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E400)&gt;0,ROUND(E400-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B400="",C400="",D400="",E400="",F400=""),"",IF(OR(B400="",C400="",E400=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E400)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H400&lt;&gt;0,F400=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G400&lt;&gt;0,F400=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F400&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F400)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C400)*($E$5:$E$504=E400)*(($D$5:$D$504=D400)*(D400&lt;&gt;"")+($B$5:$B$504=B400)*(B400&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C400="Оплата",K400&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E400)&gt;0,ROUND(E400-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J400" s="5">
@@ -11407,7 +11407,7 @@
         <v/>
       </c>
       <c r="I401" s="6">
-        <f>IF(AND(B401="",C401="",D401="",E401="",F401=""),"",IF(OR(B401="",C401="",E401=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E401)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H401&lt;&gt;0,F401=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G401&lt;&gt;0,F401=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F401&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F401)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C401)*($E$5:$E$504=E401)*(($D$5:$D$504=D401)*(D401&lt;&gt;"")+($B$5:$B$504=B401)*(B401&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C401="Оплата",K401&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E401)&gt;0,ROUND(E401-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B401="",C401="",D401="",E401="",F401=""),"",IF(OR(B401="",C401="",E401=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E401)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H401&lt;&gt;0,F401=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G401&lt;&gt;0,F401=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F401&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F401)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C401)*($E$5:$E$504=E401)*(($D$5:$D$504=D401)*(D401&lt;&gt;"")+($B$5:$B$504=B401)*(B401&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C401="Оплата",K401&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E401)&gt;0,ROUND(E401-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J401" s="5">
@@ -11434,7 +11434,7 @@
         <v/>
       </c>
       <c r="I402" s="6">
-        <f>IF(AND(B402="",C402="",D402="",E402="",F402=""),"",IF(OR(B402="",C402="",E402=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E402)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H402&lt;&gt;0,F402=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G402&lt;&gt;0,F402=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F402&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F402)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C402)*($E$5:$E$504=E402)*(($D$5:$D$504=D402)*(D402&lt;&gt;"")+($B$5:$B$504=B402)*(B402&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C402="Оплата",K402&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E402)&gt;0,ROUND(E402-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B402="",C402="",D402="",E402="",F402=""),"",IF(OR(B402="",C402="",E402=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E402)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H402&lt;&gt;0,F402=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G402&lt;&gt;0,F402=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F402&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F402)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C402)*($E$5:$E$504=E402)*(($D$5:$D$504=D402)*(D402&lt;&gt;"")+($B$5:$B$504=B402)*(B402&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C402="Оплата",K402&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E402)&gt;0,ROUND(E402-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J402" s="5">
@@ -11461,7 +11461,7 @@
         <v/>
       </c>
       <c r="I403" s="6">
-        <f>IF(AND(B403="",C403="",D403="",E403="",F403=""),"",IF(OR(B403="",C403="",E403=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E403)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H403&lt;&gt;0,F403=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G403&lt;&gt;0,F403=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F403&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F403)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C403)*($E$5:$E$504=E403)*(($D$5:$D$504=D403)*(D403&lt;&gt;"")+($B$5:$B$504=B403)*(B403&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C403="Оплата",K403&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E403)&gt;0,ROUND(E403-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B403="",C403="",D403="",E403="",F403=""),"",IF(OR(B403="",C403="",E403=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E403)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H403&lt;&gt;0,F403=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G403&lt;&gt;0,F403=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F403&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F403)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C403)*($E$5:$E$504=E403)*(($D$5:$D$504=D403)*(D403&lt;&gt;"")+($B$5:$B$504=B403)*(B403&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C403="Оплата",K403&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E403)&gt;0,ROUND(E403-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J403" s="5">
@@ -11488,7 +11488,7 @@
         <v/>
       </c>
       <c r="I404" s="6">
-        <f>IF(AND(B404="",C404="",D404="",E404="",F404=""),"",IF(OR(B404="",C404="",E404=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E404)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H404&lt;&gt;0,F404=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G404&lt;&gt;0,F404=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F404&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F404)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C404)*($E$5:$E$504=E404)*(($D$5:$D$504=D404)*(D404&lt;&gt;"")+($B$5:$B$504=B404)*(B404&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C404="Оплата",K404&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E404)&gt;0,ROUND(E404-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B404="",C404="",D404="",E404="",F404=""),"",IF(OR(B404="",C404="",E404=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E404)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H404&lt;&gt;0,F404=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G404&lt;&gt;0,F404=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F404&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F404)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C404)*($E$5:$E$504=E404)*(($D$5:$D$504=D404)*(D404&lt;&gt;"")+($B$5:$B$504=B404)*(B404&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C404="Оплата",K404&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E404)&gt;0,ROUND(E404-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J404" s="5">
@@ -11515,7 +11515,7 @@
         <v/>
       </c>
       <c r="I405" s="6">
-        <f>IF(AND(B405="",C405="",D405="",E405="",F405=""),"",IF(OR(B405="",C405="",E405=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E405)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H405&lt;&gt;0,F405=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G405&lt;&gt;0,F405=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F405&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F405)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C405)*($E$5:$E$504=E405)*(($D$5:$D$504=D405)*(D405&lt;&gt;"")+($B$5:$B$504=B405)*(B405&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C405="Оплата",K405&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E405)&gt;0,ROUND(E405-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B405="",C405="",D405="",E405="",F405=""),"",IF(OR(B405="",C405="",E405=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E405)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H405&lt;&gt;0,F405=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G405&lt;&gt;0,F405=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F405&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F405)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C405)*($E$5:$E$504=E405)*(($D$5:$D$504=D405)*(D405&lt;&gt;"")+($B$5:$B$504=B405)*(B405&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C405="Оплата",K405&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E405)&gt;0,ROUND(E405-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J405" s="5">
@@ -11542,7 +11542,7 @@
         <v/>
       </c>
       <c r="I406" s="6">
-        <f>IF(AND(B406="",C406="",D406="",E406="",F406=""),"",IF(OR(B406="",C406="",E406=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E406)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H406&lt;&gt;0,F406=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G406&lt;&gt;0,F406=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F406&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F406)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C406)*($E$5:$E$504=E406)*(($D$5:$D$504=D406)*(D406&lt;&gt;"")+($B$5:$B$504=B406)*(B406&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C406="Оплата",K406&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E406)&gt;0,ROUND(E406-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B406="",C406="",D406="",E406="",F406=""),"",IF(OR(B406="",C406="",E406=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E406)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H406&lt;&gt;0,F406=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G406&lt;&gt;0,F406=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F406&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F406)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C406)*($E$5:$E$504=E406)*(($D$5:$D$504=D406)*(D406&lt;&gt;"")+($B$5:$B$504=B406)*(B406&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C406="Оплата",K406&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E406)&gt;0,ROUND(E406-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J406" s="5">
@@ -11569,7 +11569,7 @@
         <v/>
       </c>
       <c r="I407" s="6">
-        <f>IF(AND(B407="",C407="",D407="",E407="",F407=""),"",IF(OR(B407="",C407="",E407=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E407)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H407&lt;&gt;0,F407=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G407&lt;&gt;0,F407=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F407&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F407)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C407)*($E$5:$E$504=E407)*(($D$5:$D$504=D407)*(D407&lt;&gt;"")+($B$5:$B$504=B407)*(B407&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C407="Оплата",K407&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E407)&gt;0,ROUND(E407-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B407="",C407="",D407="",E407="",F407=""),"",IF(OR(B407="",C407="",E407=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E407)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H407&lt;&gt;0,F407=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G407&lt;&gt;0,F407=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F407&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F407)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C407)*($E$5:$E$504=E407)*(($D$5:$D$504=D407)*(D407&lt;&gt;"")+($B$5:$B$504=B407)*(B407&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C407="Оплата",K407&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E407)&gt;0,ROUND(E407-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J407" s="5">
@@ -11596,7 +11596,7 @@
         <v/>
       </c>
       <c r="I408" s="6">
-        <f>IF(AND(B408="",C408="",D408="",E408="",F408=""),"",IF(OR(B408="",C408="",E408=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E408)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H408&lt;&gt;0,F408=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G408&lt;&gt;0,F408=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F408&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F408)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C408)*($E$5:$E$504=E408)*(($D$5:$D$504=D408)*(D408&lt;&gt;"")+($B$5:$B$504=B408)*(B408&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C408="Оплата",K408&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E408)&gt;0,ROUND(E408-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B408="",C408="",D408="",E408="",F408=""),"",IF(OR(B408="",C408="",E408=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E408)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H408&lt;&gt;0,F408=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G408&lt;&gt;0,F408=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F408&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F408)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C408)*($E$5:$E$504=E408)*(($D$5:$D$504=D408)*(D408&lt;&gt;"")+($B$5:$B$504=B408)*(B408&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C408="Оплата",K408&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E408)&gt;0,ROUND(E408-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J408" s="5">
@@ -11623,7 +11623,7 @@
         <v/>
       </c>
       <c r="I409" s="6">
-        <f>IF(AND(B409="",C409="",D409="",E409="",F409=""),"",IF(OR(B409="",C409="",E409=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E409)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H409&lt;&gt;0,F409=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G409&lt;&gt;0,F409=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F409&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F409)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C409)*($E$5:$E$504=E409)*(($D$5:$D$504=D409)*(D409&lt;&gt;"")+($B$5:$B$504=B409)*(B409&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C409="Оплата",K409&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E409)&gt;0,ROUND(E409-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B409="",C409="",D409="",E409="",F409=""),"",IF(OR(B409="",C409="",E409=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E409)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H409&lt;&gt;0,F409=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G409&lt;&gt;0,F409=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F409&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F409)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C409)*($E$5:$E$504=E409)*(($D$5:$D$504=D409)*(D409&lt;&gt;"")+($B$5:$B$504=B409)*(B409&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C409="Оплата",K409&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E409)&gt;0,ROUND(E409-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J409" s="5">
@@ -11650,7 +11650,7 @@
         <v/>
       </c>
       <c r="I410" s="6">
-        <f>IF(AND(B410="",C410="",D410="",E410="",F410=""),"",IF(OR(B410="",C410="",E410=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E410)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H410&lt;&gt;0,F410=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G410&lt;&gt;0,F410=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F410&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F410)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C410)*($E$5:$E$504=E410)*(($D$5:$D$504=D410)*(D410&lt;&gt;"")+($B$5:$B$504=B410)*(B410&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C410="Оплата",K410&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E410)&gt;0,ROUND(E410-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B410="",C410="",D410="",E410="",F410=""),"",IF(OR(B410="",C410="",E410=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E410)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H410&lt;&gt;0,F410=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G410&lt;&gt;0,F410=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F410&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F410)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C410)*($E$5:$E$504=E410)*(($D$5:$D$504=D410)*(D410&lt;&gt;"")+($B$5:$B$504=B410)*(B410&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C410="Оплата",K410&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E410)&gt;0,ROUND(E410-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J410" s="5">
@@ -11677,7 +11677,7 @@
         <v/>
       </c>
       <c r="I411" s="6">
-        <f>IF(AND(B411="",C411="",D411="",E411="",F411=""),"",IF(OR(B411="",C411="",E411=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E411)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H411&lt;&gt;0,F411=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G411&lt;&gt;0,F411=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F411&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F411)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C411)*($E$5:$E$504=E411)*(($D$5:$D$504=D411)*(D411&lt;&gt;"")+($B$5:$B$504=B411)*(B411&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C411="Оплата",K411&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E411)&gt;0,ROUND(E411-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B411="",C411="",D411="",E411="",F411=""),"",IF(OR(B411="",C411="",E411=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E411)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H411&lt;&gt;0,F411=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G411&lt;&gt;0,F411=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F411&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F411)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C411)*($E$5:$E$504=E411)*(($D$5:$D$504=D411)*(D411&lt;&gt;"")+($B$5:$B$504=B411)*(B411&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C411="Оплата",K411&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E411)&gt;0,ROUND(E411-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J411" s="5">
@@ -11704,7 +11704,7 @@
         <v/>
       </c>
       <c r="I412" s="6">
-        <f>IF(AND(B412="",C412="",D412="",E412="",F412=""),"",IF(OR(B412="",C412="",E412=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E412)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H412&lt;&gt;0,F412=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G412&lt;&gt;0,F412=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F412&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F412)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C412)*($E$5:$E$504=E412)*(($D$5:$D$504=D412)*(D412&lt;&gt;"")+($B$5:$B$504=B412)*(B412&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C412="Оплата",K412&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E412)&gt;0,ROUND(E412-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B412="",C412="",D412="",E412="",F412=""),"",IF(OR(B412="",C412="",E412=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E412)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H412&lt;&gt;0,F412=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G412&lt;&gt;0,F412=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F412&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F412)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C412)*($E$5:$E$504=E412)*(($D$5:$D$504=D412)*(D412&lt;&gt;"")+($B$5:$B$504=B412)*(B412&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C412="Оплата",K412&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E412)&gt;0,ROUND(E412-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J412" s="5">
@@ -11731,7 +11731,7 @@
         <v/>
       </c>
       <c r="I413" s="6">
-        <f>IF(AND(B413="",C413="",D413="",E413="",F413=""),"",IF(OR(B413="",C413="",E413=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E413)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H413&lt;&gt;0,F413=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G413&lt;&gt;0,F413=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F413&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F413)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C413)*($E$5:$E$504=E413)*(($D$5:$D$504=D413)*(D413&lt;&gt;"")+($B$5:$B$504=B413)*(B413&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C413="Оплата",K413&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E413)&gt;0,ROUND(E413-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B413="",C413="",D413="",E413="",F413=""),"",IF(OR(B413="",C413="",E413=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E413)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H413&lt;&gt;0,F413=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G413&lt;&gt;0,F413=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F413&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F413)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C413)*($E$5:$E$504=E413)*(($D$5:$D$504=D413)*(D413&lt;&gt;"")+($B$5:$B$504=B413)*(B413&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C413="Оплата",K413&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E413)&gt;0,ROUND(E413-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J413" s="5">
@@ -11758,7 +11758,7 @@
         <v/>
       </c>
       <c r="I414" s="6">
-        <f>IF(AND(B414="",C414="",D414="",E414="",F414=""),"",IF(OR(B414="",C414="",E414=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E414)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H414&lt;&gt;0,F414=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G414&lt;&gt;0,F414=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F414&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F414)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C414)*($E$5:$E$504=E414)*(($D$5:$D$504=D414)*(D414&lt;&gt;"")+($B$5:$B$504=B414)*(B414&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C414="Оплата",K414&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E414)&gt;0,ROUND(E414-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B414="",C414="",D414="",E414="",F414=""),"",IF(OR(B414="",C414="",E414=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E414)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H414&lt;&gt;0,F414=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G414&lt;&gt;0,F414=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F414&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F414)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C414)*($E$5:$E$504=E414)*(($D$5:$D$504=D414)*(D414&lt;&gt;"")+($B$5:$B$504=B414)*(B414&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C414="Оплата",K414&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E414)&gt;0,ROUND(E414-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J414" s="5">
@@ -11785,7 +11785,7 @@
         <v/>
       </c>
       <c r="I415" s="6">
-        <f>IF(AND(B415="",C415="",D415="",E415="",F415=""),"",IF(OR(B415="",C415="",E415=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E415)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H415&lt;&gt;0,F415=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G415&lt;&gt;0,F415=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F415&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F415)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C415)*($E$5:$E$504=E415)*(($D$5:$D$504=D415)*(D415&lt;&gt;"")+($B$5:$B$504=B415)*(B415&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C415="Оплата",K415&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E415)&gt;0,ROUND(E415-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B415="",C415="",D415="",E415="",F415=""),"",IF(OR(B415="",C415="",E415=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E415)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H415&lt;&gt;0,F415=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G415&lt;&gt;0,F415=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F415&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F415)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C415)*($E$5:$E$504=E415)*(($D$5:$D$504=D415)*(D415&lt;&gt;"")+($B$5:$B$504=B415)*(B415&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C415="Оплата",K415&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E415)&gt;0,ROUND(E415-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J415" s="5">
@@ -11812,7 +11812,7 @@
         <v/>
       </c>
       <c r="I416" s="6">
-        <f>IF(AND(B416="",C416="",D416="",E416="",F416=""),"",IF(OR(B416="",C416="",E416=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E416)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H416&lt;&gt;0,F416=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G416&lt;&gt;0,F416=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F416&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F416)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C416)*($E$5:$E$504=E416)*(($D$5:$D$504=D416)*(D416&lt;&gt;"")+($B$5:$B$504=B416)*(B416&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C416="Оплата",K416&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E416)&gt;0,ROUND(E416-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B416="",C416="",D416="",E416="",F416=""),"",IF(OR(B416="",C416="",E416=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E416)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H416&lt;&gt;0,F416=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G416&lt;&gt;0,F416=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F416&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F416)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C416)*($E$5:$E$504=E416)*(($D$5:$D$504=D416)*(D416&lt;&gt;"")+($B$5:$B$504=B416)*(B416&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C416="Оплата",K416&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E416)&gt;0,ROUND(E416-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J416" s="5">
@@ -11839,7 +11839,7 @@
         <v/>
       </c>
       <c r="I417" s="6">
-        <f>IF(AND(B417="",C417="",D417="",E417="",F417=""),"",IF(OR(B417="",C417="",E417=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E417)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H417&lt;&gt;0,F417=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G417&lt;&gt;0,F417=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F417&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F417)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C417)*($E$5:$E$504=E417)*(($D$5:$D$504=D417)*(D417&lt;&gt;"")+($B$5:$B$504=B417)*(B417&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C417="Оплата",K417&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E417)&gt;0,ROUND(E417-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B417="",C417="",D417="",E417="",F417=""),"",IF(OR(B417="",C417="",E417=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E417)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H417&lt;&gt;0,F417=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G417&lt;&gt;0,F417=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F417&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F417)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C417)*($E$5:$E$504=E417)*(($D$5:$D$504=D417)*(D417&lt;&gt;"")+($B$5:$B$504=B417)*(B417&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C417="Оплата",K417&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E417)&gt;0,ROUND(E417-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J417" s="5">
@@ -11866,7 +11866,7 @@
         <v/>
       </c>
       <c r="I418" s="6">
-        <f>IF(AND(B418="",C418="",D418="",E418="",F418=""),"",IF(OR(B418="",C418="",E418=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E418)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H418&lt;&gt;0,F418=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G418&lt;&gt;0,F418=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F418&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F418)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C418)*($E$5:$E$504=E418)*(($D$5:$D$504=D418)*(D418&lt;&gt;"")+($B$5:$B$504=B418)*(B418&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C418="Оплата",K418&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E418)&gt;0,ROUND(E418-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B418="",C418="",D418="",E418="",F418=""),"",IF(OR(B418="",C418="",E418=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E418)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H418&lt;&gt;0,F418=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G418&lt;&gt;0,F418=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F418&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F418)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C418)*($E$5:$E$504=E418)*(($D$5:$D$504=D418)*(D418&lt;&gt;"")+($B$5:$B$504=B418)*(B418&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C418="Оплата",K418&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E418)&gt;0,ROUND(E418-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J418" s="5">
@@ -11893,7 +11893,7 @@
         <v/>
       </c>
       <c r="I419" s="6">
-        <f>IF(AND(B419="",C419="",D419="",E419="",F419=""),"",IF(OR(B419="",C419="",E419=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E419)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H419&lt;&gt;0,F419=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G419&lt;&gt;0,F419=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F419&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F419)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C419)*($E$5:$E$504=E419)*(($D$5:$D$504=D419)*(D419&lt;&gt;"")+($B$5:$B$504=B419)*(B419&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C419="Оплата",K419&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E419)&gt;0,ROUND(E419-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B419="",C419="",D419="",E419="",F419=""),"",IF(OR(B419="",C419="",E419=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E419)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H419&lt;&gt;0,F419=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G419&lt;&gt;0,F419=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F419&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F419)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C419)*($E$5:$E$504=E419)*(($D$5:$D$504=D419)*(D419&lt;&gt;"")+($B$5:$B$504=B419)*(B419&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C419="Оплата",K419&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E419)&gt;0,ROUND(E419-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J419" s="5">
@@ -11920,7 +11920,7 @@
         <v/>
       </c>
       <c r="I420" s="6">
-        <f>IF(AND(B420="",C420="",D420="",E420="",F420=""),"",IF(OR(B420="",C420="",E420=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E420)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H420&lt;&gt;0,F420=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G420&lt;&gt;0,F420=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F420&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F420)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C420)*($E$5:$E$504=E420)*(($D$5:$D$504=D420)*(D420&lt;&gt;"")+($B$5:$B$504=B420)*(B420&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C420="Оплата",K420&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E420)&gt;0,ROUND(E420-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B420="",C420="",D420="",E420="",F420=""),"",IF(OR(B420="",C420="",E420=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E420)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H420&lt;&gt;0,F420=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G420&lt;&gt;0,F420=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F420&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F420)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C420)*($E$5:$E$504=E420)*(($D$5:$D$504=D420)*(D420&lt;&gt;"")+($B$5:$B$504=B420)*(B420&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C420="Оплата",K420&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E420)&gt;0,ROUND(E420-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J420" s="5">
@@ -11947,7 +11947,7 @@
         <v/>
       </c>
       <c r="I421" s="6">
-        <f>IF(AND(B421="",C421="",D421="",E421="",F421=""),"",IF(OR(B421="",C421="",E421=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E421)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H421&lt;&gt;0,F421=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G421&lt;&gt;0,F421=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F421&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F421)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C421)*($E$5:$E$504=E421)*(($D$5:$D$504=D421)*(D421&lt;&gt;"")+($B$5:$B$504=B421)*(B421&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C421="Оплата",K421&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E421)&gt;0,ROUND(E421-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B421="",C421="",D421="",E421="",F421=""),"",IF(OR(B421="",C421="",E421=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E421)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H421&lt;&gt;0,F421=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G421&lt;&gt;0,F421=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F421&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F421)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C421)*($E$5:$E$504=E421)*(($D$5:$D$504=D421)*(D421&lt;&gt;"")+($B$5:$B$504=B421)*(B421&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C421="Оплата",K421&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E421)&gt;0,ROUND(E421-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J421" s="5">
@@ -11974,7 +11974,7 @@
         <v/>
       </c>
       <c r="I422" s="6">
-        <f>IF(AND(B422="",C422="",D422="",E422="",F422=""),"",IF(OR(B422="",C422="",E422=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E422)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H422&lt;&gt;0,F422=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G422&lt;&gt;0,F422=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F422&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F422)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C422)*($E$5:$E$504=E422)*(($D$5:$D$504=D422)*(D422&lt;&gt;"")+($B$5:$B$504=B422)*(B422&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C422="Оплата",K422&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E422)&gt;0,ROUND(E422-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B422="",C422="",D422="",E422="",F422=""),"",IF(OR(B422="",C422="",E422=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E422)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H422&lt;&gt;0,F422=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G422&lt;&gt;0,F422=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F422&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F422)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C422)*($E$5:$E$504=E422)*(($D$5:$D$504=D422)*(D422&lt;&gt;"")+($B$5:$B$504=B422)*(B422&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C422="Оплата",K422&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E422)&gt;0,ROUND(E422-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J422" s="5">
@@ -12001,7 +12001,7 @@
         <v/>
       </c>
       <c r="I423" s="6">
-        <f>IF(AND(B423="",C423="",D423="",E423="",F423=""),"",IF(OR(B423="",C423="",E423=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E423)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H423&lt;&gt;0,F423=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G423&lt;&gt;0,F423=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F423&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F423)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C423)*($E$5:$E$504=E423)*(($D$5:$D$504=D423)*(D423&lt;&gt;"")+($B$5:$B$504=B423)*(B423&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C423="Оплата",K423&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E423)&gt;0,ROUND(E423-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B423="",C423="",D423="",E423="",F423=""),"",IF(OR(B423="",C423="",E423=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E423)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H423&lt;&gt;0,F423=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G423&lt;&gt;0,F423=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F423&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F423)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C423)*($E$5:$E$504=E423)*(($D$5:$D$504=D423)*(D423&lt;&gt;"")+($B$5:$B$504=B423)*(B423&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C423="Оплата",K423&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E423)&gt;0,ROUND(E423-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J423" s="5">
@@ -12028,7 +12028,7 @@
         <v/>
       </c>
       <c r="I424" s="6">
-        <f>IF(AND(B424="",C424="",D424="",E424="",F424=""),"",IF(OR(B424="",C424="",E424=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E424)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H424&lt;&gt;0,F424=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G424&lt;&gt;0,F424=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F424&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F424)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C424)*($E$5:$E$504=E424)*(($D$5:$D$504=D424)*(D424&lt;&gt;"")+($B$5:$B$504=B424)*(B424&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C424="Оплата",K424&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E424)&gt;0,ROUND(E424-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B424="",C424="",D424="",E424="",F424=""),"",IF(OR(B424="",C424="",E424=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E424)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H424&lt;&gt;0,F424=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G424&lt;&gt;0,F424=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F424&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F424)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C424)*($E$5:$E$504=E424)*(($D$5:$D$504=D424)*(D424&lt;&gt;"")+($B$5:$B$504=B424)*(B424&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C424="Оплата",K424&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E424)&gt;0,ROUND(E424-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J424" s="5">
@@ -12055,7 +12055,7 @@
         <v/>
       </c>
       <c r="I425" s="6">
-        <f>IF(AND(B425="",C425="",D425="",E425="",F425=""),"",IF(OR(B425="",C425="",E425=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E425)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H425&lt;&gt;0,F425=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G425&lt;&gt;0,F425=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F425&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F425)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C425)*($E$5:$E$504=E425)*(($D$5:$D$504=D425)*(D425&lt;&gt;"")+($B$5:$B$504=B425)*(B425&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C425="Оплата",K425&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E425)&gt;0,ROUND(E425-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B425="",C425="",D425="",E425="",F425=""),"",IF(OR(B425="",C425="",E425=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E425)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H425&lt;&gt;0,F425=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G425&lt;&gt;0,F425=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F425&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F425)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C425)*($E$5:$E$504=E425)*(($D$5:$D$504=D425)*(D425&lt;&gt;"")+($B$5:$B$504=B425)*(B425&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C425="Оплата",K425&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E425)&gt;0,ROUND(E425-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J425" s="5">
@@ -12082,7 +12082,7 @@
         <v/>
       </c>
       <c r="I426" s="6">
-        <f>IF(AND(B426="",C426="",D426="",E426="",F426=""),"",IF(OR(B426="",C426="",E426=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E426)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H426&lt;&gt;0,F426=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G426&lt;&gt;0,F426=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F426&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F426)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C426)*($E$5:$E$504=E426)*(($D$5:$D$504=D426)*(D426&lt;&gt;"")+($B$5:$B$504=B426)*(B426&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C426="Оплата",K426&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E426)&gt;0,ROUND(E426-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B426="",C426="",D426="",E426="",F426=""),"",IF(OR(B426="",C426="",E426=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E426)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H426&lt;&gt;0,F426=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G426&lt;&gt;0,F426=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F426&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F426)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C426)*($E$5:$E$504=E426)*(($D$5:$D$504=D426)*(D426&lt;&gt;"")+($B$5:$B$504=B426)*(B426&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C426="Оплата",K426&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E426)&gt;0,ROUND(E426-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J426" s="5">
@@ -12109,7 +12109,7 @@
         <v/>
       </c>
       <c r="I427" s="6">
-        <f>IF(AND(B427="",C427="",D427="",E427="",F427=""),"",IF(OR(B427="",C427="",E427=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E427)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H427&lt;&gt;0,F427=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G427&lt;&gt;0,F427=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F427&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F427)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C427)*($E$5:$E$504=E427)*(($D$5:$D$504=D427)*(D427&lt;&gt;"")+($B$5:$B$504=B427)*(B427&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C427="Оплата",K427&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E427)&gt;0,ROUND(E427-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B427="",C427="",D427="",E427="",F427=""),"",IF(OR(B427="",C427="",E427=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E427)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H427&lt;&gt;0,F427=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G427&lt;&gt;0,F427=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F427&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F427)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C427)*($E$5:$E$504=E427)*(($D$5:$D$504=D427)*(D427&lt;&gt;"")+($B$5:$B$504=B427)*(B427&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C427="Оплата",K427&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E427)&gt;0,ROUND(E427-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J427" s="5">
@@ -12136,7 +12136,7 @@
         <v/>
       </c>
       <c r="I428" s="6">
-        <f>IF(AND(B428="",C428="",D428="",E428="",F428=""),"",IF(OR(B428="",C428="",E428=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E428)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H428&lt;&gt;0,F428=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G428&lt;&gt;0,F428=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F428&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F428)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C428)*($E$5:$E$504=E428)*(($D$5:$D$504=D428)*(D428&lt;&gt;"")+($B$5:$B$504=B428)*(B428&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C428="Оплата",K428&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E428)&gt;0,ROUND(E428-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B428="",C428="",D428="",E428="",F428=""),"",IF(OR(B428="",C428="",E428=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E428)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H428&lt;&gt;0,F428=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G428&lt;&gt;0,F428=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F428&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F428)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C428)*($E$5:$E$504=E428)*(($D$5:$D$504=D428)*(D428&lt;&gt;"")+($B$5:$B$504=B428)*(B428&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C428="Оплата",K428&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E428)&gt;0,ROUND(E428-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J428" s="5">
@@ -12163,7 +12163,7 @@
         <v/>
       </c>
       <c r="I429" s="6">
-        <f>IF(AND(B429="",C429="",D429="",E429="",F429=""),"",IF(OR(B429="",C429="",E429=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E429)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H429&lt;&gt;0,F429=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G429&lt;&gt;0,F429=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F429&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F429)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C429)*($E$5:$E$504=E429)*(($D$5:$D$504=D429)*(D429&lt;&gt;"")+($B$5:$B$504=B429)*(B429&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C429="Оплата",K429&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E429)&gt;0,ROUND(E429-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B429="",C429="",D429="",E429="",F429=""),"",IF(OR(B429="",C429="",E429=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E429)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H429&lt;&gt;0,F429=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G429&lt;&gt;0,F429=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F429&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F429)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C429)*($E$5:$E$504=E429)*(($D$5:$D$504=D429)*(D429&lt;&gt;"")+($B$5:$B$504=B429)*(B429&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C429="Оплата",K429&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E429)&gt;0,ROUND(E429-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J429" s="5">
@@ -12190,7 +12190,7 @@
         <v/>
       </c>
       <c r="I430" s="6">
-        <f>IF(AND(B430="",C430="",D430="",E430="",F430=""),"",IF(OR(B430="",C430="",E430=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E430)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H430&lt;&gt;0,F430=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G430&lt;&gt;0,F430=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F430&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F430)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C430)*($E$5:$E$504=E430)*(($D$5:$D$504=D430)*(D430&lt;&gt;"")+($B$5:$B$504=B430)*(B430&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C430="Оплата",K430&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E430)&gt;0,ROUND(E430-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B430="",C430="",D430="",E430="",F430=""),"",IF(OR(B430="",C430="",E430=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E430)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H430&lt;&gt;0,F430=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G430&lt;&gt;0,F430=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F430&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F430)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C430)*($E$5:$E$504=E430)*(($D$5:$D$504=D430)*(D430&lt;&gt;"")+($B$5:$B$504=B430)*(B430&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C430="Оплата",K430&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E430)&gt;0,ROUND(E430-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J430" s="5">
@@ -12217,7 +12217,7 @@
         <v/>
       </c>
       <c r="I431" s="6">
-        <f>IF(AND(B431="",C431="",D431="",E431="",F431=""),"",IF(OR(B431="",C431="",E431=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E431)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H431&lt;&gt;0,F431=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G431&lt;&gt;0,F431=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F431&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F431)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C431)*($E$5:$E$504=E431)*(($D$5:$D$504=D431)*(D431&lt;&gt;"")+($B$5:$B$504=B431)*(B431&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C431="Оплата",K431&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E431)&gt;0,ROUND(E431-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B431="",C431="",D431="",E431="",F431=""),"",IF(OR(B431="",C431="",E431=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E431)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H431&lt;&gt;0,F431=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G431&lt;&gt;0,F431=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F431&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F431)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C431)*($E$5:$E$504=E431)*(($D$5:$D$504=D431)*(D431&lt;&gt;"")+($B$5:$B$504=B431)*(B431&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C431="Оплата",K431&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E431)&gt;0,ROUND(E431-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J431" s="5">
@@ -12244,7 +12244,7 @@
         <v/>
       </c>
       <c r="I432" s="6">
-        <f>IF(AND(B432="",C432="",D432="",E432="",F432=""),"",IF(OR(B432="",C432="",E432=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E432)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H432&lt;&gt;0,F432=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G432&lt;&gt;0,F432=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F432&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F432)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C432)*($E$5:$E$504=E432)*(($D$5:$D$504=D432)*(D432&lt;&gt;"")+($B$5:$B$504=B432)*(B432&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C432="Оплата",K432&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E432)&gt;0,ROUND(E432-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B432="",C432="",D432="",E432="",F432=""),"",IF(OR(B432="",C432="",E432=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E432)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H432&lt;&gt;0,F432=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G432&lt;&gt;0,F432=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F432&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F432)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C432)*($E$5:$E$504=E432)*(($D$5:$D$504=D432)*(D432&lt;&gt;"")+($B$5:$B$504=B432)*(B432&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C432="Оплата",K432&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E432)&gt;0,ROUND(E432-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J432" s="5">
@@ -12271,7 +12271,7 @@
         <v/>
       </c>
       <c r="I433" s="6">
-        <f>IF(AND(B433="",C433="",D433="",E433="",F433=""),"",IF(OR(B433="",C433="",E433=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E433)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H433&lt;&gt;0,F433=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G433&lt;&gt;0,F433=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F433&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F433)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C433)*($E$5:$E$504=E433)*(($D$5:$D$504=D433)*(D433&lt;&gt;"")+($B$5:$B$504=B433)*(B433&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C433="Оплата",K433&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E433)&gt;0,ROUND(E433-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B433="",C433="",D433="",E433="",F433=""),"",IF(OR(B433="",C433="",E433=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E433)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H433&lt;&gt;0,F433=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G433&lt;&gt;0,F433=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F433&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F433)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C433)*($E$5:$E$504=E433)*(($D$5:$D$504=D433)*(D433&lt;&gt;"")+($B$5:$B$504=B433)*(B433&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C433="Оплата",K433&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E433)&gt;0,ROUND(E433-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J433" s="5">
@@ -12298,7 +12298,7 @@
         <v/>
       </c>
       <c r="I434" s="6">
-        <f>IF(AND(B434="",C434="",D434="",E434="",F434=""),"",IF(OR(B434="",C434="",E434=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E434)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H434&lt;&gt;0,F434=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G434&lt;&gt;0,F434=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F434&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F434)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C434)*($E$5:$E$504=E434)*(($D$5:$D$504=D434)*(D434&lt;&gt;"")+($B$5:$B$504=B434)*(B434&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C434="Оплата",K434&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E434)&gt;0,ROUND(E434-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B434="",C434="",D434="",E434="",F434=""),"",IF(OR(B434="",C434="",E434=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E434)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H434&lt;&gt;0,F434=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G434&lt;&gt;0,F434=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F434&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F434)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C434)*($E$5:$E$504=E434)*(($D$5:$D$504=D434)*(D434&lt;&gt;"")+($B$5:$B$504=B434)*(B434&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C434="Оплата",K434&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E434)&gt;0,ROUND(E434-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J434" s="5">
@@ -12325,7 +12325,7 @@
         <v/>
       </c>
       <c r="I435" s="6">
-        <f>IF(AND(B435="",C435="",D435="",E435="",F435=""),"",IF(OR(B435="",C435="",E435=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E435)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H435&lt;&gt;0,F435=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G435&lt;&gt;0,F435=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F435&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F435)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C435)*($E$5:$E$504=E435)*(($D$5:$D$504=D435)*(D435&lt;&gt;"")+($B$5:$B$504=B435)*(B435&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C435="Оплата",K435&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E435)&gt;0,ROUND(E435-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B435="",C435="",D435="",E435="",F435=""),"",IF(OR(B435="",C435="",E435=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E435)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H435&lt;&gt;0,F435=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G435&lt;&gt;0,F435=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F435&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F435)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C435)*($E$5:$E$504=E435)*(($D$5:$D$504=D435)*(D435&lt;&gt;"")+($B$5:$B$504=B435)*(B435&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C435="Оплата",K435&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E435)&gt;0,ROUND(E435-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J435" s="5">
@@ -12352,7 +12352,7 @@
         <v/>
       </c>
       <c r="I436" s="6">
-        <f>IF(AND(B436="",C436="",D436="",E436="",F436=""),"",IF(OR(B436="",C436="",E436=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E436)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H436&lt;&gt;0,F436=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G436&lt;&gt;0,F436=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F436&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F436)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C436)*($E$5:$E$504=E436)*(($D$5:$D$504=D436)*(D436&lt;&gt;"")+($B$5:$B$504=B436)*(B436&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C436="Оплата",K436&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E436)&gt;0,ROUND(E436-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B436="",C436="",D436="",E436="",F436=""),"",IF(OR(B436="",C436="",E436=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E436)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H436&lt;&gt;0,F436=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G436&lt;&gt;0,F436=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F436&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F436)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C436)*($E$5:$E$504=E436)*(($D$5:$D$504=D436)*(D436&lt;&gt;"")+($B$5:$B$504=B436)*(B436&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C436="Оплата",K436&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E436)&gt;0,ROUND(E436-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J436" s="5">
@@ -12379,7 +12379,7 @@
         <v/>
       </c>
       <c r="I437" s="6">
-        <f>IF(AND(B437="",C437="",D437="",E437="",F437=""),"",IF(OR(B437="",C437="",E437=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E437)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H437&lt;&gt;0,F437=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G437&lt;&gt;0,F437=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F437&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F437)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C437)*($E$5:$E$504=E437)*(($D$5:$D$504=D437)*(D437&lt;&gt;"")+($B$5:$B$504=B437)*(B437&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C437="Оплата",K437&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E437)&gt;0,ROUND(E437-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B437="",C437="",D437="",E437="",F437=""),"",IF(OR(B437="",C437="",E437=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E437)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H437&lt;&gt;0,F437=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G437&lt;&gt;0,F437=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F437&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F437)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C437)*($E$5:$E$504=E437)*(($D$5:$D$504=D437)*(D437&lt;&gt;"")+($B$5:$B$504=B437)*(B437&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C437="Оплата",K437&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E437)&gt;0,ROUND(E437-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J437" s="5">
@@ -12406,7 +12406,7 @@
         <v/>
       </c>
       <c r="I438" s="6">
-        <f>IF(AND(B438="",C438="",D438="",E438="",F438=""),"",IF(OR(B438="",C438="",E438=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E438)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H438&lt;&gt;0,F438=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G438&lt;&gt;0,F438=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F438&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F438)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C438)*($E$5:$E$504=E438)*(($D$5:$D$504=D438)*(D438&lt;&gt;"")+($B$5:$B$504=B438)*(B438&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C438="Оплата",K438&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E438)&gt;0,ROUND(E438-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B438="",C438="",D438="",E438="",F438=""),"",IF(OR(B438="",C438="",E438=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E438)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H438&lt;&gt;0,F438=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G438&lt;&gt;0,F438=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F438&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F438)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C438)*($E$5:$E$504=E438)*(($D$5:$D$504=D438)*(D438&lt;&gt;"")+($B$5:$B$504=B438)*(B438&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C438="Оплата",K438&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E438)&gt;0,ROUND(E438-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J438" s="5">
@@ -12433,7 +12433,7 @@
         <v/>
       </c>
       <c r="I439" s="6">
-        <f>IF(AND(B439="",C439="",D439="",E439="",F439=""),"",IF(OR(B439="",C439="",E439=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E439)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H439&lt;&gt;0,F439=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G439&lt;&gt;0,F439=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F439&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F439)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C439)*($E$5:$E$504=E439)*(($D$5:$D$504=D439)*(D439&lt;&gt;"")+($B$5:$B$504=B439)*(B439&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C439="Оплата",K439&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E439)&gt;0,ROUND(E439-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B439="",C439="",D439="",E439="",F439=""),"",IF(OR(B439="",C439="",E439=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E439)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H439&lt;&gt;0,F439=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G439&lt;&gt;0,F439=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F439&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F439)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C439)*($E$5:$E$504=E439)*(($D$5:$D$504=D439)*(D439&lt;&gt;"")+($B$5:$B$504=B439)*(B439&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C439="Оплата",K439&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E439)&gt;0,ROUND(E439-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J439" s="5">
@@ -12460,7 +12460,7 @@
         <v/>
       </c>
       <c r="I440" s="6">
-        <f>IF(AND(B440="",C440="",D440="",E440="",F440=""),"",IF(OR(B440="",C440="",E440=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E440)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H440&lt;&gt;0,F440=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G440&lt;&gt;0,F440=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F440&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F440)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C440)*($E$5:$E$504=E440)*(($D$5:$D$504=D440)*(D440&lt;&gt;"")+($B$5:$B$504=B440)*(B440&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C440="Оплата",K440&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E440)&gt;0,ROUND(E440-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B440="",C440="",D440="",E440="",F440=""),"",IF(OR(B440="",C440="",E440=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E440)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H440&lt;&gt;0,F440=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G440&lt;&gt;0,F440=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F440&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F440)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C440)*($E$5:$E$504=E440)*(($D$5:$D$504=D440)*(D440&lt;&gt;"")+($B$5:$B$504=B440)*(B440&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C440="Оплата",K440&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E440)&gt;0,ROUND(E440-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J440" s="5">
@@ -12487,7 +12487,7 @@
         <v/>
       </c>
       <c r="I441" s="6">
-        <f>IF(AND(B441="",C441="",D441="",E441="",F441=""),"",IF(OR(B441="",C441="",E441=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E441)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H441&lt;&gt;0,F441=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G441&lt;&gt;0,F441=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F441&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F441)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C441)*($E$5:$E$504=E441)*(($D$5:$D$504=D441)*(D441&lt;&gt;"")+($B$5:$B$504=B441)*(B441&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C441="Оплата",K441&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E441)&gt;0,ROUND(E441-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B441="",C441="",D441="",E441="",F441=""),"",IF(OR(B441="",C441="",E441=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E441)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H441&lt;&gt;0,F441=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G441&lt;&gt;0,F441=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F441&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F441)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C441)*($E$5:$E$504=E441)*(($D$5:$D$504=D441)*(D441&lt;&gt;"")+($B$5:$B$504=B441)*(B441&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C441="Оплата",K441&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E441)&gt;0,ROUND(E441-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J441" s="5">
@@ -12514,7 +12514,7 @@
         <v/>
       </c>
       <c r="I442" s="6">
-        <f>IF(AND(B442="",C442="",D442="",E442="",F442=""),"",IF(OR(B442="",C442="",E442=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E442)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H442&lt;&gt;0,F442=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G442&lt;&gt;0,F442=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F442&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F442)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C442)*($E$5:$E$504=E442)*(($D$5:$D$504=D442)*(D442&lt;&gt;"")+($B$5:$B$504=B442)*(B442&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C442="Оплата",K442&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E442)&gt;0,ROUND(E442-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B442="",C442="",D442="",E442="",F442=""),"",IF(OR(B442="",C442="",E442=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E442)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H442&lt;&gt;0,F442=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G442&lt;&gt;0,F442=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F442&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F442)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C442)*($E$5:$E$504=E442)*(($D$5:$D$504=D442)*(D442&lt;&gt;"")+($B$5:$B$504=B442)*(B442&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C442="Оплата",K442&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E442)&gt;0,ROUND(E442-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J442" s="5">
@@ -12541,7 +12541,7 @@
         <v/>
       </c>
       <c r="I443" s="6">
-        <f>IF(AND(B443="",C443="",D443="",E443="",F443=""),"",IF(OR(B443="",C443="",E443=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E443)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H443&lt;&gt;0,F443=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G443&lt;&gt;0,F443=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F443&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F443)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C443)*($E$5:$E$504=E443)*(($D$5:$D$504=D443)*(D443&lt;&gt;"")+($B$5:$B$504=B443)*(B443&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C443="Оплата",K443&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E443)&gt;0,ROUND(E443-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B443="",C443="",D443="",E443="",F443=""),"",IF(OR(B443="",C443="",E443=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E443)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H443&lt;&gt;0,F443=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G443&lt;&gt;0,F443=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F443&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F443)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C443)*($E$5:$E$504=E443)*(($D$5:$D$504=D443)*(D443&lt;&gt;"")+($B$5:$B$504=B443)*(B443&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C443="Оплата",K443&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E443)&gt;0,ROUND(E443-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J443" s="5">
@@ -12568,7 +12568,7 @@
         <v/>
       </c>
       <c r="I444" s="6">
-        <f>IF(AND(B444="",C444="",D444="",E444="",F444=""),"",IF(OR(B444="",C444="",E444=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E444)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H444&lt;&gt;0,F444=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G444&lt;&gt;0,F444=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F444&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F444)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C444)*($E$5:$E$504=E444)*(($D$5:$D$504=D444)*(D444&lt;&gt;"")+($B$5:$B$504=B444)*(B444&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C444="Оплата",K444&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E444)&gt;0,ROUND(E444-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B444="",C444="",D444="",E444="",F444=""),"",IF(OR(B444="",C444="",E444=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E444)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H444&lt;&gt;0,F444=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G444&lt;&gt;0,F444=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F444&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F444)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C444)*($E$5:$E$504=E444)*(($D$5:$D$504=D444)*(D444&lt;&gt;"")+($B$5:$B$504=B444)*(B444&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C444="Оплата",K444&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E444)&gt;0,ROUND(E444-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J444" s="5">
@@ -12595,7 +12595,7 @@
         <v/>
       </c>
       <c r="I445" s="6">
-        <f>IF(AND(B445="",C445="",D445="",E445="",F445=""),"",IF(OR(B445="",C445="",E445=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E445)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H445&lt;&gt;0,F445=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G445&lt;&gt;0,F445=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F445&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F445)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C445)*($E$5:$E$504=E445)*(($D$5:$D$504=D445)*(D445&lt;&gt;"")+($B$5:$B$504=B445)*(B445&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C445="Оплата",K445&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E445)&gt;0,ROUND(E445-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B445="",C445="",D445="",E445="",F445=""),"",IF(OR(B445="",C445="",E445=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E445)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H445&lt;&gt;0,F445=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G445&lt;&gt;0,F445=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F445&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F445)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C445)*($E$5:$E$504=E445)*(($D$5:$D$504=D445)*(D445&lt;&gt;"")+($B$5:$B$504=B445)*(B445&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C445="Оплата",K445&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E445)&gt;0,ROUND(E445-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J445" s="5">
@@ -12622,7 +12622,7 @@
         <v/>
       </c>
       <c r="I446" s="6">
-        <f>IF(AND(B446="",C446="",D446="",E446="",F446=""),"",IF(OR(B446="",C446="",E446=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E446)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H446&lt;&gt;0,F446=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G446&lt;&gt;0,F446=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F446&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F446)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C446)*($E$5:$E$504=E446)*(($D$5:$D$504=D446)*(D446&lt;&gt;"")+($B$5:$B$504=B446)*(B446&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C446="Оплата",K446&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E446)&gt;0,ROUND(E446-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B446="",C446="",D446="",E446="",F446=""),"",IF(OR(B446="",C446="",E446=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E446)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H446&lt;&gt;0,F446=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G446&lt;&gt;0,F446=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F446&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F446)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C446)*($E$5:$E$504=E446)*(($D$5:$D$504=D446)*(D446&lt;&gt;"")+($B$5:$B$504=B446)*(B446&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C446="Оплата",K446&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E446)&gt;0,ROUND(E446-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J446" s="5">
@@ -12649,7 +12649,7 @@
         <v/>
       </c>
       <c r="I447" s="6">
-        <f>IF(AND(B447="",C447="",D447="",E447="",F447=""),"",IF(OR(B447="",C447="",E447=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E447)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H447&lt;&gt;0,F447=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G447&lt;&gt;0,F447=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F447&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F447)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C447)*($E$5:$E$504=E447)*(($D$5:$D$504=D447)*(D447&lt;&gt;"")+($B$5:$B$504=B447)*(B447&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C447="Оплата",K447&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E447)&gt;0,ROUND(E447-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B447="",C447="",D447="",E447="",F447=""),"",IF(OR(B447="",C447="",E447=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E447)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H447&lt;&gt;0,F447=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G447&lt;&gt;0,F447=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F447&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F447)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C447)*($E$5:$E$504=E447)*(($D$5:$D$504=D447)*(D447&lt;&gt;"")+($B$5:$B$504=B447)*(B447&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C447="Оплата",K447&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E447)&gt;0,ROUND(E447-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J447" s="5">
@@ -12676,7 +12676,7 @@
         <v/>
       </c>
       <c r="I448" s="6">
-        <f>IF(AND(B448="",C448="",D448="",E448="",F448=""),"",IF(OR(B448="",C448="",E448=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E448)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H448&lt;&gt;0,F448=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G448&lt;&gt;0,F448=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F448&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F448)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C448)*($E$5:$E$504=E448)*(($D$5:$D$504=D448)*(D448&lt;&gt;"")+($B$5:$B$504=B448)*(B448&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C448="Оплата",K448&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E448)&gt;0,ROUND(E448-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B448="",C448="",D448="",E448="",F448=""),"",IF(OR(B448="",C448="",E448=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E448)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H448&lt;&gt;0,F448=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G448&lt;&gt;0,F448=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F448&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F448)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C448)*($E$5:$E$504=E448)*(($D$5:$D$504=D448)*(D448&lt;&gt;"")+($B$5:$B$504=B448)*(B448&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C448="Оплата",K448&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E448)&gt;0,ROUND(E448-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J448" s="5">
@@ -12703,7 +12703,7 @@
         <v/>
       </c>
       <c r="I449" s="6">
-        <f>IF(AND(B449="",C449="",D449="",E449="",F449=""),"",IF(OR(B449="",C449="",E449=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E449)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H449&lt;&gt;0,F449=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G449&lt;&gt;0,F449=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F449&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F449)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C449)*($E$5:$E$504=E449)*(($D$5:$D$504=D449)*(D449&lt;&gt;"")+($B$5:$B$504=B449)*(B449&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C449="Оплата",K449&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E449)&gt;0,ROUND(E449-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B449="",C449="",D449="",E449="",F449=""),"",IF(OR(B449="",C449="",E449=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E449)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H449&lt;&gt;0,F449=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G449&lt;&gt;0,F449=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F449&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F449)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C449)*($E$5:$E$504=E449)*(($D$5:$D$504=D449)*(D449&lt;&gt;"")+($B$5:$B$504=B449)*(B449&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C449="Оплата",K449&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E449)&gt;0,ROUND(E449-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J449" s="5">
@@ -12730,7 +12730,7 @@
         <v/>
       </c>
       <c r="I450" s="6">
-        <f>IF(AND(B450="",C450="",D450="",E450="",F450=""),"",IF(OR(B450="",C450="",E450=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E450)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H450&lt;&gt;0,F450=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G450&lt;&gt;0,F450=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F450&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F450)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C450)*($E$5:$E$504=E450)*(($D$5:$D$504=D450)*(D450&lt;&gt;"")+($B$5:$B$504=B450)*(B450&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C450="Оплата",K450&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E450)&gt;0,ROUND(E450-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B450="",C450="",D450="",E450="",F450=""),"",IF(OR(B450="",C450="",E450=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E450)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H450&lt;&gt;0,F450=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G450&lt;&gt;0,F450=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F450&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F450)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C450)*($E$5:$E$504=E450)*(($D$5:$D$504=D450)*(D450&lt;&gt;"")+($B$5:$B$504=B450)*(B450&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C450="Оплата",K450&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E450)&gt;0,ROUND(E450-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J450" s="5">
@@ -12757,7 +12757,7 @@
         <v/>
       </c>
       <c r="I451" s="6">
-        <f>IF(AND(B451="",C451="",D451="",E451="",F451=""),"",IF(OR(B451="",C451="",E451=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E451)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H451&lt;&gt;0,F451=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G451&lt;&gt;0,F451=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F451&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F451)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C451)*($E$5:$E$504=E451)*(($D$5:$D$504=D451)*(D451&lt;&gt;"")+($B$5:$B$504=B451)*(B451&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C451="Оплата",K451&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E451)&gt;0,ROUND(E451-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B451="",C451="",D451="",E451="",F451=""),"",IF(OR(B451="",C451="",E451=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E451)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H451&lt;&gt;0,F451=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G451&lt;&gt;0,F451=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F451&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F451)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C451)*($E$5:$E$504=E451)*(($D$5:$D$504=D451)*(D451&lt;&gt;"")+($B$5:$B$504=B451)*(B451&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C451="Оплата",K451&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E451)&gt;0,ROUND(E451-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J451" s="5">
@@ -12784,7 +12784,7 @@
         <v/>
       </c>
       <c r="I452" s="6">
-        <f>IF(AND(B452="",C452="",D452="",E452="",F452=""),"",IF(OR(B452="",C452="",E452=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E452)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H452&lt;&gt;0,F452=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G452&lt;&gt;0,F452=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F452&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F452)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C452)*($E$5:$E$504=E452)*(($D$5:$D$504=D452)*(D452&lt;&gt;"")+($B$5:$B$504=B452)*(B452&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C452="Оплата",K452&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E452)&gt;0,ROUND(E452-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B452="",C452="",D452="",E452="",F452=""),"",IF(OR(B452="",C452="",E452=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E452)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H452&lt;&gt;0,F452=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G452&lt;&gt;0,F452=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F452&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F452)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C452)*($E$5:$E$504=E452)*(($D$5:$D$504=D452)*(D452&lt;&gt;"")+($B$5:$B$504=B452)*(B452&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C452="Оплата",K452&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E452)&gt;0,ROUND(E452-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J452" s="5">
@@ -12811,7 +12811,7 @@
         <v/>
       </c>
       <c r="I453" s="6">
-        <f>IF(AND(B453="",C453="",D453="",E453="",F453=""),"",IF(OR(B453="",C453="",E453=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E453)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H453&lt;&gt;0,F453=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G453&lt;&gt;0,F453=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F453&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F453)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C453)*($E$5:$E$504=E453)*(($D$5:$D$504=D453)*(D453&lt;&gt;"")+($B$5:$B$504=B453)*(B453&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C453="Оплата",K453&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E453)&gt;0,ROUND(E453-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B453="",C453="",D453="",E453="",F453=""),"",IF(OR(B453="",C453="",E453=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E453)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H453&lt;&gt;0,F453=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G453&lt;&gt;0,F453=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F453&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F453)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C453)*($E$5:$E$504=E453)*(($D$5:$D$504=D453)*(D453&lt;&gt;"")+($B$5:$B$504=B453)*(B453&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C453="Оплата",K453&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E453)&gt;0,ROUND(E453-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J453" s="5">
@@ -12838,7 +12838,7 @@
         <v/>
       </c>
       <c r="I454" s="6">
-        <f>IF(AND(B454="",C454="",D454="",E454="",F454=""),"",IF(OR(B454="",C454="",E454=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E454)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H454&lt;&gt;0,F454=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G454&lt;&gt;0,F454=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F454&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F454)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C454)*($E$5:$E$504=E454)*(($D$5:$D$504=D454)*(D454&lt;&gt;"")+($B$5:$B$504=B454)*(B454&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C454="Оплата",K454&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E454)&gt;0,ROUND(E454-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B454="",C454="",D454="",E454="",F454=""),"",IF(OR(B454="",C454="",E454=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E454)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H454&lt;&gt;0,F454=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G454&lt;&gt;0,F454=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F454&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F454)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C454)*($E$5:$E$504=E454)*(($D$5:$D$504=D454)*(D454&lt;&gt;"")+($B$5:$B$504=B454)*(B454&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C454="Оплата",K454&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E454)&gt;0,ROUND(E454-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J454" s="5">
@@ -12865,7 +12865,7 @@
         <v/>
       </c>
       <c r="I455" s="6">
-        <f>IF(AND(B455="",C455="",D455="",E455="",F455=""),"",IF(OR(B455="",C455="",E455=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E455)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H455&lt;&gt;0,F455=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G455&lt;&gt;0,F455=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F455&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F455)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C455)*($E$5:$E$504=E455)*(($D$5:$D$504=D455)*(D455&lt;&gt;"")+($B$5:$B$504=B455)*(B455&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C455="Оплата",K455&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E455)&gt;0,ROUND(E455-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B455="",C455="",D455="",E455="",F455=""),"",IF(OR(B455="",C455="",E455=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E455)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H455&lt;&gt;0,F455=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G455&lt;&gt;0,F455=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F455&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F455)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C455)*($E$5:$E$504=E455)*(($D$5:$D$504=D455)*(D455&lt;&gt;"")+($B$5:$B$504=B455)*(B455&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C455="Оплата",K455&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E455)&gt;0,ROUND(E455-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J455" s="5">
@@ -12892,7 +12892,7 @@
         <v/>
       </c>
       <c r="I456" s="6">
-        <f>IF(AND(B456="",C456="",D456="",E456="",F456=""),"",IF(OR(B456="",C456="",E456=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E456)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H456&lt;&gt;0,F456=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G456&lt;&gt;0,F456=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F456&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F456)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C456)*($E$5:$E$504=E456)*(($D$5:$D$504=D456)*(D456&lt;&gt;"")+($B$5:$B$504=B456)*(B456&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C456="Оплата",K456&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E456)&gt;0,ROUND(E456-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B456="",C456="",D456="",E456="",F456=""),"",IF(OR(B456="",C456="",E456=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E456)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H456&lt;&gt;0,F456=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G456&lt;&gt;0,F456=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F456&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F456)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C456)*($E$5:$E$504=E456)*(($D$5:$D$504=D456)*(D456&lt;&gt;"")+($B$5:$B$504=B456)*(B456&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C456="Оплата",K456&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E456)&gt;0,ROUND(E456-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J456" s="5">
@@ -12919,7 +12919,7 @@
         <v/>
       </c>
       <c r="I457" s="6">
-        <f>IF(AND(B457="",C457="",D457="",E457="",F457=""),"",IF(OR(B457="",C457="",E457=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E457)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H457&lt;&gt;0,F457=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G457&lt;&gt;0,F457=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F457&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F457)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C457)*($E$5:$E$504=E457)*(($D$5:$D$504=D457)*(D457&lt;&gt;"")+($B$5:$B$504=B457)*(B457&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C457="Оплата",K457&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E457)&gt;0,ROUND(E457-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B457="",C457="",D457="",E457="",F457=""),"",IF(OR(B457="",C457="",E457=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E457)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H457&lt;&gt;0,F457=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G457&lt;&gt;0,F457=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F457&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F457)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C457)*($E$5:$E$504=E457)*(($D$5:$D$504=D457)*(D457&lt;&gt;"")+($B$5:$B$504=B457)*(B457&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C457="Оплата",K457&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E457)&gt;0,ROUND(E457-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J457" s="5">
@@ -12946,7 +12946,7 @@
         <v/>
       </c>
       <c r="I458" s="6">
-        <f>IF(AND(B458="",C458="",D458="",E458="",F458=""),"",IF(OR(B458="",C458="",E458=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E458)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H458&lt;&gt;0,F458=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G458&lt;&gt;0,F458=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F458&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F458)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C458)*($E$5:$E$504=E458)*(($D$5:$D$504=D458)*(D458&lt;&gt;"")+($B$5:$B$504=B458)*(B458&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C458="Оплата",K458&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E458)&gt;0,ROUND(E458-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B458="",C458="",D458="",E458="",F458=""),"",IF(OR(B458="",C458="",E458=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E458)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H458&lt;&gt;0,F458=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G458&lt;&gt;0,F458=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F458&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F458)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C458)*($E$5:$E$504=E458)*(($D$5:$D$504=D458)*(D458&lt;&gt;"")+($B$5:$B$504=B458)*(B458&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C458="Оплата",K458&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E458)&gt;0,ROUND(E458-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J458" s="5">
@@ -12973,7 +12973,7 @@
         <v/>
       </c>
       <c r="I459" s="6">
-        <f>IF(AND(B459="",C459="",D459="",E459="",F459=""),"",IF(OR(B459="",C459="",E459=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E459)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H459&lt;&gt;0,F459=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G459&lt;&gt;0,F459=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F459&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F459)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C459)*($E$5:$E$504=E459)*(($D$5:$D$504=D459)*(D459&lt;&gt;"")+($B$5:$B$504=B459)*(B459&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C459="Оплата",K459&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E459)&gt;0,ROUND(E459-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B459="",C459="",D459="",E459="",F459=""),"",IF(OR(B459="",C459="",E459=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E459)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H459&lt;&gt;0,F459=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G459&lt;&gt;0,F459=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F459&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F459)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C459)*($E$5:$E$504=E459)*(($D$5:$D$504=D459)*(D459&lt;&gt;"")+($B$5:$B$504=B459)*(B459&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C459="Оплата",K459&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E459)&gt;0,ROUND(E459-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J459" s="5">
@@ -13000,7 +13000,7 @@
         <v/>
       </c>
       <c r="I460" s="6">
-        <f>IF(AND(B460="",C460="",D460="",E460="",F460=""),"",IF(OR(B460="",C460="",E460=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E460)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H460&lt;&gt;0,F460=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G460&lt;&gt;0,F460=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F460&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F460)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C460)*($E$5:$E$504=E460)*(($D$5:$D$504=D460)*(D460&lt;&gt;"")+($B$5:$B$504=B460)*(B460&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C460="Оплата",K460&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E460)&gt;0,ROUND(E460-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B460="",C460="",D460="",E460="",F460=""),"",IF(OR(B460="",C460="",E460=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E460)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H460&lt;&gt;0,F460=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G460&lt;&gt;0,F460=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F460&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F460)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C460)*($E$5:$E$504=E460)*(($D$5:$D$504=D460)*(D460&lt;&gt;"")+($B$5:$B$504=B460)*(B460&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C460="Оплата",K460&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E460)&gt;0,ROUND(E460-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J460" s="5">
@@ -13027,7 +13027,7 @@
         <v/>
       </c>
       <c r="I461" s="6">
-        <f>IF(AND(B461="",C461="",D461="",E461="",F461=""),"",IF(OR(B461="",C461="",E461=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E461)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H461&lt;&gt;0,F461=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G461&lt;&gt;0,F461=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F461&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F461)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C461)*($E$5:$E$504=E461)*(($D$5:$D$504=D461)*(D461&lt;&gt;"")+($B$5:$B$504=B461)*(B461&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C461="Оплата",K461&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E461)&gt;0,ROUND(E461-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B461="",C461="",D461="",E461="",F461=""),"",IF(OR(B461="",C461="",E461=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E461)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H461&lt;&gt;0,F461=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G461&lt;&gt;0,F461=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F461&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F461)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C461)*($E$5:$E$504=E461)*(($D$5:$D$504=D461)*(D461&lt;&gt;"")+($B$5:$B$504=B461)*(B461&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C461="Оплата",K461&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E461)&gt;0,ROUND(E461-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J461" s="5">
@@ -13054,7 +13054,7 @@
         <v/>
       </c>
       <c r="I462" s="6">
-        <f>IF(AND(B462="",C462="",D462="",E462="",F462=""),"",IF(OR(B462="",C462="",E462=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E462)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H462&lt;&gt;0,F462=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G462&lt;&gt;0,F462=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F462&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F462)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C462)*($E$5:$E$504=E462)*(($D$5:$D$504=D462)*(D462&lt;&gt;"")+($B$5:$B$504=B462)*(B462&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C462="Оплата",K462&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E462)&gt;0,ROUND(E462-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B462="",C462="",D462="",E462="",F462=""),"",IF(OR(B462="",C462="",E462=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E462)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H462&lt;&gt;0,F462=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G462&lt;&gt;0,F462=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F462&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F462)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C462)*($E$5:$E$504=E462)*(($D$5:$D$504=D462)*(D462&lt;&gt;"")+($B$5:$B$504=B462)*(B462&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C462="Оплата",K462&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E462)&gt;0,ROUND(E462-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J462" s="5">
@@ -13081,7 +13081,7 @@
         <v/>
       </c>
       <c r="I463" s="6">
-        <f>IF(AND(B463="",C463="",D463="",E463="",F463=""),"",IF(OR(B463="",C463="",E463=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E463)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H463&lt;&gt;0,F463=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G463&lt;&gt;0,F463=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F463&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F463)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C463)*($E$5:$E$504=E463)*(($D$5:$D$504=D463)*(D463&lt;&gt;"")+($B$5:$B$504=B463)*(B463&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C463="Оплата",K463&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E463)&gt;0,ROUND(E463-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B463="",C463="",D463="",E463="",F463=""),"",IF(OR(B463="",C463="",E463=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E463)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H463&lt;&gt;0,F463=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G463&lt;&gt;0,F463=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F463&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F463)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C463)*($E$5:$E$504=E463)*(($D$5:$D$504=D463)*(D463&lt;&gt;"")+($B$5:$B$504=B463)*(B463&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C463="Оплата",K463&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E463)&gt;0,ROUND(E463-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J463" s="5">
@@ -13108,7 +13108,7 @@
         <v/>
       </c>
       <c r="I464" s="6">
-        <f>IF(AND(B464="",C464="",D464="",E464="",F464=""),"",IF(OR(B464="",C464="",E464=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E464)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H464&lt;&gt;0,F464=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G464&lt;&gt;0,F464=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F464&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F464)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C464)*($E$5:$E$504=E464)*(($D$5:$D$504=D464)*(D464&lt;&gt;"")+($B$5:$B$504=B464)*(B464&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C464="Оплата",K464&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E464)&gt;0,ROUND(E464-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B464="",C464="",D464="",E464="",F464=""),"",IF(OR(B464="",C464="",E464=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E464)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H464&lt;&gt;0,F464=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G464&lt;&gt;0,F464=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F464&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F464)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C464)*($E$5:$E$504=E464)*(($D$5:$D$504=D464)*(D464&lt;&gt;"")+($B$5:$B$504=B464)*(B464&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C464="Оплата",K464&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E464)&gt;0,ROUND(E464-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J464" s="5">
@@ -13135,7 +13135,7 @@
         <v/>
       </c>
       <c r="I465" s="6">
-        <f>IF(AND(B465="",C465="",D465="",E465="",F465=""),"",IF(OR(B465="",C465="",E465=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E465)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H465&lt;&gt;0,F465=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G465&lt;&gt;0,F465=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F465&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F465)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C465)*($E$5:$E$504=E465)*(($D$5:$D$504=D465)*(D465&lt;&gt;"")+($B$5:$B$504=B465)*(B465&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C465="Оплата",K465&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E465)&gt;0,ROUND(E465-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B465="",C465="",D465="",E465="",F465=""),"",IF(OR(B465="",C465="",E465=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E465)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H465&lt;&gt;0,F465=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G465&lt;&gt;0,F465=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F465&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F465)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C465)*($E$5:$E$504=E465)*(($D$5:$D$504=D465)*(D465&lt;&gt;"")+($B$5:$B$504=B465)*(B465&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C465="Оплата",K465&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E465)&gt;0,ROUND(E465-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J465" s="5">
@@ -13162,7 +13162,7 @@
         <v/>
       </c>
       <c r="I466" s="6">
-        <f>IF(AND(B466="",C466="",D466="",E466="",F466=""),"",IF(OR(B466="",C466="",E466=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E466)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H466&lt;&gt;0,F466=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G466&lt;&gt;0,F466=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F466&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F466)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C466)*($E$5:$E$504=E466)*(($D$5:$D$504=D466)*(D466&lt;&gt;"")+($B$5:$B$504=B466)*(B466&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C466="Оплата",K466&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E466)&gt;0,ROUND(E466-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B466="",C466="",D466="",E466="",F466=""),"",IF(OR(B466="",C466="",E466=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E466)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H466&lt;&gt;0,F466=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G466&lt;&gt;0,F466=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F466&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F466)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C466)*($E$5:$E$504=E466)*(($D$5:$D$504=D466)*(D466&lt;&gt;"")+($B$5:$B$504=B466)*(B466&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C466="Оплата",K466&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E466)&gt;0,ROUND(E466-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J466" s="5">
@@ -13189,7 +13189,7 @@
         <v/>
       </c>
       <c r="I467" s="6">
-        <f>IF(AND(B467="",C467="",D467="",E467="",F467=""),"",IF(OR(B467="",C467="",E467=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E467)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H467&lt;&gt;0,F467=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G467&lt;&gt;0,F467=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F467&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F467)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C467)*($E$5:$E$504=E467)*(($D$5:$D$504=D467)*(D467&lt;&gt;"")+($B$5:$B$504=B467)*(B467&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C467="Оплата",K467&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E467)&gt;0,ROUND(E467-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B467="",C467="",D467="",E467="",F467=""),"",IF(OR(B467="",C467="",E467=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E467)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H467&lt;&gt;0,F467=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G467&lt;&gt;0,F467=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F467&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F467)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C467)*($E$5:$E$504=E467)*(($D$5:$D$504=D467)*(D467&lt;&gt;"")+($B$5:$B$504=B467)*(B467&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C467="Оплата",K467&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E467)&gt;0,ROUND(E467-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J467" s="5">
@@ -13216,7 +13216,7 @@
         <v/>
       </c>
       <c r="I468" s="6">
-        <f>IF(AND(B468="",C468="",D468="",E468="",F468=""),"",IF(OR(B468="",C468="",E468=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E468)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H468&lt;&gt;0,F468=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G468&lt;&gt;0,F468=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F468&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F468)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C468)*($E$5:$E$504=E468)*(($D$5:$D$504=D468)*(D468&lt;&gt;"")+($B$5:$B$504=B468)*(B468&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C468="Оплата",K468&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E468)&gt;0,ROUND(E468-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B468="",C468="",D468="",E468="",F468=""),"",IF(OR(B468="",C468="",E468=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E468)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H468&lt;&gt;0,F468=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G468&lt;&gt;0,F468=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F468&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F468)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C468)*($E$5:$E$504=E468)*(($D$5:$D$504=D468)*(D468&lt;&gt;"")+($B$5:$B$504=B468)*(B468&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C468="Оплата",K468&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E468)&gt;0,ROUND(E468-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J468" s="5">
@@ -13243,7 +13243,7 @@
         <v/>
       </c>
       <c r="I469" s="6">
-        <f>IF(AND(B469="",C469="",D469="",E469="",F469=""),"",IF(OR(B469="",C469="",E469=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E469)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H469&lt;&gt;0,F469=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G469&lt;&gt;0,F469=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F469&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F469)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C469)*($E$5:$E$504=E469)*(($D$5:$D$504=D469)*(D469&lt;&gt;"")+($B$5:$B$504=B469)*(B469&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C469="Оплата",K469&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E469)&gt;0,ROUND(E469-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B469="",C469="",D469="",E469="",F469=""),"",IF(OR(B469="",C469="",E469=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E469)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H469&lt;&gt;0,F469=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G469&lt;&gt;0,F469=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F469&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F469)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C469)*($E$5:$E$504=E469)*(($D$5:$D$504=D469)*(D469&lt;&gt;"")+($B$5:$B$504=B469)*(B469&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C469="Оплата",K469&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E469)&gt;0,ROUND(E469-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J469" s="5">
@@ -13270,7 +13270,7 @@
         <v/>
       </c>
       <c r="I470" s="6">
-        <f>IF(AND(B470="",C470="",D470="",E470="",F470=""),"",IF(OR(B470="",C470="",E470=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E470)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H470&lt;&gt;0,F470=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G470&lt;&gt;0,F470=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F470&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F470)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C470)*($E$5:$E$504=E470)*(($D$5:$D$504=D470)*(D470&lt;&gt;"")+($B$5:$B$504=B470)*(B470&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C470="Оплата",K470&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E470)&gt;0,ROUND(E470-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B470="",C470="",D470="",E470="",F470=""),"",IF(OR(B470="",C470="",E470=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E470)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H470&lt;&gt;0,F470=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G470&lt;&gt;0,F470=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F470&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F470)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C470)*($E$5:$E$504=E470)*(($D$5:$D$504=D470)*(D470&lt;&gt;"")+($B$5:$B$504=B470)*(B470&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C470="Оплата",K470&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E470)&gt;0,ROUND(E470-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J470" s="5">
@@ -13297,7 +13297,7 @@
         <v/>
       </c>
       <c r="I471" s="6">
-        <f>IF(AND(B471="",C471="",D471="",E471="",F471=""),"",IF(OR(B471="",C471="",E471=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E471)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H471&lt;&gt;0,F471=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G471&lt;&gt;0,F471=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F471&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F471)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C471)*($E$5:$E$504=E471)*(($D$5:$D$504=D471)*(D471&lt;&gt;"")+($B$5:$B$504=B471)*(B471&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C471="Оплата",K471&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E471)&gt;0,ROUND(E471-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B471="",C471="",D471="",E471="",F471=""),"",IF(OR(B471="",C471="",E471=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E471)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H471&lt;&gt;0,F471=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G471&lt;&gt;0,F471=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F471&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F471)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C471)*($E$5:$E$504=E471)*(($D$5:$D$504=D471)*(D471&lt;&gt;"")+($B$5:$B$504=B471)*(B471&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C471="Оплата",K471&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E471)&gt;0,ROUND(E471-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J471" s="5">
@@ -13324,7 +13324,7 @@
         <v/>
       </c>
       <c r="I472" s="6">
-        <f>IF(AND(B472="",C472="",D472="",E472="",F472=""),"",IF(OR(B472="",C472="",E472=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E472)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H472&lt;&gt;0,F472=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G472&lt;&gt;0,F472=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F472&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F472)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C472)*($E$5:$E$504=E472)*(($D$5:$D$504=D472)*(D472&lt;&gt;"")+($B$5:$B$504=B472)*(B472&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C472="Оплата",K472&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E472)&gt;0,ROUND(E472-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B472="",C472="",D472="",E472="",F472=""),"",IF(OR(B472="",C472="",E472=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E472)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H472&lt;&gt;0,F472=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G472&lt;&gt;0,F472=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F472&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F472)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C472)*($E$5:$E$504=E472)*(($D$5:$D$504=D472)*(D472&lt;&gt;"")+($B$5:$B$504=B472)*(B472&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C472="Оплата",K472&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E472)&gt;0,ROUND(E472-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J472" s="5">
@@ -13351,7 +13351,7 @@
         <v/>
       </c>
       <c r="I473" s="6">
-        <f>IF(AND(B473="",C473="",D473="",E473="",F473=""),"",IF(OR(B473="",C473="",E473=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E473)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H473&lt;&gt;0,F473=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G473&lt;&gt;0,F473=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F473&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F473)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C473)*($E$5:$E$504=E473)*(($D$5:$D$504=D473)*(D473&lt;&gt;"")+($B$5:$B$504=B473)*(B473&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C473="Оплата",K473&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E473)&gt;0,ROUND(E473-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B473="",C473="",D473="",E473="",F473=""),"",IF(OR(B473="",C473="",E473=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E473)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H473&lt;&gt;0,F473=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G473&lt;&gt;0,F473=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F473&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F473)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C473)*($E$5:$E$504=E473)*(($D$5:$D$504=D473)*(D473&lt;&gt;"")+($B$5:$B$504=B473)*(B473&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C473="Оплата",K473&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E473)&gt;0,ROUND(E473-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J473" s="5">
@@ -13378,7 +13378,7 @@
         <v/>
       </c>
       <c r="I474" s="6">
-        <f>IF(AND(B474="",C474="",D474="",E474="",F474=""),"",IF(OR(B474="",C474="",E474=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E474)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H474&lt;&gt;0,F474=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G474&lt;&gt;0,F474=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F474&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F474)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C474)*($E$5:$E$504=E474)*(($D$5:$D$504=D474)*(D474&lt;&gt;"")+($B$5:$B$504=B474)*(B474&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C474="Оплата",K474&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E474)&gt;0,ROUND(E474-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B474="",C474="",D474="",E474="",F474=""),"",IF(OR(B474="",C474="",E474=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E474)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H474&lt;&gt;0,F474=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G474&lt;&gt;0,F474=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F474&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F474)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C474)*($E$5:$E$504=E474)*(($D$5:$D$504=D474)*(D474&lt;&gt;"")+($B$5:$B$504=B474)*(B474&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C474="Оплата",K474&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E474)&gt;0,ROUND(E474-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J474" s="5">
@@ -13405,7 +13405,7 @@
         <v/>
       </c>
       <c r="I475" s="6">
-        <f>IF(AND(B475="",C475="",D475="",E475="",F475=""),"",IF(OR(B475="",C475="",E475=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E475)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H475&lt;&gt;0,F475=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G475&lt;&gt;0,F475=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F475&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F475)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C475)*($E$5:$E$504=E475)*(($D$5:$D$504=D475)*(D475&lt;&gt;"")+($B$5:$B$504=B475)*(B475&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C475="Оплата",K475&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E475)&gt;0,ROUND(E475-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B475="",C475="",D475="",E475="",F475=""),"",IF(OR(B475="",C475="",E475=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E475)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H475&lt;&gt;0,F475=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G475&lt;&gt;0,F475=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F475&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F475)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C475)*($E$5:$E$504=E475)*(($D$5:$D$504=D475)*(D475&lt;&gt;"")+($B$5:$B$504=B475)*(B475&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C475="Оплата",K475&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E475)&gt;0,ROUND(E475-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J475" s="5">
@@ -13432,7 +13432,7 @@
         <v/>
       </c>
       <c r="I476" s="6">
-        <f>IF(AND(B476="",C476="",D476="",E476="",F476=""),"",IF(OR(B476="",C476="",E476=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E476)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H476&lt;&gt;0,F476=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G476&lt;&gt;0,F476=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F476&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F476)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C476)*($E$5:$E$504=E476)*(($D$5:$D$504=D476)*(D476&lt;&gt;"")+($B$5:$B$504=B476)*(B476&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C476="Оплата",K476&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E476)&gt;0,ROUND(E476-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B476="",C476="",D476="",E476="",F476=""),"",IF(OR(B476="",C476="",E476=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E476)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H476&lt;&gt;0,F476=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G476&lt;&gt;0,F476=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F476&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F476)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C476)*($E$5:$E$504=E476)*(($D$5:$D$504=D476)*(D476&lt;&gt;"")+($B$5:$B$504=B476)*(B476&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C476="Оплата",K476&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E476)&gt;0,ROUND(E476-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J476" s="5">
@@ -13459,7 +13459,7 @@
         <v/>
       </c>
       <c r="I477" s="6">
-        <f>IF(AND(B477="",C477="",D477="",E477="",F477=""),"",IF(OR(B477="",C477="",E477=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E477)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H477&lt;&gt;0,F477=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G477&lt;&gt;0,F477=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F477&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F477)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C477)*($E$5:$E$504=E477)*(($D$5:$D$504=D477)*(D477&lt;&gt;"")+($B$5:$B$504=B477)*(B477&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C477="Оплата",K477&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E477)&gt;0,ROUND(E477-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B477="",C477="",D477="",E477="",F477=""),"",IF(OR(B477="",C477="",E477=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E477)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H477&lt;&gt;0,F477=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G477&lt;&gt;0,F477=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F477&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F477)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C477)*($E$5:$E$504=E477)*(($D$5:$D$504=D477)*(D477&lt;&gt;"")+($B$5:$B$504=B477)*(B477&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C477="Оплата",K477&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E477)&gt;0,ROUND(E477-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J477" s="5">
@@ -13486,7 +13486,7 @@
         <v/>
       </c>
       <c r="I478" s="6">
-        <f>IF(AND(B478="",C478="",D478="",E478="",F478=""),"",IF(OR(B478="",C478="",E478=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E478)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H478&lt;&gt;0,F478=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G478&lt;&gt;0,F478=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F478&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F478)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C478)*($E$5:$E$504=E478)*(($D$5:$D$504=D478)*(D478&lt;&gt;"")+($B$5:$B$504=B478)*(B478&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C478="Оплата",K478&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E478)&gt;0,ROUND(E478-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B478="",C478="",D478="",E478="",F478=""),"",IF(OR(B478="",C478="",E478=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E478)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H478&lt;&gt;0,F478=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G478&lt;&gt;0,F478=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F478&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F478)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C478)*($E$5:$E$504=E478)*(($D$5:$D$504=D478)*(D478&lt;&gt;"")+($B$5:$B$504=B478)*(B478&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C478="Оплата",K478&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E478)&gt;0,ROUND(E478-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J478" s="5">
@@ -13513,7 +13513,7 @@
         <v/>
       </c>
       <c r="I479" s="6">
-        <f>IF(AND(B479="",C479="",D479="",E479="",F479=""),"",IF(OR(B479="",C479="",E479=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E479)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H479&lt;&gt;0,F479=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G479&lt;&gt;0,F479=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F479&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F479)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C479)*($E$5:$E$504=E479)*(($D$5:$D$504=D479)*(D479&lt;&gt;"")+($B$5:$B$504=B479)*(B479&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C479="Оплата",K479&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E479)&gt;0,ROUND(E479-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B479="",C479="",D479="",E479="",F479=""),"",IF(OR(B479="",C479="",E479=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E479)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H479&lt;&gt;0,F479=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G479&lt;&gt;0,F479=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F479&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F479)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C479)*($E$5:$E$504=E479)*(($D$5:$D$504=D479)*(D479&lt;&gt;"")+($B$5:$B$504=B479)*(B479&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C479="Оплата",K479&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E479)&gt;0,ROUND(E479-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J479" s="5">
@@ -13540,7 +13540,7 @@
         <v/>
       </c>
       <c r="I480" s="6">
-        <f>IF(AND(B480="",C480="",D480="",E480="",F480=""),"",IF(OR(B480="",C480="",E480=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E480)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H480&lt;&gt;0,F480=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G480&lt;&gt;0,F480=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F480&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F480)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C480)*($E$5:$E$504=E480)*(($D$5:$D$504=D480)*(D480&lt;&gt;"")+($B$5:$B$504=B480)*(B480&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C480="Оплата",K480&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E480)&gt;0,ROUND(E480-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B480="",C480="",D480="",E480="",F480=""),"",IF(OR(B480="",C480="",E480=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E480)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H480&lt;&gt;0,F480=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G480&lt;&gt;0,F480=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F480&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F480)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C480)*($E$5:$E$504=E480)*(($D$5:$D$504=D480)*(D480&lt;&gt;"")+($B$5:$B$504=B480)*(B480&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C480="Оплата",K480&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E480)&gt;0,ROUND(E480-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J480" s="5">
@@ -13567,7 +13567,7 @@
         <v/>
       </c>
       <c r="I481" s="6">
-        <f>IF(AND(B481="",C481="",D481="",E481="",F481=""),"",IF(OR(B481="",C481="",E481=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E481)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H481&lt;&gt;0,F481=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G481&lt;&gt;0,F481=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F481&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F481)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C481)*($E$5:$E$504=E481)*(($D$5:$D$504=D481)*(D481&lt;&gt;"")+($B$5:$B$504=B481)*(B481&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C481="Оплата",K481&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E481)&gt;0,ROUND(E481-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B481="",C481="",D481="",E481="",F481=""),"",IF(OR(B481="",C481="",E481=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E481)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H481&lt;&gt;0,F481=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G481&lt;&gt;0,F481=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F481&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F481)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C481)*($E$5:$E$504=E481)*(($D$5:$D$504=D481)*(D481&lt;&gt;"")+($B$5:$B$504=B481)*(B481&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C481="Оплата",K481&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E481)&gt;0,ROUND(E481-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J481" s="5">
@@ -13594,7 +13594,7 @@
         <v/>
       </c>
       <c r="I482" s="6">
-        <f>IF(AND(B482="",C482="",D482="",E482="",F482=""),"",IF(OR(B482="",C482="",E482=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E482)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H482&lt;&gt;0,F482=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G482&lt;&gt;0,F482=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F482&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F482)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C482)*($E$5:$E$504=E482)*(($D$5:$D$504=D482)*(D482&lt;&gt;"")+($B$5:$B$504=B482)*(B482&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C482="Оплата",K482&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E482)&gt;0,ROUND(E482-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B482="",C482="",D482="",E482="",F482=""),"",IF(OR(B482="",C482="",E482=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E482)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H482&lt;&gt;0,F482=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G482&lt;&gt;0,F482=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F482&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F482)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C482)*($E$5:$E$504=E482)*(($D$5:$D$504=D482)*(D482&lt;&gt;"")+($B$5:$B$504=B482)*(B482&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C482="Оплата",K482&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E482)&gt;0,ROUND(E482-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J482" s="5">
@@ -13621,7 +13621,7 @@
         <v/>
       </c>
       <c r="I483" s="6">
-        <f>IF(AND(B483="",C483="",D483="",E483="",F483=""),"",IF(OR(B483="",C483="",E483=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E483)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H483&lt;&gt;0,F483=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G483&lt;&gt;0,F483=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F483&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F483)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C483)*($E$5:$E$504=E483)*(($D$5:$D$504=D483)*(D483&lt;&gt;"")+($B$5:$B$504=B483)*(B483&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C483="Оплата",K483&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E483)&gt;0,ROUND(E483-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B483="",C483="",D483="",E483="",F483=""),"",IF(OR(B483="",C483="",E483=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E483)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H483&lt;&gt;0,F483=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G483&lt;&gt;0,F483=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F483&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F483)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C483)*($E$5:$E$504=E483)*(($D$5:$D$504=D483)*(D483&lt;&gt;"")+($B$5:$B$504=B483)*(B483&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C483="Оплата",K483&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E483)&gt;0,ROUND(E483-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J483" s="5">
@@ -13648,7 +13648,7 @@
         <v/>
       </c>
       <c r="I484" s="6">
-        <f>IF(AND(B484="",C484="",D484="",E484="",F484=""),"",IF(OR(B484="",C484="",E484=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E484)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H484&lt;&gt;0,F484=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G484&lt;&gt;0,F484=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F484&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F484)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C484)*($E$5:$E$504=E484)*(($D$5:$D$504=D484)*(D484&lt;&gt;"")+($B$5:$B$504=B484)*(B484&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C484="Оплата",K484&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E484)&gt;0,ROUND(E484-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B484="",C484="",D484="",E484="",F484=""),"",IF(OR(B484="",C484="",E484=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E484)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H484&lt;&gt;0,F484=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G484&lt;&gt;0,F484=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F484&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F484)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C484)*($E$5:$E$504=E484)*(($D$5:$D$504=D484)*(D484&lt;&gt;"")+($B$5:$B$504=B484)*(B484&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C484="Оплата",K484&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E484)&gt;0,ROUND(E484-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J484" s="5">
@@ -13675,7 +13675,7 @@
         <v/>
       </c>
       <c r="I485" s="6">
-        <f>IF(AND(B485="",C485="",D485="",E485="",F485=""),"",IF(OR(B485="",C485="",E485=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E485)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H485&lt;&gt;0,F485=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G485&lt;&gt;0,F485=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F485&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F485)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C485)*($E$5:$E$504=E485)*(($D$5:$D$504=D485)*(D485&lt;&gt;"")+($B$5:$B$504=B485)*(B485&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C485="Оплата",K485&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E485)&gt;0,ROUND(E485-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B485="",C485="",D485="",E485="",F485=""),"",IF(OR(B485="",C485="",E485=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E485)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H485&lt;&gt;0,F485=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G485&lt;&gt;0,F485=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F485&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F485)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C485)*($E$5:$E$504=E485)*(($D$5:$D$504=D485)*(D485&lt;&gt;"")+($B$5:$B$504=B485)*(B485&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C485="Оплата",K485&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E485)&gt;0,ROUND(E485-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J485" s="5">
@@ -13702,7 +13702,7 @@
         <v/>
       </c>
       <c r="I486" s="6">
-        <f>IF(AND(B486="",C486="",D486="",E486="",F486=""),"",IF(OR(B486="",C486="",E486=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E486)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H486&lt;&gt;0,F486=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G486&lt;&gt;0,F486=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F486&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F486)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C486)*($E$5:$E$504=E486)*(($D$5:$D$504=D486)*(D486&lt;&gt;"")+($B$5:$B$504=B486)*(B486&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C486="Оплата",K486&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E486)&gt;0,ROUND(E486-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B486="",C486="",D486="",E486="",F486=""),"",IF(OR(B486="",C486="",E486=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E486)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H486&lt;&gt;0,F486=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G486&lt;&gt;0,F486=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F486&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F486)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C486)*($E$5:$E$504=E486)*(($D$5:$D$504=D486)*(D486&lt;&gt;"")+($B$5:$B$504=B486)*(B486&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C486="Оплата",K486&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E486)&gt;0,ROUND(E486-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J486" s="5">
@@ -13729,7 +13729,7 @@
         <v/>
       </c>
       <c r="I487" s="6">
-        <f>IF(AND(B487="",C487="",D487="",E487="",F487=""),"",IF(OR(B487="",C487="",E487=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E487)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H487&lt;&gt;0,F487=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G487&lt;&gt;0,F487=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F487&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F487)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C487)*($E$5:$E$504=E487)*(($D$5:$D$504=D487)*(D487&lt;&gt;"")+($B$5:$B$504=B487)*(B487&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C487="Оплата",K487&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E487)&gt;0,ROUND(E487-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B487="",C487="",D487="",E487="",F487=""),"",IF(OR(B487="",C487="",E487=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E487)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H487&lt;&gt;0,F487=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G487&lt;&gt;0,F487=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F487&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F487)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C487)*($E$5:$E$504=E487)*(($D$5:$D$504=D487)*(D487&lt;&gt;"")+($B$5:$B$504=B487)*(B487&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C487="Оплата",K487&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E487)&gt;0,ROUND(E487-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J487" s="5">
@@ -13756,7 +13756,7 @@
         <v/>
       </c>
       <c r="I488" s="6">
-        <f>IF(AND(B488="",C488="",D488="",E488="",F488=""),"",IF(OR(B488="",C488="",E488=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E488)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H488&lt;&gt;0,F488=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G488&lt;&gt;0,F488=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F488&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F488)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C488)*($E$5:$E$504=E488)*(($D$5:$D$504=D488)*(D488&lt;&gt;"")+($B$5:$B$504=B488)*(B488&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C488="Оплата",K488&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E488)&gt;0,ROUND(E488-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B488="",C488="",D488="",E488="",F488=""),"",IF(OR(B488="",C488="",E488=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E488)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H488&lt;&gt;0,F488=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G488&lt;&gt;0,F488=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F488&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F488)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C488)*($E$5:$E$504=E488)*(($D$5:$D$504=D488)*(D488&lt;&gt;"")+($B$5:$B$504=B488)*(B488&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C488="Оплата",K488&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E488)&gt;0,ROUND(E488-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J488" s="5">
@@ -13783,7 +13783,7 @@
         <v/>
       </c>
       <c r="I489" s="6">
-        <f>IF(AND(B489="",C489="",D489="",E489="",F489=""),"",IF(OR(B489="",C489="",E489=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E489)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H489&lt;&gt;0,F489=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G489&lt;&gt;0,F489=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F489&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F489)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C489)*($E$5:$E$504=E489)*(($D$5:$D$504=D489)*(D489&lt;&gt;"")+($B$5:$B$504=B489)*(B489&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C489="Оплата",K489&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E489)&gt;0,ROUND(E489-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B489="",C489="",D489="",E489="",F489=""),"",IF(OR(B489="",C489="",E489=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E489)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H489&lt;&gt;0,F489=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G489&lt;&gt;0,F489=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F489&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F489)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C489)*($E$5:$E$504=E489)*(($D$5:$D$504=D489)*(D489&lt;&gt;"")+($B$5:$B$504=B489)*(B489&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C489="Оплата",K489&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E489)&gt;0,ROUND(E489-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J489" s="5">
@@ -13810,7 +13810,7 @@
         <v/>
       </c>
       <c r="I490" s="6">
-        <f>IF(AND(B490="",C490="",D490="",E490="",F490=""),"",IF(OR(B490="",C490="",E490=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E490)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H490&lt;&gt;0,F490=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G490&lt;&gt;0,F490=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F490&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F490)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C490)*($E$5:$E$504=E490)*(($D$5:$D$504=D490)*(D490&lt;&gt;"")+($B$5:$B$504=B490)*(B490&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C490="Оплата",K490&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E490)&gt;0,ROUND(E490-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B490="",C490="",D490="",E490="",F490=""),"",IF(OR(B490="",C490="",E490=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E490)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H490&lt;&gt;0,F490=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G490&lt;&gt;0,F490=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F490&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F490)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C490)*($E$5:$E$504=E490)*(($D$5:$D$504=D490)*(D490&lt;&gt;"")+($B$5:$B$504=B490)*(B490&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C490="Оплата",K490&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E490)&gt;0,ROUND(E490-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J490" s="5">
@@ -13837,7 +13837,7 @@
         <v/>
       </c>
       <c r="I491" s="6">
-        <f>IF(AND(B491="",C491="",D491="",E491="",F491=""),"",IF(OR(B491="",C491="",E491=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E491)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H491&lt;&gt;0,F491=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G491&lt;&gt;0,F491=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F491&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F491)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C491)*($E$5:$E$504=E491)*(($D$5:$D$504=D491)*(D491&lt;&gt;"")+($B$5:$B$504=B491)*(B491&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C491="Оплата",K491&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E491)&gt;0,ROUND(E491-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B491="",C491="",D491="",E491="",F491=""),"",IF(OR(B491="",C491="",E491=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E491)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H491&lt;&gt;0,F491=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G491&lt;&gt;0,F491=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F491&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F491)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C491)*($E$5:$E$504=E491)*(($D$5:$D$504=D491)*(D491&lt;&gt;"")+($B$5:$B$504=B491)*(B491&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C491="Оплата",K491&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E491)&gt;0,ROUND(E491-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J491" s="5">
@@ -13864,7 +13864,7 @@
         <v/>
       </c>
       <c r="I492" s="6">
-        <f>IF(AND(B492="",C492="",D492="",E492="",F492=""),"",IF(OR(B492="",C492="",E492=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E492)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H492&lt;&gt;0,F492=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G492&lt;&gt;0,F492=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F492&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F492)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C492)*($E$5:$E$504=E492)*(($D$5:$D$504=D492)*(D492&lt;&gt;"")+($B$5:$B$504=B492)*(B492&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C492="Оплата",K492&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E492)&gt;0,ROUND(E492-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B492="",C492="",D492="",E492="",F492=""),"",IF(OR(B492="",C492="",E492=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E492)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H492&lt;&gt;0,F492=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G492&lt;&gt;0,F492=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F492&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F492)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C492)*($E$5:$E$504=E492)*(($D$5:$D$504=D492)*(D492&lt;&gt;"")+($B$5:$B$504=B492)*(B492&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C492="Оплата",K492&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E492)&gt;0,ROUND(E492-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J492" s="5">
@@ -13891,7 +13891,7 @@
         <v/>
       </c>
       <c r="I493" s="6">
-        <f>IF(AND(B493="",C493="",D493="",E493="",F493=""),"",IF(OR(B493="",C493="",E493=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E493)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H493&lt;&gt;0,F493=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G493&lt;&gt;0,F493=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F493&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F493)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C493)*($E$5:$E$504=E493)*(($D$5:$D$504=D493)*(D493&lt;&gt;"")+($B$5:$B$504=B493)*(B493&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C493="Оплата",K493&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E493)&gt;0,ROUND(E493-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B493="",C493="",D493="",E493="",F493=""),"",IF(OR(B493="",C493="",E493=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E493)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H493&lt;&gt;0,F493=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G493&lt;&gt;0,F493=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F493&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F493)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C493)*($E$5:$E$504=E493)*(($D$5:$D$504=D493)*(D493&lt;&gt;"")+($B$5:$B$504=B493)*(B493&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C493="Оплата",K493&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E493)&gt;0,ROUND(E493-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J493" s="5">
@@ -13918,7 +13918,7 @@
         <v/>
       </c>
       <c r="I494" s="6">
-        <f>IF(AND(B494="",C494="",D494="",E494="",F494=""),"",IF(OR(B494="",C494="",E494=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E494)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H494&lt;&gt;0,F494=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G494&lt;&gt;0,F494=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F494&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F494)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C494)*($E$5:$E$504=E494)*(($D$5:$D$504=D494)*(D494&lt;&gt;"")+($B$5:$B$504=B494)*(B494&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C494="Оплата",K494&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E494)&gt;0,ROUND(E494-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B494="",C494="",D494="",E494="",F494=""),"",IF(OR(B494="",C494="",E494=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E494)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H494&lt;&gt;0,F494=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G494&lt;&gt;0,F494=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F494&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F494)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C494)*($E$5:$E$504=E494)*(($D$5:$D$504=D494)*(D494&lt;&gt;"")+($B$5:$B$504=B494)*(B494&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C494="Оплата",K494&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E494)&gt;0,ROUND(E494-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J494" s="5">
@@ -13945,7 +13945,7 @@
         <v/>
       </c>
       <c r="I495" s="6">
-        <f>IF(AND(B495="",C495="",D495="",E495="",F495=""),"",IF(OR(B495="",C495="",E495=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E495)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H495&lt;&gt;0,F495=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G495&lt;&gt;0,F495=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F495&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F495)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C495)*($E$5:$E$504=E495)*(($D$5:$D$504=D495)*(D495&lt;&gt;"")+($B$5:$B$504=B495)*(B495&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C495="Оплата",K495&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E495)&gt;0,ROUND(E495-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B495="",C495="",D495="",E495="",F495=""),"",IF(OR(B495="",C495="",E495=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E495)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H495&lt;&gt;0,F495=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G495&lt;&gt;0,F495=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F495&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F495)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C495)*($E$5:$E$504=E495)*(($D$5:$D$504=D495)*(D495&lt;&gt;"")+($B$5:$B$504=B495)*(B495&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C495="Оплата",K495&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E495)&gt;0,ROUND(E495-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J495" s="5">
@@ -13972,7 +13972,7 @@
         <v/>
       </c>
       <c r="I496" s="6">
-        <f>IF(AND(B496="",C496="",D496="",E496="",F496=""),"",IF(OR(B496="",C496="",E496=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E496)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H496&lt;&gt;0,F496=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G496&lt;&gt;0,F496=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F496&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F496)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C496)*($E$5:$E$504=E496)*(($D$5:$D$504=D496)*(D496&lt;&gt;"")+($B$5:$B$504=B496)*(B496&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C496="Оплата",K496&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E496)&gt;0,ROUND(E496-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B496="",C496="",D496="",E496="",F496=""),"",IF(OR(B496="",C496="",E496=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E496)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H496&lt;&gt;0,F496=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G496&lt;&gt;0,F496=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F496&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F496)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C496)*($E$5:$E$504=E496)*(($D$5:$D$504=D496)*(D496&lt;&gt;"")+($B$5:$B$504=B496)*(B496&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C496="Оплата",K496&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E496)&gt;0,ROUND(E496-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J496" s="5">
@@ -13999,7 +13999,7 @@
         <v/>
       </c>
       <c r="I497" s="6">
-        <f>IF(AND(B497="",C497="",D497="",E497="",F497=""),"",IF(OR(B497="",C497="",E497=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E497)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H497&lt;&gt;0,F497=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G497&lt;&gt;0,F497=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F497&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F497)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C497)*($E$5:$E$504=E497)*(($D$5:$D$504=D497)*(D497&lt;&gt;"")+($B$5:$B$504=B497)*(B497&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C497="Оплата",K497&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E497)&gt;0,ROUND(E497-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B497="",C497="",D497="",E497="",F497=""),"",IF(OR(B497="",C497="",E497=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E497)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H497&lt;&gt;0,F497=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G497&lt;&gt;0,F497=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F497&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F497)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C497)*($E$5:$E$504=E497)*(($D$5:$D$504=D497)*(D497&lt;&gt;"")+($B$5:$B$504=B497)*(B497&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C497="Оплата",K497&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E497)&gt;0,ROUND(E497-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J497" s="5">
@@ -14026,7 +14026,7 @@
         <v/>
       </c>
       <c r="I498" s="6">
-        <f>IF(AND(B498="",C498="",D498="",E498="",F498=""),"",IF(OR(B498="",C498="",E498=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E498)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H498&lt;&gt;0,F498=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G498&lt;&gt;0,F498=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F498&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F498)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C498)*($E$5:$E$504=E498)*(($D$5:$D$504=D498)*(D498&lt;&gt;"")+($B$5:$B$504=B498)*(B498&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C498="Оплата",K498&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E498)&gt;0,ROUND(E498-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B498="",C498="",D498="",E498="",F498=""),"",IF(OR(B498="",C498="",E498=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E498)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H498&lt;&gt;0,F498=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G498&lt;&gt;0,F498=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F498&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F498)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C498)*($E$5:$E$504=E498)*(($D$5:$D$504=D498)*(D498&lt;&gt;"")+($B$5:$B$504=B498)*(B498&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C498="Оплата",K498&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E498)&gt;0,ROUND(E498-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J498" s="5">
@@ -14053,7 +14053,7 @@
         <v/>
       </c>
       <c r="I499" s="6">
-        <f>IF(AND(B499="",C499="",D499="",E499="",F499=""),"",IF(OR(B499="",C499="",E499=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E499)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H499&lt;&gt;0,F499=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G499&lt;&gt;0,F499=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F499&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F499)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C499)*($E$5:$E$504=E499)*(($D$5:$D$504=D499)*(D499&lt;&gt;"")+($B$5:$B$504=B499)*(B499&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C499="Оплата",K499&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E499)&gt;0,ROUND(E499-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B499="",C499="",D499="",E499="",F499=""),"",IF(OR(B499="",C499="",E499=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E499)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H499&lt;&gt;0,F499=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G499&lt;&gt;0,F499=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F499&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F499)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C499)*($E$5:$E$504=E499)*(($D$5:$D$504=D499)*(D499&lt;&gt;"")+($B$5:$B$504=B499)*(B499&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C499="Оплата",K499&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E499)&gt;0,ROUND(E499-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J499" s="5">
@@ -14080,7 +14080,7 @@
         <v/>
       </c>
       <c r="I500" s="6">
-        <f>IF(AND(B500="",C500="",D500="",E500="",F500=""),"",IF(OR(B500="",C500="",E500=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E500)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H500&lt;&gt;0,F500=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G500&lt;&gt;0,F500=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F500&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F500)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C500)*($E$5:$E$504=E500)*(($D$5:$D$504=D500)*(D500&lt;&gt;"")+($B$5:$B$504=B500)*(B500&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C500="Оплата",K500&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E500)&gt;0,ROUND(E500-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B500="",C500="",D500="",E500="",F500=""),"",IF(OR(B500="",C500="",E500=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E500)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H500&lt;&gt;0,F500=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G500&lt;&gt;0,F500=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F500&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F500)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C500)*($E$5:$E$504=E500)*(($D$5:$D$504=D500)*(D500&lt;&gt;"")+($B$5:$B$504=B500)*(B500&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C500="Оплата",K500&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E500)&gt;0,ROUND(E500-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J500" s="5">
@@ -14107,7 +14107,7 @@
         <v/>
       </c>
       <c r="I501" s="6">
-        <f>IF(AND(B501="",C501="",D501="",E501="",F501=""),"",IF(OR(B501="",C501="",E501=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E501)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H501&lt;&gt;0,F501=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G501&lt;&gt;0,F501=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F501&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F501)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C501)*($E$5:$E$504=E501)*(($D$5:$D$504=D501)*(D501&lt;&gt;"")+($B$5:$B$504=B501)*(B501&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C501="Оплата",K501&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E501)&gt;0,ROUND(E501-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B501="",C501="",D501="",E501="",F501=""),"",IF(OR(B501="",C501="",E501=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E501)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H501&lt;&gt;0,F501=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G501&lt;&gt;0,F501=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F501&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F501)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C501)*($E$5:$E$504=E501)*(($D$5:$D$504=D501)*(D501&lt;&gt;"")+($B$5:$B$504=B501)*(B501&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C501="Оплата",K501&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E501)&gt;0,ROUND(E501-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J501" s="5">
@@ -14134,7 +14134,7 @@
         <v/>
       </c>
       <c r="I502" s="6">
-        <f>IF(AND(B502="",C502="",D502="",E502="",F502=""),"",IF(OR(B502="",C502="",E502=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E502)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H502&lt;&gt;0,F502=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G502&lt;&gt;0,F502=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F502&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F502)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C502)*($E$5:$E$504=E502)*(($D$5:$D$504=D502)*(D502&lt;&gt;"")+($B$5:$B$504=B502)*(B502&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C502="Оплата",K502&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E502)&gt;0,ROUND(E502-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B502="",C502="",D502="",E502="",F502=""),"",IF(OR(B502="",C502="",E502=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E502)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H502&lt;&gt;0,F502=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G502&lt;&gt;0,F502=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F502&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F502)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C502)*($E$5:$E$504=E502)*(($D$5:$D$504=D502)*(D502&lt;&gt;"")+($B$5:$B$504=B502)*(B502&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C502="Оплата",K502&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E502)&gt;0,ROUND(E502-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J502" s="5">
@@ -14161,7 +14161,7 @@
         <v/>
       </c>
       <c r="I503" s="6">
-        <f>IF(AND(B503="",C503="",D503="",E503="",F503=""),"",IF(OR(B503="",C503="",E503=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E503)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H503&lt;&gt;0,F503=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G503&lt;&gt;0,F503=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F503&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F503)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C503)*($E$5:$E$504=E503)*(($D$5:$D$504=D503)*(D503&lt;&gt;"")+($B$5:$B$504=B503)*(B503&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C503="Оплата",K503&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E503)&gt;0,ROUND(E503-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B503="",C503="",D503="",E503="",F503=""),"",IF(OR(B503="",C503="",E503=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E503)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H503&lt;&gt;0,F503=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G503&lt;&gt;0,F503=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F503&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F503)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C503)*($E$5:$E$504=E503)*(($D$5:$D$504=D503)*(D503&lt;&gt;"")+($B$5:$B$504=B503)*(B503&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C503="Оплата",K503&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E503)&gt;0,ROUND(E503-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J503" s="5">
@@ -14188,7 +14188,7 @@
         <v/>
       </c>
       <c r="I504" s="6">
-        <f>IF(AND(B504="",C504="",D504="",E504="",F504=""),"",IF(OR(B504="",C504="",E504=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E504)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H504&lt;&gt;0,F504=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G504&lt;&gt;0,F504=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F504&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F504)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C504)*($E$5:$E$504=E504)*(($D$5:$D$504=D504)*(D504&lt;&gt;"")+($B$5:$B$504=B504)*(B504&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C504="Оплата",K504&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E504)&gt;0,ROUND(E504-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
+        <f>IF(AND(B504="",C504="",D504="",E504="",F504=""),"",IF(OR(B504="",C504="",E504=""),"БЛОК: нужны дата, тип операции и сумма",IF(N(E504)&lt;=0,"БЛОК: сумма должна быть больше нуля",IF(AND(H504&lt;&gt;0,F504=""),"БЛОК: у спорной операции не указан акт — укажите акт, к которому относится удержание, зачёт, неустойка или допработы: без этого бесспорную часть по акту не отделить",IF(AND(G504&lt;&gt;0,F504=""),"БЛОК: не указан акт — платёж не отнесён к конкретному акту. Распределите его документально (назначение платежа, соглашение, письмо) и укажите акт: без этого долг на первый день просрочки и проценты посчитать нельзя",IF(AND(F504&lt;&gt;"",COUNTIF('Долг по актам'!$B$5:$B$34,F504)=0),"БЛОК: такого акта нет на листе «Долг по актам» — добавьте акт или исправьте идентификатор",IF(SUMPRODUCT((($C$5:$C$504="Оплата")+($C$5:$C$504="Зачёт аванса по договору")&gt;0)*($C$5:$C$504&lt;&gt;C504)*($E$5:$E$504=E504)*(($D$5:$D$504=D504)*(D504&lt;&gt;"")+($B$5:$B$504=B504)*(B504&lt;&gt;"")&gt;0))&gt;0,"БЛОК: двойной учёт аванса — эта сумма введена и как «Оплата», и как «Зачёт аванса по договору» с тем же документом или той же датой. Аванс, зачтённый в акт, учитывается один раз: оставьте одну операцию",IF(AND(C504="Оплата",K504&lt;&gt;"Отдельный платёж — не сам аванс (сверено с выпиской банка)",OR(COUNTIFS($C$5:$C$504,"Зачёт аванса по договору",$E$5:$E$504,E504)&gt;0,ROUND(E504-$M$6,2)=0)),"БЛОК: нужна сверка с авансом — сумма этой оплаты равна зачёту аванса. Если это сам авансовый платёж, удалите строку: аванс учитывается один раз, зачётом. "&amp;"Если это отдельный платёж, сверьте его с выпиской банка и выберите в колонке K «Отдельный платёж — не сам аванс (сверено с выпиской банка)»","ок"))))))))</f>
         <v/>
       </c>
       <c r="J504" s="5">

</xml_diff>